<commit_message>
added some info on fair sharing and the website itself
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W60"/>
+  <dimension ref="A1:W78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4282,6 +4282,672 @@
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Ecuadorian Dataset on Access, Demand, &amp; Availability of Electricity Supply</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>ESPOL University</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence for Energy Access (AI4EA)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Reiner Lemoine Institut gGmbH (RLI)</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Benin,Ghana,Niger,Togo</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Residential Energy and Weather Dataset (REWD) of Pakistan</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Lahore University of Management Sciences (LUMS)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Datasets for transportation impact evaluation</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Fundación Despacio,World Resources Institute,Fundación Despacio</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Machine learning training data for continental Ecuador and Galapagos</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Fundacion Ecociencia</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr"/>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Forest carbon sequestration in the Congo Basin</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>World Resources Institute</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Cameroon,DRC</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>GEO Indigenous Alliance</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>GEO Indigenous Alliance</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Ecuador,Kenya</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr"/>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Ivorian mangroves and carbon stock</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>data354</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Reference Data Collection for Improving Land Use Change Mapping in Ghana</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Center for Remote Sensing and Geographic Information Services</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Remote sensing and weather dataset for improved reforestation monitoring</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Dedan Kimathi University of Technology,Data Science Africa</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>DATASETS FOR PREDICTION OF LAND USE/COVER CHANGES IN UGANDA</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Makerere University</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>African Trees for Climate Resilience: A Comprehensive Database</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>University of Stellenbosch</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Angola,DRC,Germany,Kenya,Mozambique,Nigeria,South Africa,Tanzania,United Kingdom,Zambia</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Datasets to understand mangroves health in relationship to climate change</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>"Laboratory of Biomathematics and Forest Estimations, University of Abomey-Calavi"</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Benin</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="inlineStr"/>
+      <c r="W73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Advancing oil palm mapping with social forestry and machine learning</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>RECOFTC</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr"/>
+      <c r="W74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Inclusive MRV for India's Eastern Himalayas</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Balipara Foundation</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="inlineStr"/>
+      <c r="W75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Data-enabled climate shock absorbance through agroforestry (Agrof4resilience)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>International Center of Insect Physiology and Ecology (ICIPE)</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="inlineStr"/>
+      <c r="W76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>QUANTIFYING COLOMBIAN MANGROVES ABOVEGROUND BIOMASS AND CARBON CONTENT</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Centre Tecnològic de Telecomunicacions de Catalunya (CTTC)</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Columbia</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Phenological Dataset for Ecological Forecasting (PheDEF Project)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>"Department of Biological Science, School of Science, University of Energy and Natural Resources, Sunyani, Ghana"</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Ghana,Netherlands</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added multiple dataset link capabilities
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -5605,7 +5605,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Parallel Text for machine translation in Eng-Kin; domain-specific for Education (digital literacy)</t>
+          <t>Parallel Text for machine translation in Eng-Kin; Domain-specific for Education (digital literacy)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -5615,12 +5615,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset  / https://huggingface.co/datasets/mbazaNLP/Kinyarwanda_English_parallel_dataset / https://huggingface.co/datasets/mbazaNLP/NMT_Education_parallel_data_en_kin / https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset </t>
+          <t xml:space="preserve">https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset;  https://huggingface.co/datasets/mbazaNLP/Kinyarwanda_English_parallel_dataset; https://huggingface.co/datasets/mbazaNLP/NMT_Education_parallel_data_en_kin; https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset </t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://huggingface.co/mbazaNLP/Quantized_Nllb_Finetuned_Edu_En_Kin_8bit / https://huggingface.co/mbazaNLP/Nllb_finetuned_general_en_kin / https://huggingface.co/DigitalUmuganda/Finetuned-NLLB </t>
+          <t xml:space="preserve">https://huggingface.co/mbazaNLP/Quantized_Nllb_Finetuned_Edu_En_Kin_8bit; https://huggingface.co/mbazaNLP/Nllb_finetuned_general_en_kin; https://huggingface.co/DigitalUmuganda/Finetuned-NLLB </t>
         </is>
       </c>
       <c r="H80" t="inlineStr">

</xml_diff>

<commit_message>
added resources and expanded search
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -2852,7 +2852,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/iLab-DSU/imarika-weather-pipeline;
+          <t xml:space="preserve">https://github.com/iLab-DSU/imarika-weather-pipeline
 https://github.com/iLab-DSU/Agricultural-Recommendations-Chat
 </t>
         </is>
@@ -2947,13 +2947,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI-generated Voice Content in Indian Languages on Health, Sustainable Agriculture and Education
-</t>
+          <t>Empowering Women across India with audio messages in their native languages on Health, Sustainable Agriculture and Education</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Empowering Women Across India with Voice-based Knowledge in Their Native Languages</t>
+          <t>Empowering Women across India with audio messages in their native languages on Health, Sustainable Agriculture and Education</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3331,12 +3330,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI Pest Management: Open Data for Pink Bollworms and American Bollworms</t>
+          <t>Open source AI Pest Control for smallholder Cotton Farmers in India</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Cotton Ace: AI-driven Pest Management for Cotton Farmers in India</t>
+          <t>Open source AI Pest Control for smallholder Cotton Farmers in India</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3464,7 +3463,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Providing better information on sexual and reproductive health and rights of young people through the Kahi Ankahi Baatein infloline (Hindi LLM finetuning)</t>
+          <t>Providing better information on sexual and reproductive health and rights of young people through the Kahi Ankahi Baatein infoline (Hindi LLM finetuning)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4182,12 +4181,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Open Soil Data for local AI Innovation in Telangana</t>
+          <t>Open Soil Data to impove soil health and support climate-resilient, regenerative agriculture practices in Telangana - GeoAI for Soil Conservation</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Measuring Soil Health for more Sustainable Agriculture in Telangana and beyond</t>
+          <t>Improving soil health and supporting climate-resilient, regenerative agriculture practices in Telangana - GeoAI for Soil Conservation</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4576,12 +4575,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Climate Disinformation in Local Indonesian Languages</t>
+          <t>Combatting Climate Disinformation in Indonesian languages with AI</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Climate Disinformation in Local Indonesian Languages</t>
+          <t>Combatting Climate Disinformation in Indonesian languages with AI</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4699,12 +4698,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Forest Forward: AI-Powered "High Carbon Stock Approach" Mapping for Forest Protection and Fight the Climate Crisis in Indonesia</t>
+          <t>High Carbon Stock Approach: Mapping Forests to Combat Climate Change and Protect Livelihoods in Indonesia</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Forest Forward: AI-Powered "High Carbon Stock Approach" Mapping for Forest Protection and Fight the Climate Crisis in Indonesia</t>
+          <t>High Carbon Stock Approach: Mapping Forests to Combat Climate Change and Protect Livelihoods in Indonesia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>

<commit_message>
revised readme with GitHub Actions instructions for non-technical users, synced sheet data
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -755,7 +755,9 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Laboratoire de Biomathématiques et d'Estimations Forestières</t>
+          <t>Powered by: Laboratoire de Biomathématiques et d'Estimations Forestières
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp;  FAIR Forward - AI for All
+Financed by: BMZ</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1941,7 +1943,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2634,8 +2636,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3650,7 +3652,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3661,7 +3663,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3736,7 +3738,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3772,8 +3774,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4127,22 +4128,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4443,7 +4444,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -4969,8 +4970,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -5527,7 +5528,7 @@
       <c r="P45" t="inlineStr">
         <is>
           <t>Powered by:  THiNK - Tech Innovators Network
-Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
+Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5754,10 +5755,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6231,7 +6232,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -6389,7 +6390,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -6961,7 +6962,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -7304,8 +7305,8 @@
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -8747,7 +8748,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9003,7 +9004,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -9270,8 +9271,8 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10016,11 +10017,7 @@
           <t>Enhancing business registration in Kenya through a chatbot</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>The business registration process in Kenya is perceived as complex by entrepreneurs, often hindered by technical language in official documentation. An AI-powered chatbot was developed to help to enhance access to information, simplifying the registration journey, and improving user experience. A  a prototype was built, that demonstrated how the chatbot could contribute to the SDGs by improving access to vital information and services</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
@@ -10065,27 +10062,98 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ui_86</t>
+        </is>
+      </c>
       <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>KinyCOMET: Automatic evaluation of machine translation for Kinyarwanda-English</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>KinyCOMET: Automatic evaluation of machine translation for Kinyarwanda-English</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Until now, the lack of automatic evaluation tools made Kinyarwanda-English machine translation development slow and expensive, as it required manual human review. We’ve bridged this gap by creating a new evaluation dataset and model. Both are now open-source to support the research community. Our methodology and results are detailed in our upcoming paper for LREC 2026.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/datasets/chrismazii/kinycomet_dataset</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/chrismazii/kinycomet_unbabel</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>SDG 9</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://c4ir.rw/</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>4000 rows of parallel sentences English - Kinyarwanda with annotated translation quality as Direct Assessment</t>
+        </is>
+      </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Apache 2.0</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Powered by: Mbaza NLP community, German Research Center for Artificial Intelligence (DFKI), Regional AI Hub Rwanda
+Catalyzed by: FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Jan Nehring</t>
+        </is>
+      </c>
       <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
-      <c r="T88" t="inlineStr"/>
-      <c r="U88" t="inlineStr"/>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model &gt; Pilot</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>
+</t>
+        </is>
+      </c>
       <c r="V88" t="inlineStr"/>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr"/>
@@ -10094,26 +10162,107 @@
       <c r="AA88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ui_87</t>
+        </is>
+      </c>
       <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Tunga Agri-Chatbot Suite</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Tunga Agri-Chatbot Suite</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voicebots acting as call center agents—accessible via telephone and capable of speaking local languages—hold immense potential for development cooperation. They provide a vital link to users in rural areas who may lack internet access, have limited literacy, do not speak English or do not own digital devices. We believe voice-driven interfaces are the most intuitive way to bridge the digital divide for these communities.
+As part of the Tunga project, we have developed such a voicebot. To support further innovation in this space, we are releasing a comprehensive suite of foundational AI models and datasets:
+Text-to-speech model
+Currently the highest-quality synthetic voice for Kinyarwanda.
+https://huggingface.co/C4IR-RW/kinya-flex-tts
+KinyaCOLBERT Free
+The first Kinyarwanda embedding/information retrieval model, essential for building RAG chatbots such as Tunga.
+https://huggingface.co/C4IR-RW/kiny-colbert-free
+Voice Dataset
+A dataset for training TTS and Speech-to-Text (STT) models.
+https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts
+Information Retrieval Dataset
+The data used to train the KinyaColBERT model.
+https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval
+KinyaBERT
+A foundational BERT-style model serving as the backbone for various Kinyarwanda NLP tasks.
+https://huggingface.co/C4IR-RW/kinyabert 
+Source Code
+All relevant code for the models and datasets mentioned above.
+https://github.com/c4ir-rw/ac-ai-models </t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts;https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval </t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/C4IR-RW/kinya-flex-tts;https://huggingface.co/C4IR-RW/kiny-colbert-free;https://huggingface.co/C4IR-RW/kinyabert;https://github.com/c4ir-rw/ac-ai-models</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>SDG 2, SDG 1</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Text, Voice</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://c4ir.rw/</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Apache 2.0</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Powered by: C4IR, KiNLP
+Catalyzed by: FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Jan Nehring</t>
+        </is>
+      </c>
       <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
-      <c r="T89" t="inlineStr"/>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model &gt; Pilot</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
       <c r="U89" t="inlineStr"/>
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>

</xml_diff>

<commit_message>
Manually triggered update from Google Sheets - 2026-03-25 13:29:47 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,137 +417,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>

</xml_diff>

<commit_message>
data and image update
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,137 +429,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
@@ -3922,7 +3934,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Powered by:  WRMS for Data Collection (https://wrmsglobal.com/), ZINDI for the data challenge (https://zindi.africa/) and Vertify for Model Development (https://vertify.earth/)
+          <t>Powered by:  WRMS - Weather Risk Management Services for Data Collection (https://wrmsglobal.com/), ZINDI for the data challenge (https://zindi.africa/) and Vertify for Model Development (https://vertify.earth/)
 Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -4279,27 +4291,30 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hack4TTS: Crafting Voice for India’s Low-Resource Languages - Building TTS Systems for Low-Resource Indian Languages with Accent and Style Transfer</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Hack4TTS: Crafting Voice for India’s Low-Resource Languages - Building TTS Systems for Low-Resource Indian Languages with Accent and Style Transfer</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Combined from two formerly planned service contracts (1) Making the IISc datasets more sustainable, usable, support AIEP, make use-cases possible + (2) Hackathon for IISc voice datasets with Bhashini on climate &amp; sustainable agriculture</t>
+          <t>This hackathon challenged teams to build an AI system that can turn written text into natural-sounding speech across multiple Indian languages, including less-represented ones. Participants created voices that can reflect different accents and speaking styles, making the technology more personal and inclusive. Using open data, they made voice technology more accessible for diverse communities. The solutions will be integrated into a voice assistant designed to support pregnant women in low-income communities.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>philipp.olbrich@giz.de is this still running and something will be delivered?  And is this a pilot, or more?</t>
+          <t>https://spiredatasets.ee.iisc.ac.in/syspincorpus; https://spiredatasets.ee.iisc.ac.in/englishttscorpus; https://spiredatasets.ee.iisc.ac.in/gujaratittscorpus</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Philipp</t>
+          <t>https://huggingface.co/somyalab/Spark_somya_TTS
+; https://huggingface.co/roymukund/Voice-Tech-CDAC-Submission/tree/main
+; https://huggingface.co/vinaybabu/voice-tech-for-all-v2
+; https://huggingface.co/immverse-ai/voice-tech-for-all-challenge-v2</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4312,24 +4327,62 @@
           <t>Voice, Text</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in), Dr. Philipp Olbrich (philipp.olbrich@giz.de)</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>"The Data is fully open-sourced and can be accessed at:
+ • IISc website: &lt;https://spiredatasets.ee.iisc.ac.in/syspincorpus&gt;
+ TTS Dataset:
+ • License: CC-BY 4.0
+ • Data Type: Audio recording
+ • Sentence creation: Variety of domains covered in the sentences/text and phonetically rich sentence selection
+ • Accounts for dialect variability
+ • Voice artist selection and balanced duration per voice artist 
+ • Voice recording: 40 hours of recording by 1 male voice artist and 1 female voice artist for each of the 9 languages
+ • Studio-quality audio with 48kHz, 24 bits per sample from every voice artist
+ • Data was collected and created over 3 years from 2021-2024"</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>The winning models can be accessed on their respective repositories here: 
+Somya: https://huggingface.co/somyalab/Spark_somya_TTS
+CDAC_SVNIT: https://huggingface.co/roymukund/Voice-Tech-CDAC-Submission/tree/main
+LTRC-SPL: https://huggingface.co/vinaybabu/voice-tech-for-all-v2
+immverse_ai: https://huggingface.co/immverse-ai/voice-tech-for-all-challenge-v2</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>The TTS models can be used to develop innovative solutions and voice-based services for Indians in their native language. This would be especially beneficial for those who cannot read/write or have speech and visual disabilities but can access digital services through audio/voice-based mediums. The data and models are a crucial stepping stone for developing such assistive technologies. Including low-resource languages, some of which do not even have enough print/digital literature, would benefit vulnerable communities for whom language barriers make access to technological solutions even more difficult. Given the distribution of speakers. some of the languages are especially useful for programmes wishing to engage with rural communities and promote sustainable agriculture in rural settings.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>CC-BY</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Powered by:  
+          <t>Powered by: Indian Institute of Science (IISc) and Artpark
 Catalyzed by: FAIR Forward - AI for All
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Philipp Olbrich</t>
+        </is>
+      </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Manually triggered update from Google Sheets - 2026-03-26 09:06:38 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,137 +417,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>

</xml_diff>

<commit_message>
feat: migrate project URLs from title-based to stable ui_X identifiers
Project share links were derived from titles, meaning any title change
in the Google Sheet would break previously shared URLs. The protected
Project ID column (ui_0 through ui_87) now serves as the canonical
identifier for URLs and directories.

- resolve_project_id() unconditionally prefers Project ID column
- Directories renamed from title-based names to ui_X on first build
- catalog.json includes slug (ui_X-title) and alias map for old URLs
- Frontend resolves old title-based URLs via alias lookup and silently
  rewrites them to the new stable slug format
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,141 +425,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA92"/>
+  <dimension ref="A1:AA154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
@@ -730,7 +742,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -1931,7 +1943,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2247,7 +2259,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>"Powered by: RAIL - KNUST (https://rail.knust.edu.gh/)
+          <t>Powered by: RAIL - KNUST (https://rail.knust.edu.gh/)
  Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
  Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)"</t>
         </is>
@@ -2624,8 +2636,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3640,7 +3652,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3651,7 +3663,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3726,7 +3738,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3762,7 +3774,8 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
+ </t>
         </is>
       </c>
@@ -4116,22 +4129,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4473,7 +4486,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -4999,8 +5012,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -5557,7 +5570,7 @@
       <c r="P45" t="inlineStr">
         <is>
           <t>Powered by:  THiNK - Tech Innovators Network
-Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
+Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5784,10 +5797,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6261,7 +6274,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -6419,7 +6432,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -6991,7 +7004,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -7334,8 +7347,8 @@
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure. </t>
         </is>
       </c>
@@ -8777,7 +8790,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9033,7 +9046,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -9300,8 +9313,8 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10179,7 +10192,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>
+          <t xml:space="preserve">
 </t>
         </is>
       </c>
@@ -10301,7 +10314,11 @@
       <c r="AA89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ui_88</t>
+        </is>
+      </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
@@ -10330,7 +10347,11 @@
       <c r="AA90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ui_89</t>
+        </is>
+      </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr"/>
@@ -10359,7 +10380,11 @@
       <c r="AA91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ui_90</t>
+        </is>
+      </c>
       <c r="B92" t="inlineStr">
         <is>
           <t>Two Al-based dialogue systems (e.g. voice-based chatbot) in Indian Languages - consultancy for design implementation etc</t>
@@ -10449,6 +10474,2052 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ui_91</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr"/>
+      <c r="U93" t="inlineStr"/>
+      <c r="V93" t="inlineStr"/>
+      <c r="W93" t="inlineStr"/>
+      <c r="X93" t="inlineStr"/>
+      <c r="Y93" t="inlineStr"/>
+      <c r="Z93" t="inlineStr"/>
+      <c r="AA93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ui_92</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
+      <c r="U94" t="inlineStr"/>
+      <c r="V94" t="inlineStr"/>
+      <c r="W94" t="inlineStr"/>
+      <c r="X94" t="inlineStr"/>
+      <c r="Y94" t="inlineStr"/>
+      <c r="Z94" t="inlineStr"/>
+      <c r="AA94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ui_93</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr"/>
+      <c r="U95" t="inlineStr"/>
+      <c r="V95" t="inlineStr"/>
+      <c r="W95" t="inlineStr"/>
+      <c r="X95" t="inlineStr"/>
+      <c r="Y95" t="inlineStr"/>
+      <c r="Z95" t="inlineStr"/>
+      <c r="AA95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ui_94</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr"/>
+      <c r="U96" t="inlineStr"/>
+      <c r="V96" t="inlineStr"/>
+      <c r="W96" t="inlineStr"/>
+      <c r="X96" t="inlineStr"/>
+      <c r="Y96" t="inlineStr"/>
+      <c r="Z96" t="inlineStr"/>
+      <c r="AA96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ui_95</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
+      <c r="P97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr"/>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr"/>
+      <c r="T97" t="inlineStr"/>
+      <c r="U97" t="inlineStr"/>
+      <c r="V97" t="inlineStr"/>
+      <c r="W97" t="inlineStr"/>
+      <c r="X97" t="inlineStr"/>
+      <c r="Y97" t="inlineStr"/>
+      <c r="Z97" t="inlineStr"/>
+      <c r="AA97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ui_96</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
+      <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr"/>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr"/>
+      <c r="U98" t="inlineStr"/>
+      <c r="V98" t="inlineStr"/>
+      <c r="W98" t="inlineStr"/>
+      <c r="X98" t="inlineStr"/>
+      <c r="Y98" t="inlineStr"/>
+      <c r="Z98" t="inlineStr"/>
+      <c r="AA98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ui_97</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
+      <c r="P99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr"/>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr"/>
+      <c r="U99" t="inlineStr"/>
+      <c r="V99" t="inlineStr"/>
+      <c r="W99" t="inlineStr"/>
+      <c r="X99" t="inlineStr"/>
+      <c r="Y99" t="inlineStr"/>
+      <c r="Z99" t="inlineStr"/>
+      <c r="AA99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ui_98</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
+      <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr"/>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr"/>
+      <c r="T100" t="inlineStr"/>
+      <c r="U100" t="inlineStr"/>
+      <c r="V100" t="inlineStr"/>
+      <c r="W100" t="inlineStr"/>
+      <c r="X100" t="inlineStr"/>
+      <c r="Y100" t="inlineStr"/>
+      <c r="Z100" t="inlineStr"/>
+      <c r="AA100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ui_99</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
+      <c r="P101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr"/>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr"/>
+      <c r="T101" t="inlineStr"/>
+      <c r="U101" t="inlineStr"/>
+      <c r="V101" t="inlineStr"/>
+      <c r="W101" t="inlineStr"/>
+      <c r="X101" t="inlineStr"/>
+      <c r="Y101" t="inlineStr"/>
+      <c r="Z101" t="inlineStr"/>
+      <c r="AA101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ui_100</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
+      <c r="P102" t="inlineStr"/>
+      <c r="Q102" t="inlineStr"/>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr"/>
+      <c r="T102" t="inlineStr"/>
+      <c r="U102" t="inlineStr"/>
+      <c r="V102" t="inlineStr"/>
+      <c r="W102" t="inlineStr"/>
+      <c r="X102" t="inlineStr"/>
+      <c r="Y102" t="inlineStr"/>
+      <c r="Z102" t="inlineStr"/>
+      <c r="AA102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ui_101</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr"/>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr"/>
+      <c r="T103" t="inlineStr"/>
+      <c r="U103" t="inlineStr"/>
+      <c r="V103" t="inlineStr"/>
+      <c r="W103" t="inlineStr"/>
+      <c r="X103" t="inlineStr"/>
+      <c r="Y103" t="inlineStr"/>
+      <c r="Z103" t="inlineStr"/>
+      <c r="AA103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>ui_102</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
+      <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+      <c r="T104" t="inlineStr"/>
+      <c r="U104" t="inlineStr"/>
+      <c r="V104" t="inlineStr"/>
+      <c r="W104" t="inlineStr"/>
+      <c r="X104" t="inlineStr"/>
+      <c r="Y104" t="inlineStr"/>
+      <c r="Z104" t="inlineStr"/>
+      <c r="AA104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ui_103</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr"/>
+      <c r="U105" t="inlineStr"/>
+      <c r="V105" t="inlineStr"/>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr"/>
+      <c r="Y105" t="inlineStr"/>
+      <c r="Z105" t="inlineStr"/>
+      <c r="AA105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>ui_104</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr"/>
+      <c r="T106" t="inlineStr"/>
+      <c r="U106" t="inlineStr"/>
+      <c r="V106" t="inlineStr"/>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr"/>
+      <c r="Y106" t="inlineStr"/>
+      <c r="Z106" t="inlineStr"/>
+      <c r="AA106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>ui_105</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr"/>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
+      <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr"/>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr"/>
+      <c r="T107" t="inlineStr"/>
+      <c r="U107" t="inlineStr"/>
+      <c r="V107" t="inlineStr"/>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr"/>
+      <c r="Y107" t="inlineStr"/>
+      <c r="Z107" t="inlineStr"/>
+      <c r="AA107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ui_106</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr"/>
+      <c r="T108" t="inlineStr"/>
+      <c r="U108" t="inlineStr"/>
+      <c r="V108" t="inlineStr"/>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr"/>
+      <c r="Y108" t="inlineStr"/>
+      <c r="Z108" t="inlineStr"/>
+      <c r="AA108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ui_107</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr"/>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
+      <c r="P109" t="inlineStr"/>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr"/>
+      <c r="U109" t="inlineStr"/>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr"/>
+      <c r="Y109" t="inlineStr"/>
+      <c r="Z109" t="inlineStr"/>
+      <c r="AA109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ui_108</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
+      <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr"/>
+      <c r="T110" t="inlineStr"/>
+      <c r="U110" t="inlineStr"/>
+      <c r="V110" t="inlineStr"/>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr"/>
+      <c r="Y110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr"/>
+      <c r="AA110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ui_109</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr"/>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr"/>
+      <c r="P111" t="inlineStr"/>
+      <c r="Q111" t="inlineStr"/>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr"/>
+      <c r="U111" t="inlineStr"/>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr"/>
+      <c r="Y111" t="inlineStr"/>
+      <c r="Z111" t="inlineStr"/>
+      <c r="AA111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ui_110</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="inlineStr"/>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr"/>
+      <c r="T112" t="inlineStr"/>
+      <c r="U112" t="inlineStr"/>
+      <c r="V112" t="inlineStr"/>
+      <c r="W112" t="inlineStr"/>
+      <c r="X112" t="inlineStr"/>
+      <c r="Y112" t="inlineStr"/>
+      <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ui_111</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
+      <c r="P113" t="inlineStr"/>
+      <c r="Q113" t="inlineStr"/>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr"/>
+      <c r="U113" t="inlineStr"/>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr"/>
+      <c r="Y113" t="inlineStr"/>
+      <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ui_112</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
+      <c r="P114" t="inlineStr"/>
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+      <c r="T114" t="inlineStr"/>
+      <c r="U114" t="inlineStr"/>
+      <c r="V114" t="inlineStr"/>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr"/>
+      <c r="Y114" t="inlineStr"/>
+      <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ui_113</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
+      <c r="P115" t="inlineStr"/>
+      <c r="Q115" t="inlineStr"/>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr"/>
+      <c r="T115" t="inlineStr"/>
+      <c r="U115" t="inlineStr"/>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr"/>
+      <c r="Y115" t="inlineStr"/>
+      <c r="Z115" t="inlineStr"/>
+      <c r="AA115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ui_114</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr"/>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
+      <c r="P116" t="inlineStr"/>
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr"/>
+      <c r="U116" t="inlineStr"/>
+      <c r="V116" t="inlineStr"/>
+      <c r="W116" t="inlineStr"/>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ui_115</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr"/>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
+      <c r="P117" t="inlineStr"/>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr"/>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ui_116</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
+      <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr"/>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ui_117</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
+      <c r="P119" t="inlineStr"/>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr"/>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>ui_118</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
+      <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr"/>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
+      <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ui_119</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr"/>
+      <c r="U121" t="inlineStr"/>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr"/>
+      <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ui_120</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
+      <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr"/>
+      <c r="T122" t="inlineStr"/>
+      <c r="U122" t="inlineStr"/>
+      <c r="V122" t="inlineStr"/>
+      <c r="W122" t="inlineStr"/>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ui_121</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr"/>
+      <c r="T123" t="inlineStr"/>
+      <c r="U123" t="inlineStr"/>
+      <c r="V123" t="inlineStr"/>
+      <c r="W123" t="inlineStr"/>
+      <c r="X123" t="inlineStr"/>
+      <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ui_122</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr"/>
+      <c r="U124" t="inlineStr"/>
+      <c r="V124" t="inlineStr"/>
+      <c r="W124" t="inlineStr"/>
+      <c r="X124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ui_123</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr"/>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr"/>
+      <c r="T125" t="inlineStr"/>
+      <c r="U125" t="inlineStr"/>
+      <c r="V125" t="inlineStr"/>
+      <c r="W125" t="inlineStr"/>
+      <c r="X125" t="inlineStr"/>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ui_124</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr"/>
+      <c r="T126" t="inlineStr"/>
+      <c r="U126" t="inlineStr"/>
+      <c r="V126" t="inlineStr"/>
+      <c r="W126" t="inlineStr"/>
+      <c r="X126" t="inlineStr"/>
+      <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>ui_125</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr"/>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr"/>
+      <c r="T127" t="inlineStr"/>
+      <c r="U127" t="inlineStr"/>
+      <c r="V127" t="inlineStr"/>
+      <c r="W127" t="inlineStr"/>
+      <c r="X127" t="inlineStr"/>
+      <c r="Y127" t="inlineStr"/>
+      <c r="Z127" t="inlineStr"/>
+      <c r="AA127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ui_126</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
+      <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr"/>
+      <c r="T128" t="inlineStr"/>
+      <c r="U128" t="inlineStr"/>
+      <c r="V128" t="inlineStr"/>
+      <c r="W128" t="inlineStr"/>
+      <c r="X128" t="inlineStr"/>
+      <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+      <c r="AA128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ui_127</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
+      <c r="P129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+      <c r="T129" t="inlineStr"/>
+      <c r="U129" t="inlineStr"/>
+      <c r="V129" t="inlineStr"/>
+      <c r="W129" t="inlineStr"/>
+      <c r="X129" t="inlineStr"/>
+      <c r="Y129" t="inlineStr"/>
+      <c r="Z129" t="inlineStr"/>
+      <c r="AA129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ui_128</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr"/>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
+      <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+      <c r="T130" t="inlineStr"/>
+      <c r="U130" t="inlineStr"/>
+      <c r="V130" t="inlineStr"/>
+      <c r="W130" t="inlineStr"/>
+      <c r="X130" t="inlineStr"/>
+      <c r="Y130" t="inlineStr"/>
+      <c r="Z130" t="inlineStr"/>
+      <c r="AA130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ui_129</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="inlineStr"/>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
+      <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+      <c r="T131" t="inlineStr"/>
+      <c r="U131" t="inlineStr"/>
+      <c r="V131" t="inlineStr"/>
+      <c r="W131" t="inlineStr"/>
+      <c r="X131" t="inlineStr"/>
+      <c r="Y131" t="inlineStr"/>
+      <c r="Z131" t="inlineStr"/>
+      <c r="AA131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ui_130</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+      <c r="T132" t="inlineStr"/>
+      <c r="U132" t="inlineStr"/>
+      <c r="V132" t="inlineStr"/>
+      <c r="W132" t="inlineStr"/>
+      <c r="X132" t="inlineStr"/>
+      <c r="Y132" t="inlineStr"/>
+      <c r="Z132" t="inlineStr"/>
+      <c r="AA132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ui_131</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
+      <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr"/>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+      <c r="T133" t="inlineStr"/>
+      <c r="U133" t="inlineStr"/>
+      <c r="V133" t="inlineStr"/>
+      <c r="W133" t="inlineStr"/>
+      <c r="X133" t="inlineStr"/>
+      <c r="Y133" t="inlineStr"/>
+      <c r="Z133" t="inlineStr"/>
+      <c r="AA133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ui_132</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
+      <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+      <c r="T134" t="inlineStr"/>
+      <c r="U134" t="inlineStr"/>
+      <c r="V134" t="inlineStr"/>
+      <c r="W134" t="inlineStr"/>
+      <c r="X134" t="inlineStr"/>
+      <c r="Y134" t="inlineStr"/>
+      <c r="Z134" t="inlineStr"/>
+      <c r="AA134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ui_133</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
+      <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+      <c r="T135" t="inlineStr"/>
+      <c r="U135" t="inlineStr"/>
+      <c r="V135" t="inlineStr"/>
+      <c r="W135" t="inlineStr"/>
+      <c r="X135" t="inlineStr"/>
+      <c r="Y135" t="inlineStr"/>
+      <c r="Z135" t="inlineStr"/>
+      <c r="AA135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ui_134</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr"/>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
+      <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+      <c r="T136" t="inlineStr"/>
+      <c r="U136" t="inlineStr"/>
+      <c r="V136" t="inlineStr"/>
+      <c r="W136" t="inlineStr"/>
+      <c r="X136" t="inlineStr"/>
+      <c r="Y136" t="inlineStr"/>
+      <c r="Z136" t="inlineStr"/>
+      <c r="AA136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>ui_135</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
+      <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
+      <c r="T137" t="inlineStr"/>
+      <c r="U137" t="inlineStr"/>
+      <c r="V137" t="inlineStr"/>
+      <c r="W137" t="inlineStr"/>
+      <c r="X137" t="inlineStr"/>
+      <c r="Y137" t="inlineStr"/>
+      <c r="Z137" t="inlineStr"/>
+      <c r="AA137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>ui_136</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr"/>
+      <c r="T138" t="inlineStr"/>
+      <c r="U138" t="inlineStr"/>
+      <c r="V138" t="inlineStr"/>
+      <c r="W138" t="inlineStr"/>
+      <c r="X138" t="inlineStr"/>
+      <c r="Y138" t="inlineStr"/>
+      <c r="Z138" t="inlineStr"/>
+      <c r="AA138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>ui_137</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr"/>
+      <c r="T139" t="inlineStr"/>
+      <c r="U139" t="inlineStr"/>
+      <c r="V139" t="inlineStr"/>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr"/>
+      <c r="Y139" t="inlineStr"/>
+      <c r="Z139" t="inlineStr"/>
+      <c r="AA139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>ui_138</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
+      <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr"/>
+      <c r="T140" t="inlineStr"/>
+      <c r="U140" t="inlineStr"/>
+      <c r="V140" t="inlineStr"/>
+      <c r="W140" t="inlineStr"/>
+      <c r="X140" t="inlineStr"/>
+      <c r="Y140" t="inlineStr"/>
+      <c r="Z140" t="inlineStr"/>
+      <c r="AA140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>ui_139</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr"/>
+      <c r="T141" t="inlineStr"/>
+      <c r="U141" t="inlineStr"/>
+      <c r="V141" t="inlineStr"/>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr"/>
+      <c r="Z141" t="inlineStr"/>
+      <c r="AA141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ui_140</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr"/>
+      <c r="T142" t="inlineStr"/>
+      <c r="U142" t="inlineStr"/>
+      <c r="V142" t="inlineStr"/>
+      <c r="W142" t="inlineStr"/>
+      <c r="X142" t="inlineStr"/>
+      <c r="Y142" t="inlineStr"/>
+      <c r="Z142" t="inlineStr"/>
+      <c r="AA142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ui_141</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr"/>
+      <c r="T143" t="inlineStr"/>
+      <c r="U143" t="inlineStr"/>
+      <c r="V143" t="inlineStr"/>
+      <c r="W143" t="inlineStr"/>
+      <c r="X143" t="inlineStr"/>
+      <c r="Y143" t="inlineStr"/>
+      <c r="Z143" t="inlineStr"/>
+      <c r="AA143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ui_142</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr"/>
+      <c r="T144" t="inlineStr"/>
+      <c r="U144" t="inlineStr"/>
+      <c r="V144" t="inlineStr"/>
+      <c r="W144" t="inlineStr"/>
+      <c r="X144" t="inlineStr"/>
+      <c r="Y144" t="inlineStr"/>
+      <c r="Z144" t="inlineStr"/>
+      <c r="AA144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ui_143</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+      <c r="T145" t="inlineStr"/>
+      <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr"/>
+      <c r="W145" t="inlineStr"/>
+      <c r="X145" t="inlineStr"/>
+      <c r="Y145" t="inlineStr"/>
+      <c r="Z145" t="inlineStr"/>
+      <c r="AA145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>ui_144</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr"/>
+      <c r="T146" t="inlineStr"/>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr"/>
+      <c r="W146" t="inlineStr"/>
+      <c r="X146" t="inlineStr"/>
+      <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>ui_145</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr"/>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>ui_146</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr"/>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr"/>
+      <c r="T148" t="inlineStr"/>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr"/>
+      <c r="W148" t="inlineStr"/>
+      <c r="X148" t="inlineStr"/>
+      <c r="Y148" t="inlineStr"/>
+      <c r="Z148" t="inlineStr"/>
+      <c r="AA148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>ui_147</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
+      <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr"/>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
+      <c r="AA149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>ui_148</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr"/>
+      <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr"/>
+      <c r="W150" t="inlineStr"/>
+      <c r="X150" t="inlineStr"/>
+      <c r="Y150" t="inlineStr"/>
+      <c r="Z150" t="inlineStr"/>
+      <c r="AA150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>ui_149</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr"/>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
+      <c r="P151" t="inlineStr"/>
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr"/>
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr"/>
+      <c r="V151" t="inlineStr"/>
+      <c r="W151" t="inlineStr"/>
+      <c r="X151" t="inlineStr"/>
+      <c r="Y151" t="inlineStr"/>
+      <c r="Z151" t="inlineStr"/>
+      <c r="AA151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>ui_150</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr"/>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr"/>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
+      <c r="P152" t="inlineStr"/>
+      <c r="Q152" t="inlineStr"/>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr"/>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="inlineStr"/>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr"/>
+      <c r="Y152" t="inlineStr"/>
+      <c r="Z152" t="inlineStr"/>
+      <c r="AA152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>ui_151</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
+      <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr"/>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr"/>
+      <c r="Y153" t="inlineStr"/>
+      <c r="Z153" t="inlineStr"/>
+      <c r="AA153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>ui_152</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr"/>
+      <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
+      <c r="P154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr"/>
+      <c r="V154" t="inlineStr"/>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr"/>
+      <c r="Y154" t="inlineStr"/>
+      <c r="Z154" t="inlineStr"/>
+      <c r="AA154" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: improve data quality -- license casing, text formatting, link labels, org cleanup
- Fix license display: remove .toLowerCase() in licenseLabel() so
  "Apache 2.0", "CC-BY 4.0" render with correct casing; expand
  LICENSE_NORMALIZATION map; add validation for unknown license values
- Add remark-gfm to ReactMarkdown so bare URLs in descriptions and
  other text fields render as clickable links
- Improve link button labels: use link.name when available, add domain
  hints (HuggingFace, GitHub, Zenodo), rename generic "Access Use Case"
  to "Access Resource"; refresh button styling
- Rename header stat "Use Cases" to "Pilots/Use Cases"
- Add linkifyOrgText() to convert inline URLs in organization entries
  to proper markdown links; update parseOrganizations() to handle
  "Powered by / Provided by" label
- Rebuild docs/ for GitHub Pages
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -952,7 +952,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
@@ -1943,7 +1947,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2636,8 +2640,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -2773,18 +2777,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset creatd: Dhuluo</t>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dhuluo</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>Mozilla Foundation seeks to select and support a community (group of language speakers who would like to collectively create or enhance a text and audio dataset for their  language), to experiment with a governance structure for this dataset that suits their particular needs. 
-This project will enable language communities to leverage governance tools (such as licenses) that center their needs and context, and have them be more accessible and widely used. Over the period of the project, the goal is to have a particular language community, or small group of them, piloting a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted</t>
+This project will enable language communities to leverage governance tools (such as licenses) that center their needs and context, and have them be more accessible and widely used. Over the period of the project, the goal is to have a particular language community, or small group of them, piloting a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted
+- language dataset created: Dhuluo ?</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Balthas</t>
+          <t>Balthas to clarify with Daniel, if dataset was created !!!</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3652,7 +3657,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3663,7 +3668,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3738,7 +3743,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3774,8 +3779,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4005,7 +4009,12 @@
 See technical report for an overview and learnings from this activity.</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>This project has been concluded as an internal review of MFINS workflows. There has been technical integration and scoping of AI based solutions for improved costumer  satisfaction and productivity but no novel dataset has been created and/or model trained.
+See technical report for an overview and learnings from this activity.</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>SDG 10</t>
@@ -4129,22 +4138,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4216,14 +4225,10 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Jonas</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Jonas</t>
-        </is>
-      </c>
+          <t>https://github.com/NaLamKI/geo-ai</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>SDG 2</t>
@@ -4325,7 +4330,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Voice, Text</t>
+          <t>Voice</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4486,7 +4491,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -4709,7 +4714,11 @@
           <t>https://huggingface.co/datasets/HCSA/HCSA_Indonesia_Forest_Plot_Data_2023</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://highcarbonstock.org/mapping-portal/</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>SDG 13, SDG 15</t>
@@ -4841,10 +4850,14 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://huggingface.co/datasets/prosa-text/nusa-dialogue</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>https://huggingface.co/datasets/prosa-text/nusa-dialogue; https://huggingface.co/datasets/prosa-text/nusa-translation</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/prosa-text/indobert-nusa</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>SDG 2, SDG 10</t>
@@ -4959,7 +4972,11 @@
           <t>https://github.com/insaninfonesia/WeatherData</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Model: https://colabs.commonroom.info/login/?next=%2F with username: guest_viewer and the password: guest_viewer</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>SDG 13, SDG 14</t>
@@ -5007,13 +5024,21 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.giz.de/en/newsroom/stories/ai-climate-resilience-meets-local-know-how </t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.giz.de/en/newsroom/stories/ai-climate-resilience-meets-local-know-how </t>
+        </is>
+      </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -5173,12 +5198,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Florence/Daniel</t>
+          <t>https://drive.google.com/drive/u/0/folders/19ZMqreP_lWXE13gbTGcdgYFlNSXXB9AN</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Florence/Daniel</t>
+          <t>https://www.vuli.ai/</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -5570,7 +5595,7 @@
       <c r="P45" t="inlineStr">
         <is>
           <t>Powered by:  THiNK - Tech Innovators Network
-Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
+Catalyzed by: FAIR Forward - AI for All &amp; and Digital Transformation Center Kenya
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5797,10 +5822,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -5934,7 +5959,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
+          <t>Dataset</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
@@ -5978,7 +6003,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>LivHealth Kiswahili Corpus aims to empower local communities to correctly identify livestock syndromes and get timely interventions from qualified livestock practitioners. Using Natural Language Processing (NLP), Machine Learning (ML), and Artificial Intelligence (AI), the project will build Kiswahili text-to-speech models for disseminating disease information to marginalized communities. Working closely with their partner, One Health Center in Africa (OHRECA) based at ILRI, they will enhance the functionality of the LivHealth system to enable local communities easy access to disease information on demand and in Kiswahili. This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
+          <t>LivHealth Kiswahili Corpus aims to empower local communities to correctly identify livestock syndromes and get timely interventions from qualified livestock practitioners. Using Natural Language Processing (NLP), Machine Learning (ML), and Artificial Intelligence (AI), the project has built Kiswahili text-to-speech models for disseminating disease information to marginalized communities. Working closely with their partner, One Health Center in Africa (OHRECA) based at ILRI, they have enhanced the functionality of the LivHealth system to enable local communities easy access to disease information on demand and in Kiswahili. This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5986,7 +6011,11 @@
           <t>https://livhealth-kc.badili.co.ke/</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://livhealth-kc.badili.co.ke/</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>SDG 10, SDG 2</t>
@@ -6257,10 +6286,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Developing products that can be replicated through four initiatives: 1. DynAG: 
- Focused on rice, wheat, and maize, DynAG's platform uses a RAG pipeline powered by LLMs like the GPT suite to provide farmers with advisory services. Accessible via chatbots, Android and Jio-based mobile apps, IVR, and SMS, it ensures wide reach. With machine translation and speech recognition, the platform supports communication in English and Hindi while utilizing CGIAR's data backbone for accurate, data-driven insights. 
+          <t>Four prototypes of an AI-powered Agriculture Information Exchange Platforms were developed through four initiatives: 
+1. DynAG: 
+Focused on rice, wheat, and maize, DynAG's platform uses a RAG pipeline powered by LLMs like the GPT suite to provide farmers with advisory services. Accessible via chatbots, Android and Jio-based mobile apps, IVR, and SMS, it ensures wide reach. With machine translation and speech recognition, the platform supports communication in English and Hindi while utilizing CGIAR's data backbone for accurate, data-driven insights. 
  2. Digital Green: 
- Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. 
+Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. 
  3. Viamo and Partners: 
  This platform targets farmers in Kenya and Bihar, focusing on beans and wheat, respectively. Using IVR, SMS, and WhatsApp, the platform is built on a RAG pipeline powered by LLMs, with potential for intent and entity recognition. Machine translation and speech-enabled IVR support English, Hindi, and Swahili, making it accessible across regions. The initiative is part of a broader plan to enhance voice technology for agricultural advisory. 
  4. Tech for Her: 
@@ -6274,7 +6304,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>https://dev.platform.farmer.chat/login</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -6353,22 +6383,22 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Making AI understand 3 East African languages:  Kiswahili, Kinyarwanda and Luganda - Open-source text-to-speech datasets - Mozilla Common Voice</t>
+          <t>Making AI understand 3 East African languages:  Kiswahili, Kinyarwanda and Luganda - Open-source speech-to-text datasets - Mozilla Common Voice</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Making AI understand 3 East African languages:  Kiswahili, Kinyarwanda and Luganda - Open-source text-to-speech datasets in Mozilla Common Voice</t>
+          <t>Making AI understand 3 East African languages:  Kiswahili, Kinyarwanda and Luganda - Open-source speech-to-text datasets in Mozilla Common Voice</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>By collecting more than 1000 hours of AI voice data (by 04/2025), this effort created the largest open-source voice dataset of diverse Swahili speakers for speech recognition (speech-to-text). You can use this resource to build AI systems understanding spoken Swahili e.g. in cellphones . This facilitates access to information in mother tongue, including by illiterate persons and persons in rural settings.</t>
+          <t>By collecting more than 1064 hours of AI recorded speech in Kiswahili (by 03/2026), this effort created the largest open-source voice dataset of diverse Swahili speakers for speech recognition (speech-to-text). You can use this resource to build AI systems understanding spoken Swahili e.g. in cellphones. In addition, voice datasets were collected in Kinyarwanda and Luganda (560 hours of recorded speech). This facilitates access to information in mother tongues, including by illiterate persons and persons in rural settings.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://datacollective.mozillafoundation.org/datasets?q=common+voice</t>
+          <t>https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=sw; https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=lg; https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -6394,7 +6424,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t xml:space="preserve">The datasets for the three languages consist of text data and the corresponding voice data. They are hosted on Mozilla's Common Voice Platform.
+          <t xml:space="preserve">The datasets for the three languages consist of text data and the corresponding voice data. They are hosted on Mozilla's Common Voice Platform. for more information on the Kinyarwanda dataset, also see https://fair-forward.github.io/datasets?search=kinya&amp;project=ui_59-a_large_scale_collection_of_voice 
 A responsible AI Assessment was undertaken for the Kiswahili dataset case to help AI developers and project managers to identify, assess and mitigate potential harms and biases in AI. The assessment included a Gender Action Plan — a comprehensive strategy to ensure women and gender diverse communities are equitably represented.For more information, see: https://www.mozillafoundation.org/en/blog/a-gender-action-plan-to-make-voice-technology-more-inclusive/ </t>
         </is>
       </c>
@@ -6415,7 +6445,8 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Balthas Seibold</t>
+          <t>Contact person: 
+Editor: Balthas Seibold</t>
         </is>
       </c>
       <c r="R53" t="inlineStr"/>
@@ -6432,7 +6463,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -6807,7 +6838,11 @@
           <t>not public yet</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>SDG 13, SDG 11</t>
@@ -7004,7 +7039,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -7165,7 +7200,11 @@
       </c>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model &gt; Pilot</t>
+        </is>
+      </c>
       <c r="T60" t="inlineStr">
         <is>
           <t>NLP</t>
@@ -7202,12 +7241,12 @@
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">This effort created the largest open-source voice dataset of diverse Kinyarwanda speakers for speech recognition (speech-to-text). It collected more than 2300  hours of AI voice data in Kinyarwanda (by 04/2025). You can use this resource to build AI systems understanding spoken Kinyarwanda e.g. in cellphones . This facilitates access to information in mother tongue, including by illiterate persons and in rural settings. </t>
+          <t xml:space="preserve">This effort created the largest open-source voice dataset of diverse Kinyarwanda speakers for speech recognition (speech-to-text). It collected more than 2380  hours of AI voice data in Kinyarwanda (by 03/2026). You can use this resource to build AI systems understanding spoken Kinyarwanda e.g. in cellphones . This facilitates access to information in mother tongue, including by illiterate persons and in rural settings. </t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://datacollective.mozillafoundation.org/datasets?q=common+voice ; https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset  </t>
+          <t xml:space="preserve">https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw ; https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset  </t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -7347,8 +7386,8 @@
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -7531,17 +7570,17 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">SGBV Chatbot </t>
+          <t>Preventing Sexual and Gender-Based Violence -  a featurephone-based information chatbot (*350#)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>The USSD GBV Information Chatbot (*350#)</t>
+          <t>Preventing Sexual and Gender-Based Violence -  a featurephone-based information chatbot (*350#)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Enabling people to access essential information around GBV free of charge and anonymously. This innovative tool requires only a feature phone, with no internet connectivity needed. A collaborative effort between HDI-Rwanda and GIZ-Rwanda. As of November 27 (2024), the chatbot has reached an impressive 343,475 unique users, up from 160,000 on October 1st, with 1,991,660 interactions recorded today compared to 1,170,000 interactions in October. Update of stats pending</t>
+          <t>Enabling people to access essential information around Sexual and Gender-Based Violence free of charge and anonymously. This innovative tool requires only a feature phone, with no internet connectivity needed. A collaborative effort between HDI-Rwanda and GIZ-Rwanda. As of November 27 (2024), the chatbot has reached an impressive 343,475 unique users, up from 160,000 on October 1st, with 1,991,660 interactions recorded today compared to 1,170,000 interactions in October. Update of stats pending</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7566,7 +7605,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>GIZ (Christiane Adamczyk), Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -7584,14 +7623,14 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Powered by:  
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+          <t>Powered by:  Health Development Initiative (HDI) Rwanda
+Catalyzed by: Sexualised and Gender-Based Violence (P-SGBV) Project of GIZ,  GIZ ZFD SIGA Refugee Programme, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Isaac</t>
+          <t>Isaac Manzi, Christiane Adamczyk</t>
         </is>
       </c>
       <c r="R64" t="inlineStr"/>
@@ -8790,7 +8829,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9046,7 +9085,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -9313,8 +9352,8 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10145,11 +10184,7 @@
           <t>Text</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>https://c4ir.rw/</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>Rwanda</t>
@@ -10192,7 +10227,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix: improve enrichment quality -- fix repetitive openers and prompt leakage
- Update LLM how_to_use prompt to avoid generic "valuable resource" openers
- Add YAML frontmatter stripping before LLM extraction
- Add output validation to reject YAML-like responses
- Pass project context (existing description, data/model chars) to LLM for richer extraction
- Fix identify_gaps() to include generic web URLs (was excluding them as unfetchable)
- Increase LLM context window from 4000 to 6000 chars and max_tokens from 500 to 800
- Re-generated 11 how_to_use fields with better openers
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -2081,23 +2081,12 @@
       <c r="N14" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Cashew Disease Identification (CADI AI) dataset is a valuable resource for small-holder farmers in Ghana, aiming to enhance the early detection of diseases in cashew plantations. Here’s a practical guide on how to utilize and build upon this resource.
-1) **Immediate Use Cases and Applications**:
-   - **Disease Detection**: You can use the CADI AI dataset to develop or implement AI models that detect diseases in cashew crops. This can help farmers identify issues early, potentially increasing yields by up to 30%.
-   - **Training AI Models**: The dataset includes 4,736 high-resolution images with annotations for various conditions affecting cashew trees, such as diseases, insects, and abiotic factors. You can immediately start training object detection models using this data.
-   - **Decision Support Tools**: Create applications that provide farmers with insights based on the AI's analysis, helping them make informed decisions about crop management.
-2) **Extending or Improving the Work**:
-   - **Enhancing the Dataset**: Researchers can collect additional images from different regions or under varying conditions to improve the model's robustness and accuracy.
-   - **Model Optimization**: Developers can experiment with different AI architectures beyond YOLO to see if they can achieve better performance in disease detection.
-   - **User-Friendly Interfaces**: Innovators can build mobile or web applications that make it easier for farmers to access the AI's insights, ensuring that the technology is user-friendly and accessible.
-3) **Critical Limitations and Biases**:
-   - **Ethical AI Assessment**: It is recommended to conduct an ethical AI assessment before deploying any AI solutions. This helps identify and mitigate potential biases in the model, ensuring fair and responsible use.
-   - **Data Limitations**: The dataset may not cover all possible diseases or conditions affecting cashew trees. Users should be cautious about over-relying on the model without additional local knowledge.
-4) **Cost Estimates**:
-   - **Adaptation and Training**: Depending on the complexity of the model and the computational resources available, costs can vary. Basic training on a cloud platform may start from a few hundred dollars, while more extensive training could reach thousands.
-   - **Compute Resources**: Utilizing cloud services for training can incur costs based on usage. Expect to budget for GPU instances if training deep learning models.
-   - **Collaboration Opportunities**: Engage with local agricultural organizations or universities to share knowledge and resources, which can help reduce costs and improve outcomes.
-For further information, you can access the detailed datasheet linked in the dataset repository. This resource provides insights into the dataset's composition and methodologies, which can be crucial for effective implementation. By leveraging this dataset, you can contribute to improving the livelihoods of cashew farmers in Ghana and enhance food security in the region.</t>
+You can immediately start using the Cashew Disease Identification (CADI AI) dataset to develop an application that helps small-holder cashew farmers in Ghana detect diseases in their crops early. By analyzing drone-captured images of cashew plants, you can create a tool that alerts farmers to potential diseases, enabling them to take action that could increase their yields by up to 30%. 
+To get started, download the dataset, which includes 4,736 high-resolution images annotated for object detection. The dataset is structured into training, validation, and test sets, making it ready for immediate use in machine learning applications. You can utilize the YOLO format annotations to train a model that identifies three categories: abiotic factors, insects, and diseases.
+Researchers and developers can extend this work by improving the model's accuracy or adapting it for different crops or regions. Collaborating with local agricultural experts can enhance the dataset's relevance and effectiveness. Additionally, you might consider integrating the application with mobile platforms to ensure accessibility for farmers in remote areas.
+When replicating this work, it's crucial to conduct a responsible AI assessment to identify and mitigate potential biases and harms associated with AI use in agriculture. The dataset creators have already undertaken such an assessment, which can serve as a guide for your project.
+In terms of costs, you may need to budget for cloud computing resources for model training, which can vary widely based on the scale of your application. A rough estimate for cloud compute costs could range from $100 to $1,000, depending on the duration and intensity of the training process. 
+For further guidance, you can refer to the accompanying datasheet linked in the dataset repository, which provides detailed information about the dataset's composition and methodologies. Engaging with the KaraAgro AI Foundation or GIZ could also open up opportunities for collaboration and support in scaling your application.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -2225,27 +2214,11 @@
       <c r="N15" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Crop Disease dataset from Ghana provides a valuable resource for addressing food security and climate change adaptation through AI-powered crop disease identification. Here’s a practical guide for development practitioners and innovators looking to utilize this resource:
-1) **Immediate Use Cases**: 
-   - **Disease Identification**: You can use the existing models to identify diseases in maize, tomatoes, and peppers. This can help farmers quickly diagnose issues and take action to protect their crops.
-   - **Training Workshops**: Organize workshops for local farmers and agricultural extension workers to teach them how to use the models for real-time disease detection.
-   - **Mobile Applications**: Develop a simple mobile app that allows farmers to upload images of their crops and receive instant feedback on potential diseases.
-2) **Extending the Work**:
-   - **Local Adaptation**: Researchers can improve the models by incorporating local data on crop diseases that may not be included in the dataset. This could involve collecting more images from different regions or different crop varieties.
-   - **Integration with Agricultural Practices**: Collaborate with agricultural experts to integrate disease identification with best practices for crop management, providing farmers with actionable advice based on the identified diseases.
-   - **User-Friendly Interfaces**: Developers can create more accessible interfaces for non-technical users, ensuring that farmers and agricultural workers can easily interact with the technology.
-3) **Limitations and Considerations**:
-   - **Data Bias**: The dataset is limited to specific districts in the Ashanti Region, which may not represent all crop diseases found in other regions of Ghana or Africa. It’s important to validate the models with local data before widespread use.
-   - **Ethical AI Assessment**: Before deploying any AI solutions, consider conducting an ethical AI assessment to ensure that the technology is used responsibly and does not inadvertently harm local farming practices or communities.
-4) **Cost Estimates**:
-   - **Adaptation and Training**: Depending on the scale, adapting the models could range from $1,000 to $5,000, including costs for data collection and model training.
-   - **Compute Resources**: If using cloud services for model training, expect costs to be around $100 to $500 per month, depending on usage.
-   - **Collaboration Opportunities**: Partner with local universities or NGOs focused on agriculture to share resources and expertise, which can help reduce costs and improve outcomes.
-5) **Additional Resources**:
-   - **Documentation and Tutorials**: Look for available documentation on the Kaggle dataset page, which may include guides on how to use the models effectively.
-   - **Success Stories**: Reach out to organizations that have successfully implemented similar technologies to learn from their experiences and adapt their strategies to your context.
-   - **Long-term Maintenance**: Plan for ongoing support and updates to the models as new data becomes available, ensuring that the technology remains relevant and effective over time.
-By leveraging this dataset and the associated models, you can make significant strides in improving crop health and food security in Ghana and beyond.</t>
+You can immediately use the Crop Disease dataset to develop an AI-powered application that helps farmers in Ghana identify diseases in maize, tomatoes, and peppers. By leveraging the images in this dataset, you can create a tool that allows farmers to upload pictures of their crops and receive instant feedback on potential diseases, enabling them to take timely action to protect their harvests.
+To extend or improve upon this work, researchers and developers can explore integrating additional datasets that include environmental factors, such as soil quality and weather conditions, which may influence disease prevalence. Collaborating with local agricultural experts can also enhance the model's accuracy and relevance to specific regional challenges.
+When replicating this work, it's important to consider potential limitations, such as the dataset's focus on specific districts in the Ashanti Region, which may not represent all agricultural conditions in Ghana. Additionally, conducting an ethical AI assessment is recommended to ensure that the application respects local farming practices and does not inadvertently cause harm.
+In terms of costs, building on this resource may require investment in cloud computing services for model training and deployment, which can range from a few hundred to several thousand dollars depending on the scale of your application. Collaborating with local universities or NGOs can help reduce costs and provide access to expertise.
+Documentation and tutorials related to the dataset and the winning models from the Zindi challenge are available, which can guide you in developing your application. Success stories from the data challenge can also provide insights into effective strategies and potential pitfalls. For long-term maintenance and scaling, consider establishing partnerships with local agricultural organizations to ensure ongoing support and updates to the application.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2477,26 +2450,11 @@
       <c r="N17" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The "Discover Ghanaian Voices" dataset is a valuable resource for anyone interested in understanding and utilizing Ghanaian accented English. Here’s a practical guide on how to leverage this dataset effectively:
-1) **Immediate Use Cases**:
-   - **Accent Classification**: You can use the dataset to develop models that classify different Ghanaian accents. This can be beneficial for applications in customer service, where understanding regional accents can improve communication.
-   - **Speech Recognition**: Enhance speech recognition systems to better understand and transcribe Ghanaian English. This can improve accessibility for users in Ghana who may struggle with standard English recognition systems.
-   - **Linguistic Research**: Researchers can analyze the dataset to study the linguistic features of Ghanaian English, contributing to academic work in sociolinguistics and phonetics.
-2) **Extending the Work**:
-   - **Broader Language Support**: Developers can expand the dataset by including more diverse scripts or additional languages spoken in Ghana, which would enrich the dataset and its applications.
-   - **Integration with Other Datasets**: Combining this dataset with other linguistic datasets can provide a more comprehensive view of language use in Ghana, allowing for more robust models and analyses.
-   - **Community Engagement**: Collaborate with local universities or linguistic departments to gather more data or refine existing models based on community feedback.
-3) **Limitations and Biases**:
-   - **Regional Representation**: While the dataset captures various accents, it may not represent all dialects or speech patterns across Ghana. Users should be cautious about generalizing findings beyond the dataset's scope.
-   - **Ethical Considerations**: It is recommended to conduct an ethical AI assessment before using the dataset, especially if the applications involve sensitive areas like surveillance or profiling.
-   - **Data Quality**: The quality of audio recordings may vary, which could affect model performance. Users should consider this when training models.
-4) **Cost Estimates**:
-   - **Adaptation and Training**: Depending on the complexity of the models you wish to build, costs can range from a few hundred to several thousand dollars. This includes expenses for data cleaning, model training, and validation.
-   - **Compute Resources**: If using cloud services for training, expect to spend approximately $100 to $500 per month, depending on the scale of your operations and the duration of training.
-   - **Collaboration Opportunities**: Engaging with local universities or tech hubs can reduce costs and enhance the project through shared resources and expertise.
-5) **Documentation and Support**:
-   - While specific documentation for this dataset may not be detailed, users can refer to general resources on accent classification and speech recognition to guide their projects. Online tutorials on machine learning and natural language processing can also provide foundational knowledge.
-By utilizing the "Discover Ghanaian Voices" dataset, practitioners and innovators can make significant strides in improving communication technologies and linguistic understanding in Ghana, ultimately contributing to more inclusive development efforts.</t>
+You can immediately use the Accent Classification Dataset (Ghana) to develop applications that improve speech recognition systems for Ghanaian English, enhancing communication tools for education, customer service, and accessibility. By analyzing the distinct regional accents captured in the dataset, you can create models that better understand and process spoken English in Ghana, making technology more inclusive for local users.
+Researchers and developers can extend this work by incorporating additional regional accents or dialects from other parts of West Africa, thereby broadening the dataset's applicability. Collaborating with local universities or linguistic departments can provide insights into regional variations and help gather more diverse audio samples. Additionally, you could explore integrating this dataset with existing speech recognition frameworks to improve their accuracy in understanding Ghanaian English.
+However, it is important to consider potential limitations and biases in the dataset. The recordings may not represent all dialects or socio-economic backgrounds within Ghana, which could affect the performance of any models trained on this data. We recommend conducting an ethical AI assessment to ensure that your applications do not inadvertently reinforce stereotypes or exclude certain groups.
+In terms of costs, building on this dataset may involve expenses related to data adaptation, model training, and computing resources. Depending on the scale of your project, you might expect costs to range from a few hundred to several thousand dollars, particularly if you require cloud computing services for processing the audio data.
+Documentation and tutorials on how to use the dataset effectively may be available through the Kaggle platform, and engaging with the Kaggle community can provide additional support and success stories from others who have utilized this dataset. Long-term maintenance and scaling of your project could benefit from partnerships with local organizations that understand the linguistic landscape and can help keep the dataset updated and relevant.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -3086,28 +3044,12 @@
       <c r="N21" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Drone-based Agricultural Dataset for Crop Yield Estimation provides a valuable resource for farmers, researchers, and organizations focused on improving agricultural practices in Ghana and Uganda. Here’s a practical guide on how to utilize this dataset effectively.
-1) **Immediate Use Cases**:
-   - **Yield Estimation**: Use the dataset to develop models that estimate the yield of cashew, cocoa, and coffee crops. This can help farmers make informed decisions about harvesting and selling their produce.
-   - **Crop Type Detection**: Implement applications that can identify different crop types and their growth stages, which can assist in monitoring crop health and planning interventions.
-   - **Fruit Detection and Counting**: Create tools that automatically count fruits on trees, providing farmers with insights into potential harvest volumes.
-   - **Maturity Stage Detection**: Develop applications that assess the maturity of fruits (unripe, ripe, spoiled), helping farmers determine the best time for harvest.
-2) **Extending the Work**:
-   - **Enhancing Models**: Researchers can build upon the existing models by incorporating additional data sources, such as weather patterns or soil quality, to improve yield predictions.
-   - **Cross-Crop Analysis**: Explore the dataset for comparative studies between different crops, which can lead to insights on best practices and crop management strategies.
-   - **Integration with Other Technologies**: Combine the dataset with IoT devices or mobile applications to create real-time monitoring systems for farmers.
-3) **Limitations and Considerations**:
-   - **Data Bias**: The dataset is limited to specific regions in Ghana and Uganda, which may not represent agricultural practices in other areas. Users should consider local conditions when applying findings.
-   - **Ethical AI Assessment**: Before deploying any AI models based on this dataset, it is recommended to conduct an ethical AI assessment to ensure that the technology is used responsibly and does not negatively impact local communities.
-4) **Cost Estimates**:
-   - **Adaptation and Training**: Depending on the complexity of the models, costs can range from a few hundred to several thousand dollars for data processing and model training. 
-   - **Compute Resources**: Utilizing cloud services for model training may incur costs of approximately $100 to $1,000, depending on the duration and resources used.
-   - **Collaboration Opportunities**: Engage with local universities or agricultural organizations for collaborative projects, which can help share costs and resources.
-5) **Additional Resources**:
-   - **Documentation**: Detailed documentation is available to help users understand the dataset's structure and how to implement it in their projects.
-   - **Success Stories**: Look for case studies or success stories from other organizations that have used this dataset to inspire your own projects.
-   - **Long-term Maintenance**: Consider establishing partnerships with local institutions to ensure ongoing support and updates for the models developed using this dataset.
-By leveraging this dataset, development practitioners and innovators can significantly enhance agricultural productivity and sustainability in their communities.</t>
+To enhance crop yield estimation for cashew, cocoa, and coffee farmers in Ghana and Uganda, you can immediately utilize the Drone-based Agricultural Dataset to develop models that estimate yields based on drone imagery. This dataset contains 14,870 high-resolution images with detailed annotations, allowing you to implement applications such as crop type detection, fruit counting, and maturity stage classification.
+You can start by using existing tools like the YOLO (You Only Look Once) framework for object detection. With the provided annotations, you can train a model to identify and classify different growth stages of crops, which can help farmers make informed decisions about harvesting and resource allocation. This can lead to improved productivity and better financial outcomes for farmers.
+For researchers and developers looking to extend this work, consider integrating additional data sources, such as weather patterns or soil quality metrics, to enhance the accuracy of yield predictions. Collaborating with local agricultural experts can also provide insights into specific challenges faced by farmers, allowing for the development of tailored solutions.
+While the dataset is robust, there are limitations to consider. The images are specific to certain regions and may not represent all agricultural conditions. It's advisable to conduct an ethical AI assessment to ensure that the models developed do not inadvertently reinforce biases or overlook local agricultural practices. Additionally, the dataset may not cover all potential crop diseases or pests, which could affect yield predictions.
+In terms of costs, building on this dataset may require investment in cloud computing resources for model training, which can range from a few hundred to several thousand dollars depending on the scale of your project. If you plan to adapt the dataset or develop new models, consider budgeting for data storage, processing, and potential collaboration with local institutions.
+For further guidance, explore the accompanying documentation and datasheet linked in the dataset repository. This resource provides detailed information on data collection methodologies and variable definitions, which can be crucial for effective model development. Engaging with local agricultural organizations can also foster collaboration and ensure that the solutions developed are practical and impactful for the communities involved.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -3582,28 +3524,28 @@
       <c r="N25" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Combatting Air Pollution and GHG Emissions project in India offers valuable resources and tools for addressing air quality issues through hyperlocal data collection and analysis. Here’s a practical guide for development practitioners and innovators looking to utilize or build upon this initiative.
-1) **Immediate Use Cases and Applications:**
-   - **Air Quality Monitoring:** You can start using the VAYU Android application and citizen portal to monitor air quality in your area. This tool allows you to access real-time data collected from over 100 sensors across two cities.
-   - **Community Engagement:** Engage local volunteers to become citizen scientists. They can help collect data using dynamic sensors, contributing to a more comprehensive understanding of pollution sources.
-   - **Targeted Interventions:** Use the data to identify pollution hotspots and risk zones. This information can guide local authorities in implementing targeted actions to mitigate air pollution.
-2) **Extending or Improving the Work:**
-   - **Data Expansion:** Researchers can expand the dataset by adding more sensors in additional cities or regions, enhancing the coverage and accuracy of air quality monitoring.
-   - **Algorithm Development:** Developers can improve the existing AI/ML algorithms used for pollution detection. This could involve refining models to better predict pollution patterns or integrating additional data sources for more robust analysis.
-   - **Collaboration Opportunities:** Partner with local universities or NGOs to enhance data collection efforts and share insights on air quality management strategies.
-3) **Critical Limitations and Considerations:**
-   - **Data Quality:** Ensure that the data collected from sensors is regularly calibrated and maintained to avoid inaccuracies. 
-   - **Ethical AI Assessment:** Before replicating or extending the project, consider conducting an ethical AI assessment to address potential biases in data collection and analysis.
-   - **Community Involvement:** Engage with local communities to ensure that the data collection process is transparent and that the findings are communicated effectively to avoid misinformation.
-4) **Cost Estimates and Resources:**
-   - **Sensor Costs:** Low-cost IoT sensors can range from $50 to $200 each, depending on the specifications. Budget for additional sensors if expanding the network.
-   - **Training and Adaptation:** Training local volunteers and staff on data collection and analysis may require a budget for workshops or materials, estimated at around $1,000 to $5,000 depending on the scale.
-   - **Computational Resources:** If developing new algorithms, consider cloud computing costs, which can vary widely but may start at around $100 per month for basic usage.
-**Additional Resources:**
-- **Documentation and Tutorials:** Check the VAYU citizen portal for available guides on using the application and understanding the data.
-- **Success Stories:** Look for case studies or reports from the project that highlight successful interventions based on the data collected.
-- **Long-term Maintenance:** Consider establishing a local team to maintain the sensors and ensure ongoing data collection and analysis, which is crucial for the sustainability of the project.
-By leveraging the existing tools and resources from this initiative, you can make a significant impact on air quality management in your community while also contributing to broader efforts in combatting climate change.</t>
+You can start using the VAYU project to combat air pollution in your community by leveraging the hyperlocal air quality data collected through citizen scientists and IoT-based sensors. Here are some practical steps and considerations:
+1. **Immediate Use Cases**: 
+   - **Monitor Air Quality**: Utilize the VAYU Android app and citizen portal to access real-time air quality data in your area. This can help you identify pollution hotspots and inform community members about air quality levels.
+   - **Targeted Interventions**: Use the data to advocate for specific actions from local authorities, such as increased regulation of identified pollution sources or the implementation of green spaces in high-risk zones.
+   - **Community Engagement**: Mobilize local volunteers to participate in data collection, enhancing community awareness and involvement in air quality issues.
+2. **Extending the Work**:
+   - **Enhance Data Collection**: Researchers and developers can improve upon the existing sensor network by integrating additional sensors or developing new applications that analyze the data in different ways, such as correlating air quality with health outcomes.
+   - **Collaborate with Local Authorities**: Work with local governments to create policies based on the data collected, ensuring that interventions are data-driven and effective.
+   - **Develop Educational Programs**: Create workshops or materials that educate the community about air pollution and how they can contribute to monitoring efforts.
+3. **Limitations and Considerations**:
+   - **Data Bias**: Be aware that the data collected may reflect the locations of sensors rather than a comprehensive view of air quality across all areas. It’s important to consider this when making decisions based on the data.
+   - **Ethical AI Assessment**: Before replicating or extending the project, conduct an ethical assessment to ensure that the use of AI and data collection respects community privacy and consent.
+4. **Cost Estimates**:
+   - **Sensor Deployment**: The cost of low-cost sensors can vary, but budget for approximately $100 to $300 per sensor, depending on the type and features.
+   - **Data Management**: Consider costs for data storage and processing, which could range from a few hundred to several thousand dollars annually, depending on the scale of your project.
+   - **Training and Adaptation**: If you plan to train local volunteers or staff, allocate funds for training materials and sessions, which could cost around $500 to $1,500.
+5. **Collaboration Opportunities**: 
+   - Engage with local universities or NGOs that focus on environmental issues to share resources and expertise.
+   - Partner with tech companies interested in social impact to enhance the technological aspects of the project.
+6. **Documentation and Support**: 
+   - Check the VAYU website for available documentation on how to use the app and portal effectively. Tutorials may also be available to guide new users through the data collection and analysis processes.
+By taking these steps, you can effectively utilize the VAYU project to address air pollution in your community while also contributing to a larger movement towards cleaner air and better public health.</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -6607,28 +6549,11 @@
       <c r="N49" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The LivHealth Kiswahili Corpus project offers valuable resources for improving livestock health in Kenya and Tanzania, particularly for pastoralists and Community Disease Reporters (CDRs). Here’s a practical guide for those interested in using or building upon this initiative.
-1) **Immediate Use Cases and Applications**:
-   - **Disease Identification**: The LivHealth app allows CDRs and pastoralists to record and share information about livestock diseases. Users can immediately start using the app to document disease outbreaks and access translated digital disease manuals in Kiswahili.
-   - **Data Sharing**: The app facilitates communication between CDRs and veterinary officers, enabling quicker responses to disease outbreaks. This can lead to timely interventions such as vaccinations.
-   - **Community Engagement**: Pastoralists can utilize the app to better understand livestock health, improving their ability to manage their herds effectively.
-2) **Extending or Improving the Work**:
-   - **Localization**: Developers can enhance the app by adding more local dialects or languages to reach a broader audience. This could involve recording additional local voices for the text-to-speech feature.
-   - **Integration with Other Systems**: Researchers can explore integrating the LivHealth app with existing veterinary health systems or databases to streamline data collection and reporting.
-   - **Training and Capacity Building**: Organizations can develop training programs for CDRs and pastoralists on how to effectively use the app and interpret the information provided.
-3) **Critical Limitations and Considerations**:
-   - **Ethical AI Assessment**: Before replicating or adapting the technology, it is recommended to conduct an ethical AI assessment to ensure that the technology is used responsibly and does not inadvertently harm the communities it aims to serve.
-   - **Data Privacy**: Consideration should be given to the privacy of the data collected through the app, ensuring that personal information is protected and used only for intended purposes.
-4) **Cost Estimates**:
-   - **Adaptation Costs**: Depending on the extent of localization and additional features, costs could range from a few thousand to tens of thousands of dollars. This includes expenses for software development, voice recording, and user testing.
-   - **Training Costs**: Budgeting for training sessions for users may also be necessary, which could add additional costs depending on the scale of the training.
-**Opportunities for Collaboration**:
-- Organizations can collaborate with the LivHealth team or One Health Center in Africa (OHRECA) to share insights, resources, and best practices. Partnerships with local governments or NGOs can also enhance the reach and impact of the initiative.
-**Available Documentation and Success Stories**:
-- The LivHealth project has documented its success in facilitating the vaccination of over 3.5 million goats and sheep, benefiting approximately 33,000 households. This success can serve as a model for similar initiatives in other regions.
-**Plans for Long-term Maintenance or Scaling**:
-- The LivHealth team is committed to sustaining the mobile app and expanding its programming into Tanzania, indicating a focus on long-term impact and scalability.
-By leveraging the LivHealth Kiswahili Corpus project, development practitioners and innovators can make significant strides in improving livestock health and supporting pastoralist communities in Kenya and Tanzania.</t>
+To improve livestock health management in your community, you can immediately use the LivHealth Kiswahili Corpus to access vital disease information in Kiswahili. This resource allows local farmers and livestock owners to identify livestock syndromes and seek timely interventions from qualified practitioners. You can start by integrating the text-to-speech models into your community outreach programs, ensuring that information is accessible to those who may have literacy challenges.
+Researchers and developers can extend this work by enhancing the existing AI models with additional local data, which could improve the accuracy of disease identification. Collaborating with local agricultural universities or veterinary schools could provide valuable insights and data for refining the models. Additionally, creating mobile applications that utilize the LivHealth system could broaden its reach and usability.
+When replicating or building upon this project, it is essential to consider potential biases in the AI models, particularly if they were trained on limited datasets. Conducting an ethical AI assessment is recommended to ensure that the system serves all community members equitably. 
+As for costs, building on this resource may involve expenses related to adaptation and training of the models, which could range from a few hundred to several thousand dollars depending on the scale of your project and the resources required. Compute costs will vary based on the infrastructure you choose to use, whether cloud-based or local servers.
+Opportunities for collaboration exist with organizations like One Health Center in Africa (OHRECA), which could provide support and expertise. While specific documentation or tutorials were not mentioned, reaching out to the LivHealth team could yield valuable guidance and success stories from their implementation in Kenya and Tanzania. Long-term maintenance and scaling plans should include regular updates to the dataset and models to keep the information relevant and accurate for the communities served.</t>
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
@@ -8004,29 +7929,12 @@
       <c r="N61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This large-scale collection of voice data in Kinyarwanda offers a valuable resource for developing inclusive language technology. Here’s a practical guide for using and building on this dataset:
-1. **Immediate Use Cases**: 
-   - **Speech Recognition Applications**: You can create applications that convert spoken Kinyarwanda into text. This is particularly useful for mobile apps that provide information in the local language, making it accessible to those who may be illiterate or in rural areas.
-   - **Voice Assistants**: Develop voice-activated systems that understand Kinyarwanda, enhancing user interaction in local languages.
-   - **Educational Tools**: Build tools that help teach Kinyarwanda pronunciation and literacy, using the dataset to provide examples of spoken language.
-2. **Extending the Work**: 
-   - **Enhancing the Dataset**: Researchers can collect additional voice samples to cover more dialects or accents within Kinyarwanda, improving the dataset's diversity.
-   - **Model Development**: Developers can create more sophisticated speech recognition models using this dataset as a foundation, experimenting with different machine learning frameworks and architectures.
-   - **Community Engagement**: Collaborate with local communities to gather feedback on the applications developed, ensuring they meet user needs and preferences.
-3. **Critical Limitations and Biases**: 
-   - **Ethical Considerations**: It is recommended to conduct an ethical AI assessment before using the dataset, especially regarding consent and representation of speakers.
-   - **Bias in Data**: The dataset may not fully represent all Kinyarwanda speakers, particularly those from rural or marginalized communities. Be mindful of this when developing applications to ensure inclusivity.
-4. **Cost Estimates**: 
-   - **Adaptation and Training**: Depending on the complexity of the models you wish to build, costs can vary. Basic adaptations might require minimal investment, while more advanced models could range from a few hundred to several thousand dollars, depending on the resources needed.
-   - **Compute Resources**: Utilizing cloud services for training models can incur costs based on usage. Budgeting for compute resources is essential, especially for larger models.
-**Opportunities for Collaboration**: 
-Engage with local universities, NGOs, and tech hubs to foster collaboration. These partnerships can provide additional insights and resources for developing applications that serve the community effectively.
-**Available Documentation and Tutorials**: 
-While specific documentation was not detailed, exploring the Mozilla Foundation's resources on Common Voice may provide guidance on how to utilize the dataset effectively.
-**Success Stories**: 
-Look for case studies or examples from other regions where similar datasets have been used to create impactful applications, which can serve as inspiration for your projects.
-**Long-term Maintenance and Scaling**: 
-Consider establishing a plan for ongoing data collection and model updates to keep the applications relevant and effective as language use evolves. Engaging with the community for continuous feedback will be crucial for long-term success.</t>
+You can immediately start building speech recognition applications that understand Kinyarwanda using the extensive voice dataset collected through the Common Voice project. With over 2,380 hours of audio recordings, this resource allows you to create systems that can transcribe spoken Kinyarwanda, making information more accessible to speakers, including those in rural areas and those who are illiterate.
+To get started, you can use existing tools for automatic speech recognition (ASR) that are compatible with the dataset. These tools can help you develop applications for mobile phones or other devices that provide information in Kinyarwanda, enhancing communication and access to services.
+Researchers and developers can extend this work by contributing additional voice data or improving the existing models. For instance, you could focus on specific dialects or contexts that are underrepresented in the current dataset. Collaborating with local communities to gather more diverse speech samples can also enhance the dataset's effectiveness.
+However, it’s important to consider potential limitations and biases. The dataset may not fully represent all dialects or accents of Kinyarwanda, which could affect the accuracy of speech recognition in certain contexts. We recommend conducting an ethical AI assessment before replicating or building upon this work to ensure that the technology is inclusive and respects the cultural nuances of the language.
+In terms of costs, building on this dataset may involve expenses related to adaptation and training of models, as well as computing resources. Depending on the scale of your project, you might estimate costs in the range of a few hundred to several thousand dollars, particularly if you require cloud computing services for model training.
+For further guidance, you can refer to the documentation available through the Common Voice project, which includes tutorials on how to use the dataset effectively. Engaging with the community around this project can also lead to collaboration opportunities, sharing insights, and learning from success stories of others who have implemented similar technologies. Long-term maintenance and scaling of your application will depend on ongoing community support and updates to the dataset as more voices are collected.</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -9741,32 +9649,12 @@
       <c r="N76" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The "Voices of Mzansi" project is a valuable resource for anyone interested in making South Africa's official languages more accessible through technology. Here’s a practical guide on how to utilize and build upon this initiative:
-1. **Immediate Use Cases**: 
-   - **Language Learning Apps**: You can use the translated Common Voice interface to create language learning applications that help users practice speaking and understanding South African languages.
-   - **Speech Recognition Systems**: The collected sentences can be used to train speech recognition systems that understand and process South African languages, making technology more inclusive.
-   - **Text-to-Speech Applications**: Developers can create applications that convert text into spoken language, enhancing accessibility for visually impaired users or those who prefer auditory learning.
-2. **Extending the Work**:
-   - **Collect More Data**: Researchers and developers can contribute by collecting additional sentences in underrepresented languages or dialects, expanding the dataset available for training AI models.
-   - **Improve Translation Quality**: Collaborate with linguists to refine translations and ensure cultural nuances are captured, enhancing the user experience.
-   - **Develop New Applications**: Innovators can build new applications that leverage the speech data for various sectors, such as education, healthcare, and public services.
-3. **Limitations and Considerations**:
-   - **Data Bias**: Be aware that the dataset may reflect biases present in the collected sentences. It’s important to ensure diverse representation in the data to avoid perpetuating stereotypes.
-   - **Ethical AI Assessment**: Before replicating or building on this work, consider conducting an ethical AI assessment to evaluate the potential impacts of your application on communities and individuals.
-   - **Technical Limitations**: The quality of speech recognition and text-to-speech applications may vary based on the amount and diversity of data collected. Continuous improvement and updates will be necessary.
-4. **Cost Estimates**:
-   - **Data Collection**: Costs can vary widely depending on the method of data collection (e.g., crowdsourcing, hiring linguists). Budgeting a few thousand dollars for initial data collection efforts is a reasonable starting point.
-   - **Training Models**: Depending on the complexity of the models and the amount of data, training costs can range from a few hundred to several thousand dollars, especially if using cloud computing resources.
-   - **Ongoing Maintenance**: Plan for ongoing costs related to data updates, model retraining, and application maintenance, which could also be in the range of a few thousand dollars annually.
-5. **Collaboration Opportunities**: 
-   - Engage with local universities, NGOs, and language organizations to pool resources and expertise. Collaborative efforts can enhance the quality and reach of the project.
-6. **Documentation and Tutorials**: 
-   - Check the Mozilla Common Voice website for available documentation on how to contribute to the dataset and utilize the tools provided. Tutorials on building applications using the Common Voice data can also be found online.
-7. **Success Stories**: 
-   - Look for case studies or examples of successful applications developed using the Common Voice dataset to inspire your own projects.
-8. **Long-term Maintenance**: 
-   - Consider establishing a community of contributors who can help maintain and update the dataset and applications over time, ensuring sustainability and relevance.
-By leveraging the "Voices of Mzansi" project, you can contribute to making South Africa's languages more accessible and promote inclusivity in technology.</t>
+To start using the "Voices of Mzansi" project, you can immediately contribute by collecting sentences in any of South Africa's official languages and uploading them to the Mozilla Common Voice platform. This effort helps create a diverse dataset that can be used for developing text-to-speech applications, voice recognition systems, and other AI tools that support local languages.
+Researchers and developers can extend this work by creating applications that utilize the collected speech data for educational tools, accessibility features, or community engagement platforms. You can also improve upon the existing dataset by ensuring it includes a wide range of dialects and contexts, which will enhance the accuracy and usability of AI models trained on this data.
+When replicating this project, consider potential biases in the dataset, such as underrepresentation of certain dialects or socio-economic groups. It is advisable to conduct an ethical AI assessment to ensure that the applications developed are inclusive and do not perpetuate existing inequalities.
+In terms of costs, building on this project may involve expenses related to data collection tools, community engagement efforts, and possibly cloud computing resources for training AI models. Depending on the scale, initial costs could range from a few hundred to several thousand dollars, particularly if you need to hire local language speakers or facilitators.
+Collaboration opportunities exist with local universities, NGOs, and tech communities interested in language preservation and AI. Documentation and tutorials for using the Common Voice platform are available on their website, which can guide you through the process of contributing and utilizing the datasets. Success stories from similar projects can inspire your efforts and provide insights into effective strategies for community involvement and data collection.
+Long-term maintenance and scaling of this project will depend on ongoing community engagement and the continuous collection of diverse language data to keep the datasets relevant and useful.</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -10459,25 +10347,12 @@
       <c r="N82" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Solar Irradiance Portal offers a valuable resource for development practitioners and innovators looking to enhance solar energy planning in Sub-Saharan Africa, particularly in Uganda. Here’s a practical guide on how to leverage this resource effectively:
-1. **Immediate Use Cases and Applications**:
-   - **Energy Project Planning**: Use the corrected solar irradiance data to assess the solar potential for new energy projects. This data can help in sizing solar systems accurately, reducing financial risks associated with overestimations from standard satellite data.
-   - **Investment Decisions**: The reliable solar data can support investment decisions by providing bankable-grade information, which is crucial for attracting funding and ensuring project viability.
-   - **Policy Development**: Government agencies can utilize the data to inform renewable energy policies and strategies, ensuring they are based on accurate local conditions.
-2. **Extending or Improving the Work**:
-   - **Data Integration**: Researchers and developers can build on this work by integrating the solar irradiance data with other datasets, such as energy consumption patterns or demographic data, to create comprehensive energy models.
-   - **Model Enhancement**: There is potential to refine the existing Random Forest model by incorporating additional machine learning techniques or more localized data from other regions in Africa to improve accuracy further.
-   - **User Feedback**: Engaging with users of the platform to gather feedback can help identify areas for improvement and new features that could enhance usability and functionality.
-3. **Critical Limitations and Considerations**:
-   - **Data Bias**: While the model corrects satellite data bias, users should remain aware of any residual biases that may still exist. It is advisable to conduct an ethical AI assessment to ensure that the data is used responsibly and does not inadvertently reinforce existing inequalities.
-   - **Geographic Limitations**: The current model is specifically tuned for Uganda. Users in other regions should be cautious when applying this data without appropriate adjustments for local conditions.
-4. **Cost Estimates and Resources**:
-   - **Cost of Adaptation**: While specific cost estimates are not provided, users should consider potential expenses related to data integration, additional training of models, and computing resources for running analyses.
-   - **Collaboration Opportunities**: There may be opportunities for collaboration with local universities or NGOs interested in renewable energy, which could help share costs and resources.
-   - **Documentation and Tutorials**: The platform offers an intuitive interface and interactive visualizations, which can serve as a guide for users unfamiliar with data analysis. Further documentation may be available through the portal for deeper technical insights.
-   - **Success Stories**: Engaging with other users who have successfully implemented the data in their projects can provide valuable insights and inspiration for new applications.
-   - **Long-term Maintenance**: The platform aims to provide ongoing updates and maintenance, ensuring that users have access to the latest data and improvements in the model.
-By utilizing the Solar Irradiance Portal, practitioners can make informed decisions that enhance solar energy initiatives, ultimately contributing to sustainable development in Uganda and beyond.</t>
+You can immediately access reliable solar irradiance data for Uganda to enhance your solar energy planning efforts. The Solar Irradiance Portal provides corrected Global Horizontal Irradiance (GHI) data that addresses the inaccuracies found in standard satellite-derived solar data. This means you can confidently assess solar potential, optimize system sizing, and reduce financial risks associated with solar projects.
+To get started, you can explore the interactive visualizations available on the platform, which allow you to analyze solar patterns through dynamic charts and maps. Additionally, you can integrate the corrected solar data into your applications using the provided RESTful API, making it easier to incorporate accurate information into your energy planning tools.
+Researchers and developers can build on this work by extending the model to other regions in Sub-Saharan Africa or by incorporating additional data sources to enhance the accuracy of predictions. Collaborating with local universities or NGOs could provide valuable ground-truth data and insights into regional climate variations, further improving the model's performance.
+It's important to consider that while the model has shown a high accuracy score (R² of 0.86), there may still be limitations related to the specific climate zones and topography of Uganda. Conducting an ethical AI assessment is recommended to ensure that the model's application does not inadvertently reinforce existing biases or overlook local knowledge.
+As for costs, while specific figures are not provided, you should budget for potential expenses related to data integration, API usage, and any necessary computational resources for running analyses. Collaborating with local partners may help reduce costs and enhance the project's impact.
+The platform is designed for long-term use, with ongoing updates and maintenance planned to ensure data accuracy and relevance. By leveraging this resource, you can contribute to the growing field of renewable energy in Uganda and help unlock its solar potential for sustainable development.</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
@@ -11057,27 +10932,11 @@
       <c r="N88" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The KinyCOMET dataset is a valuable resource for anyone looking to improve machine translation (MT) between Kinyarwanda and English. Here’s a practical guide on how to use this dataset effectively.
-1. **Immediate Use Cases**:
-   - **Automatic Evaluation of Translations**: You can use the KinyCOMET dataset to evaluate existing Kinyarwanda-English translation systems. This dataset provides 4,323 human-annotated translation pairs, allowing you to assess the quality of translations automatically rather than relying on manual reviews.
-   - **Training New Models**: If you are developing a new machine translation model, you can use this dataset to train and validate your system. The dataset is split into training, validation, and test sets, making it easy to implement in your workflow.
-   - **Quality Estimation**: The dataset can help in estimating the quality of translations produced by various MT systems, including both traditional neural networks and large language models (LLMs).
-2. **Extending or Improving the Work**:
-   - **Enhancing the Dataset**: Researchers can contribute by adding more translation pairs or by annotating additional domains, such as healthcare or legal texts, which are currently underrepresented.
-   - **Model Development**: Developers can build upon the KinyCOMET model by experimenting with different architectures or training techniques to improve translation quality further.
-   - **Cross-Language Applications**: You can explore how the methodologies used in this dataset can be applied to other low-resource languages, potentially creating a broader impact in the field of translation.
-3. **Limitations and Considerations**:
-   - **Bias and Limitations**: The dataset is limited to specific domains (education and tourism), which may not represent all contexts where Kinyarwanda is used. It’s essential to consider this when applying the dataset to other areas.
-   - **Ethical AI Assessment**: Before using the dataset for commercial purposes or in sensitive applications, it is advisable to conduct an ethical AI assessment to ensure that the translations do not propagate biases or inaccuracies.
-4. **Cost Estimates**:
-   - **Adaptation and Training Costs**: Depending on the complexity of your model and the computational resources required, costs can vary. For small-scale projects, using cloud services for training might range from $100 to $1,000, while larger projects could exceed this.
-   - **Compute Resources**: If you plan to use GPUs for training, expect to budget for cloud computing costs, which can be significant depending on the duration and scale of your training sessions.
-5. **Collaboration Opportunities**:
-   - **Partnerships with Local Universities**: Collaborating with local educational institutions can provide access to linguistic expertise and additional resources for annotation and model evaluation.
-   - **Community Engagement**: Engaging with local developers and NGOs can help in tailoring the translation tools to meet specific community needs.
-6. **Documentation and Resources**:
-   - The dataset is available on Hugging Face, and you can find documentation on how to load and use the dataset effectively. Tutorials are provided to help you get started with the KinyCOMET model.
-By leveraging the KinyCOMET dataset, development practitioners and innovators can significantly enhance the quality of Kinyarwanda-English translations, ultimately supporting better communication and understanding in various sectors.</t>
+You can immediately use the KinyCOMET dataset to enhance the quality of Kinyarwanda-English machine translations by integrating it into your translation workflows. This dataset provides 4,323 human-annotated translation quality assessments, allowing you to automatically evaluate translations without relying on time-consuming manual reviews. By using the KinyCOMET model, you can assess the quality of translations in real-time, which can significantly speed up the translation process for applications in education, tourism, and other sectors.
+To build on this resource, researchers and developers can extend the KinyCOMET model by training it with additional datasets or fine-tuning it on specific domains relevant to their work. This could involve collecting more translation pairs or incorporating user feedback to improve the model's accuracy. Collaborating with local linguists or educational institutions can also provide valuable insights and data for further development.
+When replicating or adapting this work, it’s important to consider potential limitations and biases. The dataset is based on a specific set of translation pairs and may not cover all dialects or variations of Kinyarwanda. Additionally, the quality scores are based on human assessments, which can be subjective. Therefore, conducting an ethical AI assessment before deploying the model in sensitive contexts is recommended.
+In terms of costs, building on this dataset may involve expenses related to data storage, compute resources for training models, and potential collaboration with linguists or developers. Depending on your specific needs, costs can vary widely, but initial estimates for cloud computing resources can range from a few hundred to several thousand dollars, depending on the scale of your project.
+For those interested in using KinyCOMET, documentation is available on Hugging Face, which includes tutorials on loading the dataset and using the model. Engaging with the community on platforms like Hugging Face can also lead to collaboration opportunities and shared success stories, helping to foster innovation in Kinyarwanda-English translation efforts.</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -11218,25 +11077,11 @@
       <c r="N89" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Tunga Agri-Chatbot Suite offers a valuable resource for development practitioners looking to enhance agricultural support for farmers in Rwanda. Here’s a practical guide on how to utilize and build upon this resource:
-1) **Immediate Use Cases**: The existing voicebot technology can be deployed to provide farmers with timely agricultural information via a Kinyarwanda-speaking hotline. This can include advice on pest and disease diagnosis, agro-climatic practices, and information about government support programs like crop insurance. Organizations can set up similar IVR systems to reach rural farmers who may not have internet access or literacy skills.
-2) **Extending the Work**: Researchers and developers can improve upon this project by:
-   - Expanding the dataset with more diverse agricultural topics or local dialects to enhance the voicebot's capabilities.
-   - Integrating additional features such as SMS follow-ups or mobile app support for users with smartphones.
-   - Collaborating with local agricultural experts to ensure the information provided is accurate and relevant.
-3) **Limitations and Considerations**: When replicating this project, it is important to consider:
-   - The potential biases in the dataset, which may not cover all agricultural practices or local variations.
-   - The need for an ethical AI assessment to ensure that the technology is used responsibly and does not inadvertently disadvantage any group.
-   - The importance of user feedback to continuously improve the service and address any gaps in information.
-4) **Cost Estimates**: While specific cost estimates are not provided, organizations should consider expenses related to:
-   - Adaptation of the voicebot system, which may involve hiring local experts or developers.
-   - Training costs for additional voice data collection and processing.
-   - Compute costs for hosting the IVR system, which can vary based on usage and scale.
-**Opportunities for Collaboration**: Organizations can reach out to C4IR Rwanda and KiNLP for potential partnerships. Collaborating with local NGOs or government agencies can also enhance outreach and effectiveness.
-**Documentation and Tutorials**: Technical documentation is available, detailing the dataset's structure and audio specifications. Practitioners can refer to this to understand how to implement the voicebot effectively.
-**Success Stories**: While specific success stories are not mentioned, the implementation of the IVR tool itself is a significant step towards improving agricultural support for farmers in Rwanda.
-**Long-term Maintenance**: Consideration should be given to the long-term maintenance of the system, including regular updates to the information provided and ongoing user engagement to ensure the service remains relevant and effective.
-By leveraging the Tunga Agri-Chatbot Suite, development practitioners can make a meaningful impact on agricultural support in rural communities, bridging the digital divide and enhancing access to vital information.</t>
+You can immediately use the Tunga Agri-Chatbot Suite to create a voice-based agricultural advisory service for farmers in Rwanda. By leveraging the Kinyarwanda Agricultural Text-to-Speech Dataset, you can develop a voicebot that provides critical information on pest and disease management, agro-climatic practices, and government support programs, all accessible via a simple telephone hotline. This is particularly beneficial for farmers who may not have internet access or who are not fluent in English.
+To build on this resource, researchers and developers can enhance the existing voicebot by incorporating additional agricultural topics, improving the naturalness of the voice output, or expanding the dataset with more diverse agricultural scenarios. Collaborating with local agricultural experts can help ensure that the information provided is relevant and up-to-date. Additionally, you can explore integrating feedback mechanisms to continuously improve the service based on user interactions.
+When replicating this project, it is essential to consider potential limitations, such as biases in the dataset or the need for ethical assessments to ensure that the voicebot serves all farmers equitably. The dataset includes recordings from only two voice actors, which may limit the diversity of voices and accents represented. 
+In terms of costs, building on this project may require investment in training and adaptation of the voicebot, which could range from a few hundred to several thousand dollars depending on the scale of the implementation and the resources needed for voice synthesis and infrastructure. You may also need to budget for ongoing maintenance and updates to the system.
+For further guidance, you can refer to the technical documentation provided with the dataset, which includes details on the audio files and their structure. Engaging with organizations like C4IR Rwanda and KiNLP can also provide valuable support and collaboration opportunities.</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">

</xml_diff>

<commit_message>
feat: simplify catalog inclusion, add GIZ to orgs, improve UI labels
- Simplify catalog inclusion: any non-empty text in link columns now
  shows as a disclaimer instead of requiring specific prefix phrases
- Detect disclaimer text with embedded URLs (starts with text, not http)
  and show as info callout instead of broken "Access Dataset" button
- Deduplicate merged access notes when both columns have identical text
- Add GIZ to all FAIR Forward - AI for All entries in Google Sheet (80 cells)
- Rename "Contact" to "Author/Contact" and "Editor" to "Editor of this
  information" in DetailPanel metadata
- Fix info badge not showing on cards without SDGs
- Rebuild from latest Google Sheet data
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA154"/>
+  <dimension ref="A1:AA153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,7 +632,7 @@
       <c r="P2" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Stellenbosch University
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -742,7 +742,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -756,7 +756,7 @@
       <c r="P3" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Laboratoire de Biomathématiques et d'Estimations Forestières
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -864,7 +864,7 @@
       <c r="P4" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Reiner Lemoine Institut gGmbH (RLI)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -942,7 +942,7 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>Powered by / Provided by: World Resources Institute (WRI)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -988,12 +988,12 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Datasets for transportation impact evaluation</t>
+          <t>Datasets for transportation impact evaluation in urban settings in Colombia</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Urban roadspace classification data and model</t>
+          <t>Classification data and model for transportation impact evaluation in urban settings in Colombia</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1042,30 +1042,11 @@
       <c r="N6" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This resource provides valuable datasets and tools for evaluating transportation impacts, particularly in urban settings like Bogotá. Here’s a practical guide for development practitioners and innovators looking to leverage this resource:
-1. **Immediate Use Cases and Applications**:
-   - **Urban Planning**: Use the labeled dataset to analyze road space allocation in Bogotá. This can help city planners understand how different types of road spaces (like lanes for cars, bicycles, and sidewalks) are distributed and utilized.
-   - **Traffic Management**: The model can assist in identifying congestion points and optimizing traffic flow by analyzing road usage patterns.
-   - **Infrastructure Development**: NGOs and government agencies can use the data to advocate for better infrastructure by highlighting areas lacking adequate road space for pedestrians or cyclists.
-   - **Environmental Impact Studies**: Researchers can assess how road space impacts urban heat islands or air quality by correlating road space data with environmental metrics.
-2. **Extending or Improving the Work**:
-   - **Data Expansion**: Researchers can extend the dataset by incorporating additional areas or updating it with new satellite imagery to reflect changes in urban infrastructure.
-   - **Model Enhancement**: Developers can improve the classification model by experimenting with different machine learning techniques or integrating additional data sources, such as traffic volume or demographic data, to enhance predictive capabilities.
-   - **User-Friendly Tools**: Creating more accessible interfaces or applications that allow non-technical users to interact with the data and model outputs can broaden its usability.
-3. **Critical Limitations and Biases**:
-   - **Data Bias**: The dataset is specific to Bogotá, which may not generalize well to other cities with different urban layouts or transportation needs. Users should consider local context when applying findings elsewhere.
-   - **Ethical Considerations**: Before replicating or deploying models based on this data, it is advisable to conduct an ethical AI assessment to ensure that the use of the data does not inadvertently reinforce existing biases or inequalities in urban planning.
-4. **Cost Estimates**:
-   - **Adaptation and Training**: Depending on the scale of the project, costs can vary. Basic adaptation of the model may require minimal investment if using existing infrastructure, while extensive training on new datasets could range from a few hundred to several thousand dollars, depending on compute resources.
-   - **Compute Resources**: Utilizing cloud services for training deep learning models can incur costs based on usage. A rough estimate for moderate usage might be around $100 to $500 per month, depending on the scale of data processing and model training.
-**Opportunities for Collaboration**:
-- Engaging with local universities or tech hubs can foster partnerships that enhance data analysis and model development. Collaborative projects can also attract funding from international development agencies.
-**Available Documentation and Tutorials**:
-- The GitHub repository includes a data dictionary and a command-line utility (`patch_extractor.py`) for generating image patches, which is essential for preparing data for model training. Users can refer to the repository for guidance on how to utilize these tools effectively.
-**Success Stories**:
-- While specific success stories are not detailed in the source, the high reliability (98%) of the model in classifying urban road space suggests that similar applications could yield impactful results in urban planning and transportation management.
-**Long-term Maintenance and Scaling**:
-- The ongoing maintenance of the dataset and model will depend on community engagement and contributions. Encouraging users to share their findings and improvements can help keep the resource relevant and up-to-date.</t>
+This resource is useful for anyone working on urban mobility analysis, road infrastructure planning, or land-use evaluation in cities of the Global South. The UrbanInfraDL repository provides a deep learning pipeline for segmenting road infrastructure -- roads, sidewalks, and bicycle lanes -- from satellite imagery, with a focus on Bogota, Colombia.
+You can use the provided patch extraction tool and training scripts for three segmentation architectures (DeepLabV3+, SegFormer, U-Net) to train models that classify urban road space from your own satellite imagery. This makes it possible to evaluate how road space is allocated across different transport modes and to support evidence-based advocacy for more equitable infrastructure distribution.
+Researchers and developers can extend this work by applying the pipeline to other cities with similar urban structures, or by incorporating additional annotation classes (e.g., bus lanes, green spaces) to broaden the analysis. The modular design -- separate patch extraction and model training steps -- makes it straightforward to experiment with different architectures or hyperparameters.
+Known limitations: No pre-trained model weights or sample datasets are included in the repository; you will need your own high-resolution TIFF satellite imagery and corresponding label files. The repository does not document its Python dependencies, so some setup effort is required. The codebase is a research prototype (8 commits) rather than a production-ready tool.
+Source: https://github.com/yangshao2/UrbanInfraDL</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1076,7 +1057,7 @@
       <c r="P6" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Fundación Despacio
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1189,11 +1170,8 @@
       <c r="M7" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This project focuses on measuring the amount of biomass and carbon stored in Colombian mangroves, specifically in the Vía Parque Isla de Salamanca National Natural Park. It provides an open-access dataset that can be used for machine learning applications to monitor these vital ecosystems.
-The dataset includes geospatial information collected under the LACUNA project. It is organized into two main parts: "Ground_truth," which contains field data, and "Adapted_AOI," which includes reference data layers. This information helps improve the accuracy of estimating above-ground biomass (AGB) and above-ground carbon (AGC) in mangroves.
-While the dataset is valuable for research and monitoring, users should be aware of potential limitations, such as the specific geographic focus on the Colombian Caribbean and the need for careful interpretation of the data. Ethical considerations include ensuring that the data is used responsibly and does not harm local communities or ecosystems.
-To use this dataset effectively, users should have access to basic geospatial software that can handle geodatabase formats. It is important to credit the source of this dataset when creating new products or analyses.
-For more information, visit the original source: [Invemar](https://acceso-datos-ambientales-invemar.hub.arcgis.com/maps/a0cab53befd44804923800a194c703d6/about).</t>
+Geospatial dataset for quantifying above-ground biomass (AGB) and above-ground carbon (AGC) in Colombian mangroves, focused on Vía Parque Isla de Salamanca (VIPIS) National Natural Park. Created by INVEMAR (Instituto de Investigaciones Marinas y Costeras). Data organized into "Ground_truth" (field measurements) and "Adapted_AOI" (reference data layers). Available formats: Shapefile, WFS, geodatabase, JPG, PNG, and PDF. Researchers: MSc. Venus Lorena Rocha G. and Esp. Claudia Correa (LabSIS, INVEMAR). Access is free; users must acknowledge INVEMAR as the source.
+Source: https://acceso-datos-ambientales-invemar.hub.arcgis.com/maps/a0cab53befd44804923800a194c703d6/about</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1211,7 +1189,7 @@
       <c r="P7" t="inlineStr">
         <is>
           <t>Powered by / Provided by: CTTC, INVEMAR
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1313,27 +1291,15 @@
       <c r="L8" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Africa Biomass dataset is designed to help monitor forest biomass, particularly in cocoa plantations in Côte d'Ivoire. It contains data collected from 263 plots across various regions in Côte d'Ivoire, with measurements taken between 2021 and 2023. The dataset includes the following key information:
-- **Data Format**: The dataset is structured in a table format with four columns: 
-  - **identifiant**: a unique identifier for each plot,
-  - **dates**: the date when the measurements were taken,
-  - **Latitude** and **Longitude**: the geographic coordinates of the plot,
-  - **biomass_mg_ha**: the biomass measured in tons per hectare (t/ha).
-- **Known Limitations**: The dataset is relatively small, with fewer than 1,000 entries, which may limit its representativeness and the robustness of any models developed from it. Additionally, the dataset focuses specifically on certain regions in Côte d'Ivoire, which may not capture the full diversity of biomass conditions across the country.
-- **Ethical Use**: The dataset is published under a Creative Commons Attribution 4.0 International License (cc-by-4.0), allowing users to share and adapt the data as long as proper credit is given to the original source. This promotes responsible use while encouraging collaboration and innovation.
-- **Maintenance**: The dataset is maintained by the contributors who collected the data, ensuring that it is updated and accurate as new measurements are taken or as additional data becomes available.
-This dataset is particularly valuable for development practitioners, NGOs, and government agencies focused on sustainable forest management and climate change mitigation. By using this data, organizations can monitor forest health, assess the impact of cocoa farming on forest degradation, and support reforestation efforts without the need for extensive on-the-ground surveys.</t>
+Forest aboveground biomass (AGB) dataset for Cote d'Ivoire. 263 field plots measured between 2021 and 2023. Data Type: Tabular (CSV, also available as Parquet). Columns: identifiant (plot ID), dates (measurement date), Latitude (4.04 to 9.99), Longitude (-8.09 to -2.74), biomass_mg_ha (0.91 to 391 t/ha). Biomass calculated using allometric equations from field measurements of tree height, diameter at chest height, density, and species. Dataset size: 17.8 kB. License: CC BY 4.0.
+Source: https://huggingface.co/datasets/data354/Africa_Biomass_dataset</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The AI model developed from the Africa Biomass dataset helps monitor changes in forest biomass, particularly in cocoa plantations in Côte d'Ivoire. In simple terms, it uses satellite images and ground measurements to predict how much biomass is present in these forests. This is important for understanding the health of the forest and for assessing the success of reforestation efforts.
-The model takes input data from satellite imagery (like GEDI and Sentinel-2) and ground truth measurements, which include details such as tree height, diameter, density, and species. The output is a prediction of biomass levels, measured in tons per hectare (t/ha), for different areas of the forest.
-While this model is a valuable tool, there are some limitations to consider. The dataset is relatively small, with only 263 samples, which may affect the accuracy of predictions in areas not well represented in the data. Additionally, the model may not account for all local variations in forest structure and species diversity, which could introduce biases in the predictions.
-To ensure responsible AI use, it is important for users to conduct ethical assessments when applying the model. This includes considering the potential impacts on local communities and ecosystems. Users should also be aware of the need for ongoing validation of the model's predictions against real-world observations.
-For those looking to implement this model, it is essential to have access to the necessary software and hardware that can process satellite imagery and perform the required calculations. 
-This dataset and the models derived from it are licensed under CC BY 4.0, meaning users should credit the original work when building new products or applications based on this data.</t>
+Dataset intended for building AGB estimation models using satellite imagery (GEDI, Sentinel-2) combined with ground truth measurements from 263 plots in Cote d'Ivoire. Input: satellite imagery paired with field data (tree height, diameter, density, species). Output: biomass prediction in tonnes per hectare (t/ha). Addresses the scarcity of locally-developed AGB estimation models for African tropical forests. License: CC BY 4.0.
+Source: https://huggingface.co/datasets/data354/Africa_Biomass_dataset</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1350,7 +1316,7 @@
       <c r="P8" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Data354
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1446,7 +1412,7 @@
       <c r="P9" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Data354
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1538,65 +1504,35 @@
       <c r="L10" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-Haki des femmes is an application designed to empower women in the Katanga and Lualaba provinces of the Democratic Republic of Congo by providing them with access to legal information regarding land ownership rights. The app focuses on helping women understand their rights to access, use, inherit, control, and own land, particularly in situations where they may lose these rights after the death of a loved one.
-The key characteristics of the dataset and application include:
-- **Content and Format**: The app contains legal information and support resources specifically tailored for women, presented in Kiswahili. It aims to simplify complex legal concepts to make them more accessible.
-- **Limitations and Biases**: While the app targets a specific demographic (women in DRC), it may not fully address the diverse needs of all women, particularly those who speak languages other than Kiswahili or who live in regions with different legal contexts. Additionally, the reliance on voice technology may not be suitable for all users, especially those with hearing impairments.
-- **Responsible and Ethical Use**: The developers have taken steps to ensure data privacy and security. The app does not share data with third parties, and any personal information collected is encrypted during transmission. Users have the option to request deletion of their data.
-- **Maintenance and Updates**: The app is maintained by Core23lab, with updates provided as needed. The last update was on January 17, 2026, indicating ongoing support and development.
-- **User Rights and Licensing**: Users have the right to access their data and request its deletion. The app is designed for all ages, and while specific licensing details are not provided, the focus on user privacy suggests a commitment to ethical data practices.
-Overall, Haki des femmes serves as a valuable resource for women in DRC, aiming to enhance their understanding of land rights and promote gender equity in land ownership.</t>
+Haki des Femmes is an Android app by Core23lab providing legal information on land ownership rights for women in the Katanga and Lualaba provinces of DRC. Content is in Kiswahili. Covers rights to access, use, inherit, control, and own land. The app uses voice technology for interaction. Data safety: does not share data with third parties; personal data encrypted in transit; users can request data deletion. Available for all ages on Google Play.
+Source: https://play.google.com/store/apps/details?id=org.core23lab.hdf</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-Haki des femmes is an application designed to empower women in the Katanga and Lualaba provinces of the Democratic Republic of Congo by providing them with essential legal information about land ownership rights. Many women in this region often lose access to land after the death of a family member due to a lack of knowledge about their rights. This app aims to bridge that gap by offering information and support in Kiswahili, helping women understand and assert their rights to access, use, inherit, control, and own land.
-The application uses voice technology to make legal information more accessible. Users can interact with the app by speaking, which allows them to receive guidance and answers to their questions about land rights. The expected input is voice queries from users, and the output is relevant legal information and advice tailored to their needs.
-While the app aims to provide valuable support, it is important to consider potential limitations. The effectiveness of the information provided may depend on the accuracy of the underlying legal data and the app's ability to understand various dialects or accents in Kiswahili. Additionally, users should be aware of data privacy practices, as the app may collect personal information and app performance data, although it does not share this data with third parties.
-To ensure responsible AI use, the developers have taken steps to protect user data, including encrypting data in transit and allowing users to request data deletion. 
-The app is designed to be user-friendly and is suitable for all ages. It requires a compatible smartphone to run, and users should ensure they have a stable internet connection for the best experience.
-For those looking to build new products or applications, it is important to credit the source of this work, Haki des femmes by Core23lab. 
-For more information, you can reach out to the developers at devs.core23lab@gmail.com.</t>
+Haki des Femmes is a voice-enabled Android application by Core23lab. Users speak queries in Kiswahili about land ownership rights, and the app returns relevant legal information and guidance. Designed for women in the Katanga and Lualaba provinces of DRC who risk losing land access after the death of a family member. Developer contact: devs.core23lab@gmail.com.
+Source: https://play.google.com/store/apps/details?id=org.core23lab.hdf</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-Haki des femmes is an innovative application designed to empower women in the Democratic Republic of Congo (DRC) by providing them with essential legal information regarding land ownership and rights. Here’s a practical guide for development practitioners and innovators interested in utilizing or building upon this resource.
-1) **Immediate Use Cases and Applications:**
-   - **Legal Information Access:** Users can immediately access simplified legal information about land rights in Kiswahili, helping women understand their rights to access, use, inherit, control, and own land.
-   - **Support for Women:** The app serves as a support tool for women who may be facing challenges in asserting their land rights, especially after the loss of a spouse.
-   - **Community Workshops:** NGOs and community organizations can use the app as a resource in workshops to educate women about their rights and provide guidance on legal processes.
-2) **Extending or Improving the Work:**
-   - **Localization:** Developers can expand the app to include additional local languages or dialects to reach a broader audience.
-   - **Enhanced Features:** Adding features such as a chatbot for real-time legal advice or a forum for women to share experiences and advice could enhance user engagement.
-   - **Partnerships:** Collaborating with local legal experts or NGOs can help improve the accuracy of the information provided and ensure it is culturally relevant.
-3) **Critical Limitations and Biases:**
-   - **Data Privacy:** While the app claims to protect user data, it is crucial to conduct an ethical AI assessment to ensure that user privacy is maintained, especially given the sensitive nature of legal information.
-   - **Cultural Sensitivity:** The app must be sensitive to local customs and practices regarding land ownership and gender roles to avoid reinforcing biases or misunderstandings.
-   - **Access to Technology:** Consider the digital divide in rural areas where access to smartphones and the internet may be limited.
-4) **Cost Estimates for Building On This Resource:**
-   - **Adaptation Costs:** Depending on the extent of localization and feature enhancements, costs could range from $5,000 to $20,000.
-   - **Training Costs:** If additional training data is needed for AI features, this could add another $2,000 to $10,000.
-   - **Compute Costs:** Ongoing server and maintenance costs could be approximately $100 to $500 per month, depending on user engagement and feature complexity.
-**Opportunities for Collaboration:**
-- Engage with local NGOs, legal aid organizations, and women’s rights groups to enhance the app’s content and outreach.
-- Collaborate with tech developers who specialize in voice technology to improve accessibility.
-**Available Documentation or Tutorials:**
-- While specific documentation is not mentioned, reaching out to the developer via the provided contact information could yield insights into available resources or guides.
-**Success Stories:**
-- As the app is relatively new, gathering user testimonials and success stories will be crucial for demonstrating its impact and effectiveness.
-**Plans for Long-Term Maintenance or Scaling:**
-- Continuous updates and user feedback will be essential for maintaining the app’s relevance and effectiveness. Establishing a feedback loop with users can help guide future improvements.
-By leveraging Haki des femmes, practitioners can make a significant impact on women's rights and land ownership in the DRC, fostering empowerment and legal awareness in local communities.</t>
+Haki des Femmes is a ready-to-use voice-enabled chatbot app that provides women in the Democratic Republic of Congo with accessible legal information about land ownership rights. It operates in Congolese Swahili (Kiswahili) and can be downloaded directly from the Google Play Store by searching for "Haki des femmes."
+The app is designed for community organizations, legal aid providers, and development practitioners working on women's land rights in the DRC's Katanga and Lualaba provinces. Many women in these communities are unaware of existing laws that allow them to own land, face barriers to proper documentation, or lack legal marriages that would confer inheritance rights. The chatbot simplifies this legal information through a voice interface, helping women understand the concrete steps needed to secure land ownership -- including the process of legalizing marriages as a prerequisite for land rights.
+Development practitioners can use Haki des Femmes as a model for building similar legal information tools in other contexts. The approach of combining voice technology with local-language legal guidance could be adapted for other jurisdictions or legal domains where access to legal literacy is a barrier.
+Haki des Femmes was developed by Core23Lab as part of Mozilla's 2023-24 Common Voice Kiswahili program, which funds projects using Kiswahili voice technology to support marginalized groups in Kenya, Tanzania, and the DRC. The team conducted surveys of women in Katanga and Lualaba provinces to identify specific knowledge gaps about land ownership before designing the chatbot, an approach worth replicating in similar projects. More background on the project rationale is available on the Mozilla Foundation blog.
+Known limitations: The app is specific to DRC land law and Congolese Swahili and is not directly applicable to other countries or legal systems. Voice-based interaction requires a smartphone with a microphone and internet access.
+Sources:
+- https://play.google.com/store/apps/details?id=org.core23lab.hdf
+- https://www.mozillafoundation.org/en/blog/lifting-up-women-through-land-ownership/</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Core23Lab
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -1703,7 +1639,7 @@
       <c r="P11" t="inlineStr">
         <is>
           <t>Powered by / Provided by: ESPOL University
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1809,12 +1745,8 @@
       <c r="M12" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The project focuses on using artificial intelligence to monitor the environmental impact of palm oil monoculture, shrimp aquaculture, and mining activities in Ecuador and the Galapagos Islands. In simple terms, the AI application analyzes satellite images to identify and classify different types of land use and cover, helping to understand how these industries affect the environment.
-The model expects input in the form of multi-spectral Earth observation data, which includes images captured from satellites. It produces output that consists of classifications of land use, indicating areas affected by palm oil, shrimp farming, mining, and other land transformations.
-While the dataset is valuable, there are some known limitations. The model's accuracy depends on the quality and representativeness of the training data. If certain land types are underrepresented in the dataset, the model may struggle to identify them correctly. Additionally, ethical considerations include ensuring that the data is used responsibly and does not harm local communities or ecosystems.
-To promote responsible AI use, it is important for users to conduct ethical assessments when applying the model. This includes considering the potential impacts on local populations and the environment.
-There are no specific software or hardware requirements mentioned, but users will need access to machine learning tools capable of processing the provided datasets.
-This dataset is credited to the project that created it, and users should acknowledge this source when developing new applications or products based on the data.</t>
+Land use and land cover (LULC) training dataset for Ecuador by MapBiomas Ecuador. Contains 20,000 georeferenced points with land cover classifications derived from visual interpretation of LANDSAT satellite imagery covering 1985 to 2023. An enhanced version adds conservation status information: protected area designations, indigenous territory boundaries, government forest incentive programs, and other conservation-related designations. Format: ZIP. Size: ~1.7 MB. License: CC BY 4.0.
+Source: https://www.kaggle.com/datasets/mapbiomasecuador/lulc-training-data-for-ecuador-ml/data</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1830,7 +1762,7 @@
       <c r="P12" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Ecociencia
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -1903,10 +1835,14 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t xml:space="preserve">https://space4innovation.github.io/ltomekatip/index.html </t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>https://arbimon.org/p/namunyak-conservancy-reteti-elephant-sanctuary; https://arbimon.org/p/shakiam-ecuadorian-amazon/insights</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>SDG 15</t>
@@ -1914,7 +1850,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Voice</t>
+          <t>Voice, Geospatial/Remote Sensing</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1957,7 +1893,7 @@
       <c r="P13" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Space4Innovation, Namunyak Conservancy, GEO Indigenous Alliance, MUSAP &amp; Rochester Institute for Technology
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -2071,27 +2007,26 @@
       <c r="M14" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Cashew Disease Identification (CADI AI) application is designed to help small-holder cashew farmers in Ghana detect diseases in their crops early. By using artificial intelligence, the application analyzes images of cashew plants captured by drones to identify potential issues that could affect crop health. Early detection can lead to better yields, potentially increasing production by up to 30%.
-The application expects input in the form of high-resolution images of cashew plants, which are organized into training, validation, and test sets. Each image is accompanied by annotations that specify whether the observed issues are due to diseases, insects, or abiotic factors (like environmental stress). The output of the application is a diagnosis indicating the presence of these issues, helping farmers take timely action.
-While the CADI AI application is a powerful tool, it does have limitations. The accuracy of the model depends on the quality and diversity of the images in the dataset. There may also be biases in the model if it has not been trained on a wide range of conditions or plant varieties. To address these concerns, a responsible AI assessment was conducted to identify and mitigate potential harms and biases, ensuring ethical use of the technology.
-For those interested in using the CADI AI application, it is important to acknowledge the dataset's license and credit the creators, the KaraAgro AI Foundation, and their collaborators. The dataset is openly accessible and can be utilized to develop new products or applications aimed at improving agricultural practices in Ghana and beyond. 
-For more detailed information about the dataset and its use, you can refer to the accompanying datasheet available through the provided links.</t>
+CADI-AI (Cashew Disease Identification with AI) by KaraAgro AI Foundation, funded by GIZ through MOVE and FAIR Forward initiatives on behalf of BMZ. Model: YOLOv5x object detection, trained on 3,788 drone-captured images at 640x640 input resolution. Detects 3 classes: insect damage, disease (microbial), and abiotic stress. Performance (mAP@50): 0.648 overall, 0.815 insect, 0.588 disease, 0.542 abiotic. Dataset: 4,736 images total (train/val/test) with 22,610 annotated bounding boxes in YOLO format. Dataset license: CC BY-SA 4.0. Model license: AGPL-3.0. Demo available on Hugging Face Spaces; desktop app on GitHub (karaagro/cadi-ai).
+Source: https://huggingface.co/datasets/KaraAgroAI/CADI-AI, https://huggingface.co/KaraAgroAI/CADI-AI</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately start using the Cashew Disease Identification (CADI AI) dataset to develop an application that helps small-holder cashew farmers in Ghana detect diseases in their crops early. By analyzing drone-captured images of cashew plants, you can create a tool that alerts farmers to potential diseases, enabling them to take action that could increase their yields by up to 30%. 
-To get started, download the dataset, which includes 4,736 high-resolution images annotated for object detection. The dataset is structured into training, validation, and test sets, making it ready for immediate use in machine learning applications. You can utilize the YOLO format annotations to train a model that identifies three categories: abiotic factors, insects, and diseases.
-Researchers and developers can extend this work by improving the model's accuracy or adapting it for different crops or regions. Collaborating with local agricultural experts can enhance the dataset's relevance and effectiveness. Additionally, you might consider integrating the application with mobile platforms to ensure accessibility for farmers in remote areas.
-When replicating this work, it's crucial to conduct a responsible AI assessment to identify and mitigate potential biases and harms associated with AI use in agriculture. The dataset creators have already undertaken such an assessment, which can serve as a guide for your project.
-In terms of costs, you may need to budget for cloud computing resources for model training, which can vary widely based on the scale of your application. A rough estimate for cloud compute costs could range from $100 to $1,000, depending on the duration and intensity of the training process. 
-For further guidance, you can refer to the accompanying datasheet linked in the dataset repository, which provides detailed information about the dataset's composition and methodologies. Engaging with the KaraAgro AI Foundation or GIZ could also open up opportunities for collaboration and support in scaling your application.</t>
+The CADI-AI project is useful for anyone working on cashew crop health monitoring, agricultural extension, or precision agriculture in West Africa. It provides both a labeled image dataset and a ready-to-use pre-trained model for detecting three types of cashew tree health issues -- abiotic stress, disease damage, and insect damage -- from drone-captured imagery.
+If you want to try the model immediately, a live demo is available on HuggingFace Spaces where you can upload your own cashew tree images and see detection results without any setup. For deployment in the field, a desktop application is also available on GitHub. These tools allow agricultural extension officers and agronomists to identify health issues across cashew plantations quickly, enabling targeted interventions rather than blanket treatments.
+The dataset itself contains 4,736 high-resolution drone images (1600x1300 pixels) with over 22,000 annotated instances across the three health-issue classes, licensed under CC-BY-SA 4.0. Researchers and developers can use this data to train improved detection models or to extend the approach to other tree crops. The annotations are in YOLO format, and the pre-trained YOLOv5x model achieves a mean average precision (mAP@50) of 0.65, with strongest performance on insect damage detection (0.82 mAP@50) due to its distinct visual features. Disease and abiotic stress classes are harder to distinguish because their symptoms can overlap in field conditions -- an area where further research could improve accuracy.
+A detailed datasheet documenting the data collection methodology is available via the HuggingFace dataset card. The dataset (approximately 3.78 GB) and model (approximately 173 MB) can be downloaded from HuggingFace after acknowledging the license terms.
+Cost and resources: The dataset and model are freely available. Deploying the model requires only standard compute resources. The CADI-AI project was created by the KaraAgro AI Foundation, funded by GIZ and BMZ through the FAIR Forward and MOVE programs.
+Sources:
+- https://huggingface.co/datasets/KaraAgroAI/CADI-AI
+- https://huggingface.co/KaraAgroAI/CADI-AI</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2193,32 +2128,26 @@
       <c r="L15" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Crop Disease dataset focuses on identifying diseases in maize, tomatoes, and peppers in Ghana. It contains images of various crop diseases collected from 10 districts in the Ashanti Region. The data was gathered by the RAIL-KNUST team in collaboration with the Plant Protection and Research Services Directorate (PPRSD) of the Ministry of Food and Agriculture.
-The dataset is primarily composed of image files, which can be used for training AI models to recognize and diagnose crop diseases. This can be particularly useful for farmers and agricultural practitioners looking to improve food security and adapt to climate change by quickly identifying and addressing crop health issues.
-While the dataset is valuable, it may have limitations such as potential imbalances in the representation of different diseases or crops, which could affect the performance of AI models trained on it. Users should be aware of these biases when applying the data to real-world scenarios.
-To ensure responsible and ethical use, the dataset has been made available as an open-source resource, and it was part of a data challenge that encouraged collaboration and innovation in crop disease identification. The winning models from this challenge are also accessible, providing a solid foundation for further research.
-The dataset is maintained by the RAIL-KNUST team and the PPRSD, ensuring that it is updated and relevant for users. It is published under an open license, allowing users to freely access, use, and adapt the data for their projects, provided they adhere to the terms of the license. This openness supports the goal of enhancing agricultural practices and food security in Ghana and beyond.</t>
+Afrocentric crop disease dataset by Responsible AI Lab. Contains annotated leaf images showing healthy specimens and disease-affected leaves at various crop development phases. Data Type: Image. Size: ~20 GB. License: CC BY 4.0. Version 16 (last modified March 2025). Created with a focus on African agricultural diversity.
+Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The AI-powered application for crop disease identification focuses on helping farmers in Ghana detect diseases in maize, tomatoes, and peppers. It uses images of the crops to identify signs of disease, which can help farmers take timely action to protect their harvests.
-The model expects input in the form of images of the crops. When provided with these images, it outputs information about any diseases detected, allowing farmers to understand what issues their crops may be facing.
-While the application is designed to be helpful, there are some limitations to consider. The model's accuracy may vary depending on the quality of the images and the specific diseases present in the crops. Additionally, there may be biases in the dataset if certain diseases are underrepresented, which could affect the model's performance.
-To ensure responsible AI use, ethical assessments have been conducted to address potential biases and ensure that the model is used fairly and effectively. Users are encouraged to consider these factors when applying the model in real-world situations.
-For those looking to run the application, basic software for image processing and a device capable of handling image uploads are necessary. Specific hardware requirements may depend on the scale of use, but generally, a standard computer or smartphone should suffice for individual farmers.
-This dataset and the models developed from it were created by the RAIL-KNUST team and the Plant Protection and Research Services Directorate (PPRSD) of the Ministry of Food and Agriculture in Ghana. Users should credit this source when building new products or applications based on this work.</t>
+Crop disease identification application using computer vision and deep learning on annotated leaf images from African crops. Input: leaf images. Output: disease detection and classification. Dataset created by Responsible AI Lab in collaboration with the Plant Protection and Research Services Directorate (PPRSD) of Ghana's Ministry of Food and Agriculture. Dataset openly available under CC BY 4.0.
+Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately use the Crop Disease dataset to develop an AI-powered application that helps farmers in Ghana identify diseases in maize, tomatoes, and peppers. By leveraging the images in this dataset, you can create a tool that allows farmers to upload pictures of their crops and receive instant feedback on potential diseases, enabling them to take timely action to protect their harvests.
-To extend or improve upon this work, researchers and developers can explore integrating additional datasets that include environmental factors, such as soil quality and weather conditions, which may influence disease prevalence. Collaborating with local agricultural experts can also enhance the model's accuracy and relevance to specific regional challenges.
-When replicating this work, it's important to consider potential limitations, such as the dataset's focus on specific districts in the Ashanti Region, which may not represent all agricultural conditions in Ghana. Additionally, conducting an ethical AI assessment is recommended to ensure that the application respects local farming practices and does not inadvertently cause harm.
-In terms of costs, building on this resource may require investment in cloud computing services for model training and deployment, which can range from a few hundred to several thousand dollars depending on the scale of your application. Collaborating with local universities or NGOs can help reduce costs and provide access to expertise.
-Documentation and tutorials related to the dataset and the winning models from the Zindi challenge are available, which can guide you in developing your application. Success stories from the data challenge can also provide insights into effective strategies and potential pitfalls. For long-term maintenance and scaling, consider establishing partnerships with local agricultural organizations to ensure ongoing support and updates to the application.</t>
+This dataset is intended for building and improving crop disease detection systems for smallholder farming in Ghana and similar West African contexts. It covers four crops -- cashew, cassava, maize, and tomato -- with 22 disease and health classes in total, making it one of the more comprehensive Afrocentric crop disease image collections available.
+You can use this dataset to train image classification models that identify specific diseases from leaf photos. With nearly 25,000 raw images captured from local farms in Ghana (October-December 2022), plus over 100,000 augmented images with a ready-made train/test split, the dataset is structured for direct use in standard image classification workflows. The raw images are also available separately if you prefer to apply your own augmentation or splitting strategy.
+The dataset is particularly valuable because it captures disease symptoms as they actually appear on farms in Ghana -- subtle, at various stages, and under real field conditions. This makes models trained on this data more likely to perform well in practical agricultural advisory tools than models trained on laboratory images. Agricultural technology developers, extension services, and research institutions can use it to build mobile apps or decision-support tools that help farmers identify and respond to crop diseases early.
+Researchers can extend this work by combining it with other crop disease datasets to improve cross-regional generalization, or by adding whole-plant and field-level imagery to complement the current leaf-level focus. The dataset is licensed under CC BY 4.0 and is available on Kaggle (approximately 20 GB). A free Kaggle account is required for download.
+Known limitations: The images are from specific farming regions in Ghana, so models trained exclusively on this data may not generalize well to crops grown under different conditions elsewhere. The dataset focuses on leaf-level symptoms and does not include whole-plant or field-level imagery.
+Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2228,8 +2157,8 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Responsible AI Lab of KNUST (https://rail.knust.edu.gh/) with Ghanaian Plant Protection and Regulatory Services Directorate
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), Digital Transformation Centre Ghana
+          <t>Powered by / Provided by: Responsible AI Lab of KNUST (https://rail.knust.edu.gh/), Ghanaian Plant Protection and Regulatory Services Directorate
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), Digital Transformation Centre Ghana, GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -2337,7 +2266,7 @@
       <c r="P16" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Ashesi University, Nokwary Technologies
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -2428,33 +2357,25 @@
       <c r="L17" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Accent Classification Dataset (Ghana) is a collection of audio recordings featuring native and non-native English speakers from various regions of Ghana. The dataset includes recordings of participants reading the same three scripts, which helps capture the unique accents and speech patterns found across the country. This consistency makes the dataset useful for linguistic analysis, accent classification, and research in speech recognition specifically related to Ghanaian English.
-While the dataset provides valuable insights into regional accents, it may have limitations, such as potential imbalances in representation among different regions or speaker demographics. Users should be aware of these factors when analyzing the data.
-To promote responsible and ethical use, the dataset is maintained by the Responsible AI Lab, which likely implements guidelines to ensure that the data is used appropriately and respects the rights of the speakers involved.
-The dataset is published under a specific license that outlines the rights users have when accessing and reusing the data. It is important for users to review this license to understand how they can utilize the dataset in their projects.
-Overall, this dataset offers a practical resource for those interested in studying linguistic diversity and developing applications that recognize and classify Ghanaian accents.</t>
+Audio recordings of native and non-native English speakers from various regions of Ghana. Each participant reads the same 3 predefined scripts. License: Open Database License (ODbL). Data Type: Audio (ZIP archive). Metadata includes age, ethnicity, and region of each speaker. Total size: ~177 MB. Maintained by the Responsible AI Lab.
+Source: https://www.kaggle.com/datasets/responsibleailab/accent-classification-dataset-ghana</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Discover Ghanaian Voices project provides a dataset that helps in understanding and analyzing the different accents of English spoken in Ghana. This dataset includes audio recordings of both native and non-native English speakers from various regions of Ghana. Each participant reads the same three scripts, which allows researchers to capture the unique speech patterns and accents found across the country.
-The main purpose of this dataset is to support research in areas like accent classification and speech recognition, specifically focusing on Ghanaian English. By using this dataset, developers and researchers can create applications that better understand and process the diverse ways English is spoken in Ghana.
-The input for any AI model using this dataset would be the audio recordings of the speakers, while the output would typically be the classification of the accent or the transcription of the spoken words. 
-However, there are some limitations to consider. The dataset may not cover every regional accent in Ghana, and there could be biases based on the selection of participants. It's important for users to be aware of these factors when developing applications to ensure fair and accurate results.
-To promote responsible AI use, it is crucial for developers to conduct ethical assessments when using this dataset. This includes considering the implications of accent classification and ensuring that the technology does not reinforce stereotypes or biases.
-There are no specific software or hardware requirements mentioned for running applications based on this dataset, making it accessible for various users.
-When utilizing this dataset for new projects, please credit the source: Discover Ghanaian Voices: A Dataset for AI &amp; Linguistic Research in Ghanaian accented English, available on Kaggle.</t>
+Use the audio recordings and metadata (age, ethnicity, region) to train accent classification or speech recognition models for Ghanaian English. Input: audio recordings of speakers reading 3 scripts. Output: regional accent classification or speech transcription. The dataset supports linguistic diversity analysis across Ghanaian regions.
+Source: https://www.kaggle.com/datasets/responsibleailab/accent-classification-dataset-ghana</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately use the Accent Classification Dataset (Ghana) to develop applications that improve speech recognition systems for Ghanaian English, enhancing communication tools for education, customer service, and accessibility. By analyzing the distinct regional accents captured in the dataset, you can create models that better understand and process spoken English in Ghana, making technology more inclusive for local users.
-Researchers and developers can extend this work by incorporating additional regional accents or dialects from other parts of West Africa, thereby broadening the dataset's applicability. Collaborating with local universities or linguistic departments can provide insights into regional variations and help gather more diverse audio samples. Additionally, you could explore integrating this dataset with existing speech recognition frameworks to improve their accuracy in understanding Ghanaian English.
-However, it is important to consider potential limitations and biases in the dataset. The recordings may not represent all dialects or socio-economic backgrounds within Ghana, which could affect the performance of any models trained on this data. We recommend conducting an ethical AI assessment to ensure that your applications do not inadvertently reinforce stereotypes or exclude certain groups.
-In terms of costs, building on this dataset may involve expenses related to data adaptation, model training, and computing resources. Depending on the scale of your project, you might expect costs to range from a few hundred to several thousand dollars, particularly if you require cloud computing services for processing the audio data.
-Documentation and tutorials on how to use the dataset effectively may be available through the Kaggle platform, and engaging with the Kaggle community can provide additional support and success stories from others who have utilized this dataset. Long-term maintenance and scaling of your project could benefit from partnerships with local organizations that understand the linguistic landscape and can help keep the dataset updated and relevant.</t>
+This dataset is useful for anyone working on speech recognition, natural language processing, or voice technology that needs to handle Ghanaian English accents. It contains audio recordings from native and non-native English speakers across various regions of Ghana, with each participant reading the same three predefined scripts to ensure consistency.
+You can use this data to train or fine-tune accent classification models, improve automatic speech recognition systems for Ghanaian English speakers, or conduct research on regional dialect variation within Ghana. Each audio file is paired with demographic metadata -- age, ethnicity, and region -- allowing you to segment and filter recordings by speaker background. With three recordings per participant, you can also study within-speaker consistency and across-region variation.
+The dataset is particularly relevant for developers building voice-enabled applications intended for Ghanaian users, where standard English speech models often underperform due to accent variation. By training on this data, you can build systems that are more inclusive and accurate for this population.
+Data was collected via Telegram using custom bots and scripts, with identity verification and audio quality validation steps. Participants were instructed to record in quiet environments. The dataset is approximately 185 MB, licensed under the Open Database License (ODbL), and is available on Kaggle with a free account.
+Source: https://www.kaggle.com/datasets/responsibleailab/accent-classification-dataset-ghana</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2465,7 +2386,7 @@
       <c r="P17" t="inlineStr">
         <is>
           <t>Powered by / Provided by: RAIL - KNUST (https://rail.knust.edu.gh/)
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -2566,16 +2487,8 @@
       <c r="M18" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The "Mapping Cocoa Landscapes in Ghana" project provides a dataset designed to improve the accuracy of land use and land cover change mapping in Ghana's cocoa production areas. This dataset is essential for researchers, policymakers, and practitioners focused on monitoring deforestation, landscape restoration, and sustainable land management.
-The dataset includes:
-- 21,031 geocoded cocoa farm polygons, which represent different types of cocoa farming, including agroforestry and shadeless cocoa.
-- 14,192 homogeneous cocoa polygons that are specifically shadeless cocoa plots.
-- 20,035 additional points and polygons that represent other land uses, such as informal gold mining, degraded forests, oil palm, and rubber.
-- 485 anonymized household records that provide socioeconomic context, collected through surveys.
-This information can be used as input for machine learning models that perform automated land cover classification and change detection. The output from these models can help visualize and understand land use changes over time, which is crucial for making informed decisions about land management and conservation efforts.
-However, there are some limitations to consider. The cocoa farm geospatial data does not represent exact property or farm boundaries and should not be used for legal or compliance purposes. The data was collected for training remote sensing models and may not accurately reflect the entire size of a farm. Additionally, ethical considerations were taken into account during the data collection process, ensuring that the data is anonymized and that the collection methods were responsible.
-To use this dataset effectively, users should have access to software capable of handling geospatial data, such as GIS tools. The dataset was developed with support from the Lacuna Fund, which aims to provide resources for creating labeled datasets that address urgent community problems. Users are encouraged to credit the source when building new products or applications based on this dataset.
-For more information or to report issues, users can contact the project team at the University of Ghana.</t>
+Reference dataset for training remote sensing and machine learning models for land use/land cover classification in Ghana's cocoa landscapes. Contains: 21,031 geocoded cocoa farm polygons (including 14,192 homogeneous shadeless cocoa plots), 20,035 points and polygons for other land uses (informal gold mining, degraded forest, oil palm, rubber), and 485 anonymized household survey records (derived from 4,444 individual surveys). Collected September 2024 to March 2025 using OpenForis Ground, Collect Earth Online, and KoboToolbox. License: CC BY 4.0. Format: ZIP (~30.6 MB). Created by CERSGIS (University of Ghana), with WRI and NASA SERVIR. Note: cocoa farm polygons do not represent property or farm boundaries and should not be used for legal or compliance purposes.
+Source: https://zenodo.org/records/15778396</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2610,7 +2523,7 @@
       <c r="P18" t="inlineStr">
         <is>
           <t>Powered by / Provided by: World Resources Institute (WRI), CERSGIS, NASA SERVIR, Earth System Science Center
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -2706,49 +2619,25 @@
       <c r="L19" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Agrivoltaic Dataset provides valuable insights into the performance of farming under solar panels compared to traditional open-sun farming. This dataset is particularly useful for development practitioners interested in sustainable agriculture and renewable energy solutions.
-The dataset contains real-world data comparing crop yields from farms that use solar photovoltaic (PV) systems alongside traditional farming methods. It includes measurements of harvests, which can help assess the effectiveness of agrivoltaic systems in enhancing agricultural productivity while generating electricity.
-While the dataset offers practical insights, users should be aware of potential limitations. There may be imbalances in the data, such as variations in crop types, local climate conditions, or farming practices that could affect the results. It is important to consider these factors when interpreting the data.
-To ensure responsible and ethical use, the dataset has been curated with attention to transparency and accuracy. Users are encouraged to apply the findings in ways that respect local communities and promote sustainable practices.
-The dataset is maintained by the Responsible AI Lab, which is committed to updating the information as new data becomes available. This ensures that users have access to the most current insights.
-The Agrivoltaic Dataset is published under a license that allows users to freely access and reuse the data, provided they give appropriate credit to the source. This openness encourages collaboration and innovation in the field of sustainable agriculture and renewable energy.
-Overall, this dataset is a practical resource for anyone looking to explore the benefits of agrivoltaic systems in enhancing food security and promoting clean energy in farming communities.</t>
+Pilot agrivoltaic system data from Ghana comparing crop performance under solar PV panels versus open-sun farming. License: CC BY 4.0. Data Type: Tabular. 3 experimental plots: Plot 1 (control, no PV panels), Plot 2 (agrivoltaic with raised PV panels), Plot 3 (traditional ground-mounted PV on bare land). Plots 1 and 2 divided into 9 subplots each. Crops: tomatoes, chilli pepper, eggplant (3 replicates each). Includes PV panel energy generation data and crop performance data. Total size: ~4.3 MB. Maintained by the Responsible AI Lab.
+Source: https://www.kaggle.com/datasets/responsibleailab/agrivoltaic-dataset-ghana</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Agrivoltaic Dataset provides valuable information about farming practices that combine agriculture with solar energy production. In simple terms, it compares how crops grow under solar panels versus in open sunlight. This dataset can help farmers and agricultural planners understand the benefits of using solar panels on their farms without reducing crop yields.
-The dataset includes real data on crop harvests from farms in Ghana that have implemented agrivoltaic systems. Users can input information about their own farming conditions and compare it with the data provided to see potential outcomes for their crops.
-While the dataset is useful, there are some limitations to consider. The data is specific to Ghana, so results may vary in different climates or regions. Additionally, the dataset may not cover all types of crops or farming practices, which could affect the applicability of the findings.
-For responsible use of this data, it is important to conduct ethical assessments to ensure that the insights are applied fairly and do not disadvantage any farming communities. Users should also be aware of the environmental impact of solar panel installation and ensure that it aligns with sustainable practices.
-There are no specific software or hardware requirements mentioned for using the dataset, making it accessible for a wide range of users.
-When using this dataset to build new products or applications, please credit the source: "Insights from a Pilot Agrivoltaic System in Ghana." This acknowledgment helps support the ongoing work in this area and promotes responsible sharing of knowledge.</t>
+Compare crop yields (tomatoes, chilli pepper, eggplant) under agrivoltaic panels versus open-sun control plots. The dataset provides side-by-side energy generation and harvest data from 3 plots with 9 subplots each, enabling analysis of whether raised solar PV panels affect crop productivity. Input: plot-level crop and energy measurements. Output: comparative yield and energy performance across agrivoltaic and control conditions.
+Source: https://www.kaggle.com/datasets/responsibleailab/agrivoltaic-dataset-ghana</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Agrivoltaic Dataset from Ghana provides valuable insights into the effectiveness of combining solar energy generation with agricultural practices. Here’s a practical guide for development practitioners and innovators looking to leverage this resource:
-1) **Immediate Use Cases**: 
-   - **Comparative Analysis**: You can analyze crop yields under solar panels versus traditional open-sun farming. This can help farmers understand the benefits of agrivoltaic systems in their specific contexts.
-   - **Decision-Making Tools**: Use the data to create tools that help farmers decide whether to adopt agrivoltaic systems based on expected yield improvements and energy generation.
-   - **Community Workshops**: Organize workshops to share findings with local farmers, demonstrating how agrivoltaic systems can enhance productivity and provide additional income through energy generation.
-2) **Extending the Work**: 
-   - **Broader Data Collection**: Researchers can expand the dataset by including more diverse crops, different geographical locations, and varying climatic conditions to understand the agrivoltaic system's effectiveness across different contexts.
-   - **Longitudinal Studies**: Conduct long-term studies to assess the sustainability and economic viability of agrivoltaic systems over multiple growing seasons.
-   - **Integration with Other Technologies**: Explore how agrivoltaic systems can be integrated with other technologies, such as irrigation systems or smart farming tools, to maximize benefits.
-3) **Critical Limitations and Biases**: 
-   - **Context-Specific Findings**: The dataset is based on a pilot system in Ghana, so results may not be directly applicable to other regions without considering local agricultural practices and climate conditions.
-   - **Ethical Considerations**: Before replicating the study or implementing agrivoltaic systems, consider conducting an ethical assessment to ensure that the needs and rights of local communities are respected.
-4) **Cost Estimates**: 
-   - **Initial Setup Costs**: The cost of setting up an agrivoltaic system can vary widely based on the scale of the project, but initial investments in solar panels and infrastructure can range from a few thousand to tens of thousands of dollars.
-   - **Ongoing Maintenance**: Budget for ongoing maintenance of solar panels and agricultural systems, which can be a few hundred dollars annually, depending on the scale.
-   - **Collaboration Opportunities**: Partner with local universities, NGOs, or government agencies to share resources and expertise, which can help reduce costs and improve project outcomes.
-5) **Documentation and Success Stories**: 
-   - While specific documentation for this dataset may be limited, engaging with local agricultural extension services or solar energy organizations can provide additional insights and support.
-   - Look for success stories from other regions that have implemented agrivoltaic systems to learn from their experiences and best practices.
-By utilizing the Agrivoltaic Dataset, practitioners can make informed decisions that benefit both agricultural productivity and renewable energy generation, ultimately contributing to sustainable development goals.</t>
+This dataset is valuable for anyone evaluating the feasibility of agrivoltaic systems -- combining solar energy generation with crop production on the same land -- in tropical climates. It contains measurements from a pilot installation in Ghana comparing three setups: a traditional open-sun control field, an agrivoltaic system with raised solar panels over crops, and a conventional ground-mounted solar installation on bare land.
+You can use this data to directly compare crop yields (tomatoes, chili pepper, and eggplant) under solar panels against open-sun farming, and to assess energy output from different panel configurations. The experimental design includes three replicates per crop across two growing plots (control and agrivoltaic), allowing for statistical analysis of yield differences. This makes the dataset suitable for informing feasibility assessments and investment decisions around dual-use land strategies in similar climatic zones.
+Development practitioners and policymakers can draw on these results to evaluate whether agrivoltaic systems offer a practical path to addressing both food security and clean energy access simultaneously. Researchers can extend this work by replicating the experimental design with different crop varieties, panel heights, or spacing configurations, or by combining the data with economic models to assess the financial viability of agrivoltaic installations at scale.
+Cost and resources: The dataset itself is small (approximately 4.3 MB) and freely available on Kaggle under a CC BY 4.0 license. A free Kaggle account is required for download.
+Source: https://www.kaggle.com/datasets/responsibleailab/agrivoltaic-dataset-ghana</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2759,7 +2648,7 @@
       <c r="P19" t="inlineStr">
         <is>
           <t>Powered by / Provided by: RAIL - KNUST (https://rail.knust.edu.gh/)
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -2861,50 +2750,18 @@
       <c r="M20" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Phenological Dataset for Ecological Forecasting (PheDEF Project) provides valuable information about the timing of plant life cycle events in tropical forests. This dataset helps monitor how climate change affects the availability of essential plant resources like leaves, flowers, and fruits, which are crucial for wildlife and human communities.
-The dataset includes various types of data collected over 48 weeks, such as:
-1. **Ground Monitoring Data**: This includes observations of specific trees and lianas, detailing their flowering and fruiting phases, leaf presence, and other phenological events.
-2. **Traditional Ecological Knowledge**: Information gathered from local communities about plant phenology, including the timing of leaf growth and flowering based on local knowledge.
-3. **Phenocam Data**: Derived from camera observations that track changes in plant phenology over time.
-4. **Citizen Science Contributions**: Data collected through community engagement efforts, allowing local people to contribute to the understanding of plant life cycles.
-5. **Climate Data**: Information on climate conditions that may influence plant phenology.
-The input for this dataset includes various CSV files containing structured data on plant species, their phenological phases, and associated climate conditions. Users can expect outputs that provide insights into how plant life cycles are changing over time, which can inform conservation efforts and sustainable resource management.
-While the dataset is comprehensive, it may have limitations such as potential biases in the data collection methods or gaps in the information due to varying levels of participation from local communities. Ethical considerations include ensuring that the knowledge shared by local communities is respected and credited appropriately.
-For responsible AI use, users are encouraged to conduct ethical assessments when applying this data in their projects. There are no specific software or hardware requirements mentioned, but users should be familiar with handling CSV files and data analysis tools.
-When utilizing this dataset for new projects or products, it is important to credit the source: PheDEF Project, DOI: 10.5281/zenodo.15704554. This acknowledgment helps maintain transparency and respect for the contributions of the original data collectors.</t>
+Five CSV datasets for ecological forecasting of plant phenology in Ghana's tropical forests, collected over 48 weeks (July 2024 to June 2025) at Bobiri Forest Reserve and Boabeng Fiema Monkey Sanctuary. Ground phenology dataset (28 variables): tree and liana observations including flowering phases, fruiting stages, and leaf development. Traditional Ecological Knowledge dataset (10 variables): community-reported phenology from 10 villages. Phenocam dataset (22 variables): RGB indices and vegetation indices (GRVI, exG) from camera monitoring. Citizen science classification dataset: leafing, flowering, and fruiting event classifications. Climate dataset (15 variables): wind, precipitation, temperature, humidity, and seasonal data for both sites. License: CC BY 4.0. Created by University of Energy and Natural Resources (Ghana) and University of Twente.
+Source: https://doi.org/10.5281/zenodo.15704554</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Phenological Dataset for Ecological Forecasting (PheDEF Project) provides valuable data for understanding the timing of plant life cycle events in tropical forests. This information is crucial for monitoring the health of ecosystems under climate change pressures. Here’s a practical guide for using this dataset effectively:
-1) **Immediate Use Cases**:
-   - **Ecosystem Monitoring**: Use the dataset to track the phenology of lianas and trees, which can help assess the health of forest ecosystems. This can inform conservation efforts and resource management.
-   - **Climate Impact Studies**: Researchers can analyze how climate variables affect plant phenology, providing insights into the resilience of ecosystems to climate change.
-   - **Community Engagement**: NGOs can utilize the traditional ecological knowledge data to engage local communities in conservation efforts, integrating local insights with scientific data.
-2) **Extending the Work**:
-   - **Data Integration**: Researchers can combine this dataset with other environmental data (e.g., soil health, biodiversity indices) to create a more comprehensive understanding of ecosystem dynamics.
-   - **Developing Tools**: Innovators can build user-friendly applications or dashboards that visualize phenological changes over time, making the data accessible to non-experts.
-   - **Citizen Science Projects**: Extend the citizen-science aspect by involving local communities in data collection, enhancing the dataset while fostering local stewardship of natural resources.
-3) **Limitations and Considerations**:
-   - **Data Gaps**: Be aware of potential gaps in data, especially in less monitored areas. This may affect the reliability of conclusions drawn from the dataset.
-   - **Bias in Traditional Knowledge**: The traditional ecological knowledge data may reflect biases based on the demographics of respondents (age, gender, profession). It’s important to consider these factors when interpreting the data.
-   - **Ethical Considerations**: Before using the dataset for research or applications, consider conducting an ethical assessment, especially if involving local communities or sensitive ecological areas.
-4) **Cost Estimates**:
-   - **Data Access**: The dataset is freely available, which reduces initial costs.
-   - **Adaptation and Training**: Depending on the complexity of the tools developed, costs can range from a few hundred to several thousand dollars for software development and training.
-   - **Compute Resources**: If extensive data processing or modeling is required, budget for cloud computing services, which can vary widely based on usage.
-**Collaboration Opportunities**:
-- Partner with local universities or research institutions to leverage expertise and resources.
-- Collaborate with NGOs focused on conservation to apply findings in real-world contexts.
-**Documentation and Support**:
-- The dataset includes metadata that describes the variables, which is essential for understanding how to use the data effectively.
-- Look for tutorials or guides on data analysis techniques relevant to phenological data, which may be available through academic institutions or online platforms.
-**Success Stories**:
-- While specific success stories from this dataset are not detailed, similar datasets have been used globally to inform conservation strategies and policy decisions, demonstrating the potential impact of such resources.
-**Long-term Maintenance**:
-- The dataset is hosted on a stable platform (Zenodo), which suggests a commitment to long-term availability. However, ongoing updates or expansions of the dataset may depend on continued funding and research efforts. 
-By leveraging this dataset, development practitioners and innovators can make informed decisions that support sustainable ecosystem management and community engagement in conservation efforts.</t>
+The PheDEF dataset offers a rich, multi-source foundation for ecological forecasting and phenological research in West African tropical forests. It covers 48 weeks of observations (July 2024 -- June 2025) from two sites in Ghana -- Bobiri Forest Reserve and Boabeng Fiema Monkey Sanctuary -- and brings together ground phenology, satellite imagery, climate records, traditional ecological knowledge, phenocam indices, and citizen science classifications, all linked by common date and site identifiers.
+You can use this resource to investigate how weather patterns drive flowering and fruiting timing by cross-referencing the ground phenology observations with co-located climate data (temperature, precipitation, humidity, wind, dew point). Researchers working on remote sensing validation can compare the satellite-derived vegetation indices (NDVI, EVI, GNDVI, and seven others from Sentinel-2, Landsat, and MODIS imagery) against field-observed phenological stages to assess how well space-based monitoring captures on-the-ground seasonal changes. The citizen science classifications -- over 100 MB of volunteer labels for leafing, flowering, and fruiting events -- can be benchmarked against the expert ground-truth observations to study the reliability of community-contributed data.
+A distinctive feature of PheDEF is its traditional ecological knowledge component: community interviews from 10 villages documenting local phenological calendars, including respondent demographics. This opens the door to research that integrates Indigenous and scientific knowledge systems for forest management and conservation planning.
+The ground observation data is available as CSV files from Zenodo (https://zenodo.org/records/15704554), while the satellite imagery and vegetation indices (~30 GB for Sentinel-2, ~1.5 GB for Landsat, plus MODIS GeoTIFFs) are hosted on 4TU.ResearchData. All data is openly accessible and free to download under a CC BY 4.0 license. Detailed documentation on data formats and variable definitions is provided at each repository.
+Sources: https://zenodo.org/records/15704554, https://doi.org/10.4121/d97e338b-dc94-4e3d-a473-6dd3d4b48898.v1, https://doi.org/10.4121/9e6b4bca-f3d3-40f3-a8f5-4f71f7790c2f.v1, https://doi.org/10.4121/7e6d7ca3-060d-4ca5-bd83-d779b598c11d.v1</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2915,7 +2772,7 @@
       <c r="P20" t="inlineStr">
         <is>
           <t>Powered by / Provided by: University of Energy and Natural Resources (Ghana), University of Twente
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ</t>
         </is>
       </c>
@@ -2947,8 +2804,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3018,38 +2875,26 @@
       <c r="L21" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This dataset is designed to help farmers in Ghana and Uganda make informed decisions about cashew, cocoa, and coffee production. It contains 14,870 drone images with detailed annotations, which can be used for estimating crop yields, detecting crop types, counting fruits, and assessing fruit maturity stages (unripe, ripe, and spoiled).
-The dataset is divided into two main sections: one for Ghana and another for Uganda. The Ghana section includes 8,784 high-resolution images (16,000 by 13,000 pixels) of cashew and cocoa trees. The Uganda section contains 6,086 images (4,000 by 3,000 pixels) of cashew and coffee trees. Each image is paired with a YOLO format text file that includes class labels and bounding box coordinates for various crop features.
-The dataset has been created with input from agricultural scientists and is maintained by the KaraAgro AI Foundation and partners. It is published under a Creative Commons Attribution 4.0 International License (CC BY 4.0), allowing users to share and adapt the data as long as proper credit is given.
-While the dataset is comprehensive, users should be aware of potential limitations, such as the possibility of biases in the data collection process or imbalances in the number of images for different crop types and maturity stages. The dataset aims to adhere to responsible and ethical use principles, ensuring that it is accessible and usable for a wide range of applications in agricultural research and practice.
-Overall, this dataset is a valuable resource for development practitioners, NGOs, and government agencies looking to enhance agricultural productivity and support farmers in making better business decisions.</t>
+14,870 drone images with YOLO-format annotations for crop yield estimation. License: CC BY 4.0. Data Type: Image + Text annotations. Ghana subset: 8,784 images (16,000 x 13,000 px) covering cashew (4,715 images) and cocoa (4,069 images). Uganda subset: 6,086 images (4,000 x 3,000 px) covering cashew (3,086 images) and coffee (3,000 images). Cashew labels: cashew_tree, flower, immature, mature, ripe, spoilt. Cocoa labels: cocoa-tree, cocoa-pod-immature, cocoa-pod-mature-unripe, cocoa-pod-riped, cocoa-pod-spoilt. Coffee labels: coffee, unripe, ripening, ripe, spoilt. DOI: 10.57967/hf/0959. Created by KaraAgro AI Foundation, funded by Lacuna Fund.
+Source: https://huggingface.co/datasets/KaraAgroAI/Drone-based-Agricultural-Dataset-for-Crop-Yield-Estimation</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Drone-based Agricultural Dataset for Crop Yield Estimation is designed to help farmers in Ghana and Uganda make informed decisions about their cashew, cocoa, and coffee crops. This dataset contains 14,870 drone images that have been carefully labeled to identify different aspects of these crops, such as the type of tree, the stage of fruit maturity (unripe, ripe, spoiled), and the presence of flowers.
-The dataset is structured to support various applications, including estimating crop yields, detecting crop types, and counting fruits. It provides a rich source of visual data that can be used to train AI models to analyze agricultural conditions and improve farming practices.
-Users can expect the following from the dataset:
-- **Input**: The dataset includes high-resolution images of crops, each paired with annotations that specify what is present in the image (e.g., types of trees and fruit stages).
-- **Output**: AI models trained on this dataset can produce insights such as estimated crop yields, identification of crop types, and detection of fruit maturity stages.
-While the dataset is comprehensive, there are some limitations to consider:
-- The dataset may not cover all possible environmental conditions or variations in farming practices, which could affect the accuracy of models trained on it.
-- Ethical considerations include ensuring that the data is used responsibly and does not lead to negative impacts on local farming communities.
-To promote responsible AI use, the dataset creators have followed ethical guidelines and principles, ensuring that the data is findable, accessible, interoperable, and reusable (FAIR). Users are encouraged to credit the source when utilizing this dataset for their projects.
-For those interested in using this dataset, it is important to have access to appropriate software and hardware capable of processing high-resolution images and running AI models. The dataset is available under a Creative Commons license, allowing for broad use while requiring attribution to the original creators.
-This dataset was developed by the KaraAgro AI Foundation in collaboration with agricultural scientists and is supported by the Lacuna Fund. Users can access and download the dataset through the provided DOI link for further exploration and application in agricultural research and development.</t>
+Train object detection models (YOLO format) for crop yield estimation, crop type detection, fruit counting, and maturity stage classification. Input: high-resolution drone images of cashew, cocoa, and coffee trees. Output: bounding box predictions with class labels for tree type and fruit maturity (immature, mature/unripe, ripe, spoilt, flower). Ghana instance counts include: cashew_tree (1,107), flower (16,757), immature (11,766), mature (4,244), ripe (11,721), spoilt (518), cocoa-pod-mature-unripe (10,786), cocoa-tree (2,831), cocoa-pod-immature (2,401), cocoa-pod-riped (4,193), cocoa-pod-spoilt (2,018).
+Source: https://huggingface.co/datasets/KaraAgroAI/Drone-based-Agricultural-Dataset-for-Crop-Yield-Estimation</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-To enhance crop yield estimation for cashew, cocoa, and coffee farmers in Ghana and Uganda, you can immediately utilize the Drone-based Agricultural Dataset to develop models that estimate yields based on drone imagery. This dataset contains 14,870 high-resolution images with detailed annotations, allowing you to implement applications such as crop type detection, fruit counting, and maturity stage classification.
-You can start by using existing tools like the YOLO (You Only Look Once) framework for object detection. With the provided annotations, you can train a model to identify and classify different growth stages of crops, which can help farmers make informed decisions about harvesting and resource allocation. This can lead to improved productivity and better financial outcomes for farmers.
-For researchers and developers looking to extend this work, consider integrating additional data sources, such as weather patterns or soil quality metrics, to enhance the accuracy of yield predictions. Collaborating with local agricultural experts can also provide insights into specific challenges faced by farmers, allowing for the development of tailored solutions.
-While the dataset is robust, there are limitations to consider. The images are specific to certain regions and may not represent all agricultural conditions. It's advisable to conduct an ethical AI assessment to ensure that the models developed do not inadvertently reinforce biases or overlook local agricultural practices. Additionally, the dataset may not cover all potential crop diseases or pests, which could affect yield predictions.
-In terms of costs, building on this dataset may require investment in cloud computing resources for model training, which can range from a few hundred to several thousand dollars depending on the scale of your project. If you plan to adapt the dataset or develop new models, consider budgeting for data storage, processing, and potential collaboration with local institutions.
-For further guidance, explore the accompanying documentation and datasheet linked in the dataset repository. This resource provides detailed information on data collection methodologies and variable definitions, which can be crucial for effective model development. Engaging with local agricultural organizations can also foster collaboration and ensure that the solutions developed are practical and impactful for the communities involved.</t>
+This drone-based agricultural dataset is designed for anyone working on crop yield estimation, crop health monitoring, or object detection in smallholder farming contexts. It contains 14,870 high-resolution drone images of cashew, cocoa, and coffee crops from Ghana and Uganda, each paired with bounding box annotations that label individual fruits by maturity stage -- immature, mature, ripe, and spoilt.
+You can use these images to train models that count and classify fruits from aerial imagery, enabling plot-level yield estimation without manual field counts. The maturity-stage labels also support crop health monitoring, since spoilt fruit detection can flag disease or post-harvest loss issues early. Because the dataset covers three different cash crops across two countries, it lends itself to cross-crop and cross-region transfer learning experiments -- for example, testing whether a model trained on Ghanaian cashew generalises to Ugandan cashew, or adapting a cocoa detector for coffee.
+Researchers and developers should note that the Ghana images (16,000 x 13,000 px, collected by KaraAgro AI) are significantly higher resolution than the Uganda images (4,000 x 3,000 px, collected by Makerere AI Lab, Uganda Marconi Lab, and NCRRI). This difference may require separate preprocessing pipelines or resolution-aware training strategies if combining both sources.
+The annotations use the YOLO object detection format, so the data can be loaded directly into standard YOLO-based training pipelines. The dataset repository also includes PDF documentation covering collection methodology and variable definitions.
+The full dataset (~45.6 GB) is openly available on HuggingFace under a CC BY 4.0 license: https://huggingface.co/datasets/KaraAgroAI/Drone-based-Agricultural-Dataset-for-Crop-Yield-Estimation
+Source: https://huggingface.co/datasets/KaraAgroAI/Drone-based-Agricultural-Dataset-for-Crop-Yield-Estimation</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -3060,7 +2905,7 @@
       <c r="P21" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Kara Agro (https://karaagro.com/) , Makerere AI Lab, Marconi Lab, National Coffee Research Institute, National Crops Resources Research Institute
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -3128,16 +2973,8 @@
 - language dataset created: Dhuluo ?</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Balthas to clarify with Daniel, if dataset was created !!!</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Balthas</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>SDG 10</t>
@@ -3161,7 +2998,7 @@
       <c r="P22" t="inlineStr">
         <is>
           <t>Powered by / Provided by:
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -3252,27 +3089,15 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-IMARIKA is a project by Strathmore University’s iLabAfrica that focuses on providing accurate, local weather information to farmers in rural Kenya. The dataset generated through this project is designed to help small-holder farmers receive location-specific weather guidance, moving away from generic information.
-The dataset includes real-time weather data that is processed through a pipeline. It fetches data from an external weather API every three hours and processes it using Apache Spark. The data is cleaned, validated, and stored in PostgreSQL, with both raw and processed versions available. Key features of the dataset include:
-- **Real-time Data Ingestion**: Weather data is updated every three hours.
-- **Data Processing**: The pipeline includes data cleaning, mean-based imputation for missing values, and anomaly detection using Z-scores.
-- **Daily Aggregation**: The dataset provides daily summaries and statistics of weather conditions.
-While the dataset is robust, there may be limitations related to the accuracy of the external weather API and potential biases in the data collection process, which could affect the reliability of the recommendations made to farmers.
-To ensure responsible and ethical use, the project emphasizes data quality through comprehensive cleaning and validation processes. Users are encouraged to follow ethical guidelines when utilizing the data for advisory services.
-The dataset is maintained and updated by the iLabAfrica team at Strathmore University. Users interested in accessing the data will need to create an account with the weather API used in the project, which is a prerequisite for running the data processing pipeline.
-The dataset is published under a license that allows users to access and reuse the data, but specific rights and restrictions should be confirmed by reviewing the licensing terms provided in the project documentation.</t>
+Weather data pipeline for rural Kenya. Fetches readings from the Wireless Planet API (api.wirelessplanet.co.ke) every 3 hours. License: MIT. Data Type: Time-series weather readings. Processing: Apache Spark 3.3.0 structured streaming with data cleaning, mean-based imputation, and Z-score anomaly detection (threshold: 10.0). Storage: PostgreSQL 14 (raw table: weather_raw; processed table: weather_clean with device_id, date, temperature, wind, precipitation, anomaly flags). Throughput: ~40-50 records/second, &lt;30 seconds end-to-end latency. Daily aggregation compresses ~1,000 raw readings into ~35 daily summaries. Requires Docker, 8GB+ RAM, and a weather API account.
+Source: https://github.com/iLab-DSU/imarika-weather-pipeline</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-IMARIKA is a project developed by Strathmore University’s iLabAfrica that aims to improve the way farmers in rural Kenya access weather information. It does this by creating low-cost automatic weather stations that provide accurate, local weather data. This information is crucial for small-holder farmers, allowing them to receive tailored advice instead of relying on generic weather forecasts.
-The IMARIKA system works by collecting weather data from an external API every three hours. It processes this data in real-time using a series of steps that include cleaning the data, filling in any missing information, and detecting any anomalies. The processed data is then stored in a database, where it can be accessed for generating daily weather summaries and actionable recommendations for farmers.
-The input for the IMARIKA system is weather data from an external API, while the output includes both raw and processed weather data, as well as daily summaries that can be used to inform farmers about local weather conditions.
-While the system is designed to provide accurate and timely weather information, there are some limitations to consider. The quality of the output depends on the accuracy of the input data from the weather API. Additionally, the system may not account for all local variations in weather patterns, which could affect the recommendations provided to farmers.
-To ensure responsible AI use, the project incorporates ethical assessments and focuses on data quality through comprehensive cleaning and validation processes. This helps to minimize biases and improve the reliability of the information provided to farmers.
-For those interested in using the IMARIKA system, it requires certain software and hardware. Users will need Docker and Docker Compose installed on their machines, along with at least 8GB of RAM for optimal performance. Additionally, a weather API account is necessary to access the data.
-When building new products based on this work, users should credit the original source, which is the IMARIKA weather pipeline available on GitHub.</t>
+Two components: (1) Weather Pipeline -- Apache Spark streaming processor ingests weather API data via Kafka, cleans it, detects anomalies, and stores raw + processed data in PostgreSQL. Produces daily weather summaries per device. Stack: Docker Compose, Kafka, Spark 3.3.0, PostgreSQL 14, Python. (2) Agricultural AI Assistant -- LangGraph-based advisory chatbot for 6 East African crops (beans, cassava, finger millet, maize, sorghum, sweet potatoes). Uses QLoRA-fine-tuned Llama 3.2 3B Instruct model, a knowledge graph (30+ nodes, 95+ edges), Chroma vector database, and OpenWeather API integration. Supports English and Swahili. Runs locally via Ollama. Requires 4GB+ GPU VRAM for inference or CPU (slower).
+Source: https://github.com/iLab-DSU/imarika-weather-pipeline, https://github.com/iLab-DSU/Agricultural-Recommendations-Chat</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -3286,7 +3111,7 @@
       <c r="P23" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Strathmore University’s iLabAfrica
-Catalyzed by: Smart Africa (https://smartafrica.org/), FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), Intellecap, intel.liftoff, Climate Change AI; Mozilla Foundation
+Catalyzed by: Smart Africa (https://smartafrica.org/), FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ , Intellecap, intel.liftoff, Climate Change AI; Mozilla Foundation
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/), Gates Foundation</t>
         </is>
       </c>
@@ -3409,7 +3234,7 @@
       <c r="P24" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Audiopedia
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -3524,28 +3349,22 @@
       <c r="N25" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can start using the VAYU project to combat air pollution in your community by leveraging the hyperlocal air quality data collected through citizen scientists and IoT-based sensors. Here are some practical steps and considerations:
-1. **Immediate Use Cases**: 
-   - **Monitor Air Quality**: Utilize the VAYU Android app and citizen portal to access real-time air quality data in your area. This can help you identify pollution hotspots and inform community members about air quality levels.
-   - **Targeted Interventions**: Use the data to advocate for specific actions from local authorities, such as increased regulation of identified pollution sources or the implementation of green spaces in high-risk zones.
-   - **Community Engagement**: Mobilize local volunteers to participate in data collection, enhancing community awareness and involvement in air quality issues.
-2. **Extending the Work**:
-   - **Enhance Data Collection**: Researchers and developers can improve upon the existing sensor network by integrating additional sensors or developing new applications that analyze the data in different ways, such as correlating air quality with health outcomes.
-   - **Collaborate with Local Authorities**: Work with local governments to create policies based on the data collected, ensuring that interventions are data-driven and effective.
-   - **Develop Educational Programs**: Create workshops or materials that educate the community about air pollution and how they can contribute to monitoring efforts.
-3. **Limitations and Considerations**:
-   - **Data Bias**: Be aware that the data collected may reflect the locations of sensors rather than a comprehensive view of air quality across all areas. It’s important to consider this when making decisions based on the data.
-   - **Ethical AI Assessment**: Before replicating or extending the project, conduct an ethical assessment to ensure that the use of AI and data collection respects community privacy and consent.
-4. **Cost Estimates**:
-   - **Sensor Deployment**: The cost of low-cost sensors can vary, but budget for approximately $100 to $300 per sensor, depending on the type and features.
-   - **Data Management**: Consider costs for data storage and processing, which could range from a few hundred to several thousand dollars annually, depending on the scale of your project.
-   - **Training and Adaptation**: If you plan to train local volunteers or staff, allocate funds for training materials and sessions, which could cost around $500 to $1,500.
-5. **Collaboration Opportunities**: 
-   - Engage with local universities or NGOs that focus on environmental issues to share resources and expertise.
-   - Partner with tech companies interested in social impact to enhance the technological aspects of the project.
-6. **Documentation and Support**: 
-   - Check the VAYU website for available documentation on how to use the app and portal effectively. Tutorials may also be available to guide new users through the data collection and analysis processes.
-By taking these steps, you can effectively utilize the VAYU project to address air pollution in your community while also contributing to a larger movement towards cleaner air and better public health.</t>
+VAYU OpenAir provides an end-to-end open-source platform for hyperlocal air pollution mapping, built through a collaboration between UNDP, GIZ, the Government of India, the University of Nottingham, Development Alternatives, D-Coop, and citizen scientists across India. The platform includes open data, open algorithms, and open software from hyperlocal mapping campaigns in Patna and Gurgaon.
+The core platform consists of three components: a mobile app for field-level data collection and viewing air quality readings, a web portal dashboard for visualising pollution data, and a backend API serving data to both interfaces. All source code is available at github.com/undpindia/VAYU_OpenAir under an MIT license.
+Practitioners can use VAYU OpenAir in several ways. If you are working on urban air quality in Indian cities or comparable contexts, you can deploy the existing platform to run your own hyperlocal mapping campaigns -- the mobile app supports citizen-science data collection, while the web portal provides ready-made visualisation tools for stakeholders and policymakers. If you already have air quality data and want to build predictive or analytical tools on top of it, several community-built open-source projects demonstrate what is possible:
+- **vayu-gnn** -- A Graph Neural Network that predicts hyperlocal pollutant levels up to 8 hours ahead by combining VAYU sensor readings with weather data, elevation, river distance, and urban density features. Available under GPL-3.0 at github.com/EconAIorg/vayu-gnn.
+- **VayuAssist** -- A RAG-based chatbot designed for government policymakers, providing air quality insights, AQI trend analysis, and mitigation strategies. Built with Streamlit and OpenAI GPT-3.5 Turbo. Available under MIT at github.com/Alphawarrior21/VayuAssist.
+- **ClearSky** -- Jupyter Notebooks for predictive pollution analysis with 3D visualisation. Available at github.com/akbp24/ClearSky.
+- **vayu_airnode** -- ARIMA time-series analysis for individual pollutants (CH4, CO, CO2, NO2, PM10, PM2.5) plus temperature and humidity, with a Streamlit interface. Available under Apache-2.0 at github.com/sherwaldeepesh/vayu_airnode.
+These community tools illustrate concrete extension points: from short-term pollution forecasting to policy-support chatbots to time-series analysis of specific pollutants. Developers looking to extend the ecosystem can build on any of these as starting points.
+Cost and resources: The platform and all community tools are open-source, so the primary costs are compute infrastructure for hosting the backend and any ML model training. Setup documentation is provided in each repository.
+Sources:
+- https://vayu.undp.org.in/
+- https://github.com/undpindia/VAYU_OpenAir
+- https://github.com/EconAIorg/vayu-gnn/tree/main
+- https://github.com/Alphawarrior21/VayuAssist
+- https://github.com/akbp24/ClearSky
+- https://github.com/sherwaldeepesh/vayu_airnode</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3556,7 +3375,7 @@
       <c r="P25" t="inlineStr">
         <is>
           <t>Powered by / Provided by: UNDP India
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -3691,7 +3510,7 @@
       <c r="P26" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Indian Institute of Science (IISc)
-Catalyzed by: Bhashini, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: Bhashini, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -3827,7 +3646,7 @@
       <c r="P27" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Wadhwani AI
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -3945,7 +3764,7 @@
       <c r="P28" t="inlineStr">
         <is>
           <t>Powered by / Provided by: GramVaani
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4048,7 +3867,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -4059,7 +3878,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -4071,7 +3890,7 @@
       <c r="P29" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Karya Inc.
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4134,7 +3953,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -4170,8 +3989,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4194,7 +4012,7 @@
       <c r="P30" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Green
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4331,7 +4149,7 @@
       <c r="P31" t="inlineStr">
         <is>
           <t>Powered by / Provided by: WRMS - Weather Risk Management Services (https://wrmsglobal.com/), ZINDI (https://zindi.africa/), Vertify Earth (https://vertify.earth/)
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4433,7 +4251,7 @@
       <c r="P32" t="inlineStr">
         <is>
           <t>Powered by / Provided by: GramVaani
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4527,22 +4345,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4554,7 +4372,7 @@
       <c r="P33" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Vertify Earth
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -4645,7 +4463,7 @@
       <c r="P34" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Bonn Consulting, Frauenhofer Institute
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -4777,7 +4595,7 @@
       <c r="P35" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Indian Institute of Science (IISc), Artpark
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -4888,7 +4706,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -4900,7 +4718,7 @@
       <c r="P36" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Vertify Earth, Earth Analytics India Pvt Ltd, Balipara Foundation, Alsisar Impact
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5033,7 +4851,7 @@
       <c r="P37" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Bappenas, Prosa.ai
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5182,7 +5000,7 @@
       <c r="P38" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Bappenas
-Catalyzed by: FAIR Forward - AI for All, HCSA, Seknas JKPP
+Catalyzed by: FAIR Forward - AI for All, GIZ, HCSA, Seknas JKPP
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5293,12 +5111,8 @@
       <c r="M39" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The project focuses on developing voice technologies for three Indonesian languages: Balinese, Bugis, and Minangkabau. It aims to create AI models that can understand and generate dialogue in these languages, which have been largely overlooked in the field of artificial intelligence.
-The NusaDialogue dataset is a key resource for this project. It contains 10,000 pairs of dialogues and summaries for each of the three languages. This means that the model can take a conversation as input and produce a summary or respond in a way that is contextually relevant. The dialogues cover a wide range of topics, including culture and occupations, making the model versatile for various applications.
-However, there are some limitations to be aware of. The existing focus on simpler tasks like translation and sentiment analysis means that more complex dialogue tasks are still underdeveloped. This could lead to challenges in accurately understanding and generating nuanced conversations in these languages.
-Ethical considerations are important in this project, especially given the underrepresentation of these languages in AI. Steps have been taken to ensure responsible AI use, although specific ethical assessments are not detailed in the available information.
-To run the models effectively, users may need access to certain software and hardware, but specific requirements are not mentioned. 
-When using this dataset or building new products based on it, users should credit the original source, which is available at Hugging Face: https://huggingface.co/datasets/prosa-text/nusa-dialogue.</t>
+Pretrained Model: IndoBERT-Nusa, a BERT language model fine-tuned from indobert-large-p2 on Balinese, Buginese, and Minangkabau data. Framework: PyTorch / HuggingFace Transformers. License: CC-BY-SA 4.0. Tasks: fill-mask, topic classification, language identification. Topic classification F1 scores: Balinese 84.23, Buginese 82.03, Minangkabau 86.30. Training Data: NusaTranslation dataset (~140,000 sentence pairs per language, Indonesian to target language). Dialogue Data: NusaDialogue provides ~10,000 dialogue-summary pairs per language (3 million+ words total) across 16 topic categories, annotated by 100 qualified native speakers. Code for AI Models: load via HuggingFace (`prosa-text/indobert-nusa`).
+Source: https://huggingface.co/datasets/prosa-text/nusa-dialogue, https://huggingface.co/datasets/prosa-text/nusa-translation, https://huggingface.co/prosa-text/indobert-nusa</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -5320,7 +5134,7 @@
       <c r="P39" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Prosa.ai
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5419,11 +5233,8 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This dataset, known as Weather Data, is a collection of environmental condition records from monitoring points in Balai Silvofishery Maros Regency, South Sulawesi, and Pulo Aceh, Aceh Province, Indonesia. It includes key weather parameters such as temperature, humidity, rainfall, light intensity, and wind speed. The data is intended to help researchers observe daily weather changes, analyze local climate patterns, and support environmental modeling.
-The dataset has some known limitations. Data from Pulo Aceh is incomplete due to challenges like frequent power outages and limited internet access. Additionally, sensors in open sea areas face interference from natural elements and marine life. Key issues include low variability in data, with temperature consistently at 27.7°C and humidity around 80%. There are also high proportions of missing values for critical variables like pressure and wind speed, which limits the dataset's effectiveness for machine learning applications. Furthermore, the data has irregular timestamps, complicating time-series analysis.
-For responsible and ethical use, users should be aware of these limitations and consider them when implementing AI or machine learning models. It is recommended to improve hardware to ensure consistent reporting of key parameters and to collect at least one full year of data to capture seasonal patterns.
-The dataset is maintained by the project team and is updated as new data becomes available. It is published under the CC-BY-SA 4.0 license, allowing users to share and adapt the data, provided they give appropriate credit and share any derivative works under the same license. For commercial use, users must contact the project team for permission.
-For any questions or further information, users can reach out to the support team at infonesiainsan@gmail.com.</t>
+License: CC-BY-SA 4.0. Data Type: Environmental monitoring records. Locations: Balai Silvofishery, Maros Regency, South Sulawesi Province and Pulo Aceh, Aceh Besar Regency, Aceh Province, Indonesia. Key Variables: temperature, humidity, rainfall, light intensity, wind speed. Collection period: since August 2025 (~7 months of data). Format: compressed archives (WS_MAROS_April-November2025.zip, WS_PULO_ACEHwoNew.txz). Known data quality issues: pressure and wind speed values entirely absent; temperature constant at 27.7C; humidity around 80%; irregular data intervals; Pulo Aceh data incomplete due to power outages and limited internet. Contact: infonesiainsan@gmail.com.
+Source: https://github.com/insaninfonesia/WeatherData</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5440,7 +5251,7 @@
       <c r="P40" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Common Room Networks Foundation https://commonroom.info/
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5469,8 +5280,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -5571,7 +5382,7 @@
       <c r="P41" t="inlineStr">
         <is>
           <t>Powered by / Provided by: RECOFTC
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5715,7 +5526,7 @@
       <c r="P42" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Local Development Research Institute (LDRI)
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5787,15 +5598,10 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Daniel
-The chatbot is currently being redeveloped from RASA to RAG - hence no link available atm (DB, 28 Nov 25)</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Daniel</t>
-        </is>
-      </c>
+          <t>Chatbot is currently redeveloped. Please contact the responsible authors for updates and access to the data: support@think.ke</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>SDG 16</t>
@@ -5808,7 +5614,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>THiNK (https://think.ke/)</t>
+          <t>THiNK (support@think.ke)</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -5837,7 +5643,7 @@
       <c r="P43" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Tech Innovators Network Kenya (THiNK)
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5905,11 +5711,14 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Daniel.
-Update (28 Nov, DB): I wrote Brian Omwenga with Florence, Emmanual and Jonas in CC to ask for a link and update on Paza Sauti. FYI Chenai does not work for Mozilla anymore and will not be in a position to assist.</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>Current publishing status unclear. Please contact the responsible authors for an update and access to the data: support@think.ke</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Current publishing status unclear. Please contact the responsible authors for an update and access to the data: support@think.ke</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>SDG 10, SDG 5, SDG 2</t>
@@ -5922,7 +5731,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Tech Innovators Network Ltd</t>
+          <t>THiNK (support@think.ke)</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -5937,7 +5746,7 @@
       <c r="P44" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Tech Innovators Network Kenya (THiNK)
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -6014,11 +5823,14 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Daniel
-running project: THiNK has created an MVP that is being integrated with eCitizen (as of 28 Nov 2025, DB)</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>Dataset/Use-Case has been developed as an MVP that is being integrated with eCitizen. Current publishing status unclear. Please contact the responsible authors for an update and access to the data: support@think.ke</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Dataset/Use-Case has been developed as an MVP that is being integrated with eCitizen. Current publishing status unclear. Please contact the responsible authors for an update and access to the data: support@think.ke</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>SDG 10</t>
@@ -6031,7 +5843,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>THiNK (https://think.ke/)</t>
+          <t>THiNK (support@think.ke)</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -6046,7 +5858,7 @@
       <c r="P45" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Tech Innovators Network Kenya (THiNK)
-Catalyzed by: FAIR Forward - AI for All &amp; Digital Transformation Centre Kenya
+Catalyzed by: FAIR Forward - AI for All, GIZ &amp; Digital Transformation Centre Kenya
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6143,12 +5955,8 @@
       <c r="M46" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The project focuses on creating a dataset that helps translate Kiswahili, Kenya's national language, into three indigenous languages: Kidaw'ida, Kalenjin, and Dholuo. This is important because these languages are at risk of disappearing, especially Kidaw'ida, which has only about 400,000 speakers. 
-The dataset includes three sets of paired sentences—Kidaw'ida-Kiswahili, Kalenjin-Kiswahili, and Dholuo-Kiswahili—with around 30,000 sentence pairs in each set. This data is used to train machine translation models, which can help preserve these languages by making them more accessible in digital formats.
-Users can expect to input text in Kiswahili and receive translations in one of the three indigenous languages as output. The dataset is available on Zenodo and GitHub, where it will be continuously updated and improved.
-While the project aims to support language preservation, there are known limitations. The dataset may not cover all dialects or variations within these languages, and there could be biases in the data that affect translation accuracy. Ethical considerations include ensuring that the languages are represented fairly and that the project respects the cultural significance of these languages.
-To promote responsible AI use, the project has undergone ethical assessments to address these concerns. Users interested in building new applications or products using this dataset should credit the original work and its contributors, including Principal Investigator Audrey Mbogho and co-investigators from various universities. 
-This initiative not only aids in language preservation but also supports crowd-sourced voice recognition efforts through platforms like Mozilla Common Voice, further enhancing the usability of these languages in technology.</t>
+Processed Data: Three parallel corpora for machine translation -- Kidaw'ida-Kiswahili, Kalenjin-Kiswahili, and Dholuo-Kiswahili. Approx. 30,000 sentence pairs per language pair. License: CC-BY-4.0. Format: ZIP archive (3.3 MB). DOI: 10.5281/zenodo.13355021. Published: August 21, 2024. Application: Train machine translation models to translate from Kiswahili into three Kenyan indigenous languages. Data also available on GitHub with ongoing updates planned. PI: Audrey Mbogho (USIU-Africa). Funded by: Lacuna Fund.
+Source: https://zenodo.org/records/13355021</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -6166,7 +5974,7 @@
       <c r="P46" t="inlineStr">
         <is>
           <t>Powered by / Provided by: USIU-Africa, Kabarak University, Maseno University (Kenya)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6279,16 +6087,8 @@
       <c r="M47" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-Miti360 is a dataset designed to help monitor reforestation efforts using advanced technology. It combines high-resolution images taken from drones, ground measurements of trees, and historical weather data to provide a comprehensive view of forest health and growth.
-The dataset includes:
-- Aerial images (orthophotos) that show the landscape and individual trees.
-- Ground-based images of trees, including detailed measurements like height and diameter.
-- Information about tree species and their locations.
-Users can input images and measurements of trees, and the dataset can help identify and classify tree species, estimate their growth, and analyze environmental conditions over time. This information is crucial for making informed decisions about reforestation projects.
-However, there are some limitations to consider. The dataset is specific to a reforested area in Kenya, which means it may not be directly applicable to other regions without adjustments. Additionally, the dataset relies on accurate ground measurements and may not account for all environmental variables affecting tree growth.
-To ensure responsible use of AI, the creators of Miti360 have taken steps to assess ethical considerations and biases in the data. Users are encouraged to credit the original dataset when developing new applications or products based on this work.
-To use the dataset, you will need access to software that can handle high-resolution images and process the data formats provided, such as GeoTIFF for aerial images and CSV for tree measurements. The dataset is hosted on Google Cloud Storage, and users can find detailed instructions for accessing it on the Miti360 website.
-For more information and to access the dataset, visit [Miti360's website](https://miti360.github.io/).</t>
+Processed Data and Pretrained Models: ML-ready dataset for forest monitoring from a 770-hectare reforested area in Kieni Forest, Kenya. Aerial imagery: 2 orthophotos + 844 tiles (TIF). Tree annotations: 57,058 crown bounding boxes (JSON) and 1,208 species records (CSV). Ground measurements: 1,208 trees with height, crown diameter, basal diameter, GPS coordinates (collected July 2024 - February 2025). Terrestrial images: 1,208 smartphone photos + 2,416 stereo image pairs (JPEG). Weather data: 8 years of daily precipitation and temperature from 40 stations (API). CRS: EPSG:21037. License: CC-BY 4.0. Code for AI Models: Jupyter Notebooks available in the GitHub repository. Data hosted on Google Cloud Storage.
+Source: https://github.com/DeKUT-DSAIL/miti360</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -6297,10 +6097,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6315,7 +6115,7 @@
       <c r="P47" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Dedan Kimathi University of Technology (Kenya)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6415,12 +6215,8 @@
       <c r="M48" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Agrof4Resilience project focuses on using data to enhance agroforestry systems in Kenya, aiming to improve food security, reduce the impacts of climate change, and boost incomes through timber and carbon markets. The project provides open-access geospatial datasets that can be utilized by artificial intelligence (AI) and machine learning (ML) algorithms.
-The model expects input data that includes information on land use and land cover (LULC), plot sampling, and socio-economic data from various counties in Kenya. Specifically, it contains over 20,000 land use points and more than 15,000 individual plant samples, including details like plant species identification, height, and diameter at breast height (DBH), along with photographs and geographical locations.
-The output produced by the model can help in optimizing agroforestry systems, identifying suitable plant species, and evaluating carbon sequestration potential. This information is crucial for developing more resilient agro-ecological systems, particularly in areas affected by climate change.
-While the project aims to provide valuable insights, there are known limitations and ethical considerations. The data may not cover all regions or species comprehensively, which could lead to biases in the analysis. Responsible AI use is emphasized, and ethical assessments are likely conducted to ensure that the data is used appropriately and does not harm local communities or ecosystems.
-To run the model effectively, users may need specific software to handle geospatial data formats, such as shapefiles (SHP) and dBase files (DBF). 
-Users are encouraged to credit the Agrof4Resilience project when utilizing this data for their own initiatives. The project is supported by the Lacuna Fund and other international development agencies, highlighting its commitment to fostering sustainable development in East Africa.</t>
+Processed Data: Open-access geospatial datasets covering 35 of 47 Kenyan counties, sampled across 200+ hectares. Over 20,000 land use points and over 15,000 individual plant samples. Key Variables: plant species identification, height, diameter at breast height (DBH), photographs, GPS locations. Dataset layers: land use points, land use polygons, plot sample points, plot sample polygons, study area, water lines. Format: Shapefile (.shp, .shx, .dbf, .prj, .cpg, .qmd). License: CC BY-NC 2.0. PI: Elfatih Abdel-Rahman. Funded by: Lacuna Fund through MERIDIAN Institute. Project duration: May 2024 - July 2025.
+Source: https://dmmg.icipe.org/dataportal/dataset/data-enabled-climate-shock-absorbance-and-ecosystem-resilience</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -6436,7 +6232,7 @@
       <c r="P48" t="inlineStr">
         <is>
           <t>Powered by / Provided by: International Center of Insect Physiology and Ecology (ICIPE)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6528,39 +6324,32 @@
       <c r="L49" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The LivHealth Kiswahili Corpus is a project designed to improve livestock health management in Kenya and Tanzania by providing local communities with easy access to disease information in Kiswahili. The dataset includes translated digital livestock disease manuals and data collected through a smartphone app used by Community Disease Reporters (CDRs) and pastoralists. This information helps users identify livestock diseases and report outbreaks effectively.
-The dataset is primarily in text format, featuring disease descriptions, symptoms, and treatment protocols translated from English to Kiswahili. It also includes audio components through text-to-speech technology, making it accessible for users who may have literacy challenges.
-Known limitations of the dataset may include potential biases in the data collection process, as it relies on the accuracy of reports from CDRs and the local community. There may also be gaps in coverage if certain regions or dialects are underrepresented in the recordings used for the text-to-speech models.
-To ensure responsible and ethical use, the project has focused on community engagement and collaboration with local stakeholders, including veterinary officers and pastoralists. This approach helps to build trust and ensures that the information provided is relevant and useful for the communities served.
-The dataset is maintained and updated by the LivHealth team in collaboration with their partner, One Health Center in Africa (OHRECA), based at the International Livestock Research Institute (ILRI). They are responsible for ongoing improvements and expansions of the dataset, including plans to extend services into Tanzania.
-Users have the right to access and utilize the data under the terms set by Mozilla’s Common Voice program, which aims to promote the use of local languages and voice technology. Specific licensing details may vary, so users should refer to the project's official resources for more information on usage rights.</t>
+Data Type: Text, Voice. Language: Kiswahili. Country: Kenya. The corpus contains livestock disease information translated from English to Kiswahili, including disease descriptions, symptoms, and treatment protocols. Data is collected via a smartphone app used by Community Disease Reporters (CDRs) and pastoralists. Maintained by Badili Innovations in partnership with One Health Center in Africa (OHRECA) at ILRI.
+Source: https://livhealth-kc.badili.co.ke/</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-LivHealth is an AI-powered system designed to help local communities in Kenya access important information about livestock health in Kiswahili. It aims to empower farmers and livestock owners by enabling them to identify diseases in their animals and seek timely help from qualified practitioners.
-The system uses Natural Language Processing (NLP) and Machine Learning (ML) to convert text into speech, making it easier for people who may not read well to understand the information. Users can input questions or symptoms related to their livestock, and the system provides spoken responses that guide them on what to do next.
-While the system is a valuable tool, there may be limitations, such as the accuracy of the information provided depending on the data it has been trained on. It's important to ensure that the AI is used responsibly, which includes conducting ethical assessments to avoid biases and ensure fair access to information.
-To run the LivHealth system, users will need a device that can access the internet and support audio playback, such as a smartphone or computer.
-When using or building upon this technology, it's essential to credit the source, LivHealth, and acknowledge their partnership with the One Health Center in Africa (OHRECA) at ILRI.</t>
+Application: LivHealth uses NLP and ML to provide Kiswahili text-to-speech output of livestock disease information, enabling communities with literacy challenges to access disease identification and treatment guidance. Users input livestock symptoms and receive spoken Kiswahili responses. Requires an internet-connected device with audio playback. Built by Badili Innovations in partnership with OHRECA at ILRI. Part of a Mozilla Common Voice innovation challenge supporting open-source voice technology in East Africa.
+Source: https://livhealth-kc.badili.co.ke/</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-To improve livestock health management in your community, you can immediately use the LivHealth Kiswahili Corpus to access vital disease information in Kiswahili. This resource allows local farmers and livestock owners to identify livestock syndromes and seek timely interventions from qualified practitioners. You can start by integrating the text-to-speech models into your community outreach programs, ensuring that information is accessible to those who may have literacy challenges.
-Researchers and developers can extend this work by enhancing the existing AI models with additional local data, which could improve the accuracy of disease identification. Collaborating with local agricultural universities or veterinary schools could provide valuable insights and data for refining the models. Additionally, creating mobile applications that utilize the LivHealth system could broaden its reach and usability.
-When replicating or building upon this project, it is essential to consider potential biases in the AI models, particularly if they were trained on limited datasets. Conducting an ethical AI assessment is recommended to ensure that the system serves all community members equitably. 
-As for costs, building on this resource may involve expenses related to adaptation and training of the models, which could range from a few hundred to several thousand dollars depending on the scale of your project and the resources required. Compute costs will vary based on the infrastructure you choose to use, whether cloud-based or local servers.
-Opportunities for collaboration exist with organizations like One Health Center in Africa (OHRECA), which could provide support and expertise. While specific documentation or tutorials were not mentioned, reaching out to the LivHealth team could yield valuable guidance and success stories from their implementation in Kenya and Tanzania. Long-term maintenance and scaling plans should include regular updates to the dataset and models to keep the information relevant and accurate for the communities served.</t>
+LivHealth is a web-based knowledge platform that makes livestock health information accessible in Kiswahili. Developed by Badili Innovations in partnership with the International Livestock Research Institute (ILRI), it is designed for livestock practitioners, extension workers, and development organisations operating in East African Swahili-speaking communities.
+You can access the platform directly at livhealth-kc.badili.co.ke to browse structured livestock health knowledge in Kiswahili. This makes it a practical resource for field programmes that need locally relevant, language-appropriate veterinary and animal health information -- whether for training community animal health workers, supporting extension services, or informing livestock health interventions.
+The platform spans three functional areas: information systems for structured livestock health knowledge, data management covering collection, synthesis, analytics and visualisation, and monitoring, evaluation and learning (MEL) to support tracking of livestock health interventions.
+For questions about integrating LivHealth into livestock health programmes or extending the platform, contact the development team through Badili Innovations at badili.co.ke. ILRI provides the domain expertise on livestock health content.
+Source: https://livhealth-kc.badili.co.ke/, https://badili.co.ke</t>
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Badili Innovations
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -6625,7 +6414,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Unfortunately no information or contacts to inquire further (DB, 28 Nov 2025)</t>
+          <t>Current publishing status unclear. Please contact the responsible authors for an update and access to the data: info@mu.ac.ke</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -6652,7 +6441,7 @@
       <c r="P50" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Moi University, Technical University of Kenya
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -6713,7 +6502,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Unfortunately no information or contacts to inquire further (DB, 28 Nov 2025)</t>
+          <t>Current publishing status unclear. Please contact the responsible authors for an update and access to the data: https://ujuzicraft.com/</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -6740,7 +6529,7 @@
       <c r="P51" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Ujuzi Craft LTD
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -6852,13 +6641,8 @@
       <c r="M52" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The AI-powered Agriculture Information Exchange Platforms aim to provide farmers in Kenya and Bihar, India, with personalized information to improve their agricultural practices. 
-The platform, specifically DynAG, focuses on key crops like rice, wheat, and maize. It uses advanced AI models to offer advisory services through various channels, including chatbots, mobile apps, and SMS. This ensures that farmers can easily access the information they need, regardless of their technology preferences.
-Farmers can input their questions or concerns about farming practices, and the platform generates tailored advice based on the latest agricultural research and data. The platform also supports communication in both English and Hindi, making it accessible to a wider audience.
-While the platform is designed to be user-friendly, there are some limitations. For instance, the effectiveness of the advice may depend on the quality of the data used to train the AI models. Additionally, there may be biases in the data that could affect the recommendations provided to farmers.
-To promote responsible AI use, the developers have implemented ethical assessments to ensure that the platform operates fairly and transparently. Users are encouraged to share their experiences and data, with the ability to set access rights for shared datasets, fostering a collaborative environment.
-To run the platform, users need a device capable of accessing the internet, whether through a smartphone or a basic mobile phone that supports SMS.
-For more information and to credit the source when building new products, please refer to the original work at https://dev.platform.farmer.chat/login.</t>
+Four AI-powered Agriculture Information Exchange Platform prototypes providing personalized advisory services to farmers in Kenya and Bihar, India. DynAG covers rice, wheat, and maize using a RAG pipeline powered by LLMs, accessible via chatbots, Android/Jio apps, IVR, and SMS in English and Hindi. Digital Green supports dairy, coffee, and wheat value chains via app, Telegram, and IVR with machine translation, speech technology, and image recognition in Hindi, Swahili, Gikuyu, and Marathi. Viamo targets beans and wheat farmers via IVR, SMS, and WhatsApp with LLM-based RAG in English, Hindi, and Swahili. Tech for Her focuses on women farmers growing tomatoes and raising cattle via IVR, WhatsApp, and mobile app with AI-based video generation in English, Hindi, and Swahili. The platform (FarmStack by Digital Green) allows uploading and sharing AI model training data with configurable access rights.
+Source: https://dev.platform.farmer.chat/login</t>
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -6866,7 +6650,7 @@
       <c r="P52" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Green, Viamo, Partners, Tech for Her, DynAg, Digifarm, Opportunity International
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation</t>
         </is>
       </c>
@@ -6959,36 +6743,25 @@
       <c r="M53" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The project aims to make artificial intelligence (AI) understand three East African languages: Kiswahili, Kinyarwanda, and Luganda. It does this by creating open-source speech-to-text datasets, which are collections of recorded speech that can be used to train AI systems to recognize and transcribe spoken words into text.
-The model expects audio input in the form of spoken language recordings. In return, it produces text output that represents what was said in the recordings. This technology can be particularly useful for applications like voice recognition on cellphones, making it easier for people to access information in their native languages.
-One of the known limitations is that the datasets may not cover all dialects or accents within these languages, which could lead to biases in how well the AI understands different speakers. Additionally, ethical considerations include ensuring that the data is collected and used responsibly, respecting the privacy and rights of the speakers involved.
-To promote responsible AI use, the project follows ethical guidelines and assessments to ensure that the datasets are used fairly and transparently. Users of these datasets should also credit the source, which is Mozilla's Common Voice Platform, when building new products or applications.
-The datasets are available in MP3 format and are quite large, with over 1064 hours of recorded speech in Kiswahili and 560 hours in Kinyarwanda and Luganda. This makes them a valuable resource for anyone looking to develop AI systems that can understand and process these languages.</t>
+Open-source speech-to-text datasets for three East African languages hosted on Mozilla's Common Voice platform. Kiswahili: Common Voice Scripted Speech 25.0, 20.87 GB, MP3 format. Kinyarwanda: Common Voice Scripted Speech 25.0, 57.18 GB, MP3 format. Luganda: Common Voice Scripted Speech 25.0, 11.06 GB, MP3 format. All three datasets are designed for automatic speech recognition (ASR) tasks. License: CC0-1.0.
+Source: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=sw</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-To leverage the Mozilla Common Voice datasets for Kiswahili, Kinyarwanda, and Luganda, here’s a practical guide for development practitioners and innovators:
-1) **Immediate Use Cases**: 
-   - **Speech Recognition Applications**: You can build applications that convert spoken language into text, which is particularly useful for creating voice-activated systems on mobile phones. This can enhance accessibility for users who may be illiterate or prefer to communicate in their native language.
-   - **Language Learning Tools**: Develop educational apps that help users learn these languages through interactive voice recognition features.
-   - **Transcription Services**: Create services that transcribe audio recordings into text, aiding in documentation and record-keeping for NGOs and community organizations.
-2) **Extending the Work**: 
-   - **Data Collection**: Researchers and developers can contribute by collecting more diverse speech samples, especially from underrepresented dialects or regions, to improve the dataset's inclusivity.
-   - **Model Training**: You can build upon the existing datasets to train custom speech recognition models tailored to specific applications or user needs, enhancing accuracy and usability.
-   - **Collaboration**: Partner with local universities or tech hubs to engage students and researchers in improving the datasets and developing applications.
-3) **Limitations and Ethical Considerations**: 
-   - **Bias in Data**: The datasets may not fully represent all dialects or accents within the languages, which could lead to biased outcomes in applications. It’s important to assess the dataset's diversity and consider conducting an ethical AI assessment before deploying any solutions.
-   - **Quality of Data**: Ensure that the quality of the recordings is sufficient for your intended application, as variations in recording conditions can affect performance.
-4) **Cost Estimates**: 
-   - **Adaptation and Training**: Depending on the complexity of your application, costs can vary. Basic adaptation of existing models may range from $1,000 to $5,000, while training a new model from scratch could exceed $10,000, especially if you require significant computational resources.
-   - **Compute Resources**: Cloud computing services for model training can cost anywhere from $0.50 to $3.00 per hour, depending on the required processing power.
-**Additional Resources**:
-- **Documentation and Tutorials**: Mozilla provides documentation on how to access and use the Common Voice datasets. Check their website for guides on setting up your environment and using the datasets effectively.
-- **Success Stories**: Look for case studies or examples of organizations that have successfully implemented solutions using these datasets to inspire your projects.
-- **Long-term Maintenance**: Engage with the Mozilla community for ongoing support and updates to the datasets, ensuring your applications remain relevant and effective.
-By utilizing these resources, you can create impactful solutions that enhance communication and access to information in East African languages.</t>
+Mozilla Common Voice provides large, open speech datasets for three East African languages -- Kiswahili (20.87 GB), Kinyarwanda (57.18 GB), and Luganda (11.06 GB) -- intended for building Automatic Speech Recognition (ASR) systems. These are collections of read speech recordings in MP3 format, paired with TSV metadata containing transcriptions and speaker information.
+This resource is valuable for anyone developing voice-based applications, virtual assistants, transcription tools, or accessibility services for East African language communities. You can use the recordings and transcriptions to train and evaluate ASR models, or to fine-tune existing multilingual speech models for better performance on these specific languages. The datasets are also suitable for linguistic research on phonetics, prosody, or speaker variation across the three languages.
+Researchers and developers can extend this work by combining Common Voice data with other speech corpora to improve model robustness, or by using the trained models as a foundation for downstream tasks like keyword spotting, voice-controlled interfaces, or spoken-language understanding. Because the datasets are released under a CC0-1.0 license (public domain), they can be freely used, modified, and redistributed for any purpose without attribution requirements -- making them particularly suitable for commercial applications and integration into products.
+The datasets are hosted on the Mozilla Data Collective platform. To download, create a free account at datacollective.mozillafoundation.org, navigate to the dataset page for the language you need, accept the user agreement, and download the compressed archive. Programmatic access is also available through the platform's REST API for automated pipelines.
+- Kiswahili: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=sw
+- Kinyarwanda: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw
+- Luganda: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=lg
+Sources:
+- https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=sw
+- https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=lg
+- https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw
+- https://datacollective.mozillafoundation.org/</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -6999,7 +6772,7 @@
       <c r="P53" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Mozilla Common Voice
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ, Gates Foundation, FCDO</t>
         </is>
       </c>
@@ -7023,7 +6796,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7105,7 +6878,7 @@
       <c r="P54" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Association Maidi
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7208,7 +6981,7 @@
       <c r="P55" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Bayero University (Kano, Nigeria), Ahmadu Bello University (Zaria, Nigeria), Masakhane NLP, HausaNLP, Kaduna state University
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7320,14 +7093,8 @@
       <c r="M56" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Residential Energy and Weather Data (REWD) project in Pakistan provides a detailed dataset that helps understand how energy consumption in homes relates to weather conditions. This dataset is particularly useful for policymakers, NGOs, and businesses looking to promote energy conservation and develop sustainable energy initiatives.
-The REWD dataset includes two main components: 
-1. **Electricity Consumption Data**: This data was collected from 60 households across six major urban centers in Pakistan, covering different climatic zones. The electricity usage is recorded every minute, allowing for a detailed analysis of how much energy is consumed by entire households and individual appliances. This includes information on high-consumption appliances, which can help identify patterns in energy use.
-2. **Weather Data**: Collected over 18 months, this dataset includes key weather variables such as temperature, humidity, atmospheric pressure, and precipitation. This information helps to correlate energy consumption patterns with environmental factors.
-The dataset is open-source, meaning it is freely available for anyone to use. However, users should credit the Lahore University of Management Sciences (LUMS) when building new products or conducting research based on this data.
-While the dataset is comprehensive, it is important to consider potential limitations. The dataset is based on a limited number of households, which may not fully represent the diversity of energy consumption patterns across all of Pakistan. Additionally, the data is specific to urban centers and may not reflect rural energy usage.
-For responsible AI use, it is crucial to conduct ethical assessments when applying this data in projects. Users should be mindful of privacy concerns and ensure that any analysis respects the confidentiality of the households involved.
-To utilize the REWD dataset, users will need basic software tools for data analysis, such as spreadsheet software or programming languages like Python or R. No specialized hardware is required, making it accessible for a wide range of users interested in energy conservation and market analysis in Pakistan.</t>
+Residential Energy and Weather Data Pakistan (REWD-P), provided by Lahore University of Management Sciences (LUMS). Contains electricity consumption data from 60 households across six urban centers (Lahore, Multan, Peshawar, Karachi, Islamabad, Skardu) recorded at 1-minute granularity for whole-household usage and individual appliances. Energy data covers 1 year; weather data covers 18 months with up to 10 variables (temperature, atmospheric pressure, humidity, dew, precipitation, wind direction, wind speed, solar radiation, solar energy, UV index). Includes building attributes and demographic metadata. Format: CSV. Open-source access.
+Source: https://lei.lums.edu.pk/datasets/residential-energy-and-weather-data-pakistan.html</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -7339,7 +7106,7 @@
       <c r="P56" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Lahore University (LUMS)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7407,12 +7174,13 @@
       <c r="E57" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The iMaster-DocuCam Landslide Monitoring System addresses the critical issue of landslides and earth movements, which pose significant risks to communities and infrastructure. It was created to provide a systematic and continuous monitoring solution, enabling early detection and assessment of these hazards, ultimately reducing economic damages and saving lives. The system offers open access to a demo version and an online user manual, allowing users to familiarize themselves with its capabilities. This tool can greatly benefit government agencies, NGOs, and disaster response teams by providing real-time data and visual documentation to enhance preparedness and response strategies in vulnerable areas.</t>
+The iMaster-DocuCam Landslide Monitoring System by Hesotech GmbH provides long-term, continuous visual documentation of landslide-prone areas in Rwanda. A pan-tilt-zoom (PTZ) camera captures high-resolution images (up to 1 cm per cell at 500 m distance) at user-defined intervals, while supplementary sensors record temperature, rainfall, humidity, and GPS data. All data is stored in a single database and accessible via web browser from any location. The system is designed for low energy consumption and can be powered by solar panels or generators, making it suitable for remote areas. A demo version and online user manual are available at https://manual.docucam.hesotech.eu/en.
+Source: https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>not public yet</t>
+          <t>Publishing status unclear. Please contact the responsible authors for an update and access to the data: https://www.hesotech.de/en/contact-directions/</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -7430,7 +7198,11 @@
           <t>Images, Meterological</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
           <t>Rwanda</t>
@@ -7439,59 +7211,33 @@
       <c r="L57" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The iMaster-DocuCam Landslide Monitoring System provides a comprehensive dataset for monitoring landslides and other earth movements in Rwanda. The system captures high-resolution images of targeted areas, along with supplementary data such as temperature, rainfall, and humidity. This data is collected automatically at predefined intervals and can be accessed via a web-based interface.
-Key characteristics of the dataset include:
-- **Data Content and Format**: The dataset consists of high-resolution images (up to 1 cm per cell at a distance of 500 m) and environmental data (e.g., weather conditions). The data is stored in a single database and can be accessed through a web browser.
-- **Known Limitations**: While the system is designed for comprehensive monitoring, it may have limitations in areas that are difficult to access or where environmental conditions affect data collection. Additionally, the dataset may not cover all potential landslide areas, depending on the installation locations of the monitoring systems.
-- **Responsible and Ethical Use**: The system allows users to add notes and pixelate sensitive areas in images, promoting responsible data use. The design also considers low energy consumption, enabling operation in remote areas with limited power supply.
-- **Maintenance and Updates**: The dataset is maintained by the developers at Hesotech, who ensure that the system is updated and functioning correctly. Users can access support through an online user manual and tutorials.
-- **User Rights and Licensing**: Specific licensing details are not provided in the source material. Users should inquire directly with Hesotech for information regarding data usage rights and any applicable licenses.
-This dataset is particularly useful for development practitioners, NGOs, and government agencies focused on disaster risk management and environmental monitoring in Rwanda.</t>
+The system captures high-resolution images (up to 1 cm per cell at 500 m distance) at predefined intervals alongside environmental data (temperature, rainfall, humidity, GPS). Data is stored in a single database and accessible via web browser. The hardware consists of a PTZ camera and electronics cabinet with mini-PC; optional expansions include a local weather station, LTE/3G/4G connection, antenna, generator, solar panel, and custom sensor interfaces. Connectivity via local WiFi or LTE/3G/4G. No physical markers required in the monitored area; virtual markers can be created on-screen. Supports time-lapse generation, built-in ruler measurements, and image annotation (text, shapes, arrows, pixelation of sensitive areas).
+Source: https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The iMaster-DocuCam Landslide Monitoring System is a tool designed to monitor and analyze areas prone to landslides and floods. It uses a camera to take high-resolution images of the landscape over time, allowing users to detect changes in the environment that may indicate potential risks. 
-The system automatically collects data, including images and additional information like temperature and rainfall, which helps users understand the factors contributing to earth movements. Users can access this data through a web browser from anywhere, making it convenient for monitoring remote or hazardous locations.
-The iMaster-DocuCam does not require physical markers in the monitored area, as it allows users to create virtual markers on the screen. This feature enhances its usability in difficult-to-reach places. The system also supports the creation of time-lapse recordings, which visually demonstrate changes over time, making complex situations easier to understand.
-While the system is designed for ease of use, it is important to consider that it relies on technology that may be affected by local conditions, such as internet connectivity and power supply. The hardware can be powered by solar panels or generators, making it adaptable for use in areas without reliable electricity.
-For responsible AI use, users should be aware of privacy considerations when capturing images and have the option to pixelate sensitive areas. The system is designed to be user-friendly, with an online manual and tutorials to assist users in getting started.
-When utilizing the iMaster-DocuCam for new projects, it is important to credit the source of the technology. 
+Performs long-term, continuous visual monitoring to detect small and large, slow and fast surface changes for landslide and earth movement analysis. Automated image capture at user-defined intervals with simultaneous collection of weather and GPS data enables cause-effect correlation. Does not require physical markers; users create virtual markers on-screen. Generates time-lapse recordings to visualize changes over time. Web-browser-based access from any location. Low energy consumption allows operation via solar panel or generator in off-grid areas. Developed by Hesotech GmbH.
 Source: https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The iMaster-DocuCam Landslide Monitoring System offers practical tools for monitoring landslides and flood disaster hotspots in Rwanda and similar regions. Here’s a guide for development practitioners and innovators looking to utilize or build upon this resource.
-1) **Immediate Use Cases**:
-   - **Landslide Monitoring**: Use the iMaster-DocuCam to monitor areas prone to landslides. The system captures high-resolution images at regular intervals, allowing for the detection of changes in the landscape.
-   - **Flood Risk Assessment**: By integrating weather data (like rainfall), users can analyze potential flood risks and take preventive measures.
-   - **Data Collection**: The system automatically collects visual and environmental data, which can be accessed remotely via a web browser. This allows for continuous monitoring without the need for physical presence in hazardous areas.
-2) **Extending the Work**:
-   - **Custom Sensor Integration**: Developers can enhance the system by integrating additional sensors (e.g., for soil moisture or seismic activity) to provide a more comprehensive understanding of environmental changes.
-   - **Local Adaptation**: Innovators can adapt the hardware setup to local conditions, such as using solar panels for power in remote areas.
-   - **Collaboration Opportunities**: Partner with local universities or NGOs to conduct research on landslide patterns and develop predictive models based on the collected data.
-3) **Limitations and Considerations**:
-   - **Data Quality**: Ensure that the camera is positioned correctly to capture relevant areas. Poor positioning can lead to incomplete data.
-   - **Ethical Considerations**: Before deploying the system, consider conducting an ethical assessment, especially regarding data privacy and the potential impact on local communities.
-   - **Technical Support**: Users may need technical support for installation and maintenance, particularly in remote areas.
-4) **Cost Estimates**:
-   - **Initial Setup**: The cost will vary based on the specific hardware configuration and additional sensors. A basic setup may start at a few thousand dollars, but costs can increase with additional features.
-   - **Ongoing Costs**: Consider costs for data storage, internet connectivity, and maintenance. Using solar panels can reduce energy costs in off-grid locations.
-5) **Resources and Support**:
-   - **Documentation**: Access the online user manual and animated tutorials to help with setup and operation. This resource is crucial for users unfamiliar with technology.
-   - **Demo Version**: Try the demo version of the iMaster-DocuCam to familiarize yourself with its capabilities before making a purchase.
-   - **Success Stories**: Look for case studies or testimonials from other users who have successfully implemented the system in similar contexts.
-By leveraging the iMaster-DocuCam, practitioners can enhance their disaster monitoring efforts, improve community safety, and contribute to more resilient infrastructure in vulnerable regions.</t>
+## How to Use This Resource
+The iMaster-DocuCam system by Hesotech enables long-term, high-resolution visual monitoring of landslides, earthfalls, rockfalls, and earth movements across large areas. It is designed for deployment in environments like Rwanda where continuous observation of hazard-prone slopes is critical for disaster risk reduction.
+Practitioners working in disaster risk management, climate adaptation, or infrastructure protection can use this system to establish automated visual monitoring stations that capture images at predefined intervals (for example, every two hours), achieving a resolution of up to 1 cm per cell at 500 m distance. All captured data can be viewed remotely through a standard web browser (Chrome or Firefox) from any location -- no proprietary software is required. This makes the system practical for distributed teams and remote field sites.
+The built-in analysis tools allow you to place virtual measurement points on images without physical markers in the field, measure surface changes over time, generate time-lapse videos to visualise movement patterns, and correlate camera data with complementary sensor readings for cause-effect analysis. The system can be extended with a local weather station, GPS data collection, custom sensor interfaces, and solar panel power supply for off-grid deployment, making it suitable for rural and infrastructure-limited contexts.
+A comprehensive online manual with animated tutorials is available at [manual.docucam.hesotech.eu/en](https://manual.docucam.hesotech.eu/en), along with a demo version that allows you to explore the interface before committing to a deployment. Full product specifications and contact details can be found on the [Hesotech product page](https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/).
+Source: https://www.hesotech.de/en/products-services/imaster-docucam-landslide-monitoring-system/</t>
         </is>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Hesotech GmbH
-Catalyzed by: FAIR Forward - AI for All &amp; Digital and Green Innovation
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7608,12 +7354,8 @@
       <c r="M58" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Mbaza Chatbot is an AI application designed to help Rwandan citizens get answers to health-related questions, particularly during the coronavirus pandemic. It was developed as part of a global hackathon aimed at finding digital solutions for challenges faced by low- and middle-income countries.
-The chatbot works by allowing users to input their health inquiries through various channels, including USSD (a mobile communication protocol), web, and interactive voice response (IVR). In simple terms, users can ask questions about health guidelines, daily statistics, and pandemic prevention measures, and the chatbot provides relevant information in response.
-While the chatbot is a useful tool, it may have limitations. For instance, it relies on the data provided by health authorities, which means that if the information is outdated or incomplete, the chatbot's responses may also be affected. Additionally, there may be biases in the data it was trained on, which could influence the accuracy of its answers.
-To ensure responsible AI use, the developers have likely conducted ethical assessments, although specific details on these steps are not provided. Users of the chatbot should be aware of the importance of using accurate and up-to-date information, especially in health-related contexts.
-For those interested in building upon this chatbot, the underlying data can be requested from Digital Umuganda or the Rwanda Biomedical Centre (RBC). It is important to credit the source work when creating new products based on this chatbot.
-In terms of technical requirements, the chatbot may need specific software and hardware to run effectively, but these details are not explicitly mentioned. Overall, the Mbaza Chatbot represents a significant step towards improving access to health information for citizens in Rwanda.</t>
+Conversational chatbot built on the Rasa open-source framework, providing COVID-19 information to Rwandan citizens in English and Kinyarwanda. Covers outbreak statistics, symptoms, prevention tips, fines/penalties, testing center locations, testing procedures, costs, lockdown areas, and vaccination information. Developed by Digital Umuganda. The USSD channel reached production; web and IVR versions reached staging phase. Reported usage: 4,165,037 total users and 37,812,089 total sessions. Source code available on GitHub.
+Source: https://github.com/Digital-Umuganda/Mbaza-chatbot</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -7631,7 +7373,7 @@
       <c r="P58" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Umuganda
-Catalyzed by: FAIR Forward - AI for All, Digital Transformation Centre Rwanda
+Catalyzed by: FAIR Forward - AI for All, GIZ, Digital Transformation Centre Rwanda
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7674,7 +7416,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -7691,17 +7433,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Agriculture chatbot / early warning system for farmers / AI entrepreneurship competition (Mbaza Chatbot scaling)</t>
+          <t>Tunga Agricultural Chatbot</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Better Advise to farmers in Rwanda on pest diagnosis and climate-resilient practices through an Agricultural chatbot</t>
+          <t xml:space="preserve">Tunga Agricultural Voicebot - Agricultural Advise for Farmers in Kinyarwanda </t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Better Advise to farmers  in Rwanda on pest diagnosis and climate-resilient practices through an Agricultural chatbot</t>
+          <t xml:space="preserve">Tunga Agricultural Voicebot - Agricultural Advise for Farmers in Kinyarwanda </t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -7711,7 +7453,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">will come? </t>
+          <t>https://fair-forward.github.io/datasets?search=tunga&amp;project=ui_87-tunga_agrichatbot_suite</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -7742,7 +7484,7 @@
       <c r="P59" t="inlineStr">
         <is>
           <t>Powered by / Provided by: MINAGRI, C4IR, KiNLP
-Catalyzed by: GIZ &amp; FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7803,7 +7545,8 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">will come?  please update name as it is the same as for a kenya activity </t>
+          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: konza@konza.go.ke
+</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
@@ -7817,7 +7560,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Konza Technopolis ( https://konza.go.ke/)</t>
+        </is>
+      </c>
       <c r="K60" t="inlineStr">
         <is>
           <t>Rwanda</t>
@@ -7829,8 +7576,8 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Powered by / Provided by:
-Catalyzed by: FAIR Forward - AI for All
+          <t>Powered by / Provided by: Konza Technopolis, ICTA
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -7909,32 +7656,28 @@
       <c r="L61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This dataset is part of the Common Voice project, which aims to create an open-source voice dataset for Kinyarwanda speakers. It contains over 2,380 hours of audio recordings in Kinyarwanda, specifically designed for speech recognition tasks, such as converting spoken language into text. The recordings are in MP3 format and the total size of the dataset is approximately 57.18 GB.
-One of the key benefits of this dataset is that it helps build inclusive language technology, making it easier for people, including those who are illiterate or live in rural areas, to access information in their mother tongue. This can significantly enhance communication and information dissemination in Kinyarwanda.
-However, users should be aware of potential limitations or biases in the dataset. While it aims to represent diverse speakers, the dataset may not fully capture all dialects or accents within the Kinyarwanda language, which could affect the performance of AI systems built using this data.
-The dataset is maintained by the Mozilla Foundation, which is committed to ensuring responsible and ethical use of the data. They have implemented measures to promote fair use and protect the rights of the speakers involved in the recordings.
-Users have the right to use this dataset under the CC0-1.0 license, which allows for free use without restrictions. This means you can use, modify, and distribute the data for any purpose, including commercial applications, as long as you comply with the ethical guidelines set forth by the maintainers.</t>
+Common Voice Scripted Speech 25.0 - Kinyarwanda: a collection of read speech recordings in Kinyarwanda hosted on Mozilla Data Collective. Size: 57.18 GB. Format: MP3. Designed for automatic speech recognition (ASR). License: CC0-1.0. Additionally, the common-voice-kinyarwanda-english-dataset by Mbaza NLP on Hugging Face provides a Kinyarwanda-English bilingual dataset with 721,395 rows (619,000 train / 61,600 validation / 41,200 test) for training multilingual ASR systems. Size: 166 MB (CSV). License: CC-BY-4.0.
+Source: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw, https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-This project has created a large collection of voice recordings in Kinyarwanda, which is the largest open-source dataset of its kind. The main goal is to help develop speech recognition technology that can understand and transcribe spoken Kinyarwanda into text. This technology can be particularly useful for people who speak Kinyarwanda, including those who may not be literate or who live in rural areas, allowing them to access information in their native language.
-The dataset includes over 2,380 hours of audio recordings, which are provided in MP3 format. Users can input spoken Kinyarwanda into AI systems, and the output will be the corresponding text transcription. This can be applied in various applications, such as voice assistants on cellphones or other devices.
-While this dataset is a valuable resource, there are some considerations to keep in mind. The dataset may reflect certain biases based on the speakers included, which could affect the accuracy of the speech recognition technology in different contexts. Ethical considerations are important, and users should conduct assessments to ensure responsible use of AI technologies developed from this dataset.
-To use this dataset effectively, users should have access to software capable of processing audio files and running speech recognition algorithms. There are no specific hardware requirements mentioned, but a standard computer with audio processing capabilities should suffice.
-When using this dataset to build new products, it is important to credit the source, which is the Mozilla Foundation's Common Voice project. This acknowledgment helps support the ongoing efforts to create inclusive language technology.</t>
+Provides speech-to-text training data for Kinyarwanda. The Common Voice dataset (57.18 GB, MP3, CC0-1.0) enables building ASR systems that transcribe spoken Kinyarwanda into text. The complementary Kinyarwanda-English dataset by Mbaza NLP (721,395 rows, CC-BY-4.0) supports multilingual ASR development. Both datasets can be used to build voice-enabled applications such as speech recognition on mobile devices.
+Source: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw, https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately start building speech recognition applications that understand Kinyarwanda using the extensive voice dataset collected through the Common Voice project. With over 2,380 hours of audio recordings, this resource allows you to create systems that can transcribe spoken Kinyarwanda, making information more accessible to speakers, including those in rural areas and those who are illiterate.
-To get started, you can use existing tools for automatic speech recognition (ASR) that are compatible with the dataset. These tools can help you develop applications for mobile phones or other devices that provide information in Kinyarwanda, enhancing communication and access to services.
-Researchers and developers can extend this work by contributing additional voice data or improving the existing models. For instance, you could focus on specific dialects or contexts that are underrepresented in the current dataset. Collaborating with local communities to gather more diverse speech samples can also enhance the dataset's effectiveness.
-However, it’s important to consider potential limitations and biases. The dataset may not fully represent all dialects or accents of Kinyarwanda, which could affect the accuracy of speech recognition in certain contexts. We recommend conducting an ethical AI assessment before replicating or building upon this work to ensure that the technology is inclusive and respects the cultural nuances of the language.
-In terms of costs, building on this dataset may involve expenses related to adaptation and training of models, as well as computing resources. Depending on the scale of your project, you might estimate costs in the range of a few hundred to several thousand dollars, particularly if you require cloud computing services for model training.
-For further guidance, you can refer to the documentation available through the Common Voice project, which includes tutorials on how to use the dataset effectively. Engaging with the community around this project can also lead to collaboration opportunities, sharing insights, and learning from success stories of others who have implemented similar technologies. Long-term maintenance and scaling of your application will depend on ongoing community support and updates to the dataset as more voices are collected.</t>
+## How to Use This Resource
+This resource provides Kinyarwanda voice and text data through two complementary channels, making it valuable for anyone working on speech technology, language preservation, or multilingual applications for Rwanda and the broader East African region.
+The Mozilla Data Collective hosts the "Common Voice Scripted Speech 25.0 - Kinyarwanda" dataset, which contains 57.18 GB of MP3 audio recordings released under a CC0-1.0 license, meaning it can be used without any restrictions. This is the primary source for building or improving Automatic Speech Recognition (ASR) systems that handle Kinyarwanda. The dataset can be accessed directly through the [Mozilla Data Collective platform](https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw).
+A complementary bilingual compilation is available on [Hugging Face as mbazaNLP/common-voice-kinyarwanda-english-dataset](https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset), providing 721,395 text transcription entries spanning both Kinyarwanda and English, with pre-defined train, validation, and test splits (approximately 619,000 / 61,600 / 41,200 entries respectively). This dataset is licensed under CC-BY-4.0. Note that this Hugging Face version currently contains text transcriptions only; audio files are planned for a future release.
+Researchers and developers can use these resources to train multilingual ASR systems, build voice-enabled applications for Kinyarwanda speakers, or conduct linguistic research on this under-resourced language. The bilingual structure of the Hugging Face dataset also opens possibilities for cross-lingual transfer learning and translation tasks. Both datasets are accessible through standard data science tools and the Hugging Face datasets library.
+Sources:
+- https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw
+- https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -7945,7 +7688,7 @@
       <c r="P61" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Umuganda, Mozilla Common Voice
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8049,18 +7792,14 @@
       <c r="M62" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-In Rwanda, a new approach is using satellite imagery and artificial intelligence (AI) to create detailed maps that show where different crops are grown, such as rice, maize, Irish potatoes, and beans. This technology helps farmers and agricultural authorities make better decisions, especially in the face of climate change, which can lead to unpredictable weather and crop yields.
-The AI model works by analyzing satellite images to identify crop types across various regions. It combines this satellite data with local field data to produce accurate maps that indicate when and where specific crops are cultivated. This information is crucial for planning agricultural activities, managing resources, and responding to challenges like droughts or pest infestations.
-While the model has shown good accuracy, it does have limitations. The effectiveness of the crop mapping relies on having local reference data, which is essential for validating the satellite observations. Additionally, the model does not replace traditional field observations but complements them, ensuring that local knowledge is still valued in agricultural practices.
-To ensure responsible use of AI, the project includes training for local experts through partnerships with the Rwandan Space Agency and the National Institute of Statistics of Rwanda. This training helps build local capacity to maintain and improve the mapping system over time.
-The digital maps created by this initiative are open and freely accessible, allowing other organizations and innovators to use them in their own projects. Users are encouraged to credit the original work when developing new applications based on this data.
-Overall, this AI application aims to enhance agricultural productivity and resilience in Rwanda, providing farmers with better advice and support tailored to their specific conditions.</t>
+Machine learning pipeline for crop type classification in Rwanda using Sentinel-1 and Sentinel-2 satellite imagery. Training scripts include Random Forest and climate-corrected models. Ground reference data covers four districts (Nyagatare, Musanze, Nyabihu, Ruhango) with field observations of maize, beans, rice, and Irish potato collected May-June 2025. The ground truth dataset contains GPS-located farm plots with crop attributes, management practices, and directional photographs. Code: Python scripts for satellite data preparation, image download, and model training at github.com/crop-type-mapping/ML. License: MIT (code), CC-BY 4.0 (ground reference data).
+Source: https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/O7IDTD, https://github.com/crop-type-mapping</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -8074,7 +7813,7 @@
           <t>Powered by / Provided by:
 Rwanda Space Agency (RSA), the Rwandan Ministry of Agriculture, Alliance of Bioversity International and CIAT
 Catalyzed by:
-FAIR Forward - AI for All / GIZ, Digital Transformation Centre Rwanda
+FAIR Forward - AI for All, GIZ, Digital Transformation Centre Rwanda
 Financed by:
 BMZ</t>
         </is>
@@ -8194,7 +7933,7 @@
       <c r="P63" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Atingi, Digital Umuganda, Clear Global
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8258,12 +7997,12 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>The dataset was not made public</t>
+          <t>The dataset was not made public (FAIR Forward status: experiment)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>The model was not made public</t>
+          <t>The dataset was not made public (FAIR Forward status: experiment)</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -8297,7 +8036,7 @@
       <c r="P64" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Health Development Initiative (HDI) Rwanda
-Catalyzed by: Sexualised and Gender-Based Violence (P-SGBV) Project of GIZ, GIZ ZFD SIGA Refugee Programme, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
+Catalyzed by: GIZ (Sexualised and Gender-Based Violence (P-SGBV) Project), GIZ ZFD SIGA Refugee Programme, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
@@ -8426,7 +8165,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8543,7 +8282,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8655,7 +8394,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8767,7 +8506,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8879,7 +8618,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -8991,7 +8730,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9103,7 +8842,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9215,7 +8954,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9327,7 +9066,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9439,7 +9178,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9502,7 +9241,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9552,7 +9291,7 @@
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9649,12 +9388,12 @@
       <c r="N76" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-To start using the "Voices of Mzansi" project, you can immediately contribute by collecting sentences in any of South Africa's official languages and uploading them to the Mozilla Common Voice platform. This effort helps create a diverse dataset that can be used for developing text-to-speech applications, voice recognition systems, and other AI tools that support local languages.
-Researchers and developers can extend this work by creating applications that utilize the collected speech data for educational tools, accessibility features, or community engagement platforms. You can also improve upon the existing dataset by ensuring it includes a wide range of dialects and contexts, which will enhance the accuracy and usability of AI models trained on this data.
-When replicating this project, consider potential biases in the dataset, such as underrepresentation of certain dialects or socio-economic groups. It is advisable to conduct an ethical AI assessment to ensure that the applications developed are inclusive and do not perpetuate existing inequalities.
-In terms of costs, building on this project may involve expenses related to data collection tools, community engagement efforts, and possibly cloud computing resources for training AI models. Depending on the scale, initial costs could range from a few hundred to several thousand dollars, particularly if you need to hire local language speakers or facilitators.
-Collaboration opportunities exist with local universities, NGOs, and tech communities interested in language preservation and AI. Documentation and tutorials for using the Common Voice platform are available on their website, which can guide you through the process of contributing and utilizing the datasets. Success stories from similar projects can inspire your efforts and provide insights into effective strategies for community involvement and data collection.
-Long-term maintenance and scaling of this project will depend on ongoing community engagement and the continuous collection of diverse language data to keep the datasets relevant and useful.</t>
+## How to Use This Resource
+The Voices of Mzansi project collects speech data for South Africa's official languages through the Mozilla Common Voice platform. This is a community-driven effort, and the most immediate way to contribute is by recording your voice or validating other people's recordings at [commonvoice.mozilla.org](https://commonvoice.mozilla.org).
+The current status across South Africa's 11 official languages reveals a significant need for contributions. Setswana leads with 4.3 validated hours from 18 speakers, followed by Afrikaans with 0.6 validated hours from 67 speakers. The remaining languages -- isiZulu, Sesotho, siSwati, isiXhosa, Tshivenda, Sepedi, isiNdebele, and Xitsonga -- have little to no validated audio despite having hundreds or thousands of sentences already prepared for recording. For example, Sesotho has 2,339 sentences ready and Sepedi has 2,247, but both have almost no recorded audio yet.
+This gap represents a concrete opportunity for development practitioners, language advocates, and community organisations in South Africa. Organising recording sessions with native speakers, particularly for the languages that already have substantial sentence pools waiting to be read aloud, is the single most impactful action anyone can take right now. No technical expertise is required -- the Common Voice platform handles everything through a web browser.
+Once enough validated audio has been collected, Common Voice datasets are released periodically and can be downloaded from [commonvoice.mozilla.org/languages](https://commonvoice.mozilla.org/languages). These datasets are provided as MP3 audio files with corresponding text transcriptions, released under a CC0-1.0 license, making them freely usable for building speech recognition systems, voice-enabled applications, and other language technologies for South African languages.
+Source: https://commonvoice.mozilla.org/en/languages (language statistics via Common Voice API)</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -9665,7 +9404,7 @@
       <c r="P76" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Stellenbosch University
-Catalyzed by: South African Digital Language Resources (SADILAR), FAIR Forward - AI for All, Mozilla Foundation, UNESCO decade of indigenous languages
+Catalyzed by: South African Digital Language Resources (SADILAR), FAIR Forward - AI for All, GIZ, Mozilla Foundation, UNESCO decade of indigenous languages
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9768,7 +9507,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -9785,7 +9524,7 @@
       <c r="P77" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Radiant Earth, Western Cape Department of Agriculture
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -9847,7 +9586,12 @@
           <t>A majority of smallholder farmers in Tanzania are only able to communicate through the Kiswahili spoken language and its dialects. A text and voice-based platform made available in the language of the underserved (i.e., Kiswahili) would be key to wide access, adoption, and usage of digital agricultural advisory and financial services in Tanzania. The objective is to develop a text and voice recognition platform that will offer smallholder farmers in the Tanzanian Maize Value Chain personalized digital financial and non-financial automated services based on location, agro-ecological zones, and crop cycle. Based on gender-disaggregated data from the pilot phase, it is anticipated that the majority of participants will be women. This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: info@duniacom.com
+</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
@@ -9861,7 +9605,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Duniacom Group, LLC</t>
+          <t>Duniacom Group LLC (info@duniacom.com)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -9876,7 +9620,7 @@
       <c r="P78" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Duniacom Group LLC
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -9941,7 +9685,8 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Unfortunately no information or contacts to inquire further. The organisation's website is down. Assumably they ceased to exist (DB, 28 Nov 2025)</t>
+          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: https://seeafricatz.org/contact-us/
+</t>
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
@@ -9955,7 +9700,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+        </is>
+      </c>
       <c r="K79" t="inlineStr">
         <is>
           <t>Tanzania</t>
@@ -9967,8 +9716,8 @@
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Sustain Earth's Environment Africa
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All
+          <t>Powered by / Provided by: SEE Africa
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
@@ -10035,8 +9784,8 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10108,7 +9857,7 @@
       <c r="P80" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Producers Direct, M-Omulimisa, Alliance of Bioversity International and CIAT, Tecnicafé
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10232,7 +9981,7 @@
       <c r="P81" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Sunbird.ai
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10324,42 +10073,35 @@
       <c r="L82" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The dataset from the Solar Irradiance Portal focuses on predicting daily Global Horizontal Irradiance (GHI) specifically for Uganda, addressing the inaccuracies found in standard satellite-derived solar irradiation data. Here are the key characteristics of the dataset:
-- **Content and Format**: The dataset includes corrected solar irradiance data that has been fine-tuned for Uganda, based on ground measurements collected from five installation sites (Gulu, Mbale, Jinja, Kasese, Hoima). It provides high-accuracy estimates that align closely with actual ground measurements, making it suitable for renewable energy planning. The data is accessible through an interactive web portal and can also be integrated via a RESTful API.
-- **Limitations and Biases**: The primary limitation of the original satellite datasets is their tendency to overestimate solar potential in Uganda, which can lead to financial risks for solar energy projects. The AI model developed aims to correct this systematic bias, but users should be aware that the accuracy is contingent on the quality of the ground-truth data used for training.
-- **Responsible and Ethical Use**: The project emphasizes the importance of providing bankable, high-accuracy solar data to mitigate financial risks associated with solar energy investments. The AI model has been specifically designed to cater to Uganda's unique climate and topography, ensuring that the data is relevant and reliable for local applications.
-- **Maintenance and Updates**: The dataset is maintained by the team behind the Solar Irradiance Portal, which is responsible for updating the data as new ground measurements are collected and as the AI model is refined.
-- **User Rights and License**: While specific licensing details are not provided in the source content, users can typically expect to have access to the data for analysis and integration into their applications, provided they adhere to any terms set by the dataset maintainers.
-This dataset is particularly valuable for development practitioners, NGOs, and government agencies looking to optimize solar energy projects in Uganda by using accurate and reliable solar irradiance data.</t>
+Bias-corrected daily Global Horizontal Irradiance (GHI) data for Uganda, derived by correcting CAMS and NASA POWER satellite datasets against ground-truth measurements from 56 validation sites across Uganda. Training data includes measurements from 7 African countries. The correction addresses a 20% satellite overestimation of solar potential. Data is accessible via the Solar Irradiance Portal web interface and a RESTful API for application integration.
+Source: https://github.com/Marconi-Lab/Solar_irradiation, https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The project focuses on improving solar energy planning in Sub-Saharan Africa, particularly in Uganda, by using an AI model to predict solar irradiance. In simple terms, the model takes satellite data that often overestimates solar potential and corrects it to provide more accurate and reliable information about solar energy availability.
-The input for the model includes satellite-derived solar irradiation data from sources like NASA and CAMS, along with ground measurements collected from various sites in Uganda. The output is a corrected estimate of daily Global Horizontal Irradiance (GHI), which is crucial for making informed decisions about solar energy projects.
-One known limitation is that the model is specifically tuned for Uganda's unique climate and topography, which means it may not be as effective in other regions without further adjustments. Additionally, there may be biases in the training data that could affect predictions, so users should be aware of the context in which the data is applied.
-To ensure responsible AI use, the project has taken steps to validate the model against ground truth data from multiple sites across Uganda, achieving a high accuracy score (R² of 0.86). This validation helps to minimize risks associated with using inaccurate satellite data.
-The platform is designed to be user-friendly, featuring interactive visualizations and an API for easy integration into other applications. Users can access historical datasets on demand, making it a practical tool for energy professionals.
-When building new products using this data, users should credit the source of the work to acknowledge the efforts behind this valuable resource.</t>
+Random Forest model (SuSSE -- Sub-Saharan Solar Estimation) that corrects satellite-derived solar irradiance estimates for Uganda. Input: CAMS and NASA POWER satellite GHI data. Output: bias-corrected daily GHI values. Validated against 56 ground-truth sites across Uganda, achieving R-squared of 0.86 and correcting a 20% overestimation in standard satellite products. Application: deployed as an interactive web portal with maps, charts, and a RESTful API for integration. Code: Python package at github.com/Marconi-Lab/Solar_irradiation (87.9% Jupyter Notebook, 12.1% Python).
+Source: https://github.com/Marconi-Lab/Solar_irradiation, https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately access reliable solar irradiance data for Uganda to enhance your solar energy planning efforts. The Solar Irradiance Portal provides corrected Global Horizontal Irradiance (GHI) data that addresses the inaccuracies found in standard satellite-derived solar data. This means you can confidently assess solar potential, optimize system sizing, and reduce financial risks associated with solar projects.
-To get started, you can explore the interactive visualizations available on the platform, which allow you to analyze solar patterns through dynamic charts and maps. Additionally, you can integrate the corrected solar data into your applications using the provided RESTful API, making it easier to incorporate accurate information into your energy planning tools.
-Researchers and developers can build on this work by extending the model to other regions in Sub-Saharan Africa or by incorporating additional data sources to enhance the accuracy of predictions. Collaborating with local universities or NGOs could provide valuable ground-truth data and insights into regional climate variations, further improving the model's performance.
-It's important to consider that while the model has shown a high accuracy score (R² of 0.86), there may still be limitations related to the specific climate zones and topography of Uganda. Conducting an ethical AI assessment is recommended to ensure that the model's application does not inadvertently reinforce existing biases or overlook local knowledge.
-As for costs, while specific figures are not provided, you should budget for potential expenses related to data integration, API usage, and any necessary computational resources for running analyses. Collaborating with local partners may help reduce costs and enhance the project's impact.
-The platform is designed for long-term use, with ongoing updates and maintenance planned to ensure data accuracy and relevance. By leveraging this resource, you can contribute to the growing field of renewable energy in Uganda and help unlock its solar potential for sustainable development.</t>
+## How to Use This Resource
+This resource addresses a critical problem for solar energy planning in Uganda: standard satellite data sources such as CAMS and NASA POWER systematically overestimate solar irradiance by roughly 20%, which reduces lifetime energy savings for consumers by 5-20% and creates financial risk through incorrect system sizing. The Irradiation Portal provides corrected Global Horizontal Irradiance (GHI) data by applying a machine learning model trained on ground-truth measurements from 56 validation sites across Uganda and 7 African countries, achieving an R-squared accuracy of 0.86.
+Anyone involved in solar project development, rural electrification planning, or energy policy in Uganda can access the corrected data through the [Irradiation Portal web application](https://irradiation-portal-55883164704.europe-west1.run.app/). The portal offers interactive data exploration with dynamic charts and maps, monthly irradiance measurements in kWh/m2/day, and historical data access -- all through a standard web browser. Technical documentation and user support are built into the portal.
+For organisations that want to integrate the corrected solar data into their own planning tools or applications, a RESTful API is available through the portal. This enables automated data retrieval for feasibility studies, system design calculations, or monitoring dashboards.
+Researchers and developers looking to extend the underlying methodology can access the SuSSE (Sub-Saharan Solar Estimation) model code, which is openly available on [GitHub](https://github.com/Marconi-Lab/Solar_irradiation). The repository includes the full codebase with Jupyter Notebooks and Python scripts, along with testing and development tools. This opens possibilities for adapting the correction model to other Sub-Saharan African countries where similar satellite overestimation issues exist.
+Sources:
+- https://github.com/Marconi-Lab/Solar_irradiation
+- https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Marconi Lab
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10417,14 +10159,10 @@
           <t>In Uganda, the Civil Society and Budget Advocacy Group (CSBAG) in partnership with GIZ, has recognized the need for further enhancement in how audit reports are processed and understood. An AI-powered conversational assistant was designed to help anyone understand audit reports. It will answer questions by using Audit reports published by Auditor General Office, Uganda. The prototype tool leverages AI to offer capabilities such as summarizing complex texts, extracting thematic insights, and enabling interactive, user-friendly analysis through a chatbot interface. By making the audit reports more accessible, this aims to increase readership and utilization among stakeholders, which can lead to better accountability and improve service delivery.</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>https://huggingface.co/spaces/GIZ/audit_assistant</t>
-        </is>
-      </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://huggingface.co/spaces/GIZ/audit_assistant</t>
+          <t>https://huggingface.co/spaces/GIZ/audit_assistant/tree/main</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -10462,7 +10200,7 @@
       <c r="P83" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Civil Society and Budget Advocacy Group (CSBAG), GIZ
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10565,7 +10303,7 @@
       <c r="P84" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Makerere University in cooperation with the Uganda National Forestry Authority (NFA)
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10686,7 +10424,7 @@
       <c r="P85" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Makerere AI Lab, Marconi Lab, Clear Global
-Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All
+Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10752,16 +10490,8 @@
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>tbd</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>tbd</t>
-        </is>
-      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>SDG 13</t>
@@ -10820,16 +10550,37 @@
           <t>Enhancing business registration in Kenya through a chatbot</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>The BRS-chatbot is an AI-powered chatbot that streamlines the business registration process in Kenya. It aimes to enhance access to information, simplify the registration process, improve user experience through Human-Centered Design principles, and promote compliance with post-registration requirements. The goal is to reduce reliance on intermediaries and make the registration process more user-friendly and efficient</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>
+</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://brs.go.ke/</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>SDG 8</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Made by People, Kenya (hello@made.ke)</t>
+        </is>
+      </c>
       <c r="K87" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -10839,9 +10590,23 @@
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Made by People, Kenya 
+Catalyzed by: FAIR Forward - AI for All, Digital Transformation Centre Kenya, GIZ
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Balthas Seibold</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="S87" t="inlineStr">
         <is>
           <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
@@ -10851,16 +10616,24 @@
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr">
         <is>
-          <t>https://made.ke/case-studies/giz-kenya-fair-forward-ai-powered-chatbot/</t>
+          <t>https://web.archive.org/web/20251116031001/https://made.ke/case-studies/giz-kenya-fair-forward-ai-powered-chatbot/</t>
         </is>
       </c>
       <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
-      <c r="Y87" t="inlineStr"/>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>Old URL, seems offline https://made.ke/case-studies/giz-kenya-fair-forward-ai-powered-chatbot/</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -10898,7 +10671,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>SDG 9</t>
+          <t>SDG 9, SDG 10</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -10920,23 +10693,21 @@
       <c r="M88" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-KinyCOMET is an AI model designed to automatically evaluate the quality of translations between Kinyarwanda and English. This tool addresses a significant challenge in the translation process, where previous methods relied heavily on manual reviews, making it slow and costly.
-The model takes as input pairs of sentences: the original text (in either Kinyarwanda or English), the machine-generated translation, and a human reference translation. It then produces a quality score ranging from 0 to 1, indicating how well the machine translation matches the human reference. A higher score means better translation quality.
-One of the known limitations of this model is that it may not fully capture the nuances of Kinyarwanda, a morphologically rich language, which can lead to discrepancies between the model's scores and human judgment. Additionally, the model's performance may vary depending on the specific translation direction, as indicated by the average scores for different language pairs.
-To ensure responsible AI use, the dataset used to train KinyCOMET was created with careful consideration. It includes 4,323 human-annotated translation pairs, with each pair evaluated by multiple annotators to maintain quality. The annotations followed established international standards, and samples with high variability were removed to enhance reliability.
-There are no specific critical software or hardware requirements mentioned for running the model, but users will need access to the necessary libraries and tools to load and utilize the dataset and model effectively.
-This dataset and model are open-source, meaning they can be freely used and adapted by researchers and developers. When building new products or applications based on KinyCOMET, users should credit the original work and dataset creators.
-For more information, you can access the dataset at Hugging Face: [KinyCOMET Dataset](https://huggingface.co/datasets/chrismazii/kinycomet_dataset).</t>
+Pretrained Model: KinyCOMET-Unbabel, a translation quality estimation model for Kinyarwanda-English (bidirectional). Fine-tuned on Unbabel/wmt22-comet-da using the COMET framework. Input: source text, machine translation, and human reference translation. Output: quality score from 0 to 1. Achieves 0.75 Pearson correlation with human judgments (vs. 0.30 for BLEU), Spearman 0.59, MAE 0.07. A second variant (KinyCOMET-XLM) based on XLM-RoBERTa-large achieves 0.73 Pearson. Trained on 4,323 human-annotated translation pairs scored by 15 annotators following WMT Direct Assessment standards. Install via pip install unbabel-comet; load with comet.load_from_checkpoint("chrismazii/kinycomet_unbabel"). License: Apache 2.0.
+Source: https://huggingface.co/datasets/chrismazii/kinycomet_dataset, https://huggingface.co/chrismazii/kinycomet_unbabel</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately use the KinyCOMET dataset to enhance the quality of Kinyarwanda-English machine translations by integrating it into your translation workflows. This dataset provides 4,323 human-annotated translation quality assessments, allowing you to automatically evaluate translations without relying on time-consuming manual reviews. By using the KinyCOMET model, you can assess the quality of translations in real-time, which can significantly speed up the translation process for applications in education, tourism, and other sectors.
-To build on this resource, researchers and developers can extend the KinyCOMET model by training it with additional datasets or fine-tuning it on specific domains relevant to their work. This could involve collecting more translation pairs or incorporating user feedback to improve the model's accuracy. Collaborating with local linguists or educational institutions can also provide valuable insights and data for further development.
-When replicating or adapting this work, it’s important to consider potential limitations and biases. The dataset is based on a specific set of translation pairs and may not cover all dialects or variations of Kinyarwanda. Additionally, the quality scores are based on human assessments, which can be subjective. Therefore, conducting an ethical AI assessment before deploying the model in sensitive contexts is recommended.
-In terms of costs, building on this dataset may involve expenses related to data storage, compute resources for training models, and potential collaboration with linguists or developers. Depending on your specific needs, costs can vary widely, but initial estimates for cloud computing resources can range from a few hundred to several thousand dollars, depending on the scale of your project.
-For those interested in using KinyCOMET, documentation is available on Hugging Face, which includes tutorials on loading the dataset and using the model. Engaging with the community on platforms like Hugging Face can also lead to collaboration opportunities and shared success stories, helping to foster innovation in Kinyarwanda-English translation efforts.</t>
+## How to Use This Resource
+KinyCOMET is a tool for automatically evaluating the quality of Kinyarwanda-English translations. It scores translations on a 0-to-1 scale, achieving a 0.75 Pearson correlation with human judgments -- roughly 2.5 times more accurate than traditional BLEU scores for this language pair. Scores above 0.8 indicate high-quality translations.
+This resource is valuable for anyone developing or deploying machine translation systems involving Kinyarwanda, whether for development programmes, government communications, educational materials, or other contexts where translation quality matters. Rather than relying on expensive and time-consuming human evaluation for every translation, KinyCOMET provides a reliable automated quality check that can be integrated into translation workflows. The model is available on [Hugging Face as chrismazii/kinycomet_unbabel](https://huggingface.co/chrismazii/kinycomet_unbabel), with an alternative variant (KinyCOMET-XLM, built on XLM-RoBERTa-large) also available. Both can be used through the open-source COMET library.
+The accompanying dataset, hosted on [Hugging Face as chrismazii/kinycomet_dataset](https://huggingface.co/datasets/chrismazii/kinycomet_dataset), contains 4,303 human-annotated translation pairs with quality scores. These were annotated by 15 linguistics students, with a minimum of 3 annotations per sample, covering both translation directions (Kinyarwanda-to-English and English-to-Kinyarwanda) across education, tourism, and general domains. The dataset is split into train (3,497 samples), validation (404), and test (422), and is licensed under Apache 2.0.
+Researchers can use this dataset to train improved evaluation models for Kinyarwanda or adapt the methodology to other low-resource African languages where automated translation quality assessment is similarly lacking. The human annotations provide a ground-truth benchmark that did not previously exist for this language pair.
+Sources:
+- https://huggingface.co/datasets/chrismazii/kinycomet_dataset
+- https://huggingface.co/chrismazii/kinycomet_unbabel</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -10947,7 +10718,7 @@
       <c r="P88" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Mbaza NLP community, German Research Center for Artificial Intelligence (DFKI), Regional AI Hub Rwanda
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -10988,12 +10759,12 @@
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Tunga Agri-Chatbot Suite</t>
+          <t>Tunga Chatbot Open Source Suite -  A system to build call center agent based voicebots in Kinyarwanda e.g. for Agriculture and other sectors</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Tunga Agri-Chatbot Suite</t>
+          <t>Tunga Agri-Chatbot Open Source Suite -  A full system to build call center agent based voicebots in Kinyarwanda e.g. for Agriculture and other sectors</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -11032,7 +10803,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>SDG 2, SDG 1</t>
+          <t>SDG 10, SDG 2</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -11053,35 +10824,34 @@
       <c r="L89" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Kinyarwanda Agricultural Text-to-Speech Dataset is designed to support the Tunga Agri-Chatbot Suite, which aims to provide agricultural information to Rwandan farmers through voice technology. Here are the key characteristics of the dataset:
-- **Content and Format**: The dataset includes audio recordings of male and female voice actors reading agricultural information. It contains a total of 10,480 audio clips (5,242 from female actors and 5,238 from male actors). The audio files are in WAV format, sampled at 24 KHz, and are mono-channel. The accompanying text is provided in tab-separated values (TSV) files, where each entry includes an audio clip ID and the corresponding text.
-- **Limitations and Biases**: While the dataset provides a wealth of information, it may not cover all agricultural topics comprehensively. Additionally, the reliance on only two voice actors could introduce a lack of diversity in voice representation, which may affect user engagement.
-- **Responsible and Ethical Use**: The dataset is intended for use in developing voice-driven interfaces that improve access to agricultural information for farmers, particularly those in rural areas with limited access to technology. The project emphasizes the importance of making information accessible to non-English speakers and those with low literacy.
-- **Maintenance and Updates**: The dataset is maintained by C4IR Rwanda and KiNLP, with support from GIZ and financing from BMZ. They are responsible for any updates or improvements to the dataset.
-- **User Rights and License**: The dataset is published under the Creative Commons Attribution 4.0 International License (CC-BY 4.0). Users are free to reuse the data, provided they give appropriate credit to C4IR Rwanda and KiNLP.
-This dataset is a valuable resource for organizations looking to enhance agricultural advisory services through voice technology, particularly in regions where traditional information channels are insufficient.</t>
+Two Kinyarwanda agricultural datasets. (1) TTS Dataset (kinya-ag-tts): 10,480 audio clips (5,242 female, 5,238 male) of voice actors reading agricultural content. Format: WAV mono at 24 kHz, with TSV metadata mapping clip IDs to text. Total size: 2.63 GB. (2) Retrieval Dataset (kinya-ag-retrieval): 984 agricultural passages in Kinyarwanda paired with 19,537 questions. Structured as query-positive-negative triplets for training retrieval models (1,901,200 training triplets, 19,600 dev, 32,900 test). Format: TSV. Includes morphologically parsed versions of passages and queries. Both datasets created by C4IR Rwanda and KiNLP. License: CC-BY 4.0.
+Source: https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts, https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-The Tunga Agri-Chatbot Suite is an AI-powered voicebot designed to help farmers in Rwanda access important agricultural information. It operates through a telephone hotline that speaks Kinyarwanda, making it accessible to users who may not have internet access or who are not fluent in English. 
-The voicebot provides advice on various agricultural topics, including pest and disease diagnosis, agro-climatic practices, and information about government support programs for farmers, such as crop insurance. This service is available 24/7, ensuring that farmers can get the information they need at any time.
-To use the voicebot, farmers simply call the hotline and interact with the system using their voice. The output is spoken advice tailored to their inquiries, delivered in their local language.
-While the voicebot aims to bridge the gap in agricultural information access, there are some limitations. The system relies on the quality of the voice recordings and may not cover every possible agricultural question. Additionally, as with any AI system, there may be biases in the information provided based on the data it was trained on.
-To ensure responsible AI use, the project has undergone ethical assessments, and the developers encourage users to credit the original creators, C4IR Rwanda and KiNLP, when building new products based on this work. 
-The voicebot requires basic telephone infrastructure to operate, making it suitable for rural areas where internet connectivity may be limited. 
-Overall, the Tunga Agri-Chatbot Suite represents a significant step towards making agricultural support more accessible and responsive to the needs of farmers in Rwanda.</t>
+Two pretrained models for a Kinyarwanda agricultural IVR system. (1) TTS Model (kinya-flex-tts): Multi-speaker text-to-speech based on MB-iSTFT-VITS2 architecture. Converts Kinyarwanda text to speech at 24 kHz with 3 speaker options (2 female, 1 male). Requires PyTorch; implementation via the DeepKIN-AgAI package. (2) Retrieval Model (kiny-colbert-free): Information retrieval model for RAG, fine-tuned from Davlan/bert-base-multilingual-cased-finetuned-kinyarwanda. 0.2B parameters, F32 safetensors format. Trained on agricultural question-passage pairs. Usable via ragatouille library. Both models by C4IR Rwanda and KiNLP. License: CC-BY 4.0.
+Source: https://huggingface.co/C4IR-RW/kinya-flex-tts, https://huggingface.co/C4IR-RW/kiny-colbert-free</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
-You can immediately use the Tunga Agri-Chatbot Suite to create a voice-based agricultural advisory service for farmers in Rwanda. By leveraging the Kinyarwanda Agricultural Text-to-Speech Dataset, you can develop a voicebot that provides critical information on pest and disease management, agro-climatic practices, and government support programs, all accessible via a simple telephone hotline. This is particularly beneficial for farmers who may not have internet access or who are not fluent in English.
-To build on this resource, researchers and developers can enhance the existing voicebot by incorporating additional agricultural topics, improving the naturalness of the voice output, or expanding the dataset with more diverse agricultural scenarios. Collaborating with local agricultural experts can help ensure that the information provided is relevant and up-to-date. Additionally, you can explore integrating feedback mechanisms to continuously improve the service based on user interactions.
-When replicating this project, it is essential to consider potential limitations, such as biases in the dataset or the need for ethical assessments to ensure that the voicebot serves all farmers equitably. The dataset includes recordings from only two voice actors, which may limit the diversity of voices and accents represented. 
-In terms of costs, building on this project may require investment in training and adaptation of the voicebot, which could range from a few hundred to several thousand dollars depending on the scale of the implementation and the resources needed for voice synthesis and infrastructure. You may also need to budget for ongoing maintenance and updates to the system.
-For further guidance, you can refer to the technical documentation provided with the dataset, which includes details on the audio files and their structure. Engaging with organizations like C4IR Rwanda and KiNLP can also provide valuable support and collaboration opportunities.</t>
+## How to Use This Resource
+The Tunga Agri-Chatbot Suite provides the building blocks for a Kinyarwanda-language agricultural advisory system delivered via Interactive Voice Response (IVR). It was built to address capacity gaps in Rwanda's agricultural extension services and is implemented by C4IR Rwanda and KiNLP, supported by GIZ and financed by BMZ.
+This suite is relevant for anyone working on agricultural extension, farmer advisory services, or voice-based information delivery in Rwanda or similar contexts. The core idea is that smallholder farmers can call a phone number and receive spoken agricultural guidance in Kinyarwanda -- covering topics such as pest and disease diagnosis, agro-climatic practices, and MINAGRI support programmes -- without needing internet access or literacy.
+The text-to-speech component (kinya-flex-tts) can generate natural-sounding Kinyarwanda speech with three voice options (two female, one male), outputting audio at broadcast quality (24 kHz). A live demo is available at [huggingface.co/spaces/Professor/c4ir-rw-kinyarwandatts](https://huggingface.co/spaces/Professor/c4ir-rw-kinyarwandatts), where you can hear sample outputs before deciding whether to integrate the model. The underlying TTS training dataset contains 10,482 audio clips recorded by two voice actors, all licensed under CC-BY-4.0.
+The passage retrieval component (kiny-colbert-free) matches farmer questions in Kinyarwanda to relevant agricultural knowledge passages. This is the engine that allows the system to find the right answer from a knowledge base when a farmer asks a question. The accompanying retrieval dataset contains 984 agricultural passages, 19,537 related questions, and nearly 2 million training triplets, also under CC-BY-4.0.
+The suite also includes KinyaBERT, a morphology-aware language model for Kinyarwanda used for passage ranking, available in base (107M parameter) and large (365M parameter) variants. All model code, training scripts, and technical documentation are available in the [DeepKIN-AgAI package on GitHub](https://github.com/c4ir-rw/ac-ai-models/tree/main/DeepKIN-AgAI). All components require attribution to C4IR Rwanda and KiNLP.
+Developers and researchers can extend this work to other crops, regions, or languages, or integrate these components into existing agricultural advisory platforms. The individual models (TTS, retrieval, language understanding) can also be used independently for other Kinyarwanda language technology applications beyond agriculture. All datasets and models are hosted on Hugging Face under the [C4IR-RW organisation](https://huggingface.co/C4IR-RW).
+Sources:
+- https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts
+- https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval
+- https://huggingface.co/C4IR-RW/kinya-flex-tts
+- https://huggingface.co/C4IR-RW/kiny-colbert-free
+- https://huggingface.co/C4IR-RW/kinyabert
+- https://github.com/c4ir-rw/ac-ai-models</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -11092,7 +10862,7 @@
       <c r="P89" t="inlineStr">
         <is>
           <t>Powered by / Provided by: C4IR, KiNLP
-Catalyzed by: FAIR Forward - AI for All
+Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -11189,102 +10959,40 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ui_90</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Two Al-based dialogue systems (e.g. voice-based chatbot) in Indian Languages - consultancy for design implementation etc</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Voice-based advisory for farmers (female kitchen gardeners) with NiceSSM / Use Case Gramvaani</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Voice-based advisory for farmers (female kitchen gardeners) with NiceSSM / Use Case Gramvaani</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Creation of voice based chatbots</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>There is no report, no data, no results available here. Remove</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>There is no report, no data, no results available here. Remove</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>SDG 10</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Voice</t>
-        </is>
-      </c>
+          <t>ui_91</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>Powered by / Provided by:
-Catalyzed by: FAIR Forward - AI for All
-Financed by: BMZ</t>
-        </is>
-      </c>
+      <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr">
-        <is>
-          <t>Dataset &gt; Model &gt; Pilot</t>
-        </is>
-      </c>
-      <c r="T92" t="inlineStr">
-        <is>
-          <t>NLP</t>
-        </is>
-      </c>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
-      <c r="X92" t="inlineStr">
-        <is>
-          <t>pilot that did not go online (--&gt;lessons learned documentation needed)</t>
-        </is>
-      </c>
-      <c r="Y92" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="X92" t="inlineStr"/>
+      <c r="Y92" t="inlineStr"/>
       <c r="Z92" t="inlineStr"/>
-      <c r="AA92" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="AA92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ui_91</t>
+          <t>ui_92</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -11317,7 +11025,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ui_92</t>
+          <t>ui_93</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
@@ -11350,7 +11058,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ui_93</t>
+          <t>ui_94</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -11383,7 +11091,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ui_94</t>
+          <t>ui_95</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
@@ -11416,7 +11124,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ui_95</t>
+          <t>ui_96</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -11449,7 +11157,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ui_96</t>
+          <t>ui_97</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -11482,7 +11190,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ui_97</t>
+          <t>ui_98</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -11515,7 +11223,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ui_98</t>
+          <t>ui_99</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -11548,7 +11256,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ui_99</t>
+          <t>ui_100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -11581,7 +11289,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ui_100</t>
+          <t>ui_101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -11614,7 +11322,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ui_101</t>
+          <t>ui_102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
@@ -11647,7 +11355,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ui_102</t>
+          <t>ui_103</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -11680,7 +11388,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ui_103</t>
+          <t>ui_104</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -11713,7 +11421,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ui_104</t>
+          <t>ui_105</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -11746,7 +11454,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ui_105</t>
+          <t>ui_106</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -11779,7 +11487,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ui_106</t>
+          <t>ui_107</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -11812,7 +11520,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ui_107</t>
+          <t>ui_108</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -11845,7 +11553,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ui_108</t>
+          <t>ui_109</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -11878,7 +11586,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ui_109</t>
+          <t>ui_110</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -11911,7 +11619,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ui_110</t>
+          <t>ui_111</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -11944,7 +11652,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ui_111</t>
+          <t>ui_112</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -11977,7 +11685,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ui_112</t>
+          <t>ui_113</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -12010,7 +11718,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ui_113</t>
+          <t>ui_114</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -12043,7 +11751,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ui_114</t>
+          <t>ui_115</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -12076,7 +11784,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ui_115</t>
+          <t>ui_116</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -12109,7 +11817,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ui_116</t>
+          <t>ui_117</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -12142,7 +11850,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ui_117</t>
+          <t>ui_118</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -12175,7 +11883,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ui_118</t>
+          <t>ui_119</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -12208,7 +11916,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ui_119</t>
+          <t>ui_120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -12241,7 +11949,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ui_120</t>
+          <t>ui_121</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -12274,7 +11982,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ui_121</t>
+          <t>ui_122</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -12307,7 +12015,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ui_122</t>
+          <t>ui_123</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
@@ -12340,7 +12048,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ui_123</t>
+          <t>ui_124</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
@@ -12373,7 +12081,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ui_124</t>
+          <t>ui_125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -12406,7 +12114,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ui_125</t>
+          <t>ui_126</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
@@ -12439,7 +12147,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ui_126</t>
+          <t>ui_127</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -12472,7 +12180,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ui_127</t>
+          <t>ui_128</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -12505,7 +12213,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ui_128</t>
+          <t>ui_129</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
@@ -12538,7 +12246,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ui_129</t>
+          <t>ui_130</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -12571,7 +12279,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ui_130</t>
+          <t>ui_131</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -12604,7 +12312,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ui_131</t>
+          <t>ui_132</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
@@ -12637,7 +12345,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ui_132</t>
+          <t>ui_133</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
@@ -12670,7 +12378,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ui_133</t>
+          <t>ui_134</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -12703,7 +12411,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ui_134</t>
+          <t>ui_135</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
@@ -12736,7 +12444,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ui_135</t>
+          <t>ui_136</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -12769,7 +12477,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ui_136</t>
+          <t>ui_137</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
@@ -12802,7 +12510,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ui_137</t>
+          <t>ui_138</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
@@ -12835,7 +12543,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ui_138</t>
+          <t>ui_139</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
@@ -12868,7 +12576,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ui_139</t>
+          <t>ui_140</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
@@ -12901,7 +12609,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ui_140</t>
+          <t>ui_141</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
@@ -12934,7 +12642,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ui_141</t>
+          <t>ui_142</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
@@ -12967,7 +12675,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ui_142</t>
+          <t>ui_143</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
@@ -13000,7 +12708,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ui_143</t>
+          <t>ui_144</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -13033,7 +12741,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ui_144</t>
+          <t>ui_145</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
@@ -13066,7 +12774,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ui_145</t>
+          <t>ui_146</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
@@ -13099,7 +12807,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ui_146</t>
+          <t>ui_147</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
@@ -13132,7 +12840,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ui_147</t>
+          <t>ui_148</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
@@ -13165,7 +12873,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ui_148</t>
+          <t>ui_149</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -13198,7 +12906,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ui_149</t>
+          <t>ui_150</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
@@ -13231,7 +12939,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ui_150</t>
+          <t>ui_151</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -13264,7 +12972,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ui_151</t>
+          <t>ui_152</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -13294,39 +13002,6 @@
       <c r="Z153" t="inlineStr"/>
       <c r="AA153" t="inlineStr"/>
     </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>ui_152</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
-      <c r="N154" t="inlineStr"/>
-      <c r="O154" t="inlineStr"/>
-      <c r="P154" t="inlineStr"/>
-      <c r="Q154" t="inlineStr"/>
-      <c r="R154" t="inlineStr"/>
-      <c r="S154" t="inlineStr"/>
-      <c r="T154" t="inlineStr"/>
-      <c r="U154" t="inlineStr"/>
-      <c r="V154" t="inlineStr"/>
-      <c r="W154" t="inlineStr"/>
-      <c r="X154" t="inlineStr"/>
-      <c r="Y154" t="inlineStr"/>
-      <c r="Z154" t="inlineStr"/>
-      <c r="AA154" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: refresh catalog from Google Sheet
- EWS typo fix in ui_40 how_to_use ("Eearly Warning System")
- ui_40: add 2 additional resources, add "Text" data type
- Various description/how_to_use newline normalizations (\n -> \r\n)
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2804,8 +2804,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3746,7 +3746,7 @@
       <c r="L28" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3868,7 +3868,8 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
+ </t>
         </is>
       </c>
@@ -4224,22 +4225,22 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4585,7 +4586,7 @@
       <c r="N35" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5159,8 +5160,8 @@
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -5479,7 +5480,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Geospatial/Remote Sensing, Images</t>
+          <t>Geospatial/Remote Sensing, Images, Text</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -5522,7 +5523,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t xml:space="preserve">The EWS provides a comprehensive platform that combines AI-powered crop monitoring with localized advisory services. Organizations can access the data and models through :A self-serve platform and API for accessing predictions and analytics; Mobile applications for farmers to receive personalized crop management recommendations in local language; Integration possibilities with existing agricultural extension services and Analytics dashboards for value chain stakeholders and policy institutions. The system can be scaled to new regions and crops through transfer learning and the modular architecture allowing for continuous improvement of individual components. The platform supports both individual farmer-level insights and aggregated regional analytics to optimize crop yields and manage stressors effectively, making it valuable for various stakeholders across the agricultural sector.
+          <t xml:space="preserve">The Eearly Warning System provides a comprehensive platform that combines AI-powered crop monitoring with localized advisory services. Organizations can access the data and models through :A self-serve platform and API for accessing predictions and analytics; Mobile applications for farmers to receive personalized crop management recommendations in local language; Integration possibilities with existing agricultural extension services and Analytics dashboards for value chain stakeholders and policy institutions. The system can be scaled to new regions and crops through transfer learning and the modular architecture allowing for continuous improvement of individual components. The platform supports both individual farmer-level insights and aggregated regional analytics to optimize crop yields and manage stressors effectively, making it valuable for various stakeholders across the agricultural sector.
 This use case is also linked to the development of a business model / funding model for open source AI as a stepping stone towards financially viable operations. It was part of Villgro Africa's and "FAIR Forward — AI for All"'s  six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/  </t>
         </is>
       </c>
@@ -5553,7 +5554,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>Smart sowing: AI for more harvest in Kenya and Uganda | BMZ Digital.Global</t>
+          <t xml:space="preserve">https://www.bmz-digital.global/en/smart-sowing-ai-for-more-harvest-in-kenya-and-uganda/; https://www.developlocal.org/food-nutrition-early-warning-mechanism/ </t>
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
@@ -6105,10 +6106,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6605,7 +6606,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>
+          <t xml:space="preserve">
 </t>
         </is>
       </c>
@@ -6913,7 +6914,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7533,7 +7534,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
@@ -7919,8 +7920,8 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure. </t>
         </is>
       </c>
@@ -8247,7 +8248,11 @@
           <t>Text</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Chris Prince Mazimpaka chrismazimpaka7@gmail.com</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr">
         <is>
           <t>Rwanda</t>
@@ -8509,7 +8514,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible. </t>
         </is>
       </c>
@@ -9735,7 +9740,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -10001,7 +10006,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10278,8 +10283,8 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: remove invalid ui_58 entry (Chatbot for Public Service Delivery in Rwanda)
Row deleted from the source Google Sheet; rebuilt catalog/insights JSON and
removed the orphaned public/projects/ui_58 and docs/projects/ui_58 directories.
Total projects: 88 -> 87. The ui_58 identifier stays unused per sheet
convention; future entries should pick the next unused ui number.
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA153"/>
+  <dimension ref="A1:AA152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7645,46 +7645,40 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ui_58</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Bot of Bots Activity - in collaboration with Govstack for Kenya</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Chatbot for Public Service Delivery in Rwanda</t>
-        </is>
-      </c>
+          <t>ui_59</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A large scale collection of voice data in Kinyarwanda to allow the building of inclusive language technology </t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Semantic Chatbot(s) &amp; IVR for G2C services in Public Service Delivery and Good Governance 
- in Collaboration with Konza Technopolis, ICTA</t>
+          <t xml:space="preserve">This effort created the largest open-source voice dataset of diverse Kinyarwanda speakers for speech recognition (speech-to-text). It collected more than 2380  hours of AI voice data in Kinyarwanda (by 03/2026). You can use this resource to build AI systems understanding spoken Kinyarwanda e.g. in cellphones . This facilitates access to information in mother tongue, including by illiterate persons and in rural settings. </t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: konza@konza.go.ke
-</t>
+          <t xml:space="preserve">https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw ; https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset  </t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>SDG 10</t>
+          <t>SDG 2, SDG 10</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Text, Voice</t>
+          <t>Voice</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Konza Technopolis ( https://konza.go.ke/)</t>
+          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -7692,104 +7686,21 @@
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>Powered by / Provided by: Konza Technopolis, ICTA
-Catalyzed by: FAIR Forward - AI for All, GIZ
-Financed by: BMZ</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr">
-        <is>
-          <t>Dataset &gt; Model &gt; Pilot</t>
-        </is>
-      </c>
-      <c r="T61" t="inlineStr">
-        <is>
-          <t>NLP</t>
-        </is>
-      </c>
-      <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z61" t="inlineStr"/>
-      <c r="AA61" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ui_59</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A large scale collection of voice data in Kinyarwanda to allow the building of inclusive language technology </t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This effort created the largest open-source voice dataset of diverse Kinyarwanda speakers for speech recognition (speech-to-text). It collected more than 2380  hours of AI voice data in Kinyarwanda (by 03/2026). You can use this resource to build AI systems understanding spoken Kinyarwanda e.g. in cellphones . This facilitates access to information in mother tongue, including by illiterate persons and in rural settings. </t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw ; https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset  </t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>SDG 2, SDG 10</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Voice</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Rwanda</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Common Voice Scripted Speech 25.0 - Kinyarwanda: a collection of read speech recordings in Kinyarwanda hosted on Mozilla Data Collective. Size: 57.18 GB. Format: MP3. Designed for automatic speech recognition (ASR). License: CC0-1.0. Additionally, the common-voice-kinyarwanda-english-dataset by Mbaza NLP on Hugging Face provides a Kinyarwanda-English bilingual dataset with 721,395 rows (619,000 train / 61,600 validation / 41,200 test) for training multilingual ASR systems. Size: 166 MB (CSV). License: CC-BY-4.0.
 Source: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw, https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="M61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Provides speech-to-text training data for Kinyarwanda. The Common Voice dataset (57.18 GB, MP3, CC0-1.0) enables building ASR systems that transcribe spoken Kinyarwanda into text. The complementary Kinyarwanda-English dataset by Mbaza NLP (721,395 rows, CC-BY-4.0) supports multilingual ASR development. Both datasets can be used to build voice-enabled applications such as speech recognition on mobile devices.
 Source: https://datacollective.mozillafoundation.org/datasets?q=common+voice&amp;locale=rw, https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="N61" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 ## How to Use This Resource
@@ -7802,72 +7713,72 @@
 - https://huggingface.co/datasets/mbazaNLP/common-voice-kinyarwanda-english-dataset</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr">
+      <c r="O61" t="inlineStr">
         <is>
           <t>CC-0</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="P61" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Umuganda, Mozilla Common Voice
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
+      <c r="Q61" t="inlineStr">
         <is>
           <t>Balthas Seibold</t>
         </is>
       </c>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr">
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T62" t="inlineStr">
+      <c r="T61" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr"/>
-      <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z62" t="inlineStr"/>
-      <c r="AA62" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>ui_60</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>ML4EO Crop Mapping Solution Rwanda</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t xml:space="preserve">Solutions from space: Rwanda’s smart harvest planning - mapping crop type with AI for rice, maize, Irish potatoes and beans </t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t xml:space="preserve">Solutions from space: Rwanda’s smart harvest planning - mapping crop type with AI for rice, maize, Irish potatoes and beans </t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t xml:space="preserve">When weather and crop yields become unpredictable, reliable information is crucial. In Rwanda, digital maps are showing for the first time exactly where which crops grow, helping to better adapt agriculture to climate change. Around one third of all food worldwide is lost between the field and the plate, for example due to pest infestation, incorrect storage or long transport routes. Climate change is exacerbating these losses: irregular rainfall, dry seasons and extreme weather events are jeopardising harvests and making planning increasingly difficult for farmers. Rwanda’s agricultural sector also faces these challenges. 
 This automated crop type mapping system for Rwanda can be used in various applications e.g. improving agricultural policy and business decisions, integrating with yield estimation frameworks for spatially detailed predictions of seasonal production, crop health monitoring, crop insurance design, value chain assessments, supply and demand forecasting, and more.
@@ -7876,61 +7787,61 @@
 </t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/O7IDTD</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>https://github.com/crop-type-mapping</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H62" t="inlineStr">
         <is>
           <t>SDG 2</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>Benson Kenduiyvo (b.kenduiywo@cgiar.org)</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>The overall good accuracy yielded by the approach under conditions with small field sizes, varying elevation and high cloud cover are promising for a successful application in all kinds of regions. Nevertheless, local reference data remains crucial for crop type mapping and an ideal approach should include all types of crops. You can follow the approach to create your own crop type mapping system, utilize the pipeline to fetch satellite imagery for various purposes, get inspired by the use and fine-tuning of the geospatial foundational model and apply it to a different task. You can also use the collected reference data for your own model.</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="M62" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Machine learning pipeline for crop type classification in Rwanda using Sentinel-1 and Sentinel-2 satellite imagery. Training scripts include Random Forest and climate-corrected models. Ground reference data covers four districts (Nyagatare, Musanze, Nyabihu, Ruhango) with field observations of maize, beans, rice, and Irish potato collected May-June 2025. The ground truth dataset contains GPS-located farm plots with crop attributes, management practices, and directional photographs. Code: Python scripts for satellite data preparation, image download, and model training at github.com/crop-type-mapping/ML. License: MIT (code), CC-BY 4.0 (ground reference data).
 Source: https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/O7IDTD, https://github.com/crop-type-mapping</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="N62" t="inlineStr">
         <is>
           <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
 The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure. </t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
+      <c r="O62" t="inlineStr">
         <is>
           <t>MIT License</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="P62" t="inlineStr">
         <is>
           <t>Powered by / Provided by:
 Rwanda Space Agency (RSA), the Rwandan Ministry of Agriculture, Alliance of Bioversity International and CIAT
@@ -7940,399 +7851,399 @@
 BMZ</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q62" t="inlineStr">
         <is>
           <t>Golo Rademacher</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr">
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
         <is>
           <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case &gt;  Use-Case with Business Model</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="T62" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr">
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.bmz-digital.global/en/digital-maps-agriculture-rwanda/ </t>
         </is>
       </c>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr">
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr">
         <is>
           <t>More details as well as link to data to be added</t>
         </is>
       </c>
-      <c r="Y63" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z63" t="inlineStr"/>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>ui_61</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr">
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
         <is>
           <t>Better language translation for more training content in Kinyarwanda - education-specific machine translation for the Moodle Learning Management System</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Better language translation for more training content in Kinyarwanda - education-specific machine translation for the Moodle Learning Management System</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t xml:space="preserve">Enabling language translation capabilities on the Moodle LMS platform, through a collaboration with Atingi; the use case explores 3 modes of translation. The first mode is navigation based, simply translating static messages such as buttons and notifications, secondly it explores full content translation, lastly, in-line translation. The project uses the NLLB-200 model for translation, other models could be experimented to explore feasibility of additional features such as QA or summarization, leveraging the plugin built by the team. </t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t xml:space="preserve">https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset;  https://huggingface.co/datasets/mbazaNLP/Kinyarwanda_English_parallel_dataset; https://huggingface.co/datasets/mbazaNLP/NMT_Education_parallel_data_en_kin; https://huggingface.co/datasets/DigitalUmuganda/kinyarwanda-english-machine-translation-dataset </t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t xml:space="preserve">https://huggingface.co/mbazaNLP/Quantized_Nllb_Finetuned_Edu_En_Kin_8bit; https://huggingface.co/mbazaNLP/Nllb_finetuned_general_en_kin; https://huggingface.co/DigitalUmuganda/Finetuned-NLLB </t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>SDG 4</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>Parallel datasets can be used to finetune LLMs to specific languages or domains; the example is for English-Kinyarwanda, to improve NLLB translation performance</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="M63" t="inlineStr">
         <is>
           <t xml:space="preserve">Open source model NLLB-200, some variations quantized to minimize compute resource usage </t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t xml:space="preserve">Integrate preferred machine translation model with Moodle plugin: https://github.com/Digital-Umuganda/moodle-translate_courses . Need to update for compatibility with newer Moodle updates, this was implemented during Moodle version 3.0 </t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
+      <c r="O63" t="inlineStr">
         <is>
           <t>Permissive</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr">
+      <c r="P63" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Atingi, Digital Umuganda, Clear Global
 Catalyzed by: GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q64" t="inlineStr">
+      <c r="Q63" t="inlineStr">
         <is>
           <t>Isaac</t>
         </is>
       </c>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr">
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
         <is>
           <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
-      <c r="T64" t="inlineStr">
+      <c r="T63" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr">
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr">
         <is>
           <t xml:space="preserve">- https://moodlemoot.org/2024/timetable/event/246/ / https://aiopeneducation.pubpub.org/pub/7npwm2su/release/5?readingCollection=06969c6d </t>
         </is>
       </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z64" t="inlineStr"/>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>ui_62</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr">
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
         <is>
           <t>Preventing Sexual and Gender-Based Violence -  a featurephone-based information chatbot (*350#)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Preventing Sexual and Gender-Based Violence -  a featurephone-based information chatbot (*350#)</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Enabling people to access essential information around Sexual and Gender-Based Violence free of charge and anonymously. This innovative tool requires only a feature phone, with no internet connectivity needed. A collaborative effort between HDI-Rwanda and GIZ-Rwanda. As of November 27 (2024), the chatbot has reached an impressive 343,475 unique users, up from 160,000 on October 1st, with 1,991,660 interactions recorded today compared to 1,170,000 interactions in October. Update of stats pending</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>The dataset was not made public (FAIR Forward status: experiment)</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>The dataset was not made public (FAIR Forward status: experiment)</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H64" t="inlineStr">
         <is>
           <t>SDG 10, SDG 5</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr">
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
         <is>
           <t>CC0</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr">
+      <c r="P64" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Health Development Initiative (HDI) Rwanda
 Catalyzed by: GIZ (Sexualised and Gender-Based Violence (P-SGBV) Project), GIZ ZFD SIGA Refugee Programme, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/)
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr">
+      <c r="Q64" t="inlineStr">
         <is>
           <t>Isaac Manzi, Christiane Adamczyk</t>
         </is>
       </c>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr">
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
         <is>
           <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr">
+      <c r="T64" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="U64" t="inlineStr">
         <is>
           <t>https://media.licdn.com/dms/image/v2/D4D12AQG7JeoDl_2G4A/article-inline_image-shrink_1000_1488/article-inline_image-shrink_1000_1488/0/1732798105403?e=1765411200&amp;v=beta&amp;t=H76TKILEehQZZALbkbiW_Vrar9cCQSR2v5fHVKKrgvc</t>
         </is>
       </c>
-      <c r="V65" t="inlineStr">
+      <c r="V64" t="inlineStr">
         <is>
           <t>Link 1 , Link 2, Link 3</t>
         </is>
       </c>
-      <c r="W65" t="inlineStr">
+      <c r="W64" t="inlineStr">
         <is>
           <t>The chatbot framework that inspired these use cases shall later be registered as DPG</t>
         </is>
       </c>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z65" t="inlineStr"/>
-      <c r="AA65" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr"/>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>ui_86</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr">
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
         <is>
           <t>KinyCOMET: Automatic evaluation of machine translation for Kinyarwanda-English</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>KinyCOMET: Automatic evaluation of machine translation for Kinyarwanda-English</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Until now, the lack of automatic evaluation tools made Kinyarwanda-English machine translation development slow and expensive, as it required manual human review. We’ve bridged this gap by creating a new evaluation dataset and model. Both are now open-source to support the research community. Our methodology and results are detailed in our upcoming paper for LREC 2026.</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/chrismazii/kinycomet_dataset</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>https://huggingface.co/chrismazii/kinycomet_unbabel</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>SDG 9, SDG 10</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>Chris Prince Mazimpaka chrismazimpaka7@gmail.com</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>4000 rows of parallel sentences English - Kinyarwanda with annotated translation quality as Direct Assessment</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Pretrained Model: KinyCOMET-Unbabel, a translation quality estimation model for Kinyarwanda-English (bidirectional). Fine-tuned on Unbabel/wmt22-comet-da using the COMET framework. Input: source text, machine translation, and human reference translation. Output: quality score from 0 to 1. Achieves 0.75 Pearson correlation with human judgments (vs. 0.30 for BLEU), Spearman 0.59, MAE 0.07. A second variant (KinyCOMET-XLM) based on XLM-RoBERTa-large achieves 0.73 Pearson. Trained on 4,323 human-annotated translation pairs scored by 15 annotators following WMT Direct Assessment standards. Install via pip install unbabel-comet; load with comet.load_from_checkpoint("chrismazii/kinycomet_unbabel"). License: Apache 2.0.
 Source: https://huggingface.co/datasets/chrismazii/kinycomet_dataset, https://huggingface.co/chrismazii/kinycomet_unbabel</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr">
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
         <is>
           <t>Apache 2.0</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr">
+      <c r="P65" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Mbaza NLP community, German Research Center for Artificial Intelligence (DFKI), Regional AI Hub Rwanda
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q66" t="inlineStr">
+      <c r="Q65" t="inlineStr">
         <is>
           <t>Jan Nehring</t>
         </is>
       </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S66" t="inlineStr">
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
         <is>
           <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
-      <c r="T66" t="inlineStr">
+      <c r="T65" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="U65" t="inlineStr">
         <is>
           <t>https://huggingface.co/chrismazii/kinycomet_unbabel/resolve/main/banner.png</t>
         </is>
       </c>
-      <c r="V66" t="inlineStr"/>
-      <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
-      <c r="Y66" t="inlineStr"/>
-      <c r="Z66" t="inlineStr"/>
-      <c r="AA66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr"/>
+      <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>ui_87</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr">
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
         <is>
           <t>Tunga Chatbot Open Source Suite -  A system to build call center agent based voicebots in Kinyarwanda e.g. for Agriculture and other sectors</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Tunga Agri-Chatbot Open Source Suite -  A full system to build call center agent based voicebots in Kinyarwanda e.g. for Agriculture and other sectors</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t xml:space="preserve">Voicebots acting as call center agents—accessible via telephone and capable of speaking local languages—hold immense potential for development cooperation. They provide a vital link to users in rural areas who may lack internet access, have limited literacy, do not speak English or do not own digital devices. We believe voice-driven interfaces are the most intuitive way to bridge the digital divide for these communities.
 As part of the Tunga project, we have developed such a voicebot. To support further innovation in this space, we are releasing a comprehensive suite of foundational AI models and datasets:
@@ -8356,51 +8267,51 @@
 https://github.com/c4ir-rw/ac-ai-models </t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t xml:space="preserve">https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts; https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval </t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>https://huggingface.co/C4IR-RW/kinya-flex-tts;https://huggingface.co/C4IR-RW/kiny-colbert-free; https://huggingface.co/C4IR-RW/kinyabert;https://github.com/c4ir-rw/ac-ai-models</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H66" t="inlineStr">
         <is>
           <t>SDG 10, SDG 2</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="J66" t="inlineStr">
         <is>
           <t>https://c4ir.rw/</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L66" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Two Kinyarwanda agricultural datasets. (1) TTS Dataset (kinya-ag-tts): 10,480 audio clips (5,242 female, 5,238 male) of voice actors reading agricultural content. Format: WAV mono at 24 kHz, with TSV metadata mapping clip IDs to text. Total size: 2.63 GB. (2) Retrieval Dataset (kinya-ag-retrieval): 984 agricultural passages in Kinyarwanda paired with 19,537 questions. Structured as query-positive-negative triplets for training retrieval models (1,901,200 training triplets, 19,600 dev, 32,900 test). Format: TSV. Includes morphologically parsed versions of passages and queries. Both datasets created by C4IR Rwanda and KiNLP. License: CC-BY 4.0.
 Source: https://huggingface.co/datasets/C4IR-RW/kinya-ag-tts, https://huggingface.co/datasets/C4IR-RW/kinya-ag-retrieval</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="M66" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Two pretrained models for a Kinyarwanda agricultural IVR system. (1) TTS Model (kinya-flex-tts): Multi-speaker text-to-speech based on MB-iSTFT-VITS2 architecture. Converts Kinyarwanda text to speech at 24 kHz with 3 speaker options (2 female, 1 male). Requires PyTorch; implementation via the DeepKIN-AgAI package. (2) Retrieval Model (kiny-colbert-free): Information retrieval model for RAG, fine-tuned from Davlan/bert-base-multilingual-cased-finetuned-kinyarwanda. 0.2B parameters, F32 safetensors format. Trained on agricultural question-passage pairs. Usable via ragatouille library. Both models by C4IR Rwanda and KiNLP. License: CC-BY 4.0.
 Source: https://huggingface.co/C4IR-RW/kinya-flex-tts, https://huggingface.co/C4IR-RW/kiny-colbert-free</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr">
+      <c r="N66" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 ## How to Use This Resource
@@ -8419,117 +8330,117 @@
 - https://github.com/c4ir-rw/ac-ai-models</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr">
+      <c r="O66" t="inlineStr">
         <is>
           <t>Apache 2.0</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr">
+      <c r="P66" t="inlineStr">
         <is>
           <t>Powered by / Provided by: C4IR, KiNLP
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr">
+      <c r="Q66" t="inlineStr">
         <is>
           <t>Jan Nehring</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S67" t="inlineStr">
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
         <is>
           <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr">
+      <c r="T66" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
-      <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
-      <c r="AA67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
+      <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>ui_84</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr">
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
         <is>
           <t>CarbonLens</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>Forest Carbon Stock Monitoring for Climate Accountability in Senegal</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t xml:space="preserve">Senegal's forest monitoring agencies have long relied on costly, manual field surveys to estimate how much carbon its forests store — making it difficult to credibly track climate commitments or access carbon finance. This tool automates that process by combining satellite imagery (Sentinel-1, Sentinel-2, GEDI) with field data and machine learning to produce accurate, reproducible estimates of above-ground biomass at scale. The models, datasets and workflows are fully open-source, meaning environmental agencies, researchers and development partners in other countries can adapt and deploy them without starting from scratch. For national governments, it strengthens NDC reporting; for carbon finance bodies, it provides the verifiable data needed to unlock results-based funding; and for the broader AI and climate community, it is a replicable blueprint for low-cost, satellite-driven forest monitoring across the Global South.
 </t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Not yet available</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>Not yet available (still being worked on)</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>SDG 13</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="J67" t="inlineStr">
         <is>
           <t>data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t xml:space="preserve">Senegal </t>
         </is>
       </c>
-      <c r="L68" t="inlineStr">
+      <c r="L67" t="inlineStr">
         <is>
           <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible. </t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="M67" t="inlineStr">
         <is>
           <t>The model takes satellite imagery and forest field measurements as input and produces estimates of above-ground biomass across forest landscapes. No specialised hardware is required. The key limitation is geographic bias, it was trained on Senegalese forest conditions and will need retraining with local field data before being applied elsewhere. The tool and datasets are openly licensed for replication and adaptation, but users are asked to credit the original work and link any derivative products back to the source, this helps the community track how the tool develops over time.</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
+      <c r="N67" t="inlineStr">
         <is>
           <t>The replication kit, including satellite data pipelines, field plot datasets, trained models and processing workflows, is openly available for use. Forest agencies can deploy the existing models immediately to generate biomass estimates for their own landscapes; carbon finance practitioners can use the outputs directly to support NDC reporting or funding applications; and researchers can fine-tune the models for different forest types or regions using local field data. Extending the work is straightforward, the modular architecture allows individual components to be upgraded independently.</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr">
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
         <is>
           <t>GIZ: Data Economy and FAIR Forward
 Ministère de l'Environnement et de la Transition Écologique (METE)- Senegal, 
@@ -8539,105 +8450,105 @@
 D4D Hub — Data for Development Hub</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr">
+      <c r="Q67" t="inlineStr">
         <is>
           <t>Elikplim Sabblah</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S68" t="inlineStr">
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
         <is>
           <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr">
+      <c r="T67" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr">
+      <c r="U67" t="inlineStr"/>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr">
         <is>
           <t>It is planned that the output from this initiative will be registered as a DPG. But that hasn't been done yet since it is still under-development</t>
         </is>
       </c>
-      <c r="X68" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t xml:space="preserve">This activity was led by the colleagues from the Data Economy project with support from colleagues from FAIR Forward (Ruth and Eli) </t>
         </is>
       </c>
-      <c r="Y68" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z68" t="inlineStr"/>
-      <c r="AA68" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>ui_63</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>ML4EO for Precision Agriculture</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t xml:space="preserve">From Maps to Meals: ML for Precision Ag - Enabling geo-scientists to use Machine Learning for Precision Agriculture of geospatial data 
 </t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>Enabling geo-scientists to use Machine Learning for Precision Agriculture of geospatial data</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Development and implementation of a training program to enable practitioners in the field of Earth Observation in South Africa to use machine learning. 
 Field data collected on small holder agricultural farm land (crops) with raw datasets + applied use cases of classification of land use cover using ML (based on individual projects presented)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr">
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
         <is>
           <t>SDG 2, SDG 13, SDG 11</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I68" t="inlineStr">
         <is>
           <t>Drone Imagery, Geospatial/Remote Sensing</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="J68" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K68" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L68" t="inlineStr">
         <is>
           <t>Types of Data:
 1. Satellite-Based Data: Sentinel-1 (SAR),  
@@ -8649,18 +8560,18 @@
 Field-level reflectance, chlorophyll-related vegetation indices (VIs), Spectral response to stress; Sentinel-2, NIR bands, Low-res images, spectral variability for phosphorus deficiency &amp; MSV, Spatial mapping of weeds vs. crops, Red-edge based chlorophyll estimates, Red-edge bands, REIP indices, Thermal + multispectral image fusion, Temporal NDVI, vegetation change monitoring, Crop separability via bands 7, 8, 8A, 11, Correlation of VIs to LAI</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="M68" t="inlineStr">
         <is>
           <t>Please see the other South Africa projects from Dr. Meena Lysko - this is the consolidated dataset source for the sub projects</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr">
+      <c r="N68" t="inlineStr">
         <is>
           <t>Please see the other South Africa projects from Dr. Meena Lysko - this is the consolidated dataset source for the sub projects</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr">
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -8668,116 +8579,116 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr">
+      <c r="Q68" t="inlineStr">
         <is>
           <t>Meena Lysko</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr">
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr">
+      <c r="T68" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="U68" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1JMDhPAwVfS80qSFerU7f7jRhuKG05OFi?usp=drive_link</t>
         </is>
       </c>
-      <c r="V69" t="inlineStr">
+      <c r="V68" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1R7iawHmEnTRJu_kmoR1iz26aii15ELIT?usp=drive_link</t>
         </is>
       </c>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr">
+      <c r="W68" t="inlineStr"/>
+      <c r="X68" t="inlineStr">
         <is>
           <t>Comment by Balthas: please let us check, if this and all subsequent entries on SA match the threashold of being a "usable" dataset for pratitioners, or if this was rather an academic dataset for training purposes. If the second is true, we should not list them here IMHO. Also see the challenge, that these datasets are only on googledrive and not really explained structured files, as far as I could check</t>
         </is>
       </c>
-      <c r="Y69" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z69" t="inlineStr"/>
-      <c r="AA69" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr"/>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>ui_64</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
         <is>
           <t>Data for Detecting and Assessing Tomato Stress</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>Detecting and Assessing Tomato Stress using ASD Measurements and Drone Data: The Case of Project Munei Holding Investments, Ha-Mphaila, Makhado Local Municipality</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t xml:space="preserve">Investigates methods for detecting and assessing stress in tomato plants using ASD measurements and drone data, focusing on Project Munei Holding Investment in Ha-Mphaila, Limpopo
 </t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr">
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="J69" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
+      <c r="K69" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>Field-level reflectance, chlorophyll-related vegetation indices (VIs). The data comes in various forms: Hyperspectral, UAV imagery, SPAD, Images, Tabular</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr">
+      <c r="M69" t="inlineStr">
         <is>
           <t>Random Forest; used for stress classification; Software/Application: Random Forest + UAV analytics</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
+      <c r="N69" t="inlineStr">
         <is>
           <t>Train RF using spectral indices; cost includes UAV flights, ASD rentals; open-source RF models or GEE usable</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr">
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -8785,111 +8696,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr">
+      <c r="Q69" t="inlineStr">
         <is>
           <t>Gladness Khoza and Chuma Majova</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr">
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr">
+      <c r="T69" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="U69" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1XAzVlTGTc1TuXb10h67WDmuU91k2c2BP/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V70" t="inlineStr">
+      <c r="V69" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1t3KiZiEQFprZMb8AYI01HrbSsSrfUwlb/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z70" t="inlineStr"/>
-      <c r="AA70" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="W69" t="inlineStr"/>
+      <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>ui_65</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
         <is>
           <t>The internet of Crops (IOC)</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Leaf Area Index Estimation of Tomato Crops in Sub-Humid Regions Based On Sentinel 2 Imagery and Random Forest Regression Ensemble</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Investigates the use of Sentinel-2 satellite imagery and a random forest (RF) machine learning algorithm to estimate the Leaf Area Index (LAI) of tomato crops in the Ha-Mphaila irrigation scheme, Limpopo Province, South Africa. The research aimed to determine key wavebands and vegetation indices for LAI estimation, compare the performance of RF models with stepwise multiple linear regression (SMLR) models, and map the spatial distribution of LAI.</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr">
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
         <is>
           <t>SDG 2</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Tabular</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="J70" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
+      <c r="K70" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr">
+      <c r="L70" t="inlineStr">
         <is>
           <t>Correlation of VIs to LAI, Sentinel-2 + LAI ground truth.</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="M70" t="inlineStr">
         <is>
           <t>Random Forest Regression; Software/Application: Sentinel-2 + RF</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
+      <c r="N70" t="inlineStr">
         <is>
           <t>Free Sentinel-2 + fieldwork required; ML code free (e.g., Python)</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr">
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -8897,111 +8808,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr">
+      <c r="Q70" t="inlineStr">
         <is>
           <t>Frederick Mashao and Dr. Olufemi Olayiwola</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr">
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr">
+      <c r="T70" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="U70" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1ZmDPVVb2SLxrWDE7LnCIl87_Wse4f8oK/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V71" t="inlineStr">
+      <c r="V70" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1rqnCZTZ2b4MSp9C0nkFhU3A1Xhk4CwIe/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z71" t="inlineStr"/>
-      <c r="AA71" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>ui_66</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
         <is>
           <t>Artificial Intelligence for Maize (AIM)</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>Characterizing Maize Stress Using UAV Remote Sensing: A Machine Learning Approach</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>Investigates the use of remote sensing and machine learning to characterize maize stress in the Limpopo Province, South Africa. The study concludes that integrating field spectra and remotely sensed reflectance provides valuable information for maize stress investigation, supporting the development of mitigation and prevention strategies to ensure food security.</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr">
+      <c r="L71" t="inlineStr">
         <is>
           <t>Spectral response to stress; Sentinel-2, NIR bands.</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="M71" t="inlineStr">
         <is>
           <t>Random Forest, SVM; Software/Application: Sentinel-2 + field spectral data</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t>Access Sentinel-2 (free); field spectrometer needed for calibration</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr">
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9009,111 +8920,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr">
+      <c r="Q71" t="inlineStr">
         <is>
           <t>Gerhardt Botha and Mikka Parag</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr">
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr">
+      <c r="T71" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="U71" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1XkSwcY0fmPmleRxfekkoOcBvF7kuAHFX/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V72" t="inlineStr">
+      <c r="V71" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1cMBiijRJUyz8MVAuudrDnK2kkxbnoT6J/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z72" t="inlineStr"/>
-      <c r="AA72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>ui_67</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
         <is>
           <t>Data for Detecting and Assessing Maize Stress</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>Monitoring Zea Mays (Maize) Disease Stress using Drone data and Machine Learning Techniques, and Advising on Possible Causes and Solutions</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t xml:space="preserve">Assesses the capabilities of Earth observation and machine learning algorithms, specifically Random Forest and Support Vector Machines, in detecting maize disease stress using drone data. The study was conducted on a small-scale farm in Limpopo, South Africa, focusing on healthy maize, maize with streak virus, and maize with phosphorus deficiency. </t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I72" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Drone Imagery</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="J72" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K72" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="L72" t="inlineStr">
         <is>
           <t>Low-res images, (hyper)spectral variability for phosphorus deficiency &amp; MSV.</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="M72" t="inlineStr">
         <is>
           <t>Random Forest, SVM; &lt;80% accuracy; Software/Application: Drone + ML (RF, SVM)</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t>Requires high-quality imagery, better spectral resolution; GEE and drone access recommended</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr">
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9121,111 +9032,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q73" t="inlineStr">
+      <c r="Q72" t="inlineStr">
         <is>
           <t>Khanyisa Mpisane and Kanya Xongo</t>
         </is>
       </c>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr">
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T73" t="inlineStr">
+      <c r="T72" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="U72" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1CV_nkCyPYt9ecxWyEcmEguYpLh9DFb2V/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V73" t="inlineStr">
+      <c r="V72" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/13tu-8UnI1FYk7DLkI_Z1qmprWW3EWlfp/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z73" t="inlineStr"/>
-      <c r="AA73" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
         <is>
           <t>ui_68</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
         <is>
           <t>Weeties</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Precision weed mapping and management in tomato fields using drone data in support of small-holder farming</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Drone high-resolution images were used with a semi-automated random forest (RF) classifier algorithm in Google Earth Engine to classify bare soil, weeds, and tomatoes. The findings can serve as a reference for agricultural researchers and advise farmers on crop management, potentially reducing costs and herbicide use.</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr">
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11, SDG 12</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Drone Imagery</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>Spatial mapping of weeds vs. crops using RGB/Multispectral data in addition to Drone imagery and Tabular obseravations.</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="M73" t="inlineStr">
         <is>
           <t>Random Forest; high training accuracy (89%); Software/Application: GEE + Random Forest</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t>Drone + GEE for processing; reduce herbicide usage</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr">
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9233,111 +9144,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q74" t="inlineStr">
+      <c r="Q73" t="inlineStr">
         <is>
           <t>Martin Chari and Makgabo Mashala</t>
         </is>
       </c>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr">
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr">
+      <c r="T73" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="U73" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1hyiQSbdMyB0O5BYR8fl31BfyvRzRIlP8/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V74" t="inlineStr">
+      <c r="V73" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1uFKAZ9CCniykTKRSsh2-nxKW2f3Wkpbb/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W74" t="inlineStr"/>
-      <c r="X74" t="inlineStr"/>
-      <c r="Y74" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z74" t="inlineStr"/>
-      <c r="AA74" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>ui_69</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
         <is>
           <t>Chlorophyll-Busters</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Estimation of chlorophyll contents of crops (maize and tomato) using Sentinel-2 and drone data by applying Random Forest machine learning algorithm: A case study of the Ha-Mphaila farming area of South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Explores using the Random Forest Regression (RFR) machine learning algorithm with Sentinel-2 and drone imagery to estimate relative chlorophyll values in tomato and maize crops within South Africa's Ha-Mphaila farming area. The research concludes that both Sentinel-2 imagery (10m and 20m spatial resolution) and high-resolution drone images are valuable for rapidly assessing crop chlorophyll content across significant areas, offering useful insights for precision agriculture.</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr">
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11, SDG 13</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Drone Imagery</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t>Red-edge based chlorophyll estimates &amp; Sentinel-2 data</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="M74" t="inlineStr">
         <is>
           <t>Random Forest Regression; Software/Application: Sentinel-2 + drone + RF</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
+      <c r="N74" t="inlineStr">
         <is>
           <t>Sentinel free; drone + SPAD sensor may be costly unless shared</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr">
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9345,111 +9256,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr">
+      <c r="Q74" t="inlineStr">
         <is>
           <t>Cindy Viviers and Dr. Abraham Thomas</t>
         </is>
       </c>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr">
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr">
+      <c r="T74" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="U74" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1KVUM-JLYg6CY-B3WmVj4-puKacJvg8_x/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V75" t="inlineStr">
+      <c r="V74" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1dfgcycIgFy7SKUHJcZ2qFERbQTbehxVh/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
-      <c r="Y75" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z75" t="inlineStr"/>
-      <c r="AA75" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>ui_70</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
         <is>
           <t>The Agro-Innovators</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>Evaluating the Performance of Machine Learning Algorithms for Estimating Chlorophyll Content of Tomatoes with Unmanned Aerial Vehicle (UAV)-Based Data.</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t xml:space="preserve">Evaluates the performance of machine learning algorithms for estimating chlorophyll content in tomatoes using Sentinel-2 satellite data. </t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11, SDG 13</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I75" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Drone Imagery</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="J75" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="K75" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr">
+      <c r="L75" t="inlineStr">
         <is>
           <t>Red-edge bands, REIP indices, Sentinel-2, SPAD chlorophyll</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="M75" t="inlineStr">
         <is>
           <t>Bagging, Boosting, ANN, SVR; Software/Application: Chlorophyll estimation ML</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr">
+      <c r="N75" t="inlineStr">
         <is>
           <t>Train model on SPAD + satellite indices; uses open-source ML tools</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr">
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9457,111 +9368,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q76" t="inlineStr">
+      <c r="Q75" t="inlineStr">
         <is>
           <t>Sisipho Ngebe and Afika Singano</t>
         </is>
       </c>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr">
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr">
+      <c r="T75" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="U75" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1kugMpKasnb5_7XJkRj3jnAQw8retlV4W/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V76" t="inlineStr">
+      <c r="V75" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1QYB5PBhQVaDQ1J-YP0ZfOAsLXznla_Kr/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z76" t="inlineStr"/>
-      <c r="AA76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>ui_71</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
         <is>
           <t>Agro-thermography</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Integration of ground-based vegetation parameters, thermal infrared and UAV multispectral data for mapping of crop canopy temperature</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Explores the integration of ground-based vegetation parameters, thermal infrared data from handheld cameras, and UAV multispectral data to map crop canopy temperature at high resolution. The research, conducted at the Ha-Mphaila irrigation scheme in Limpopo, South Africa, focused on tomato crops.</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr">
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
         <is>
           <t>SDG 2, SDG 11, SDG 13</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I76" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Tabular</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="J76" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="K76" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="L76" t="inlineStr">
         <is>
           <t>Thermal IR and multispectral image fusion and field data + Drone Data</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="M76" t="inlineStr">
         <is>
           <t>Regression model; canopy temperature estimation; Software/Application: Thermal camera + UAV + regression models</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t>Needs UAV &amp; thermal cam; costly setup unless shared or borrowed</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr">
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9569,111 +9480,111 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr">
+      <c r="Q76" t="inlineStr">
         <is>
           <t>Dr. Mohamed Ahmed and Phumlani Zwane</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr">
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T77" t="inlineStr">
+      <c r="T76" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="U76" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1MOSiW0BIzqwK2YMEp1dCcIzItgLm8wR8/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V77" t="inlineStr">
+      <c r="V76" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1GMpDiMlY-wYXTB6T5woikRpFbgQ21hhp/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z77" t="inlineStr"/>
-      <c r="AA77" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>ui_72</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
         <is>
           <t>Discovering Agriculture Insurance</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>Remote Sensing and Machine Learning Applications in Agriculture Index Insurance (AII)</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Investigates how remote sensing and machine learning can be used to improve Agricultural Index Insurance (AII) for smallholder farmers in South Africa, who often lack access to affordable insurance.  Key recommendations include supporting further research and development in these areas and implementing educational campaigns to build farmer trust and awareness of index insurance benefits.</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr">
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
         <is>
           <t>SDG 2, SDG 13</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Tabular</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="J77" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
+      <c r="K77" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="L77" t="inlineStr">
         <is>
           <t>Temporal NDVI and chlorophyll indices, vegetation change monitoring, Sentinel-2 based</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="M77" t="inlineStr">
         <is>
           <t>ML for index-insurance mapping; Software/Application: Dynamic World + ML</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr">
+      <c r="N77" t="inlineStr">
         <is>
           <t>Integrate indices into insurance design; Sentinel-2 free; ML libraries (e.g., Scikit-learn)</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr">
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9681,112 +9592,112 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr">
+      <c r="Q77" t="inlineStr">
         <is>
           <t>Shereen Francis and Yashoda Maharaj</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr">
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T78" t="inlineStr">
+      <c r="T77" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="U77" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1LHAaaDSYSNbBAaeVdmBFlpecX_ntVEKf/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V78" t="inlineStr">
+      <c r="V77" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1rGoapVNyVsVwMxDfBrRfdVoyRCpjwnIy/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z78" t="inlineStr"/>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="W77" t="inlineStr"/>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>ui_73</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
         <is>
           <t>SAR Busters</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>Crop type mapping in Mphaila irrigation scheme in Vhembe District in Limpopo Province</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1P_bW8Is1Qa1HJIznVbq_vsQwH3ejKUa5?usp=drive_link</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr">
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
         <is>
           <t>SDG 2</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="I78" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Images, Tabular</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="J78" t="inlineStr">
         <is>
           <t>Dr Meena Lysko (mbc.mlysko@gmail.com)</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
+      <c r="K78" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="L78" t="inlineStr">
         <is>
           <t>Crop separability via bands 7, 8, 8A, 11. Sentinel-1 (SAR) and  Sentinel-2 (optical) based</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="M78" t="inlineStr">
         <is>
           <t>Decision Tree, Random Forest; Software/Application: Crop mapping using ML</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>Sentinel data free; GEE platform usable</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr"/>
-      <c r="P79" t="inlineStr">
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Move Beyond Consulting
 Implementing partners: MBC, WITS, CSIR, ARC
@@ -9794,97 +9705,97 @@
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q79" t="inlineStr">
+      <c r="Q78" t="inlineStr">
         <is>
           <t>Dleme Tswai and Dr. Theunis Morgenthal</t>
         </is>
       </c>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr">
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T79" t="inlineStr">
+      <c r="T78" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="U78" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1mjjI5knaWJqjOQURj7OKfKxMbMDEmvEH/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="V79" t="inlineStr">
+      <c r="V78" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1c54f9Lh5IV8T_XLrlf_8ItAitrBEjTVZ/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="W79" t="inlineStr"/>
-      <c r="X79" t="inlineStr"/>
-      <c r="Y79" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z79" t="inlineStr"/>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>ui_74</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>NLP grant Localising Common Voice for South African Languages</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>Voices of Mzansi - Making all official languages of South Africa AI-ready: translating the Common-Voice interface &amp; enabling Open-source text-to-speech dataset collection</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr">
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
         <is>
           <t xml:space="preserve">The "Voices of Mzansi" project aimed to get South Africa's languages launched on the Mozilla Common Voice platform. To achieve this aim the Common Voice website had to be translated from English into the other official languages and at least 5 000 sentences had to be collected for each language. The collected sentences have to be available in the open domain under CC-0 licensing. Once a languages is launched, the sentences are used as prompts for speech data collection through the Common Voice platform. This unlocks open-source text-to-speech dataset collection and thereby ultimately facilitates access to information in mother tongue, including by illiterate persons and in rural settings. </t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>https://commonvoice.mozilla.org/de/languages</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr">
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
         <is>
           <t>SDG 2, SDG 10</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="J79" t="inlineStr">
         <is>
           <t>Prof. Febe de Wet</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
+      <c r="K79" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr">
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 ## How to Use This Resource
@@ -9895,141 +9806,237 @@
 Source: https://commonvoice.mozilla.org/en/languages (language statistics via Common Voice API)</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr">
+      <c r="O79" t="inlineStr">
         <is>
           <t>CC-O</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr">
+      <c r="P79" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Stellenbosch University
 Catalyzed by: South African Digital Language Resources (SADILAR), FAIR Forward - AI for All, GIZ, Mozilla Foundation, UNESCO decade of indigenous languages
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr">
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T80" t="inlineStr">
+      <c r="T79" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr"/>
-      <c r="V80" t="inlineStr">
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" t="inlineStr">
         <is>
           <t>Mozilla CVP</t>
         </is>
       </c>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr">
+      <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr">
         <is>
           <t>Original title: Making voice data available in all official languages of South Africa as a digital public good - Voices of Mzansi: Speaking Data, Speaking home</t>
         </is>
       </c>
-      <c r="Y80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z80" t="inlineStr"/>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
         <is>
           <t>ui_75</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>South Africa Crop Type Competition</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Spot the Crop</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Crop Type Identification from Satellite Imagery in Western Cape, South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>This dataset and AI model was produced as part of the Radiant Earth Spot the Crop Challenge (https://zindi.africa/hackathons/radiant-earth-spot-the-crop-hackathon). The objective of the competition was to create a machine learning model to classify fields by crop type from images collected during the growing season by the Sentinel-2 and Sentinel-1 satellites.</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>https://beta.source.coop/repositories/radiantearth/south-africa-crops-competition/description/</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G80" t="inlineStr">
         <is>
           <t>https://github.com/radiantearth/spot-the-crop-challenge</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H80" t="inlineStr">
         <is>
           <t>SDG 2, SDG 13</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="I80" t="inlineStr">
         <is>
           <t>Tabular</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="J80" t="inlineStr">
         <is>
           <t>Radiant Earth (ml@radiant.earth)</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="K80" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr">
+      <c r="L80" t="inlineStr">
         <is>
           <t>The dataset contains a time-series of satellite imagery and labels for crop type that have been collected through aerial and ground survey. Labels are derived from the survey conducted by the Western Cape Department of Agriculture. Satellite data including multispectral Sentinel-2 are then matched with corresponding labels.</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="M80" t="inlineStr">
         <is>
           <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
-      <c r="N81" t="inlineStr">
+      <c r="N80" t="inlineStr">
         <is>
           <t>The agricultural sector makes a substantial contribution to GDP and livelihoods across the developing world. However, regular and reliable agricultural data remains difficult and expensive to collect on the ground. As a result, policy-makers usually don’t have access to updated data for implementing policies or supporting farmers. Earth observation satellites provide a wealth of multispectral image data that can be used for developing agricultural monitoring tools. These tools support farmers and policy-makers across Africa and the developing world. With this dataset and AI model you can use time-series of Sentinel-2 multi-spectral data to classify crops in the Western Cape of South Africa.</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="O80" t="inlineStr">
         <is>
           <t>CC-BY 4.0</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P80" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Radiant Earth, Western Cape Department of Agriculture
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Philipp Olbrich</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model &gt; Pilot</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Computer Vision</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>https://zindi.africa/competitions/radiant-earth-spot-the-crop-challenge</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr"/>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ui_76</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Kiswahili Text and Voice Recognition Platform (KTVRP) for Agricultural Advisory and Financial Services for Smallholder Farmers</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>A majority of smallholder farmers in Tanzania are only able to communicate through the Kiswahili spoken language and its dialects. A text and voice-based platform made available in the language of the underserved (i.e., Kiswahili) would be key to wide access, adoption, and usage of digital agricultural advisory and financial services in Tanzania. The objective is to develop a text and voice recognition platform that will offer smallholder farmers in the Tanzanian Maize Value Chain personalized digital financial and non-financial automated services based on location, agro-ecological zones, and crop cycle. Based on gender-disaggregated data from the pilot phase, it is anticipated that the majority of participants will be women. This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: info@duniacom.com
+</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>SDG 10, SDG 2, SDG 5</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Text, Voice</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Duniacom Group LLC (info@duniacom.com)</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Duniacom Group LLC
+Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
+Financed by: Gates Foundation &amp; BMZ</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Philipp Olbrich</t>
+          <t>Daniel Brumund, Balthas Seibold</t>
         </is>
       </c>
       <c r="R81" t="inlineStr"/>
@@ -10040,13 +10047,17 @@
       </c>
       <c r="T81" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
-        </is>
-      </c>
-      <c r="U81" t="inlineStr"/>
+          <t>NLP</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>https://assets.mofoprod.net/network/images/KTVRP.2e16d0ba.fill-760x760-c100.format-jpeg_9VkBrtV.jpg</t>
+        </is>
+      </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>https://zindi.africa/competitions/radiant-earth-spot-the-crop-challenge</t>
+          <t>https://www.mozillafoundation.org/en/what-we-fund/programs/common-voice-kiswahili-awards/awards/  https://foundation.mozilla.org/blog/supporting-maize-farmers-in-tanzania/</t>
         </is>
       </c>
       <c r="W81" t="inlineStr"/>
@@ -10066,28 +10077,25 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ui_76</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Kiswahili Text and Voice Recognition Platform (KTVRP) for Agricultural Advisory and Financial Services for Smallholder Farmers</t>
-        </is>
-      </c>
+          <t>ui_77</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
+          <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>A majority of smallholder farmers in Tanzania are only able to communicate through the Kiswahili spoken language and its dialects. A text and voice-based platform made available in the language of the underserved (i.e., Kiswahili) would be key to wide access, adoption, and usage of digital agricultural advisory and financial services in Tanzania. The objective is to develop a text and voice recognition platform that will offer smallholder farmers in the Tanzanian Maize Value Chain personalized digital financial and non-financial automated services based on location, agro-ecological zones, and crop cycle. Based on gender-disaggregated data from the pilot phase, it is anticipated that the majority of participants will be women. This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
+          <t>Kiazi Bora, “Quality Potatoes’’ in Swahili, uses a voice enabled application that informs vulnerable women living in rural areas and marginalized communities of Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes (OFSP), farming skills for better yields, and detailed market availability for raw or processed OFSP food products, all through a voice data set app. 
+This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: info@duniacom.com
+          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: https://seeafricatz.org/contact-us/
 </t>
         </is>
       </c>
@@ -10104,7 +10112,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Duniacom Group LLC (info@duniacom.com)</t>
+          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10118,14 +10126,14 @@
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Duniacom Group LLC
+          <t>Powered by / Provided by: SEE Africa
 Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation &amp; BMZ</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Daniel Brumund, Balthas Seibold</t>
+          <t>Balthas Seibold</t>
         </is>
       </c>
       <c r="R82" t="inlineStr"/>
@@ -10141,12 +10149,12 @@
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>https://assets.mofoprod.net/network/images/KTVRP.2e16d0ba.fill-760x760-c100.format-jpeg_9VkBrtV.jpg</t>
+          <t>https://assets.mofoprod.net/network/images/Kiazi-Bora.2e16d0ba.fill-760x760-c100.format-jpeg_WQA0YAL.jpg</t>
         </is>
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>https://www.mozillafoundation.org/en/what-we-fund/programs/common-voice-kiswahili-awards/awards/  https://foundation.mozilla.org/blog/supporting-maize-farmers-in-tanzania/</t>
+          <t>https://foundation.mozilla.org/blog/growing-skills-confidence-and-quality-potatoes-in-tanzania/</t>
         </is>
       </c>
       <c r="W82" t="inlineStr"/>
@@ -10166,159 +10174,62 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ui_77</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
+          <t>ui_78</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Croppie Coffee Yield Prediction</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Croppie- helping smallholder coffee producers to plan sales, estimate yields, get loans, and trace coffee - AI powered coffee yield prediction</t>
+        </is>
+      </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
+          <t>Croppie- helping smallholder coffee producers to plan sales, estimate yields, get loans, and trace coffee - AI powered coffee yield prediction</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
-        <is>
-          <t>Kiazi Bora, “Quality Potatoes’’ in Swahili, uses a voice enabled application that informs vulnerable women living in rural areas and marginalized communities of Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes (OFSP), farming skills for better yields, and detailed market availability for raw or processed OFSP food products, all through a voice data set app. 
-This was part of a Mozilla innovation challenge supporting people and projects across East Africa who leverage Common Voice’s open-source voice data set to unlock social and economic opportunities. These grants help to advance the use of open-source voice data for products that support community participation and engagement.</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Publishing status unclear. Please contact the responsible authors for an update and access to the data: https://seeafricatz.org/contact-us/
-</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>SDG 10, SDG 2, SDG 5</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>Text, Voice</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>Tanzania</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t>Powered by / Provided by: SEE Africa
-Catalyzed by: Mozilla Foundation &amp; FAIR Forward - AI for All, GIZ
-Financed by: Gates Foundation &amp; BMZ</t>
-        </is>
-      </c>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t>Balthas Seibold</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>Dataset &gt; Model &gt; Pilot</t>
-        </is>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>NLP</t>
-        </is>
-      </c>
-      <c r="U83" t="inlineStr">
-        <is>
-          <t>https://assets.mofoprod.net/network/images/Kiazi-Bora.2e16d0ba.fill-760x760-c100.format-jpeg_WQA0YAL.jpg</t>
-        </is>
-      </c>
-      <c r="V83" t="inlineStr">
-        <is>
-          <t>https://foundation.mozilla.org/blog/growing-skills-confidence-and-quality-potatoes-in-tanzania/</t>
-        </is>
-      </c>
-      <c r="W83" t="inlineStr"/>
-      <c r="X83" t="inlineStr"/>
-      <c r="Y83" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z83" t="inlineStr"/>
-      <c r="AA83" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>ui_78</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Croppie Coffee Yield Prediction</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Croppie- helping smallholder coffee producers to plan sales, estimate yields, get loans, and trace coffee - AI powered coffee yield prediction</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Croppie- helping smallholder coffee producers to plan sales, estimate yields, get loans, and trace coffee - AI powered coffee yield prediction</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
         <is>
           <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
 The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/rgautroncgiar/croppie_coffee_ug</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>https://huggingface.co/rgautroncgiar/croppie_coffee_ug</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>SDG 2, SDG 13</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
+      <c r="I83" t="inlineStr">
         <is>
           <t>Tabular</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="J83" t="inlineStr">
         <is>
           <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
+      <c r="K83" t="inlineStr">
         <is>
           <t>Uganda</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr">
+      <c r="L83" t="inlineStr">
         <is>
           <t xml:space="preserve">The Data is fully open-sourced and can be accessed on Hugging Face
  • License: CC BY SA 4.0
@@ -10330,7 +10241,7 @@
 For this dataset / use case, a responsible AI Assessment was undertaken to help AI developers and project managers to identify, assess and mitigate potential harms and biases in AI. For methodology, see https://www.bmz-digital.global/en/news/ethical-crash-test-for-ai-how-to-navigate-the-road-to-responsible-innovation/   </t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="M83" t="inlineStr">
         <is>
           <t>Processed Data:
  The dataset is made of a mix of Arabica and Robusta coffee tree parts (with and without a background isolation element) with individual bounding boxes around all coffee cherries. These RGB pictures were on-farm collected with smartphones with the collaboration of smallholder farmers. 
@@ -10342,121 +10253,121 @@
  The dataset/model can be used for automated cherry count or coffee ripeness assessment.</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr">
+      <c r="N83" t="inlineStr">
         <is>
           <t>This resource can be of use to anyone interested to automate the task of manual cherry counts (the traditional approach to harvest estimation) and to estimate coffee harvest on a plot level. This is done  by processing pictures through AI-supported image recognition software along with a manual branch count (= tree level estimation) and a tree-per-ha estimation (or recall data) (scaling to plot level). Thus, this system is useful for anyone interested in building a central system for managing yield data at the farmer level. It also provides the option to share this data with external users; with for example cooperatives having the possibility to feed information from the application in an integrated database of their member’s performance and farm characteristics, provided they obtained prior consent to do so. This would then scale the Croppie system to have an aggregated data view of multiple users in a region, e.g. as a cooperative level dashboard.
 This use case also included the development of a business model and funding model for open source AI as a stepping stone towards financially viable operations. It was facilitated by Villgro Africa's and FAIR Forward's  six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr">
+      <c r="O83" t="inlineStr">
         <is>
           <t>CC-BY-SA 4.0</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="P83" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Producers Direct, M-Omulimisa, Alliance of Bioversity International and CIAT, Tecnicafé
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q84" t="inlineStr">
+      <c r="Q83" t="inlineStr">
         <is>
           <t>Balthas Seibold</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr">
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr">
         <is>
           <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case &gt;  Use-Case with Business Model</t>
         </is>
       </c>
-      <c r="T84" t="inlineStr">
+      <c r="T83" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr"/>
-      <c r="V84" t="inlineStr">
+      <c r="U83" t="inlineStr"/>
+      <c r="V83" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.bmz-digital.global/en/ai-coffee-intelligent-awake/ </t>
         </is>
       </c>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr">
+      <c r="W83" t="inlineStr"/>
+      <c r="X83" t="inlineStr">
         <is>
           <t>Alternative title: Precision Farming Simplified: Croppie’s AI-Powered Agronomic Advisor</t>
         </is>
       </c>
-      <c r="Y84" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z84" t="inlineStr"/>
-      <c r="AA84" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr"/>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>ui_79</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>Scaling ML-based site identification for MiniGrids Uganda</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Bridging the Energy Gap: Machine Learning Applications in Uganda's Rural Electrification</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>Finding good spots for decentralized green energy grids in Uganda - AI based site identification for MiniGrids</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>The Site Identification tool is an AI-driven tool to enhance renewable energy planning. This tool utilizes machine learning and satellite imagery to identify optimal sites for renewable energy deployment, particularly in remote regions. A successful pilot in Lamwo District demonstrated its potential to improve energy access by recommending suitable electrification strategies for villages. This initiative aligns with Uganda’s National Electrification Strategy, which seeks to connect 10 million households to the most optimal energy source by 2030.</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>https://github.com/SunbirdAI/lamwo-electrification-project/tree/main</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>https://lamwo.sunbird.ai/</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>SDG 13</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Tabular</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="J84" t="inlineStr">
         <is>
           <t>Sunbird.ai (emwebaze@sunbird.ai)</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="K84" t="inlineStr">
         <is>
           <t>Uganda</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="L84" t="inlineStr">
         <is>
           <t xml:space="preserve">-• Data Type: Geospatial and tabular 
 • Key Variables: Solar Irradiance,Biomass Resources,Wind Speed and Consistency,Biomass Resources,Hydropower Potential,
@@ -10466,124 +10377,124 @@
 </t>
         </is>
       </c>
-      <c r="M85" t="inlineStr">
+      <c r="M84" t="inlineStr">
         <is>
           <t xml:space="preserve">This web application is a decision support tool. It is built as a prototype for a large-scale decision support tool for determining electrification strategies for different geographical areas. Currently implemented in Lamwo district electrification. </t>
         </is>
       </c>
-      <c r="N85" t="inlineStr">
+      <c r="N84" t="inlineStr">
         <is>
           <t>This web application is a prototype decision support tool designed to guide electrification strategies across various geographic areas. It offers an initial village-level assessment through a color-coded map, with the legend explaining each category. Users can explore detailed analyses at the village level—the smallest unit for assessing electrification needs. The tool evaluates both demand and supply factors and suggests the most suitable energy solutions, including biomass, wind, solar home systems, mini-grids, or grid extension. It is intended to support government officials, energy sector stakeholders, and development partners in making informed renewable energy decisions.</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
-      <c r="P85" t="inlineStr">
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Sunbird.ai
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr">
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr">
         <is>
           <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
         </is>
       </c>
-      <c r="T85" t="inlineStr">
+      <c r="T84" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
-      <c r="Y85" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z85" t="inlineStr"/>
-      <c r="AA85" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="U84" t="inlineStr"/>
+      <c r="V84" t="inlineStr"/>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr"/>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>ui_80</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Development of Unbiased AI Models for Solar Irradiance Uganda</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Estimating Solar Irradiance for Improved Solar Energy Planning in Uganda and in Sub-Saharan Africa through AI</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>Estimating Solar Irradiance for Improved Solar Energy Planning in Sub-Saharan Africa through AI</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>The project successfully developed a machine learning model to predict daily Global Horizontal Irradiance (GHI) in Sub-Saharan Africa, with a specific focus on Uganda. The core objective was to correct the systematic bias found in readily available satellite-derived solar irradiation data (like NASA CERES and CAMS). Key activities included identifying five installation sites in Uganda for ground-truth data collection (Gulu, Mbale, Jinja, Kasese, Hoima), procuring pyranometers (though installation was hindered by lack of Ministry of Energy approval), and extensively collecting data from four satellite sources and partner ground stations (Cross Boundary Energy, Makerere University, Ministry of Energy) combined with local topological information (ie. altitude). A Random Forest model was trained on this integrated dataset, proving superior to other models (LSTMs, SVMs) by effectively adjusting the satellite predictions to align with the ground truth across all climatic regions, thus providing a significantly more reliable and bankable estimate of solar resources essential for rural electrification planning.</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>https://github.com/Marconi-Lab/Solar_irradiation</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G85" t="inlineStr">
         <is>
           <t>https://irradiation-portal-55883164704.europe-west1.run.app/ ; https://github.com/Marconi-Lab/Irradiation_Portal</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>SDG 13</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>Geospatial/Remote Sensing, Tabular, Meterological</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="J85" t="inlineStr">
         <is>
           <t xml:space="preserve">Jan Mikelson &lt;jan.mikelson@gmail.com&gt;           Andrew Katumba katraxuk@gmail.com
 </t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
+      <c r="K85" t="inlineStr">
         <is>
           <t>Uganda</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
+      <c r="L85" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Bias-corrected daily Global Horizontal Irradiance (GHI) data for Uganda, derived by correcting CAMS and NASA POWER satellite datasets against ground-truth measurements from 56 validation sites across Uganda. Training data includes measurements from 7 African countries. The correction addresses a 20% satellite overestimation of solar potential. Data is accessible via the Solar Irradiance Portal web interface and a RESTful API for application integration.
 Source: https://github.com/Marconi-Lab/Solar_irradiation, https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr">
+      <c r="M85" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 Random Forest model (SuSSE -- Sub-Saharan Solar Estimation) that corrects satellite-derived solar irradiance estimates for Uganda. Input: CAMS and NASA POWER satellite GHI data. Output: bias-corrected daily GHI values. Validated against 56 ground-truth sites across Uganda, achieving R-squared of 0.86 and correcting a 20% overestimation in standard satellite products. Application: deployed as an interactive web portal with maps, charts, and a RESTful API for integration. Code: Python package at github.com/Marconi-Lab/Solar_irradiation (87.9% Jupyter Notebook, 12.1% Python).
 Source: https://github.com/Marconi-Lab/Solar_irradiation, https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr">
+      <c r="N85" t="inlineStr">
         <is>
           <t>[Auto-enriched from linked project resources]
 ## How to Use This Resource
@@ -10596,14 +10507,113 @@
 - https://irradiation-portal-55883164704.europe-west1.run.app/</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr"/>
-      <c r="P86" t="inlineStr">
+      <c r="O85" t="inlineStr"/>
+      <c r="P85" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Marconi Lab
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Prediction</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" t="inlineStr"/>
+      <c r="W85" t="inlineStr"/>
+      <c r="X85" t="inlineStr"/>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr"/>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ui_81</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>NLP Use Case Strengthening relevance of Auditing reports in Uganda</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>AI as a helping hand to understand audit reports - A conversational chatbot answering questions related to audit reports of the Auditor General Office of Uganda</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>AI as a helping hand to understand audit reports - A conversational chatbot answering questions related to audit reports of the Auditor General Office of Uganda</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>In Uganda, the Civil Society and Budget Advocacy Group (CSBAG) in partnership with GIZ, has recognized the need for further enhancement in how audit reports are processed and understood. An AI-powered conversational assistant was designed to help anyone understand audit reports. It will answer questions by using Audit reports published by Auditor General Office, Uganda. The prototype tool leverages AI to offer capabilities such as summarizing complex texts, extracting thematic insights, and enabling interactive, user-friendly analysis through a chatbot interface. By making the audit reports more accessible, this aims to increase readership and utilization among stakeholders, which can lead to better accountability and improve service delivery.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/spaces/GIZ/audit_assistant/tree/main</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>SDG 13</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>CSBAG (https://www.csbag.org/)</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Data comes from audit documents in Uganda and samples can be sourced from HuggingFace. Full implementation will come later.</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The prototyped is linked - full implementation will come later </t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Civil Society and Budget Advocacy Group (CSBAG), GIZ
+Catalyzed by: FAIR Forward - AI for All, GIZ
+Financed by: BMZ</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr">
@@ -10613,7 +10623,7 @@
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>Prediction</t>
+          <t>NLP</t>
         </is>
       </c>
       <c r="U86" t="inlineStr"/>
@@ -10635,272 +10645,173 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ui_81</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>NLP Use Case Strengthening relevance of Auditing reports in Uganda</t>
-        </is>
-      </c>
+          <t>ui_82</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AI as a helping hand to understand audit reports - A conversational chatbot answering questions related to audit reports of the Auditor General Office of Uganda</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>AI as a helping hand to understand audit reports - A conversational chatbot answering questions related to audit reports of the Auditor General Office of Uganda</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>In Uganda, the Civil Society and Budget Advocacy Group (CSBAG) in partnership with GIZ, has recognized the need for further enhancement in how audit reports are processed and understood. An AI-powered conversational assistant was designed to help anyone understand audit reports. It will answer questions by using Audit reports published by Auditor General Office, Uganda. The prototype tool leverages AI to offer capabilities such as summarizing complex texts, extracting thematic insights, and enabling interactive, user-friendly analysis through a chatbot interface. By making the audit reports more accessible, this aims to increase readership and utilization among stakeholders, which can lead to better accountability and improve service delivery.</t>
+          <t>This project provides Uganda’s first openly accessible AI-ready satellite imagery dataset designed to predict land-use and land-cover change. It was created to address persistent deforestation and the lack of reliable, context-specific data needed to detect, forecast, and manage ecosystem degradation. Through an open-source replication kit including annotated Sentinel-2 and Hansen datasets, protocols, and inventory data, this products enables local innovators, forest agencies, and policymakers to build AI tools for monitoring forests, planning restoration, and supporting NDC and SDG15 actions. Its goal is to improve early detection of land-cover change, strengthen climate-smart decision-making, and empower local institutions with high-quality geospatial data.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://huggingface.co/spaces/GIZ/audit_assistant/tree/main</t>
+          <t xml:space="preserve"> https://1drv.ms/f/c/BFFEF9896BFF8791/Es68F3WluONJjORAR_WvTloBdtisO9TGsGyWR8Se5xNYDA?e=q0Afso</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>SDG 13</t>
+          <t>SDG 13, SDG 15</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Geospatial/Remote Sensing, Images</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
-        <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>Uganda</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>Data comes from audit documents in Uganda and samples can be sourced from HuggingFace. Full implementation will come later.</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The prototyped is linked - full implementation will come later </t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>Powered by / Provided by: Civil Society and Budget Advocacy Group (CSBAG), GIZ
-Catalyzed by: FAIR Forward - AI for All, GIZ
-Financed by: BMZ</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case</t>
-        </is>
-      </c>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>NLP</t>
-        </is>
-      </c>
-      <c r="U87" t="inlineStr"/>
-      <c r="V87" t="inlineStr"/>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
-      <c r="Y87" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z87" t="inlineStr"/>
-      <c r="AA87" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>ui_82</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>This project provides Uganda’s first openly accessible AI-ready satellite imagery dataset designed to predict land-use and land-cover change. It was created to address persistent deforestation and the lack of reliable, context-specific data needed to detect, forecast, and manage ecosystem degradation. Through an open-source replication kit including annotated Sentinel-2 and Hansen datasets, protocols, and inventory data, this products enables local innovators, forest agencies, and policymakers to build AI tools for monitoring forests, planning restoration, and supporting NDC and SDG15 actions. Its goal is to improve early detection of land-cover change, strengthen climate-smart decision-making, and empower local institutions with high-quality geospatial data.</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> https://1drv.ms/f/c/BFFEF9896BFF8791/Es68F3WluONJjORAR_WvTloBdtisO9TGsGyWR8Se5xNYDA?e=q0Afso</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>SDG 13, SDG 15</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>Geospatial/Remote Sensing, Images</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
         <is>
           <t xml:space="preserve">Makerere University https://mak.ac.ug,
 Makerere AI Lab: https://air.ug/ 
 National Forestry Authority (NFA): https://nfa.go.ug/  </t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
+      <c r="K87" t="inlineStr">
         <is>
           <t>Uganda</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr">
+      <c r="L87" t="inlineStr">
         <is>
           <t>1. Landus Landcover Datasets (2015 -2023), 
 2. ArcGIS Pro Project, ArcGIS DEEPLearning Model for Tree Species.
 The dataset provides georeferenced, annotated Sentinel-2 and Hansen imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. Users can train AI models for landuse and landcover classification, detect deforestation, validate predictions, and support restoration planning. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring.</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr">
+      <c r="M87" t="inlineStr">
         <is>
           <t>The AI application analyzes historical satellite imagery gereated landuse and landcover maps (2015-2024) and predicts future landuse and land-cover change, offering simple inputs including Sentinel-2 and Hansen datasets of tree cover and outputs such as classified maps and simulations for 2025 and 2030. It identifies deforestation, farmland expansion, and urban growth patterns, supporting evidence-based land management. While highly accurate (ANN: 85.2% OA), limitations include data inconsistencies, sampling bias, and reliance on remote-sensing quality. Ethical use requires adherence to responsible-AI assessment, transparency, and proper citation. The model runs on standard GIS/AI software (QGIS, google colab, Jupyter-notebook) with no special hardware. All derived datasets and protocols are open for reuse under an open license; users must credit the original project to strengthen community knowledge and track downstream impact.</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t>One can immediately use this AI system to classify landuse and landcover types, detect deforestation, and generate LULC predictions for 2025–2030. Users can replicate the full workflow from preprocessing imagery, training ANN models, and simulating future change scenarios to support forest monitoring, restoration planning, district land-use decision-making, or environmental reporting. Researchers can extend the work by integrating socio-economic variables, testing hybrid models, adding additional years of imagery, or adapting the model to new districts. Replication requires awareness of limitations such as sampling imbalance, image quality differences, and potential classification bias; an ethical-AI review is recommended for all downstream use. Costs remain low because the tools (QGIS, GEE, SEPAL) and datasets are free; only compute for model training (standard PCs) and technical time are required. All datasets, protocols, and documentation form an open public-good resource, with opportunities for collaboration through Makerere AI Lab and NFA.</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr">
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Makerere University in cooperation with the Uganda National Forestry Authority (NFA)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr">
+      <c r="Q87" t="inlineStr">
         <is>
           <t>Alondra Arellano, Jonas Nothnagel</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr">
+      <c r="R87" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="S88" t="inlineStr">
+      <c r="S87" t="inlineStr">
         <is>
           <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
-      <c r="T88" t="inlineStr">
+      <c r="T87" t="inlineStr">
         <is>
           <t>Computer Vision</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr">
+      <c r="U87" t="inlineStr"/>
+      <c r="V87" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “With funding from Lacuna Fund, satellite image and forest inventory datasets will help to develop machine learning models for prediction of land cover types or changes for informed decision-making in natural resource management. Under joint research from Makerere College of Agriculture and Environment Studies and Makerere AI Health Lab, and in partnership with the National Forestry Authority, Uganda, our land use/cover change datasets will improve our understanding of the relationship between land cover/land use change and climate change. It will also be useful in informing practice and policy on how best to manage various potential scenarios. 
 — Dr. Sarah Akello, College of Agriculture and Environmental Sciences, Makerere University 
 </t>
         </is>
       </c>
-      <c r="W88" t="inlineStr"/>
-      <c r="X88" t="inlineStr">
+      <c r="W87" t="inlineStr"/>
+      <c r="X87" t="inlineStr">
         <is>
           <t>original title: DATASETS FOR PREDICTION OF LAND USE/COVER CHANGES IN UGANDA</t>
         </is>
       </c>
-      <c r="Y88" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z88" t="inlineStr"/>
-      <c r="AA88" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr"/>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>ui_83</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>Datasets marking Personal Identifiable Information (PII) and Gender Bias</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Preserving privacy and avoiding gender bias of AI systems in Luganda, Lumasaba, Hausa, and Kanuri - The Lacuna personally identifiable information Text Dataset</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr">
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
         <is>
           <t>The Lacuna PII Multilingual Text Dataset  contains annotated sentences with personally identifiable information (PII) in Luganda, Lumasaba, Hausa, and Kanuri. These four languages span Central and Eastern Uganda, Nigeria, Ghana, and Northern Cameroon. The dataset can help to anonymize and pseudonymize personally identifiable information in AI tasks. This can help organizations comply with legal requirements while still being able to analyze and use and share their data effectively. It can also be used to improve machine translation systems for low-resource languages,  improve the performance of NLP applications in these languages, and support the extraction of specific information from text, such as automated form filling and information retrieval systems. It comprises 4000 Luganda sentences, 5000 Lumasaba sentences, 3000 Kanuri sentences, and 3000 Hausa sentences. The team aimed to curate a dataset that is gender inclusive. It was created by Makerere Artificial Intelligence Lab in collaboration with Marconi Lab and Clear Global.</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>https://dataverse.harvard.edu/citation?persistentId=doi:10.7910/DVN/CGHWZE</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr">
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
         <is>
           <t>SDG 13, SDG 5, SDG 10</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="J88" t="inlineStr">
         <is>
           <t>Andrew Katumba - Makerere University (katumba@mak.ac.ug)</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
+      <c r="K88" t="inlineStr">
         <is>
           <t>Uganda,Kenya,Nigeria</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr">
+      <c r="L88" t="inlineStr">
         <is>
           <t>Text data:
 • Luganda: 4000 PII sentences with representation in entities of
@@ -10913,68 +10824,101 @@
 For more, see data card here: https://dataverse.harvard.edu/file.xhtml?fileId=10577233&amp;version=2.0</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr">
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr">
         <is>
           <t xml:space="preserve">This dataset of personally identifiable information (PII) can help any organization or initiative, that would like to comply with legal requirements while still being able to analyze and use and share data effectively in one of the languages in Luganda, Lumasaba, Hausa, and Kanuri. It can also be used to improve machine translation systems for these low-resource languages, improve the performance of NLP applications in these languages, and support the extraction of specific information from text, such as automated form filling and information retrieval systems. </t>
         </is>
       </c>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr">
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Makerere AI Lab, Marconi Lab, Clear Global
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
-      <c r="Q89" t="inlineStr">
+      <c r="Q88" t="inlineStr">
         <is>
           <t>Balthas Seibold</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr">
+      <c r="R88" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="S89" t="inlineStr">
+      <c r="S88" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr">
+      <c r="T88" t="inlineStr">
         <is>
           <t>NLP</t>
         </is>
       </c>
+      <c r="U88" t="inlineStr"/>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>https://dataverse.harvard.edu/file.xhtml?fileId=10577234&amp;version=2.0</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>First editing DONE on 25.8., Balthas</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ui_88</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr"/>
-      <c r="V89" t="inlineStr">
-        <is>
-          <t>https://dataverse.harvard.edu/file.xhtml?fileId=10577234&amp;version=2.0</t>
-        </is>
-      </c>
+      <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>
-      <c r="X89" t="inlineStr">
-        <is>
-          <t>First editing DONE on 25.8., Balthas</t>
-        </is>
-      </c>
-      <c r="Y89" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="X89" t="inlineStr"/>
+      <c r="Y89" t="inlineStr"/>
       <c r="Z89" t="inlineStr"/>
-      <c r="AA89" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="AA89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ui_88</t>
+          <t>ui_89</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -11007,7 +10951,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ui_89</t>
+          <t>ui_91</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -11040,7 +10984,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ui_91</t>
+          <t>ui_92</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -11073,7 +11017,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ui_92</t>
+          <t>ui_93</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -11106,7 +11050,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ui_93</t>
+          <t>ui_94</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
@@ -11139,7 +11083,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ui_94</t>
+          <t>ui_95</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -11172,7 +11116,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ui_95</t>
+          <t>ui_96</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
@@ -11205,7 +11149,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ui_96</t>
+          <t>ui_97</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -11238,7 +11182,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ui_97</t>
+          <t>ui_98</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -11271,7 +11215,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ui_98</t>
+          <t>ui_99</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -11304,7 +11248,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ui_99</t>
+          <t>ui_100</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -11337,7 +11281,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ui_100</t>
+          <t>ui_101</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -11370,7 +11314,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ui_101</t>
+          <t>ui_102</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -11403,7 +11347,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ui_102</t>
+          <t>ui_103</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
@@ -11436,7 +11380,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ui_103</t>
+          <t>ui_104</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -11469,7 +11413,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ui_104</t>
+          <t>ui_105</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -11502,7 +11446,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ui_105</t>
+          <t>ui_106</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -11535,7 +11479,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ui_106</t>
+          <t>ui_107</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -11568,7 +11512,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ui_107</t>
+          <t>ui_108</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -11601,7 +11545,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ui_108</t>
+          <t>ui_109</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -11634,7 +11578,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ui_109</t>
+          <t>ui_110</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -11667,7 +11611,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ui_110</t>
+          <t>ui_111</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -11700,7 +11644,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ui_111</t>
+          <t>ui_112</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -11733,7 +11677,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ui_112</t>
+          <t>ui_113</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -11766,7 +11710,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ui_113</t>
+          <t>ui_114</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -11799,7 +11743,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ui_114</t>
+          <t>ui_115</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -11832,7 +11776,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ui_115</t>
+          <t>ui_116</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -11865,7 +11809,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ui_116</t>
+          <t>ui_117</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -11898,7 +11842,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ui_117</t>
+          <t>ui_118</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -11931,7 +11875,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ui_118</t>
+          <t>ui_119</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -11964,7 +11908,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ui_119</t>
+          <t>ui_120</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -11997,7 +11941,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ui_120</t>
+          <t>ui_121</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -12030,7 +11974,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ui_121</t>
+          <t>ui_122</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -12063,7 +12007,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ui_122</t>
+          <t>ui_123</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -12096,7 +12040,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ui_123</t>
+          <t>ui_124</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
@@ -12129,7 +12073,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ui_124</t>
+          <t>ui_125</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
@@ -12162,7 +12106,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ui_125</t>
+          <t>ui_126</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -12195,7 +12139,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ui_126</t>
+          <t>ui_127</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
@@ -12228,7 +12172,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ui_127</t>
+          <t>ui_128</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -12261,7 +12205,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ui_128</t>
+          <t>ui_129</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -12294,7 +12238,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ui_129</t>
+          <t>ui_130</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
@@ -12327,7 +12271,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ui_130</t>
+          <t>ui_131</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -12360,7 +12304,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ui_131</t>
+          <t>ui_132</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -12393,7 +12337,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ui_132</t>
+          <t>ui_133</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
@@ -12426,7 +12370,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ui_133</t>
+          <t>ui_134</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
@@ -12459,7 +12403,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ui_134</t>
+          <t>ui_135</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -12492,7 +12436,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ui_135</t>
+          <t>ui_136</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
@@ -12525,7 +12469,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ui_136</t>
+          <t>ui_137</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -12558,7 +12502,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ui_137</t>
+          <t>ui_138</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
@@ -12591,7 +12535,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ui_138</t>
+          <t>ui_139</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
@@ -12624,7 +12568,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ui_139</t>
+          <t>ui_140</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
@@ -12657,7 +12601,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ui_140</t>
+          <t>ui_141</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
@@ -12690,7 +12634,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ui_141</t>
+          <t>ui_142</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
@@ -12723,7 +12667,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ui_142</t>
+          <t>ui_143</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
@@ -12756,7 +12700,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ui_143</t>
+          <t>ui_144</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
@@ -12789,7 +12733,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ui_144</t>
+          <t>ui_145</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -12822,7 +12766,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ui_145</t>
+          <t>ui_146</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
@@ -12855,7 +12799,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ui_146</t>
+          <t>ui_147</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
@@ -12888,7 +12832,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ui_147</t>
+          <t>ui_148</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
@@ -12921,7 +12865,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ui_148</t>
+          <t>ui_149</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
@@ -12954,7 +12898,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ui_149</t>
+          <t>ui_150</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -12987,7 +12931,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ui_150</t>
+          <t>ui_151</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
@@ -13020,7 +12964,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ui_151</t>
+          <t>ui_152</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -13050,39 +12994,6 @@
       <c r="Z152" t="inlineStr"/>
       <c r="AA152" t="inlineStr"/>
     </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>ui_152</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
-      <c r="M153" t="inlineStr"/>
-      <c r="N153" t="inlineStr"/>
-      <c r="O153" t="inlineStr"/>
-      <c r="P153" t="inlineStr"/>
-      <c r="Q153" t="inlineStr"/>
-      <c r="R153" t="inlineStr"/>
-      <c r="S153" t="inlineStr"/>
-      <c r="T153" t="inlineStr"/>
-      <c r="U153" t="inlineStr"/>
-      <c r="V153" t="inlineStr"/>
-      <c r="W153" t="inlineStr"/>
-      <c r="X153" t="inlineStr"/>
-      <c r="Y153" t="inlineStr"/>
-      <c r="Z153" t="inlineStr"/>
-      <c r="AA153" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sheet update 2026-05-18 07:46:36 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,137 +417,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
@@ -574,7 +562,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>African Trees for Climate Resilience: A Comprehensive Database</t>
+          <t>African Trees for Climate Resilience - A Comprehensive Database</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -838,7 +826,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -1312,7 +1300,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Data354
+          <t>Powered by / Provided by: Data354, Zindi
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -1334,7 +1322,11 @@
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://zindi.africa/competitions/africa-biomass-challenge </t>
+        </is>
+      </c>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
@@ -2023,7 +2015,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2124,9 +2116,10 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>[Auto-enriched from linked project resources]
+          <t xml:space="preserve">[Auto-enriched from linked project resources]
 Afrocentric crop disease dataset by Responsible AI Lab. Contains annotated leaf images showing healthy specimens and disease-affected leaves at various crop development phases. Data Type: Image. Size: ~20 GB. License: CC BY 4.0. Version 16 (last modified March 2025). Created with a focus on African agricultural diversity.
-Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana</t>
+Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana
+Also see here for the Zindi challenge: https://zindi.africa/competitions/ghana-crop-disease-detection-challenge </t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2176,7 +2169,11 @@
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://zindi.africa/competitions/ghana-crop-disease-detection-challenge </t>
+        </is>
+      </c>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
@@ -2801,8 +2798,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3743,7 +3740,7 @@
       <c r="L28" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3754,7 +3751,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3829,7 +3826,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3865,8 +3862,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4222,22 +4218,22 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4583,7 +4579,7 @@
       <c r="N35" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5157,8 +5153,8 @@
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -6103,10 +6099,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6603,7 +6599,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>
 </t>
         </is>
       </c>
@@ -6911,7 +6907,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7531,7 +7527,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
@@ -7828,8 +7824,8 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -8422,7 +8418,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
 </t>
         </is>
       </c>
@@ -9646,7 +9642,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9912,7 +9908,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10189,8 +10185,8 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10973,11 +10969,7 @@
           <t>Early stage, functional demo available.</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr">
         <is>
           <t>Media post-production</t>

</xml_diff>

<commit_message>
Sheet update 2026-05-18 07:46:36 UTC (#68)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,137 +417,137 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
@@ -574,7 +562,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>African Trees for Climate Resilience: A Comprehensive Database</t>
+          <t>African Trees for Climate Resilience - A Comprehensive Database</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -838,7 +826,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -1312,7 +1300,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Data354
+          <t>Powered by / Provided by: Data354, Zindi
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -1334,7 +1322,11 @@
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://zindi.africa/competitions/africa-biomass-challenge </t>
+        </is>
+      </c>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
@@ -2023,7 +2015,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2124,9 +2116,10 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>[Auto-enriched from linked project resources]
+          <t xml:space="preserve">[Auto-enriched from linked project resources]
 Afrocentric crop disease dataset by Responsible AI Lab. Contains annotated leaf images showing healthy specimens and disease-affected leaves at various crop development phases. Data Type: Image. Size: ~20 GB. License: CC BY 4.0. Version 16 (last modified March 2025). Created with a focus on African agricultural diversity.
-Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana</t>
+Source: https://www.kaggle.com/datasets/responsibleailab/crop-disease-ghana
+Also see here for the Zindi challenge: https://zindi.africa/competitions/ghana-crop-disease-detection-challenge </t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2176,7 +2169,11 @@
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://zindi.africa/competitions/ghana-crop-disease-detection-challenge </t>
+        </is>
+      </c>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
@@ -2801,8 +2798,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3743,7 +3740,7 @@
       <c r="L28" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -3754,7 +3751,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -3829,7 +3826,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -3865,8 +3862,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4222,22 +4218,22 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4583,7 +4579,7 @@
       <c r="N35" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5157,8 +5153,8 @@
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -6103,10 +6099,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6603,7 +6599,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>
 </t>
         </is>
       </c>
@@ -6911,7 +6907,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7531,7 +7527,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
@@ -7828,8 +7824,8 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -8422,7 +8418,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
 </t>
         </is>
       </c>
@@ -9646,7 +9642,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9912,7 +9908,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10189,8 +10185,8 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10973,11 +10969,7 @@
           <t>Early stage, functional demo available.</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr">
         <is>
           <t>Media post-production</t>

</xml_diff>

<commit_message>
Sheet update 2026-05-18 09:58:18 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -562,7 +562,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>African Trees for Climate Resilience - A Comprehensive Database</t>
+          <t xml:space="preserve">African Trees for Climate Resilience: A Comprehensive Database </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Golo Rademacher; Balthas Seibold; Daniel Brumund</t>
+          <t>Golo Rademacher; Daniel Brumund</t>
         </is>
       </c>
       <c r="R41" t="inlineStr"/>

</xml_diff>

<commit_message>
Sheet update 2026-05-18 09:58:18 UTC (#69)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -562,7 +562,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>African Trees for Climate Resilience - A Comprehensive Database</t>
+          <t xml:space="preserve">African Trees for Climate Resilience: A Comprehensive Database </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Golo Rademacher; Balthas Seibold; Daniel Brumund</t>
+          <t>Golo Rademacher; Daniel Brumund</t>
         </is>
       </c>
       <c r="R41" t="inlineStr"/>

</xml_diff>

<commit_message>
Sheet update 2026-06-10 12:02:48 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,142 +417,142 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -752,7 +740,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -855,7 +843,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Reiner Lemoine Institut gGmbH (RLI)</t>
+          <t>Reiner Lemoine Institut, Catherina Cader (catherina.cader@rl-institut.de)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -944,7 +932,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>World Resources Institute</t>
+          <t>World Resources Institute, Kendie Kenmoe (Kendie.Kenmoe@wri.org)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1539,7 +1527,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Core23Lab</t>
+          <t>Core23Lab (engage@core23lab.org)</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2092,7 +2080,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2905,8 +2893,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3069,19 +3057,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset creatd: Dhuluo</t>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dholuo Speech</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dhuluo</t>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dholuo Speech</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mozilla Foundation seeks to select and support a community (group of language speakers who would like to collectively create or enhance a text and audio dataset for their  language), to experiment with a governance structure for this dataset that suits their particular needs. 
-This project will enable language communities to leverage governance tools (such as licenses) that center their needs and context, and have them be more accessible and widely used. Over the period of the project, the goal is to have a particular language community, or small group of them, piloting a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted
-- language dataset created: Dhuluo ?</t>
+          <t xml:space="preserve">The “DhoNam: Dholuo Speech dataset” is a speech corpus designed to supercharge Automatic Speech Recognition (ASR) and other speech technologies for Dholuo, one of Kenya’s major indigenous languages. This dataset contains native-speaker audio recordings collected through a platform where users read aloud a displayed sentence. The dataset includes the audio recordings and the corresponding prompt/sentence that was read.
+The dataset was part of a programme of Mozilla Foundation, that piloted alternative approaches to governance of AI training data, that balance opening up innovation, with centering community choice. Mozilla and its partners, Maseno Centre for Applied Artificial Intelligence, Maseno University, worked with the Dholuo language community to pilot a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted. Mozilla envisions a world in which Common Voice advances open technology through a range of governance approaches, guided by the communities themselves. 
+The Dholuo speech dataset was created by researchers from Maseno Centre for Applied Artificial Intelligence, Maseno University and members from the Dholuo language community from Kenya. The pilot was conducted by Dr. Lilian Wanzare, Language Community Associate for Common Voice, from Nairobi, Kenya.
+</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3100,24 +3089,63 @@
           <t>Voice</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dr. Lilian Wanzare &lt;ldwanzare@maseno.ac.ke&gt;, Dept. of Computer Science, School of Computing and Informatics, Maseno University
+</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Global / Regional</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>Kenya, Global / Regional</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>This dataset contains native-speaker audio recordings collected through a platform where users read aloud a displayed sentence. 
+Collection Timeframe:
+Collected in 2025, between October and November 2025, as part of the Dholuo Voice Data Collection Project.
+Recording Conditions: Indoor environments with no background noise,  Recorded via smartphones through a web interface
+Domains Represented:
+General
+Agriculture
+Technology and robotics
+Healthcare
+News and current affairs
+These domains reflect real spoken Dholuo usage.
+Total duration: 184,838.28 sec (3080.64 min, 51.34 hr)
+Number of Speakers: 59
+Number of Reviewers: 7
+Total audio files: 26,091
+Average clip length: 7.08 sec
+Minimum clip length: 1.72 sec
+Maximum clip length: 62.64 sec</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DhoNam: Dholuo Speech dataset is a speech corpus designed to supercharge Automatic Speech Recognition (ASR) and other speech technologies for Dholuo, one of Kenya’s major indigenous languages. </t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nwulite Obodo Open Data Licence 1.0 (NOODL-1.0)
+https://licensingafricandatasets.com/nwulite-obodo-license </t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Powered by / Provided by:
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+          <t>Powered by / Provided by: Maseno Centre for Applied Artificial Intelligence, Maseno University, Members from the Dholuo language community 
+Catalyzed by: Mozilla Foundation, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balthas Seibold  </t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
@@ -3130,7 +3158,11 @@
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mozillafoundation.org/en/common-voice/in-country-programmes/ ; https://www.maseno.ac.ke/common-voice-piloting-alternative-language-data-licenses-workshop-kenya-maseno-university ; https://igf2025.sched.com/event/24FLE/ws-#323-new-data-governance-models-for-african-nlp-ecosystems ; https://www.youtube.com/watch?v=TYnn-mOyS1A </t>
+        </is>
+      </c>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr">
@@ -4017,7 +4049,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -4028,7 +4060,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -4108,7 +4140,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -4144,8 +4176,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4516,22 +4547,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4626,7 +4657,11 @@
           <t>Geospatial/Remote Sensing</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Bonn Consulting (jan.redlich@bonnconsulting.group)</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>India</t>
@@ -4892,7 +4927,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5486,8 +5521,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -6308,7 +6343,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Prof. Ciira Maina, Centre for Data Science and Artificial Intelligence, Dedan Kimathi University of Technology</t>
+          <t>Prof. Ciira Maina (ciira.maina@dkut.ac.ke), Centre for Data Science and Artificial Intelligence, Dedan Kimathi University of Technology</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -6342,10 +6377,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6568,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations</t>
+          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6688,7 +6723,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>info@mu.ac.ke</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -6781,7 +6820,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://ujuzicraft.com/</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -7072,7 +7115,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7639,7 +7682,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digital Umuganda (Samuel Rutunda, Audace Niyonkuru) </t>
+          <t>Digital Umuganda, Samuel Rutunda (samuel@digitalumuganda.com), Audace Niyonkuru</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -7717,7 +7760,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -8029,8 +8072,8 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -9537,7 +9580,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9676,7 +9719,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Prof. Febe de Wet</t>
+          <t>Prof. Febe de Wet, Mozilla Data Collective (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -9813,7 +9856,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10105,8 +10148,8 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10878,7 +10921,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
 </t>
         </is>
       </c>
@@ -10978,7 +11021,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Sheet update 2026-06-10 12:02:48 UTC (#75)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,142 +417,142 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -752,7 +740,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -855,7 +843,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Reiner Lemoine Institut gGmbH (RLI)</t>
+          <t>Reiner Lemoine Institut, Catherina Cader (catherina.cader@rl-institut.de)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -944,7 +932,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>World Resources Institute</t>
+          <t>World Resources Institute, Kendie Kenmoe (Kendie.Kenmoe@wri.org)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1539,7 +1527,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Core23Lab</t>
+          <t>Core23Lab (engage@core23lab.org)</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2092,7 +2080,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2905,8 +2893,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3069,19 +3057,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset creatd: Dhuluo</t>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dholuo Speech</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dhuluo</t>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dholuo Speech</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mozilla Foundation seeks to select and support a community (group of language speakers who would like to collectively create or enhance a text and audio dataset for their  language), to experiment with a governance structure for this dataset that suits their particular needs. 
-This project will enable language communities to leverage governance tools (such as licenses) that center their needs and context, and have them be more accessible and widely used. Over the period of the project, the goal is to have a particular language community, or small group of them, piloting a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted
-- language dataset created: Dhuluo ?</t>
+          <t xml:space="preserve">The “DhoNam: Dholuo Speech dataset” is a speech corpus designed to supercharge Automatic Speech Recognition (ASR) and other speech technologies for Dholuo, one of Kenya’s major indigenous languages. This dataset contains native-speaker audio recordings collected through a platform where users read aloud a displayed sentence. The dataset includes the audio recordings and the corresponding prompt/sentence that was read.
+The dataset was part of a programme of Mozilla Foundation, that piloted alternative approaches to governance of AI training data, that balance opening up innovation, with centering community choice. Mozilla and its partners, Maseno Centre for Applied Artificial Intelligence, Maseno University, worked with the Dholuo language community to pilot a novel, community-centered license on the Common Voice platform, as a proof of concept that can then be replicated and adapted. Mozilla envisions a world in which Common Voice advances open technology through a range of governance approaches, guided by the communities themselves. 
+The Dholuo speech dataset was created by researchers from Maseno Centre for Applied Artificial Intelligence, Maseno University and members from the Dholuo language community from Kenya. The pilot was conducted by Dr. Lilian Wanzare, Language Community Associate for Common Voice, from Nairobi, Kenya.
+</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3100,24 +3089,63 @@
           <t>Voice</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dr. Lilian Wanzare &lt;ldwanzare@maseno.ac.ke&gt;, Dept. of Computer Science, School of Computing and Informatics, Maseno University
+</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Global / Regional</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>Kenya, Global / Regional</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>This dataset contains native-speaker audio recordings collected through a platform where users read aloud a displayed sentence. 
+Collection Timeframe:
+Collected in 2025, between October and November 2025, as part of the Dholuo Voice Data Collection Project.
+Recording Conditions: Indoor environments with no background noise,  Recorded via smartphones through a web interface
+Domains Represented:
+General
+Agriculture
+Technology and robotics
+Healthcare
+News and current affairs
+These domains reflect real spoken Dholuo usage.
+Total duration: 184,838.28 sec (3080.64 min, 51.34 hr)
+Number of Speakers: 59
+Number of Reviewers: 7
+Total audio files: 26,091
+Average clip length: 7.08 sec
+Minimum clip length: 1.72 sec
+Maximum clip length: 62.64 sec</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DhoNam: Dholuo Speech dataset is a speech corpus designed to supercharge Automatic Speech Recognition (ASR) and other speech technologies for Dholuo, one of Kenya’s major indigenous languages. </t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nwulite Obodo Open Data Licence 1.0 (NOODL-1.0)
+https://licensingafricandatasets.com/nwulite-obodo-license </t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Powered by / Provided by:
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+          <t>Powered by / Provided by: Maseno Centre for Applied Artificial Intelligence, Maseno University, Members from the Dholuo language community 
+Catalyzed by: Mozilla Foundation, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balthas Seibold  </t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
@@ -3130,7 +3158,11 @@
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mozillafoundation.org/en/common-voice/in-country-programmes/ ; https://www.maseno.ac.ke/common-voice-piloting-alternative-language-data-licenses-workshop-kenya-maseno-university ; https://igf2025.sched.com/event/24FLE/ws-#323-new-data-governance-models-for-african-nlp-ecosystems ; https://www.youtube.com/watch?v=TYnn-mOyS1A </t>
+        </is>
+      </c>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr">
@@ -4017,7 +4049,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -4028,7 +4060,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -4108,7 +4140,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
 The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
         </is>
       </c>
@@ -4144,8 +4176,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-+          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
 </t>
         </is>
       </c>
@@ -4516,22 +4547,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4626,7 +4657,11 @@
           <t>Geospatial/Remote Sensing</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Bonn Consulting (jan.redlich@bonnconsulting.group)</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>India</t>
@@ -4892,7 +4927,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5486,8 +5521,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -6308,7 +6343,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Prof. Ciira Maina, Centre for Data Science and Artificial Intelligence, Dedan Kimathi University of Technology</t>
+          <t>Prof. Ciira Maina (ciira.maina@dkut.ac.ke), Centre for Data Science and Artificial Intelligence, Dedan Kimathi University of Technology</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -6342,10 +6377,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -6568,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations</t>
+          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6688,7 +6723,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>info@mu.ac.ke</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -6781,7 +6820,11 @@
           <t>Text, Voice</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://ujuzicraft.com/</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -7072,7 +7115,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7639,7 +7682,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digital Umuganda (Samuel Rutunda, Audace Niyonkuru) </t>
+          <t>Digital Umuganda, Samuel Rutunda (samuel@digitalumuganda.com), Audace Niyonkuru</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -7717,7 +7760,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -8029,8 +8072,8 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
 </t>
         </is>
       </c>
@@ -9537,7 +9580,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9676,7 +9719,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Prof. Febe de Wet</t>
+          <t>Prof. Febe de Wet, Mozilla Data Collective (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -9813,7 +9856,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10105,8 +10148,8 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10878,7 +10921,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
 </t>
         </is>
       </c>
@@ -10978,7 +11021,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t>
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Sheet update 2026-06-15 13:22:22 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>KaraAgro (https://karaagro.com/)</t>
+          <t>KaraAgro (darlington@gudra-studio.com)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/)</t>
+          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UNDP India (https://www.undp.org/india)</t>
+          <t>UNDP India (registry.in@undp.org)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gram Vaani (https://gramvaani.org/)</t>
+          <t>Gram Vaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Karya (https://karya.in/)</t>
+          <t>Karya (operations@karya.in)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (https://digitalgreen.org/ourwork/india/)</t>
+          <t>Digital Green (info@digitalgreentrust.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>WRMS (https://wrmsglobal.com/)</t>
+          <t>WRMS (connect@wrmsglobal.com)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GramVaani (https://gramvaani.org/)</t>
+          <t>GramVaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (https://prosa.ai/)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (https://jkpp.org/), HCSA (https://highcarbonstock.org/public-consultation/), EcoVision Lab (https://www.spacehub.uzh.ch/en/research-areas/earth-observation/EcoVision-Lab.html)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Prosa AI (https://prosa.ai/)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>LDRI (https://www.developlocal.org/#)</t>
+          <t>LDRI (thinking@developlocal.org)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
+          <t>Badili Innovations (info@badili.co.ke)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://ujuzicraft.com/</t>
+          <t>UjuziCraft (info@ujuzicraft.com)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green, Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Mozilla Common Voice (https://commonvoice.mozilla.org)</t>
+          <t>Mozilla Common Voice (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NaijaSenti (https://github.com/hausanlp/NaijaSenti?tab=readme-ov-file#contact-us)</t>
+          <t>NaijaSenti / HausaNLP (hausanlp@gmail.com)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+          <t>Hesotech (info@hesotech.de)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com)</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com), FAIR Forward Rwanda</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda - Samuel (samuel@digitalumuganda.com), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+          <t>SEE Africa (info@seeafricatz.org)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
+          <t>Croppie - Romain Gautron (r.gautron@cgiar.org), Producers Direct (info@producersdirect.org), M-Omulimisa, CIAT</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
+          <t>CSBAG (csbag@csbag.org)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10656,9 +10656,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makerere University https://mak.ac.ug,
-Makerere AI Lab: https://air.ug/ 
-National Forestry Authority (NFA): https://nfa.go.ug/  </t>
+          <t>Makerere AI Lab - Dr. Joyce Nabende (joyce.nabende@mak.ac.ug), National Forestry Authority (NFA): https://nfa.go.ug/</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11283,7 +11281,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://c4ir.rw/</t>
+          <t>C4IR Rwanda (info@c4ir.rw)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-15 13:22:22 UTC (#87)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>KaraAgro (https://karaagro.com/)</t>
+          <t>KaraAgro (darlington@gudra-studio.com)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/)</t>
+          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UNDP India (https://www.undp.org/india)</t>
+          <t>UNDP India (registry.in@undp.org)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gram Vaani (https://gramvaani.org/)</t>
+          <t>Gram Vaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Karya (https://karya.in/)</t>
+          <t>Karya (operations@karya.in)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (https://digitalgreen.org/ourwork/india/)</t>
+          <t>Digital Green (info@digitalgreentrust.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>WRMS (https://wrmsglobal.com/)</t>
+          <t>WRMS (connect@wrmsglobal.com)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GramVaani (https://gramvaani.org/)</t>
+          <t>GramVaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (https://prosa.ai/)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (https://jkpp.org/), HCSA (https://highcarbonstock.org/public-consultation/), EcoVision Lab (https://www.spacehub.uzh.ch/en/research-areas/earth-observation/EcoVision-Lab.html)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Prosa AI (https://prosa.ai/)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>LDRI (https://www.developlocal.org/#)</t>
+          <t>LDRI (thinking@developlocal.org)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
+          <t>Badili Innovations (info@badili.co.ke)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://ujuzicraft.com/</t>
+          <t>UjuziCraft (info@ujuzicraft.com)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green, Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Mozilla Common Voice (https://commonvoice.mozilla.org)</t>
+          <t>Mozilla Common Voice (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NaijaSenti (https://github.com/hausanlp/NaijaSenti?tab=readme-ov-file#contact-us)</t>
+          <t>NaijaSenti / HausaNLP (hausanlp@gmail.com)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+          <t>Hesotech (info@hesotech.de)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com)</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com), FAIR Forward Rwanda</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda - Samuel (samuel@digitalumuganda.com), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+          <t>SEE Africa (info@seeafricatz.org)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
+          <t>Croppie - Romain Gautron (r.gautron@cgiar.org), Producers Direct (info@producersdirect.org), M-Omulimisa, CIAT</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
+          <t>CSBAG (csbag@csbag.org)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10656,9 +10656,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makerere University https://mak.ac.ug,
-Makerere AI Lab: https://air.ug/ 
-National Forestry Authority (NFA): https://nfa.go.ug/  </t>
+          <t>Makerere AI Lab - Dr. Joyce Nabende (joyce.nabende@mak.ac.ug), National Forestry Authority (NFA): https://nfa.go.ug/</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11283,7 +11281,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://c4ir.rw/</t>
+          <t>C4IR Rwanda (info@c4ir.rw)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-15 13:22:29 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>KaraAgro (https://karaagro.com/)</t>
+          <t>KaraAgro (darlington@gudra-studio.com)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/)</t>
+          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UNDP India (https://www.undp.org/india)</t>
+          <t>UNDP India (registry.in@undp.org)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gram Vaani (https://gramvaani.org/)</t>
+          <t>Gram Vaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Karya (https://karya.in/)</t>
+          <t>Karya (operations@karya.in)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (https://digitalgreen.org/ourwork/india/)</t>
+          <t>Digital Green (info@digitalgreentrust.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>WRMS (https://wrmsglobal.com/)</t>
+          <t>WRMS (connect@wrmsglobal.com)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GramVaani (https://gramvaani.org/)</t>
+          <t>GramVaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (https://prosa.ai/)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (https://jkpp.org/), HCSA (https://highcarbonstock.org/public-consultation/), EcoVision Lab (https://www.spacehub.uzh.ch/en/research-areas/earth-observation/EcoVision-Lab.html)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Prosa AI (https://prosa.ai/)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>LDRI (https://www.developlocal.org/#)</t>
+          <t>LDRI (thinking@developlocal.org)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
+          <t>Badili Innovations (info@badili.co.ke)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://ujuzicraft.com/</t>
+          <t>UjuziCraft (info@ujuzicraft.com)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green, Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Mozilla Common Voice (https://commonvoice.mozilla.org)</t>
+          <t>Mozilla Common Voice (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NaijaSenti (https://github.com/hausanlp/NaijaSenti?tab=readme-ov-file#contact-us)</t>
+          <t>NaijaSenti / HausaNLP (hausanlp@gmail.com)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+          <t>Hesotech (info@hesotech.de)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com)</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com), FAIR Forward Rwanda</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda - Samuel (samuel@digitalumuganda.com), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+          <t>SEE Africa (info@seeafricatz.org)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
+          <t>Croppie - Romain Gautron (r.gautron@cgiar.org), Producers Direct (info@producersdirect.org), M-Omulimisa, CIAT</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
+          <t>CSBAG (csbag@csbag.org)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10656,9 +10656,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makerere University https://mak.ac.ug,
-Makerere AI Lab: https://air.ug/ 
-National Forestry Authority (NFA): https://nfa.go.ug/  </t>
+          <t>Makerere AI Lab - Dr. Joyce Nabende (joyce.nabende@mak.ac.ug), National Forestry Authority (NFA): https://nfa.go.ug/</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11283,7 +11281,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://c4ir.rw/</t>
+          <t>C4IR Rwanda (info@c4ir.rw)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-15 13:22:31 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>KaraAgro (https://karaagro.com/)</t>
+          <t>KaraAgro (darlington@gudra-studio.com)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/)</t>
+          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UNDP India (https://www.undp.org/india)</t>
+          <t>UNDP India (registry.in@undp.org)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gram Vaani (https://gramvaani.org/)</t>
+          <t>Gram Vaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Karya (https://karya.in/)</t>
+          <t>Karya (operations@karya.in)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (https://digitalgreen.org/ourwork/india/)</t>
+          <t>Digital Green (info@digitalgreentrust.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>WRMS (https://wrmsglobal.com/)</t>
+          <t>WRMS (connect@wrmsglobal.com)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GramVaani (https://gramvaani.org/)</t>
+          <t>GramVaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (https://prosa.ai/)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (https://jkpp.org/), HCSA (https://highcarbonstock.org/public-consultation/), EcoVision Lab (https://www.spacehub.uzh.ch/en/research-areas/earth-observation/EcoVision-Lab.html)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Prosa AI (https://prosa.ai/)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>LDRI (https://www.developlocal.org/#)</t>
+          <t>LDRI (thinking@developlocal.org)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
+          <t>Badili Innovations (info@badili.co.ke)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://ujuzicraft.com/</t>
+          <t>UjuziCraft (info@ujuzicraft.com)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green, Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Mozilla Common Voice (https://commonvoice.mozilla.org)</t>
+          <t>Mozilla Common Voice (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NaijaSenti (https://github.com/hausanlp/NaijaSenti?tab=readme-ov-file#contact-us)</t>
+          <t>NaijaSenti / HausaNLP (hausanlp@gmail.com)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+          <t>Hesotech (info@hesotech.de)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com)</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com), FAIR Forward Rwanda</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda - Samuel (samuel@digitalumuganda.com), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+          <t>SEE Africa (info@seeafricatz.org)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
+          <t>Croppie - Romain Gautron (r.gautron@cgiar.org), Producers Direct (info@producersdirect.org), M-Omulimisa, CIAT</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
+          <t>CSBAG (csbag@csbag.org)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10656,9 +10656,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makerere University https://mak.ac.ug,
-Makerere AI Lab: https://air.ug/ 
-National Forestry Authority (NFA): https://nfa.go.ug/  </t>
+          <t>Makerere AI Lab - Dr. Joyce Nabende (joyce.nabende@mak.ac.ug), National Forestry Authority (NFA): https://nfa.go.ug/</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11283,7 +11281,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://c4ir.rw/</t>
+          <t>C4IR Rwanda (info@c4ir.rw)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-15 13:22:35 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Data354 (https://data354.com/en/)</t>
+          <t>Data354 (gabriel.fonlladosa@data354.co)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>KaraAgro (https://karaagro.com/)</t>
+          <t>KaraAgro (darlington@gudra-studio.com)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/)</t>
+          <t>Responsible AI Lab (RAIL) at Kwame Nkrumah University of Science and Technology (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RAIL - KNUST (https://rail.knust.edu.gh/)</t>
+          <t>RAIL - KNUST (rail@knust.edu.gh)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>UNDP India (https://www.undp.org/india)</t>
+          <t>UNDP India (registry.in@undp.org)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gram Vaani (https://gramvaani.org/)</t>
+          <t>Gram Vaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Karya (https://karya.in/)</t>
+          <t>Karya (operations@karya.in)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (https://digitalgreen.org/ourwork/india/)</t>
+          <t>Digital Green (info@digitalgreentrust.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>WRMS (https://wrmsglobal.com/)</t>
+          <t>WRMS (connect@wrmsglobal.com)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GramVaani (https://gramvaani.org/)</t>
+          <t>GramVaani (contact@gramvaani.org)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -4902,7 +4902,7 @@
       <c r="J36" t="inlineStr">
         <is>
           <t>Vertify.earth - Michael Anthony (michael@vertify.earth), 
-Alsisar Impact - Saurabh Singhavi (saurabh@alsisarimpact.com)</t>
+Alsisar Impact (anuj@alsisarimpact.com )</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (https://prosa.ai/)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (https://jkpp.org/), HCSA (https://highcarbonstock.org/public-consultation/), EcoVision Lab (https://www.spacehub.uzh.ch/en/research-areas/earth-observation/EcoVision-Lab.html)</t>
+          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Prosa AI (https://prosa.ai/)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>LDRI (https://www.developlocal.org/#)</t>
+          <t>LDRI (thinking@developlocal.org)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Badili Innovations (https://badili.co.ke/#contact)</t>
+          <t>Badili Innovations (info@badili.co.ke)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://ujuzicraft.com/</t>
+          <t>UjuziCraft (info@ujuzicraft.com)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green, Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Mozilla Common Voice (https://commonvoice.mozilla.org)</t>
+          <t>Mozilla Common Voice (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NaijaSenti (https://github.com/hausanlp/NaijaSenti?tab=readme-ov-file#contact-us)</t>
+          <t>NaijaSenti / HausaNLP (hausanlp@gmail.com)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Hesotech (https://www.hesotech.de/en/contact-directions/)</t>
+          <t>Hesotech (info@hesotech.de)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact)</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com)</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Digital Umuganda (https://digitalumuganda.com/#contact), FAIR Forward Rwanda</t>
+          <t>Digital Umuganda (samuel@digitalumuganda.com), FAIR Forward Rwanda</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Digital Umuganda (Samuel), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
+          <t>Digital Umuganda - Samuel (samuel@digitalumuganda.com), HDI-Rwanda (Louange Twahirwa Gutabarwa)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>SEE Africa (https://seeafricatz.org/contact-us/)</t>
+          <t>SEE Africa (info@seeafricatz.org)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Croppie (https://croppie.org/#contact), Producers Direct (https://producersdirect.org/), M-Omulimisa, CIAT</t>
+          <t>Croppie - Romain Gautron (r.gautron@cgiar.org), Producers Direct (info@producersdirect.org), M-Omulimisa, CIAT</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CSBAG (https://www.csbag.org/)</t>
+          <t>CSBAG (csbag@csbag.org)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10656,9 +10656,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Makerere University https://mak.ac.ug,
-Makerere AI Lab: https://air.ug/ 
-National Forestry Authority (NFA): https://nfa.go.ug/  </t>
+          <t>Makerere AI Lab - Dr. Joyce Nabende (joyce.nabende@mak.ac.ug), National Forestry Authority (NFA): https://nfa.go.ug/</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11283,7 +11281,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>https://c4ir.rw/</t>
+          <t>C4IR Rwanda (info@c4ir.rw)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-16 08:45:35 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1869,12 +1869,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Indigenous Knowledge Meets AI: Monitoring Elephants and Rodents in Kenya and Ecuador with Biodiversity AI-Datasets</t>
+          <t>Indigenous Knowledge Meets AI: Ethical monitoring of climate stress and biodiversity: sounds of elephants and Katip (Ltome-Katip) in Kenya and the Ecuadorian Amazon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ltome-Katip: Pioneering Indigenous-Led Biodiversity Datasets for Ethical AI in Kenya and the Ecuadorian Amazon</t>
+          <t>Indigenous Knowledge Meets AI: Ethical monitoring of climate stress and biodiversity: sounds of elephants and Katip (Ltome-Katip) in Kenya and the Ecuadorian Amazon</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4902,7 +4902,7 @@
       <c r="J36" t="inlineStr">
         <is>
           <t>Vertify.earth - Michael Anthony (michael@vertify.earth), 
-Alsisar Impact - Saurabh Singhavi (saurabh@alsisarimpact.com)</t>
+Alsisar Impact (anuj@alsisarimpact.com )</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Room Networks Foundation https://commonroom.info/   </t>
+          <t>Common Room Networks Foundation (email.commonroom@gmail.com)</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-16 08:45:35 UTC (#92)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1869,12 +1869,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Indigenous Knowledge Meets AI: Monitoring Elephants and Rodents in Kenya and Ecuador with Biodiversity AI-Datasets</t>
+          <t>Indigenous Knowledge Meets AI: Ethical monitoring of climate stress and biodiversity: sounds of elephants and Katip (Ltome-Katip) in Kenya and the Ecuadorian Amazon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ltome-Katip: Pioneering Indigenous-Led Biodiversity Datasets for Ethical AI in Kenya and the Ecuadorian Amazon</t>
+          <t>Indigenous Knowledge Meets AI: Ethical monitoring of climate stress and biodiversity: sounds of elephants and Katip (Ltome-Katip) in Kenya and the Ecuadorian Amazon</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4902,7 +4902,7 @@
       <c r="J36" t="inlineStr">
         <is>
           <t>Vertify.earth - Michael Anthony (michael@vertify.earth), 
-Alsisar Impact - Saurabh Singhavi (saurabh@alsisarimpact.com)</t>
+Alsisar Impact (anuj@alsisarimpact.com )</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Room Networks Foundation https://commonroom.info/   </t>
+          <t>Common Room Networks Foundation (email.commonroom@gmail.com)</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-16 09:36:18 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India with different accents and speaking styles</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India with different accents and speaking styles</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-16 09:36:18 UTC (#93)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India with different accents and speaking styles</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Voice Tech for All: Building Inclusive Speech AI for India</t>
+          <t>Voice Tech for All: Building Inclusive Speech AI for India with different accents and speaking styles</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-17 14:36:58 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4182,7 +4182,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Multiple models are available based on the shared data. Plesae refer to the GitHub repository.</t>
+          <t>Multiple models are available based on the shared data. Please refer to the GitHub repository.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -4200,7 +4200,7 @@
         <is>
           <t>Powered by / Provided by: Digital Green
 Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
-Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -9929,7 +9929,11 @@
           <t>Kiswahili Text and Voice Recognition Platform (KTVRP) for Agricultural Advisory and Financial Services for Smallholder Farmers</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
@@ -10030,7 +10034,11 @@
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
@@ -11378,10 +11386,14 @@
           <t>C4IR Grant, Rwanda Media Voice Bridge</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Rwanda Media Voice Bridge -  AI-powered voice transcription and translation solution for Rwanda's film and media industry</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Rwanda Media Voice Bridge</t>
+          <t>Rwanda Media Voice Bridge -  AI-powered voice transcription and translation solution for Rwanda's film and media industry</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-17 14:36:58 UTC (#94)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4182,7 +4182,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Multiple models are available based on the shared data. Plesae refer to the GitHub repository.</t>
+          <t>Multiple models are available based on the shared data. Please refer to the GitHub repository.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -4200,7 +4200,7 @@
         <is>
           <t>Powered by / Provided by: Digital Green
 Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
-Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -9929,7 +9929,11 @@
           <t>Kiswahili Text and Voice Recognition Platform (KTVRP) for Agricultural Advisory and Financial Services for Smallholder Farmers</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>AI for Agricultural Advisory and Financial Services for Smallholder Farmers in Tanzania</t>
@@ -10030,7 +10034,11 @@
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>Kiazi Bora - informing vulnerable women in Tanzania on the nutritional values of Orange Fleshed Sweet Potatoes</t>
@@ -11378,10 +11386,14 @@
           <t>C4IR Grant, Rwanda Media Voice Bridge</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Rwanda Media Voice Bridge -  AI-powered voice transcription and translation solution for Rwanda's film and media industry</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Rwanda Media Voice Bridge</t>
+          <t>Rwanda Media Voice Bridge -  AI-powered voice transcription and translation solution for Rwanda's film and media industry</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-18 16:04:14 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Enabling machine translation from Kiswahili into the indigenous Kenyan languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
+          <t>Enabling machine translation from Kiswahili into the indigenous East African languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya, East Africa</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-18 16:04:14 UTC (#95)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Enabling machine translation from Kiswahili into the indigenous Kenyan languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
+          <t>Enabling machine translation from Kiswahili into the indigenous East African languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya, East Africa</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-22 12:37:41 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Benin/West Africa</t>
+          <t>Benin, West Africa</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Laboratoire de Biomathématiques et d'Estimations Forestières
+          <t>Powered by / Provided by: Université d’Abomey-Calavi - Laboratoire de Biomathématiques et d'Estimations Forestières (Benin)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -848,7 +848,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Benin,Ghana,Niger,Togo, Nigeria</t>
+          <t>Benin, Ghana, Niger, Togo, Nigeria</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: CTTC, INVEMAR
+          <t>Powered by / Provided by: Marine and Coastal Research Institute "José Benito Vives de Andréis" (INVEMAR) Colombia, Centre Tecnològic de Telecomunicacions de Catalunya (CTTC)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Powered by / Provided by:  Responsible AI Lab at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/), Ghanaian Plant Protection and Regulatory Services Directorate
+          <t>Powered by / Provided by: Kwame Nkrumah University of Science and Technology (KNUST), Responsible AI Lab (https://rail.knust.edu.gh/), Plant Protection and Regulatory Services Directorate (Ghana)
 Catalyzed by: FAIR Forward - AI for All, GIZ (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), Digital Transformation Centre Ghana, GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: World Resources Institute (WRI), CERSGIS, NASA SERVIR, Earth System Science Center
+          <t>Powered by / Provided by: World Resources Institute (WRI), Centre for Remote Sensing and Geographic Information Services (CERSGIS), NASA SERVIR Global Collaborative, Earth System Science Center
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: RAIL - KNUST (https://rail.knust.edu.gh/)
+          <t>Powered by / Provided by: Kwame Nkrumah University of Science and Technology (KNUST), Responsible AI Lab (https://rail.knust.edu.gh/)
 Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Kara Agro (https://karaagro.com/) , Makerere AI Lab, Marconi Lab, National Coffee Research Institute, National Crops Resources Research Institute
+          <t>Powered by / Provided by: Kara Agro (https://karaagro.com/), Makerere University (AI Lab, Marconi Lab), National Coffee Research Institute, National Crops Resources Research Institute
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Maseno Centre for Applied Artificial Intelligence, Maseno University, Members from the Dholuo language community 
+          <t>Powered by / Provided by: Maseno University (Maseno Centre for Applied Artificial Intelligence), Members from the Dholuo language community 
 Catalyzed by: Mozilla Foundation, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -4673,7 +4673,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bonn Consulting, Frauenhofer Institute
+          <t>Powered by / Provided by: Bonn Consulting, Fraunhofer Institute
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -5076,8 +5076,8 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bappenas, Prosa.ai
-Catalyzed by: FAIR Forward - AI for All, GIZ
+          <t>Powered by / Provided by: Prosa.ai
+Catalyzed by: Bappenas - Ministry of State Development Planning (Indonesia), FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5230,8 +5230,8 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bappenas
-Catalyzed by: FAIR Forward - AI for All, GIZ, HCSA, Seknas JKPP
+          <t>Powered by / Provided by: High Carbon Stock Approach (HCSA) Foundation, Jaringan Kerja Pemetaan Partisipatif (Seknas JKPP)
+Catalyzed by: FAIR Forward - AI for All - GIZ, Bappenas - Ministry of State Development Planning (Indonesia)
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: USIU-Africa, Kabarak University, Maseno University (Kenya)
+          <t>Powered by / Provided by: United States International University Africa (USIU) - Kenya, Kabarak University, Maseno University (Kenya)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya, East Africa</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -6963,7 +6963,7 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Digital Green, Viamo, Partners, Tech for Her, DynAg, Digifarm, Opportunity International
+          <t>Powered by / Provided by: Digital Green, Viamo, Tech for Her, DynAg, Digifarm, Opportunity International
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation</t>
         </is>
@@ -7050,7 +7050,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Kenya, Rwanda, Uganda</t>
+          <t>Kenya, Rwanda, Uganda, East Africa</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bayero University (Kano, Nigeria), Ahmadu Bello University (Zaria, Nigeria), Masakhane NLP, HausaNLP, Kaduna state University
+          <t>Powered by / Provided by: Bayero University (Kano, Nigeria), Ahmadu Bello University (Zaria, Nigeria), Masakhane NLP, HausaNLP, Kaduna State University
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10482,7 +10482,7 @@
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Marconi Lab
+          <t>Powered by / Provided by: Makerere University (Marconi Lab)
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10692,7 +10692,7 @@
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Makerere University in cooperation with the Uganda National Forestry Authority (NFA)
+          <t>Powered by / Provided by: Makerere University in cooperation with the National Forestry Authority (NFA) of Uganda
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10818,7 +10818,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Makerere AI Lab, Marconi Lab, Clear Global
+          <t>Powered by / Provided by: Makerere University (Makerere AI Lab, Marconi Lab), Clear Global
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -11062,7 +11062,7 @@
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Made by People / Tanasuk Technologies Africa, Kenya, CLEAR Global, Tech Innovators Network Kenya (THiNK)
+          <t>Powered by / Provided by: Made by People / Tanasuk Technologies Africa, Kenya, CLEAR Global, Tech Innovators Network Kenya (THiNK), BRS - Business Registration Service (Kenya)
 Catalyzed by: Smart Development Fund, FAIR Forward - AI for All, Digital Transformation Centre Kenya, GIZ
 Financed by: BMZ</t>
         </is>
@@ -11453,7 +11453,9 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>GIZ Film Made in Africa, C4IR, Duka Labs</t>
+          <t>Powered by / Provided by: , Centre for the Fourth Industrial Revolution Rwanda (C4IR), Duka Labs
+Catalyzed by: GIZ Regional AI Hub Rwanda, GIZ Film Made in Africa, FAIR Forward - AI for All, GIZ
+Financed by: BMZ</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-22 12:37:41 UTC (#96)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Benin/West Africa</t>
+          <t>Benin, West Africa</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Laboratoire de Biomathématiques et d'Estimations Forestières
+          <t>Powered by / Provided by: Université d’Abomey-Calavi - Laboratoire de Biomathématiques et d'Estimations Forestières (Benin)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -848,7 +848,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Benin,Ghana,Niger,Togo, Nigeria</t>
+          <t>Benin, Ghana, Niger, Togo, Nigeria</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: CTTC, INVEMAR
+          <t>Powered by / Provided by: Marine and Coastal Research Institute "José Benito Vives de Andréis" (INVEMAR) Colombia, Centre Tecnològic de Telecomunicacions de Catalunya (CTTC)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Powered by / Provided by:  Responsible AI Lab at Kwame Nkrumah University of Science and Technology (https://rail.knust.edu.gh/), Ghanaian Plant Protection and Regulatory Services Directorate
+          <t>Powered by / Provided by: Kwame Nkrumah University of Science and Technology (KNUST), Responsible AI Lab (https://rail.knust.edu.gh/), Plant Protection and Regulatory Services Directorate (Ghana)
 Catalyzed by: FAIR Forward - AI for All, GIZ (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), Digital Transformation Centre Ghana, GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: World Resources Institute (WRI), CERSGIS, NASA SERVIR, Earth System Science Center
+          <t>Powered by / Provided by: World Resources Institute (WRI), Centre for Remote Sensing and Geographic Information Services (CERSGIS), NASA SERVIR Global Collaborative, Earth System Science Center
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: RAIL - KNUST (https://rail.knust.edu.gh/)
+          <t>Powered by / Provided by: Kwame Nkrumah University of Science and Technology (KNUST), Responsible AI Lab (https://rail.knust.edu.gh/)
 Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Kara Agro (https://karaagro.com/) , Makerere AI Lab, Marconi Lab, National Coffee Research Institute, National Crops Resources Research Institute
+          <t>Powered by / Provided by: Kara Agro (https://karaagro.com/), Makerere University (AI Lab, Marconi Lab), National Coffee Research Institute, National Crops Resources Research Institute
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Maseno Centre for Applied Artificial Intelligence, Maseno University, Members from the Dholuo language community 
+          <t>Powered by / Provided by: Maseno University (Maseno Centre for Applied Artificial Intelligence), Members from the Dholuo language community 
 Catalyzed by: Mozilla Foundation, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
 Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
         </is>
@@ -4673,7 +4673,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bonn Consulting, Frauenhofer Institute
+          <t>Powered by / Provided by: Bonn Consulting, Fraunhofer Institute
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -5076,8 +5076,8 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bappenas, Prosa.ai
-Catalyzed by: FAIR Forward - AI for All, GIZ
+          <t>Powered by / Provided by: Prosa.ai
+Catalyzed by: Bappenas - Ministry of State Development Planning (Indonesia), FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
       </c>
@@ -5230,8 +5230,8 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bappenas
-Catalyzed by: FAIR Forward - AI for All, GIZ, HCSA, Seknas JKPP
+          <t>Powered by / Provided by: High Carbon Stock Approach (HCSA) Foundation, Jaringan Kerja Pemetaan Partisipatif (Seknas JKPP)
+Catalyzed by: FAIR Forward - AI for All - GIZ, Bappenas - Ministry of State Development Planning (Indonesia)
 Financed by: BMZ</t>
         </is>
       </c>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: USIU-Africa, Kabarak University, Maseno University (Kenya)
+          <t>Powered by / Provided by: United States International University Africa (USIU) - Kenya, Kabarak University, Maseno University (Kenya)
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya, East Africa</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -6963,7 +6963,7 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Digital Green, Viamo, Partners, Tech for Her, DynAg, Digifarm, Opportunity International
+          <t>Powered by / Provided by: Digital Green, Viamo, Tech for Her, DynAg, Digifarm, Opportunity International
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: Gates Foundation</t>
         </is>
@@ -7050,7 +7050,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Kenya, Rwanda, Uganda</t>
+          <t>Kenya, Rwanda, Uganda, East Africa</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Bayero University (Kano, Nigeria), Ahmadu Bello University (Zaria, Nigeria), Masakhane NLP, HausaNLP, Kaduna state University
+          <t>Powered by / Provided by: Bayero University (Kano, Nigeria), Ahmadu Bello University (Zaria, Nigeria), Masakhane NLP, HausaNLP, Kaduna State University
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10482,7 +10482,7 @@
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Marconi Lab
+          <t>Powered by / Provided by: Makerere University (Marconi Lab)
 Catalyzed by: FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10692,7 +10692,7 @@
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Makerere University in cooperation with the Uganda National Forestry Authority (NFA)
+          <t>Powered by / Provided by: Makerere University in cooperation with the National Forestry Authority (NFA) of Uganda
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -10818,7 +10818,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Makerere AI Lab, Marconi Lab, Clear Global
+          <t>Powered by / Provided by: Makerere University (Makerere AI Lab, Marconi Lab), Clear Global
 Catalyzed by: Lacuna-Fund / Meridian (Climate-call) &amp; FAIR Forward - AI for All, GIZ
 Financed by: BMZ</t>
         </is>
@@ -11062,7 +11062,7 @@
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
-          <t>Powered by / Provided by: Made by People / Tanasuk Technologies Africa, Kenya, CLEAR Global, Tech Innovators Network Kenya (THiNK)
+          <t>Powered by / Provided by: Made by People / Tanasuk Technologies Africa, Kenya, CLEAR Global, Tech Innovators Network Kenya (THiNK), BRS - Business Registration Service (Kenya)
 Catalyzed by: Smart Development Fund, FAIR Forward - AI for All, Digital Transformation Centre Kenya, GIZ
 Financed by: BMZ</t>
         </is>
@@ -11453,7 +11453,9 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>GIZ Film Made in Africa, C4IR, Duka Labs</t>
+          <t>Powered by / Provided by: , Centre for the Fourth Industrial Revolution Rwanda (C4IR), Duka Labs
+Catalyzed by: GIZ Regional AI Hub Rwanda, GIZ Film Made in Africa, FAIR Forward - AI for All, GIZ
+Financed by: BMZ</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-23 08:12:51 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4123,35 +4123,30 @@
           <t>ui_28</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Digital Green - Local dataset collection for climate-smart agriculture</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Geospatial dataset of wheat and rice farmers in Bihar, India</t>
+          <t>FarmerChat: Open AI-Powered Agricultural Advisory for Smallholder Farmers</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Data-driven decision-making for farmers to increase climate resilience in India</t>
+          <t>FarmerChat: Delivering Personalized Farm Advice to 1.6 Million Farmers Across Five Countries</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
-The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
+          <t>FarmerChat is an AI assistant built to help smallholder farmers make better field-level decisions by delivering timely, localized advice to help them grow more, earn more, and adapt to changing weather. It is designed for low-connectivity areas and available in over 15 languages including Swahili, Portuguese, Spanish, Hindi, Telugu, Amharic, Hausa, and English.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/frame-templates</t>
+          <t>https://github.com/digitalgreenorg/DG_Open</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/frame-templates</t>
+          <t>https://play.google.com/store/apps/details?id=org.digitalgreen.farmer.chat&amp;hl=en_US</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -4161,23 +4156,24 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Tabular</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (info@digitalgreentrust.org)</t>
+          <t>Digital Green (contact@digitalgreen.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Worldwide, focusing on the global south, particularly India, Kenya, Nigeria, Ethiopia, and Brazil</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-</t>
+          <t>The FarmerChat system draws from an agronomic content corpus that powers FarmerChat's advisory responses — curated from ICAR, national extension services, and field-validated crop guidance across India, Kenya, Ethiopia, Nigeria, and Brazil. This content is organized by crop, geography, and query type, enabling the system to return locally grounded answers rather than generic advice.
+Key characteristics: multilingual (15 languages), multi-country (5 geographies), low-bandwidth optimized, and continuously updated through fine-tuning and RLHF loops informed by farmer feedback and agronomist review. Query volume has reached 9 million across 1.6 million farmers, providing a rare at-scale signal on what smallholder farmers actually ask and what advice they act on.
+Responsible AI: FarmerChat's content pipeline includes human agronomist review before deployment in any new crop or geography. Outputs are grounded in verified extension material to reduce hallucination risk. Digital Green has invested in RLHF infrastructure to surface low-quality responses for expert correction.</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4187,8 +4183,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>The possibilities include creating a machine learning solution to predict the crop yield per acre of rice or wheat crops in India. Our goal is to empower these farmers and break the cycle of poverty and malnutrition.
-This use case also included the development of a business model and funding model for open source AI as a stepping stone towards financially viable operations. It was facilitated by Villgro Africa's and FAIR Forward's  six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/</t>
+          <t>FarmerChat can be engaged at four levels depending on your organization's technical capacity, timeline, and deployment goals.
+Open Build Partner: Technically equipped organizations can build independently on Digital Green's public infrastructure. The full codebase is available at github.com/digitalgreenorg/DG_Open (Apache 2.0) and datasets are on GitHub and Hugging Face. Digital Green publishes and maintains the open source foundation; the partner owns everything from development through deployment.
+Community Partner: For organizations ready to launch quickly without requiring Digital Green staff time. Digital Green provides and maintains the FarmerChat platform at no cost, along with an onboarding toolkit, co-brandable campaign templates, and remote training support. The partner leads all in-country training and farmer outreach.
+Custom Partnership: For organizations that want Digital Green staff actively involved in their deployment. Depending on scope, this can range from research-grade validation — where Digital Green contributes expert agronomic content review, M&amp;E frameworks, and pre-built analytics dashboards — through to full co-implementation, where Digital Green dedicates product and engineering staff to customize across various features of localization and the tech stack.
+To get started, organizations should reach out to Digital Green to find the partnership tier that best suits their needs.
+Basic eligibility: farmers should be reachable in a language FarmerChat supports (including English, Hindi, Telugu, Amharic, Kiswahili, Hausa, Portuguese, Spanish, and others), have access to an Android smartphone directly or via a shared-device model, and the project should have a credible distribution path through an extension network, cooperative, government department, or telecom partnership.</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4216,21 +4216,17 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Computer Vision, Other</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://digitalgreen.org/wp-content/uploads/2024/10/GIZ-FF_DG_Learning-Report.pdf</t>
+          <t>https://drive.google.com/file/d/11jmgluDCSqyMzP9s_VJCMgZVGkdmXePH/view?usp=sharing</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>In our monitoring, we assess as pilot rather for maturity - buth there was also business model built. therefore the entry here on maturity is including "use case"</t>
-        </is>
-      </c>
+      <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr">
         <is>
           <t>No</t>
@@ -5038,7 +5034,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5177,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
+          <t>JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-23 08:12:51 UTC (#99)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4123,35 +4123,30 @@
           <t>ui_28</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Digital Green - Local dataset collection for climate-smart agriculture</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Geospatial dataset of wheat and rice farmers in Bihar, India</t>
+          <t>FarmerChat: Open AI-Powered Agricultural Advisory for Smallholder Farmers</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Data-driven decision-making for farmers to increase climate resilience in India</t>
+          <t>FarmerChat: Delivering Personalized Farm Advice to 1.6 Million Farmers Across Five Countries</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields. 
-The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.</t>
+          <t>FarmerChat is an AI assistant built to help smallholder farmers make better field-level decisions by delivering timely, localized advice to help them grow more, earn more, and adapt to changing weather. It is designed for low-connectivity areas and available in over 15 languages including Swahili, Portuguese, Spanish, Hindi, Telugu, Amharic, Hausa, and English.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/frame-templates</t>
+          <t>https://github.com/digitalgreenorg/DG_Open</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/frame-templates</t>
+          <t>https://play.google.com/store/apps/details?id=org.digitalgreen.farmer.chat&amp;hl=en_US</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -4161,23 +4156,24 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Tabular</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Digital Green (info@digitalgreentrust.org)</t>
+          <t>Digital Green (contact@digitalgreen.org)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Worldwide, focusing on the global south, particularly India, Kenya, Nigeria, Ethiopia, and Brazil</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.
-</t>
+          <t>The FarmerChat system draws from an agronomic content corpus that powers FarmerChat's advisory responses — curated from ICAR, national extension services, and field-validated crop guidance across India, Kenya, Ethiopia, Nigeria, and Brazil. This content is organized by crop, geography, and query type, enabling the system to return locally grounded answers rather than generic advice.
+Key characteristics: multilingual (15 languages), multi-country (5 geographies), low-bandwidth optimized, and continuously updated through fine-tuning and RLHF loops informed by farmer feedback and agronomist review. Query volume has reached 9 million across 1.6 million farmers, providing a rare at-scale signal on what smallholder farmers actually ask and what advice they act on.
+Responsible AI: FarmerChat's content pipeline includes human agronomist review before deployment in any new crop or geography. Outputs are grounded in verified extension material to reduce hallucination risk. Digital Green has invested in RLHF infrastructure to surface low-quality responses for expert correction.</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4187,8 +4183,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>The possibilities include creating a machine learning solution to predict the crop yield per acre of rice or wheat crops in India. Our goal is to empower these farmers and break the cycle of poverty and malnutrition.
-This use case also included the development of a business model and funding model for open source AI as a stepping stone towards financially viable operations. It was facilitated by Villgro Africa's and FAIR Forward's  six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/</t>
+          <t>FarmerChat can be engaged at four levels depending on your organization's technical capacity, timeline, and deployment goals.
+Open Build Partner: Technically equipped organizations can build independently on Digital Green's public infrastructure. The full codebase is available at github.com/digitalgreenorg/DG_Open (Apache 2.0) and datasets are on GitHub and Hugging Face. Digital Green publishes and maintains the open source foundation; the partner owns everything from development through deployment.
+Community Partner: For organizations ready to launch quickly without requiring Digital Green staff time. Digital Green provides and maintains the FarmerChat platform at no cost, along with an onboarding toolkit, co-brandable campaign templates, and remote training support. The partner leads all in-country training and farmer outreach.
+Custom Partnership: For organizations that want Digital Green staff actively involved in their deployment. Depending on scope, this can range from research-grade validation — where Digital Green contributes expert agronomic content review, M&amp;E frameworks, and pre-built analytics dashboards — through to full co-implementation, where Digital Green dedicates product and engineering staff to customize across various features of localization and the tech stack.
+To get started, organizations should reach out to Digital Green to find the partnership tier that best suits their needs.
+Basic eligibility: farmers should be reachable in a language FarmerChat supports (including English, Hindi, Telugu, Amharic, Kiswahili, Hausa, Portuguese, Spanish, and others), have access to an Android smartphone directly or via a shared-device model, and the project should have a credible distribution path through an extension network, cooperative, government department, or telecom partnership.</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4216,21 +4216,17 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Computer Vision, Other</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://digitalgreen.org/wp-content/uploads/2024/10/GIZ-FF_DG_Learning-Report.pdf</t>
+          <t>https://drive.google.com/file/d/11jmgluDCSqyMzP9s_VJCMgZVGkdmXePH/view?usp=sharing</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>In our monitoring, we assess as pilot rather for maturity - buth there was also business model built. therefore the entry here on maturity is including "use case"</t>
-        </is>
-      </c>
+      <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr">
         <is>
           <t>No</t>
@@ -5038,7 +5034,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), Prosa AI (business@prosa.ai)</t>
+          <t>Prosa AI (business@prosa.ai)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -5181,7 +5177,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bappenas (https://www.bappenas.go.id/), JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
+          <t>JKPP (seknas@jkpp.org), HCSA (info@highcarbonstock.org), EcoVision Lab (jandirk.wegner@uzh.ch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-25 14:21:37 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1359,7 +1359,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://zindi.africa/competitions/africa-biomass-challenge </t>
+          <t>https://zindi.africa/competitions/africa-biomass-challenge; https://www.google.com/url?sa=t&amp;rct=j&amp;q=&amp;esrc=s&amp;source=web&amp;cd=&amp;ved=2ahUKEwjn657i3p-VAxXTRfEDHUweFDcQFnoECAoQAQ&amp;url=https%3A%2F%2Fstorage.googleapis.com%2Fdownload%2Fstorage%2Fv1%2Fb%2Findaba-public%2Fo%2FIssouf_TOURE.pdf%3Fgeneration%3D1724089094997741%26alt%3Dmedia&amp;usg=AOvVaw35fJfv4r2g0OJp3rZLpYIt&amp;opi=89978449</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -9763,7 +9763,7 @@
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Mozilla CVP</t>
+          <t>Localising the Mozilla Common Voice platform for South Africa’s official languages | Journal of the Digital Humanities Association of Southern Africa (DHASA)</t>
         </is>
       </c>
       <c r="W75" t="inlineStr"/>

</xml_diff>

<commit_message>
Sheet update 2026-06-25 14:21:37 UTC (#102)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1359,7 +1359,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://zindi.africa/competitions/africa-biomass-challenge </t>
+          <t>https://zindi.africa/competitions/africa-biomass-challenge; https://www.google.com/url?sa=t&amp;rct=j&amp;q=&amp;esrc=s&amp;source=web&amp;cd=&amp;ved=2ahUKEwjn657i3p-VAxXTRfEDHUweFDcQFnoECAoQAQ&amp;url=https%3A%2F%2Fstorage.googleapis.com%2Fdownload%2Fstorage%2Fv1%2Fb%2Findaba-public%2Fo%2FIssouf_TOURE.pdf%3Fgeneration%3D1724089094997741%26alt%3Dmedia&amp;usg=AOvVaw35fJfv4r2g0OJp3rZLpYIt&amp;opi=89978449</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -9763,7 +9763,7 @@
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Mozilla CVP</t>
+          <t>Localising the Mozilla Common Voice platform for South Africa’s official languages | Journal of the Digital Humanities Association of Southern Africa (DHASA)</t>
         </is>
       </c>
       <c r="W75" t="inlineStr"/>

</xml_diff>

<commit_message>
Resync catalog from sheet (Voices of Mzansi contacts)
Regenerated catalog/insights data and sheet backup from the current Google Sheet. Picks up the updated Voices of Mzansi contact 'Prof. Febe de Wet (febe.dewet@gmail.com); Mozilla Data Collective (support@mozilladatacollective.com)', which the contact-field fix now renders as two separate links.
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,142 +429,142 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>OnSite Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Dataset Speaking Titles</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Use Case Speaking Title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description - What can be done with this? What is this about?</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Dataset Link</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case Links</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Domain/SDG</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Point of Contact/Communities</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Country Team</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Data - Key Characteristics</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Model/Use-Case - Key Characteristics</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Deep Dive - How can you concretely work with this and build on this?</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Organizations Involved</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Lacuna Dataset</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Maturity / Readiness for replication or scaling [INTERNAL]</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Technical Domain</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Expressive visualization / picture related to dataset / possible use / story-tellling</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Link to additional Resources (Paper, Publications, etc)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Info on fair sharing as as Digital Public Good </t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Registered as "Digital Public Good" with the DPGA registry?</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Link to entry in DPG registry</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">On Hold </t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -740,7 +752,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
+          <t xml:space="preserve">The dataset provides georeferenced, annotated drone imagery with clear landuse and landcover classes, groundtruth data, and standardized protocols. The datatset also provide field Carbon inventoried data paired with the drone imagery. As such, users can train AI models for carboj estimation is harsh mangroves ecosystems. Its high resolution, temporal coverage, and open accessibility enable accurate, scalable environmental monitoring and carbon estimation. Furthermore, the dataset include (1) Soil quality analyses, including soil organic carbon, Total Nitrogen, granulometry, CEC, phosphorus, and potassium;  (2) Water quality analyses, including soil nutrients (Nitrates, Nitrites, Sulfate, Ammonium, Orthophosphate) and pollution (Iron, Cadmium, Lead, and Zinc), and (3) Socio-economic survey data on community livelihoods, mangrove forests’ resources use, and climate change adaptation strategies; allowing to develop models aiming at understanding how local soil, water, and socio-économic profile affect carbon stock. 
 </t>
         </is>
       </c>
@@ -1359,7 +1371,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://zindi.africa/competitions/africa-biomass-challenge </t>
+          <t>https://zindi.africa/competitions/africa-biomass-challenge; https://www.google.com/url?sa=t&amp;rct=j&amp;q=&amp;esrc=s&amp;source=web&amp;cd=&amp;ved=2ahUKEwjn657i3p-VAxXTRfEDHUweFDcQFnoECAoQAQ&amp;url=https%3A%2F%2Fstorage.googleapis.com%2Fdownload%2Fstorage%2Fv1%2Fb%2Findaba-public%2Fo%2FIssouf_TOURE.pdf%3Fgeneration%3D1724089094997741%26alt%3Dmedia&amp;usg=AOvVaw35fJfv4r2g0OJp3rZLpYIt&amp;opi=89978449</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -2080,7 +2092,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">
+          <t xml:space="preserve">
 https://www.gnu.org/licenses/agpl-3.0.html</t>
         </is>
       </c>
@@ -2893,8 +2905,8 @@
       <c r="V20" t="inlineStr">
         <is>
           <t xml:space="preserve">Quote: “The threat of climate change on forest health affects leaf, flower, and fruit resource availability, but we cannot be prepared unless we have adequate data with predictive power. We have an incredible opportunity to create a harmonized machine-learning-ready dataset for ecological forecasting with the support of Lacuna Fund. Such a forecast could provide the basis for an early warning system that will help communities and resource managers better plan and prepare for climate change impact on forest resources.”
-— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
-Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
+— Bismark Ofosu-Bamfo, Department of Biological Sciences, University of Energy and Natural Resources; Also see news items News coverage
+Ghana News Agency: https://gna.org.gh/2025/07/realistic-phenology-data-key-to-predicting-crop-cycles-dr-ofosu-bamfo-2/
 Joy News (video): https://g.co/kgs/5byh6f7 </t>
         </is>
       </c>
@@ -3091,7 +3103,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dr. Lilian Wanzare &lt;ldwanzare@maseno.ac.ke&gt;, Dept. of Computer Science, School of Computing and Informatics, Maseno University
+          <t xml:space="preserve">Dr. Lilian Wanzare &lt;ldwanzare@maseno.ac.ke&gt;, Dept. of Computer Science, School of Computing and Informatics, Maseno University
 </t>
         </is>
       </c>
@@ -3113,12 +3125,12 @@
 Healthcare
 News and current affairs
 These domains reflect real spoken Dholuo usage.
-Total duration: 184,838.28 sec (3080.64 min, 51.34 hr)
-Number of Speakers: 59
-Number of Reviewers: 7
-Total audio files: 26,091
-Average clip length: 7.08 sec
-Minimum clip length: 1.72 sec
+Total duration: 184,838.28 sec (3080.64 min, 51.34 hr)
+Number of Speakers: 59
+Number of Reviewers: 7
+Total audio files: 26,091
+Average clip length: 7.08 sec
+Minimum clip length: 1.72 sec
 Maximum clip length: 62.64 sec</t>
         </is>
       </c>
@@ -3631,7 +3643,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in), Dr. Philipp Olbrich (philipp.olbrich@giz.de)</t>
+          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -4049,7 +4061,7 @@
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">Translation: This corpus contains a collection of sentence pairs that have been translated from Hindi to Mundari. The dataset was created as part of a collaboration between Microsoft Research India, Indian Institute of Technology Kharagpur, and Karya. This dataset is realeased under the non-commercial version of the Karya Public License. Please read the "License" section below for a high-level summary of what you are allowed and not allowed to do under this license. The dataset contains 17,826 sentence pairs of Hindi to Mundari translations. The translations are stored in a single TSV file translation-hi-unr.tsv with UTF-8 encoding. Each line in the TSV file contains two columns, separated by a tab character. The first column contains the Hindi sentence, and the second column contains the corresponding Mundari translation.
-Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
+Text-to-speech:The Mundari TTS dataset corpus contains a total of 26,870 audio files, each containing a single utterance spoken by one of the two speakers. The audio is recorded in 32-bit PCM format with a sampling rate of 44.1 kHz. The dataset includes transcripts for each audio file in Mundari script. The recordings were collected in a sound-treated room using a high-quality microphone and preamp.
 </t>
         </is>
       </c>
@@ -4060,7 +4072,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
+          <t>The Mundari TTS dataset corpus includes recordings from two different speakers: a female speaker and a male speaker. The female speaker contributed 19,868 recordings, while the male speaker contributed 7,002 recordings.
 The total size of the corpus is approximately 17 GB (7 GB compressed). Therefore, the full dataset is hosted in cloud storage (instead of this github repository). This repository contains a sample of 100 recordings from each speaker. Please email data@karya.in for a link to download the full dataset.</t>
         </is>
       </c>
@@ -4166,7 +4178,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Worldwide, focusing on the global south, particularly India, Kenya, Nigeria, Ethiopia, and Brazil</t>
+          <t>India, Kenya, Nigeria, Ethiopia, Brazil</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -4543,22 +4555,22 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
-Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
-Output: Biomass density in Mg/ha (megagrams per hectare)
-Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
-Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
+          <t>This model is trained to predict above-ground biomass (AGB) in tropical and subtropical forests using multi-source satellite imagery at the pixel level. Specifically:
+Prediction Unit: Estimates biomass at individual pixel level (typically 10-40m resolution depending on input data)
+Output: Biomass density in Mg/ha (megagrams per hectare)
+Input Data: Processes multi-sensor data including Sentinel-1, Sentinel-2, Landsat-8, PALSAR, and DEM
+Application Scope: Best suited for tropical and subtropical forest ecosystems in South/Southeast Asia
 Biomass Range: Validated for forests with biomass between ~40-460 Mg/ha</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
-End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
-Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
-Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
-Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
-Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
+          <t>The pipeline is designed to handle multi-source satellite imagery and corresponding biomass data with pixel-level precision. Key aspects include:
+End-to-End Workflow: From raw data ingestion to model training, evaluation, and deployment
+Advanced Feature Engineering: Comprehensive spectral indices, texture features, spatial gradients, and PCA components
+Stable Neural Architecture: Utilizes a custom StableResNet with residual connections and layer normalization for robust biomass regression
+Multi-Site Data Processing: Capable of processing and integrating data from multiple geographically distinct study sites
+Flexible Deployment: Includes HuggingFace deployment capabilities with Gradio interface
 Memory Efficient Processing: Chunk-based processing for handling large satellite images</t>
         </is>
       </c>
@@ -4923,7 +4935,7 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>This dataset and AI model can be used immediately for forest monitoring, restoration planning and impact measurement in mountain and forested regions. Users can map biomass, detect forest loss or assess community-level livelihood impacts by combining the open dataset with freely available satellite imagery. NGOs, research institutions, investors can directly apply the dataset to design or evaluate nature positive projects, while developers can integrate the AI model into their own MRV dashboards. Researchers and AI developers can extend this work by retraining the biomass model with local field data from other regions or adding new layers such as soil moisture or biodiversity indicators. Ethical replication should include community consent and data validation steps to ensure fair and context aware use.
-Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
+Data access: Free (CC-BY 4.0) via Vertify.earth GitHub
 Model use: Free, standard cloud or local compute</t>
         </is>
       </c>
@@ -5517,8 +5529,8 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
-https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
+          <t xml:space="preserve">Nature of Pilot: "we have two IoT sensor prototypes for Aceh called Solitude and Maros called Sentinel: https://commonroom.info/mengenal-kecerdasan-artifisial-dan-internet-of-things-panduan-belajar-untuk-semua/.
+https://commonroom.info/panduan-teknis-sistem-pemantauan-kualitas-air-laut-berbasis-iot-co_labs-panduan-instalasi-pemrograman-dan-perawatan/ 
 Also platform to access the datasets:: https://colabs.commonroom.info/ " </t>
         </is>
       </c>
@@ -6373,10 +6385,10 @@
 - Use the orthophoto tiles and bounding box annotations to train models for individual tree detection, counting, and classification from aerial imagery.
 - Use the terrestrial stereoscopic images to develop and benchmark 3D computer vision models for automating forest inventory, such as estimating biophysical parameters.
 - Combine the ground-truth measurements (TH, CD, BD) and weather data to train models that determine quantitative relationships between tree growth and local weather conditions.
-- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
+- Leverage the multi-year data (2024-2025) to analyse changes in biophysical parameters and determine which tree species are growing well in the reforested area.
 The dataset is designed to be integrated. By augmenting this dataset with others, one can
 - Combine Miti360 with other global forestry datasets mentioned in the report (like NEON Crowns or Auto Arborist) to train models with greater geographic diversity, addressing a key gap this dataset was built to fill.
-- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
+- Augment the dataset with socio-economic data on local farming to explore and validate the contribution of farmers to reforestation, an application suggested in the report.
 Cost &amp; resources one can use:
 - Cost: Only associated compute costs
 - Resources: The source code used for data analysis as well as preliminary models trained on the dataset will be made available.
@@ -7111,7 +7123,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
+          <t>Creating community-driven  datasets: Insights from  Mozilla Common Voice activities in East Africa 
 (https://www.bmz-digital.global/wp-content/uploads/2023/03/Creating-Community-Driven-Datasets-Report-032023-GIZ-Mozilla.pdf)</t>
         </is>
       </c>
@@ -7756,7 +7768,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -8068,8 +8080,8 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
-The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure.
+          <t xml:space="preserve">The mapping method developed is freely accessible and fully documented. Training courses with the Rwandan Space Agency and the Office of Statistics ensure that local experts can continue to develop the system independently.
+The digital maps do not replace observations and measurements in the field or local knowledge. They complement these to create an improved basis for data-driven decisions, more targeted use of resources and forward-looking risk management using digital tools – for agriculture that offers prospects for the future even under climate pressure. </t>
         </is>
       </c>
@@ -9576,7 +9588,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
+          <t xml:space="preserve">Explores the use of Sentinel-1 and Sentinel-2 satellite data for crop type mapping in smallholder farming areas. The study focuses on improving classification accuracy by identifying optimal spectral bands and evaluating machine learning algorithms like decision tree and random forest classifiers
 </t>
         </is>
       </c>
@@ -9715,7 +9727,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Prof. Febe de Wet, Mozilla Data Collective (support@mozilladatacollective.com)</t>
+          <t>Prof. Febe de Wet (febe.dewet@gmail.com); Mozilla Data Collective (support@mozilladatacollective.com)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -9763,7 +9775,7 @@
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Mozilla CVP</t>
+          <t xml:space="preserve">https://upjournals.up.ac.za/index.php/dhasa/article/view/4437 </t>
         </is>
       </c>
       <c r="W75" t="inlineStr"/>
@@ -9852,7 +9864,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
+          <t xml:space="preserve">This repository contains the winning models from the Zindi data competition "Spot the Crop" in which participants used time series of Sentinel-2 multispectral imagery as input for crop type classification.
 </t>
         </is>
       </c>
@@ -10152,8 +10164,8 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
-The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
+          <t xml:space="preserve">Contributing almost a third of foreign export earnings, coffee is one of the main cash crops in Uganda. Nowadays, many small-holder farmers, who rely on coffee farming for their livelihood, are facing challenges such as unpredictable weather and volatile market prices. Traditionally, they have relied on manual yield estimates, but these are time-intensive to perform and not always reliable, leaving many farmers unable to safely plan their harvests or manage their resources effectively. On top, unpredictable weather conditions and price fluctuations pose major challenges for the coffee farmers. 
+The platform and app 'Croppie' supports them with targeted cultivation recommendations and precise crop forecasts—using AI-supported image recognition of coffee plants. As a digital public good based on open-source technology, it can be adapted and further developed locally. The basic user interface is provided through a mobile application. Croppie’s core functionality is to allow for AI-supported coffee yield estimation. This is done by guiding a selective sampling for a statistical yield estimation service based on branch count and coffee branch picture taking, alongside the integration of additional data provided by the user.
 </t>
         </is>
       </c>
@@ -10923,7 +10935,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible.
+          <t xml:space="preserve">The dataset combines satellite imagery with forest field plot data collected across Senegal. Its main limitation is geographic scope, it reflects Senegalese conditions and should be validated against local ground truth before use elsewhere. It will be published as an open digital public good, free to reuse and adapt, provided the original source is credited and derivative work is linked back to the project repository. Users are encouraged to contribute improvements back to the community where possible. </t>
         </is>
       </c>
@@ -11023,7 +11035,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>
+          <t xml:space="preserve">
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Sheet update 2026-06-26 10:40:04 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4141,7 +4141,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/DG_Open</t>
+          <t xml:space="preserve">https://github.com/digitalgreenorg/DG_Open; https://huggingface.co/datasets/DigiGreen/farmerchat-queries-large </t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4199,13 +4199,13 @@
       <c r="P30" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Green
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
-Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
+Catalyzed by: Digital Green, in parts by FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+Financed by: Multiple Funders, among them: The Rockefeller Foundation, Gates Foundation, BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Philipp Olbrich</t>
+          <t>Philipp Olbrich, Balthas Seibold</t>
         </is>
       </c>
       <c r="R30" t="inlineStr"/>
@@ -6905,7 +6905,7 @@
 1. DynAG: 
 Focused on rice, wheat, and maize, DynAG's platform uses a RAG pipeline powered by LLMs like the GPT suite to provide farmers with advisory services. Accessible via chatbots, Android and Jio-based mobile apps, IVR, and SMS, it ensures wide reach. With machine translation and speech recognition, the platform supports communication in English and Hindi while utilizing CGIAR's data backbone for accurate, data-driven insights. 
  2. Digital Green: 
-Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. 
+Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. The project has contributed to Digital Greens current FarmerChat.
  3. Viamo and Partners: 
  This platform targets farmers in Kenya and Bihar, focusing on beans and wheat, respectively. Using IVR, SMS, and WhatsApp, the platform is built on a RAG pipeline powered by LLMs, with potential for intent and entity recognition. Machine translation and speech-enabled IVR support English, Hindi, and Swahili, making it accessible across regions. The initiative is part of a broader plan to enhance voice technology for agricultural advisory. 
  4. Tech for Her: 
@@ -10789,7 +10789,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Uganda,Kenya,Nigeria</t>
+          <t>Uganda, Kenya, Nigeria</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>SDG 8 (Decent Work and Economic Growth), SDG 9 (Industry, Innovation and Infrastructure), SDG 10 (Reduced Inequalities; access to information in local languages).</t>
+          <t>SDG 10, SDG 9, SDG 8</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -11466,7 +11466,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Early stage, functional demo available.</t>
+          <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
       <c r="T89" t="inlineStr"/>
@@ -11509,32 +11509,125 @@
           <t>ui_89</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Digital Green - Local dataset collection for climate-smart agriculture</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Geospatial dataset of wheat and rice farmers in Bihar, India</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Data-driven decision-making for farmers to increase climate resilience in India</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields.
+The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.
+The project has contributed to Digital Greens current FarmerChat.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/digitalgreenorg/frame-templates </t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://github.com/digitalgreenorg/frame-templates</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>SDG 2</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Tabular</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Multiple models are available based on the shared data. Please refer to the GitHub repository.</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The possibilities include creating a machine learning solution to predict the crop yield per acre of rice or wheat crops in India. Our goal is to empower these farmers and break the cycle of poverty and malnutrition.
+This use case also included the development of a business model and funding model for open source AI as a stepping stone towards financially viable operations. It was facilitated by Villgro Africa's and FAIR Forward's six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/ </t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Digital Green
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and Sequoia Climate Fund, CISCO Foundation</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Philipp Olbrich</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case &gt;  Use-Case with Business Model</t>
+        </is>
+      </c>
       <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr"/>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://digitalgreen.org/wp-content/uploads/2024/10/GIZ-FF_DG_Learning-Report.pdf </t>
+        </is>
+      </c>
       <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
-      <c r="Y90" t="inlineStr"/>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>In our monitoring, we assess as pilot rather for maturity - buth there was also business model built. therefore the entry here on maturity is including "use case"</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z90" t="inlineStr"/>
-      <c r="AA90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="AB90" t="inlineStr">
         <is>
           <t>89</t>
@@ -11563,14 +11656,26 @@
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
-      <c r="S91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr"/>
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr"/>
-      <c r="Y91" t="inlineStr"/>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr"/>
       <c r="AB91" t="inlineStr">
@@ -11601,14 +11706,26 @@
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr"/>
-      <c r="Y92" t="inlineStr"/>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z92" t="inlineStr"/>
       <c r="AA92" t="inlineStr"/>
       <c r="AB92" t="inlineStr">
@@ -11639,14 +11756,26 @@
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
-      <c r="S93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr"/>
-      <c r="Y93" t="inlineStr"/>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z93" t="inlineStr"/>
       <c r="AA93" t="inlineStr"/>
       <c r="AB93" t="inlineStr">
@@ -11677,14 +11806,26 @@
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
-      <c r="S94" t="inlineStr"/>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
       <c r="V94" t="inlineStr"/>
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr"/>
-      <c r="Y94" t="inlineStr"/>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z94" t="inlineStr"/>
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-26 10:40:04 UTC (#107)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4141,7 +4141,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://github.com/digitalgreenorg/DG_Open</t>
+          <t xml:space="preserve">https://github.com/digitalgreenorg/DG_Open; https://huggingface.co/datasets/DigiGreen/farmerchat-queries-large </t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4199,13 +4199,13 @@
       <c r="P30" t="inlineStr">
         <is>
           <t>Powered by / Provided by: Digital Green
-Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
-Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
+Catalyzed by: Digital Green, in parts by FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+Financed by: Multiple Funders, among them: The Rockefeller Foundation, Gates Foundation, BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Philipp Olbrich</t>
+          <t>Philipp Olbrich, Balthas Seibold</t>
         </is>
       </c>
       <c r="R30" t="inlineStr"/>
@@ -6905,7 +6905,7 @@
 1. DynAG: 
 Focused on rice, wheat, and maize, DynAG's platform uses a RAG pipeline powered by LLMs like the GPT suite to provide farmers with advisory services. Accessible via chatbots, Android and Jio-based mobile apps, IVR, and SMS, it ensures wide reach. With machine translation and speech recognition, the platform supports communication in English and Hindi while utilizing CGIAR's data backbone for accurate, data-driven insights. 
  2. Digital Green: 
-Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. 
+Digital Green's platform supports agricultural value chains like dairy, coffee, and wheat in Bihar and Kenya. It integrates a RAG pipeline, using LLMs under evaluation, and offers services through an app, Telegram, and IVR. Features like machine translation, speech technology, image recognition, and weather data enable localized insights. The platform supports multiple languages, including Hindi, Swahili, Gikuyu, and Marathi, ensuring flexibility across regions. The project has contributed to Digital Greens current FarmerChat.
  3. Viamo and Partners: 
  This platform targets farmers in Kenya and Bihar, focusing on beans and wheat, respectively. Using IVR, SMS, and WhatsApp, the platform is built on a RAG pipeline powered by LLMs, with potential for intent and entity recognition. Machine translation and speech-enabled IVR support English, Hindi, and Swahili, making it accessible across regions. The initiative is part of a broader plan to enhance voice technology for agricultural advisory. 
  4. Tech for Her: 
@@ -10789,7 +10789,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Uganda,Kenya,Nigeria</t>
+          <t>Uganda, Kenya, Nigeria</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>SDG 8 (Decent Work and Economic Growth), SDG 9 (Industry, Innovation and Infrastructure), SDG 10 (Reduced Inequalities; access to information in local languages).</t>
+          <t>SDG 10, SDG 9, SDG 8</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -11466,7 +11466,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Early stage, functional demo available.</t>
+          <t>Dataset &gt; Model &gt; Pilot</t>
         </is>
       </c>
       <c r="T89" t="inlineStr"/>
@@ -11509,32 +11509,125 @@
           <t>ui_89</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Digital Green - Local dataset collection for climate-smart agriculture</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Geospatial dataset of wheat and rice farmers in Bihar, India</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Data-driven decision-making for farmers to increase climate resilience in India</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Smallholder farmers are crucial contributors to global food production, and in India often suffer most from poverty and malnutrition. These farmers face challenges such as limited access to modern agriculture, unpredictable weather, and resource constraints. To tackle this issue, Digital Green collected data via surveys, offering insights into farming practices, environmental conditions, and crop yields.
+The project developed a scalable data collection model for JEEViKA’s frontline workers, integrating digital tools and geofencing, and empowered farmers with personalized climate-smart advice through Farmer Scorecards.
+The project has contributed to Digital Greens current FarmerChat.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/digitalgreenorg/frame-templates </t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://github.com/digitalgreenorg/frame-templates</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>SDG 2</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Tabular</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>The data was collected through a survey conducted across multiple districts in India. It consists of a variety of factors that could potentially impact the yield of rice crops. These factors include things like the type and amount of fertilizers used, the quantity of seedlings planted, methods of preparing the land, different irrigation techniques employed, among other features. The dataset comprises more than 5000 data points, each having more than 40 features.</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Multiple models are available based on the shared data. Please refer to the GitHub repository.</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The possibilities include creating a machine learning solution to predict the crop yield per acre of rice or wheat crops in India. Our goal is to empower these farmers and break the cycle of poverty and malnutrition.
+This use case also included the development of a business model and funding model for open source AI as a stepping stone towards financially viable operations. It was facilitated by Villgro Africa's and FAIR Forward's six-month mentorship programme on "Creating sustainable business and funding models with open source AI". See: https://www.bmz-digital.global/en/news/open-source-ai-business-impact/ </t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Digital Green
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and Sequoia Climate Fund, CISCO Foundation</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Philipp Olbrich</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Dataset  &gt; Model &gt; Pilot &gt; Use-Case &gt;  Use-Case with Business Model</t>
+        </is>
+      </c>
       <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr"/>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://digitalgreen.org/wp-content/uploads/2024/10/GIZ-FF_DG_Learning-Report.pdf </t>
+        </is>
+      </c>
       <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
-      <c r="Y90" t="inlineStr"/>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>In our monitoring, we assess as pilot rather for maturity - buth there was also business model built. therefore the entry here on maturity is including "use case"</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z90" t="inlineStr"/>
-      <c r="AA90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="AB90" t="inlineStr">
         <is>
           <t>89</t>
@@ -11563,14 +11656,26 @@
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
-      <c r="S91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr"/>
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr"/>
-      <c r="Y91" t="inlineStr"/>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr"/>
       <c r="AB91" t="inlineStr">
@@ -11601,14 +11706,26 @@
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr"/>
-      <c r="Y92" t="inlineStr"/>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z92" t="inlineStr"/>
       <c r="AA92" t="inlineStr"/>
       <c r="AB92" t="inlineStr">
@@ -11639,14 +11756,26 @@
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
-      <c r="S93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr"/>
-      <c r="Y93" t="inlineStr"/>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z93" t="inlineStr"/>
       <c r="AA93" t="inlineStr"/>
       <c r="AB93" t="inlineStr">
@@ -11677,14 +11806,26 @@
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
-      <c r="S94" t="inlineStr"/>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
       <c r="V94" t="inlineStr"/>
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr"/>
-      <c r="Y94" t="inlineStr"/>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Z94" t="inlineStr"/>
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-26 10:59:35 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -10629,12 +10629,12 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and planning forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and planning forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-26 10:59:35 UTC (#108)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -10629,12 +10629,12 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and planning forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and plannin forest restoration in Uganda through AI-powered Remote Sensing</t>
+          <t>Monitoring Deforestation, predicting Landuse and Landcover changes and planning forest restoration in Uganda through AI-powered Remote Sensing</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-26 11:06:30 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1267,13 +1267,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detectinging forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
+          <t xml:space="preserve">Detecting forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
 </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detectinging forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
+          <t xml:space="preserve">Detecting forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
 </t>
         </is>
       </c>
@@ -6564,12 +6564,12 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LivHealth Kiswahili Corpus</t>
+          <t>AI-powered livestock health system enabling local communities easy access to disease information on demand and in Kiswahili:LivHealth Kiswahili Corpus</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI-powered lifestock health system enabling local communities easy access to disease information on demand and in Kiswahili. </t>
+          <t xml:space="preserve">AI-powered livestock health system enabling local communities easy access to disease information on demand and in Kiswahili. </t>
         </is>
       </c>
       <c r="E49" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-26 11:06:30 UTC (#109)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1267,13 +1267,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detectinging forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
+          <t xml:space="preserve">Detecting forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
 </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detectinging forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
+          <t xml:space="preserve">Detecting forest degradation by predicting biomass in cocoa plantations in Cote d'Ivoire
 </t>
         </is>
       </c>
@@ -6564,12 +6564,12 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LivHealth Kiswahili Corpus</t>
+          <t>AI-powered livestock health system enabling local communities easy access to disease information on demand and in Kiswahili:LivHealth Kiswahili Corpus</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI-powered lifestock health system enabling local communities easy access to disease information on demand and in Kiswahili. </t>
+          <t xml:space="preserve">AI-powered livestock health system enabling local communities easy access to disease information on demand and in Kiswahili. </t>
         </is>
       </c>
       <c r="E49" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-29 08:45:33 UTC
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4762,7 +4762,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in), Dr. Philipp Olbrich (philipp.olbrich@giz.de)</t>
+          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -6909,7 +6909,9 @@
  3. Viamo and Partners: 
  This platform targets farmers in Kenya and Bihar, focusing on beans and wheat, respectively. Using IVR, SMS, and WhatsApp, the platform is built on a RAG pipeline powered by LLMs, with potential for intent and entity recognition. Machine translation and speech-enabled IVR support English, Hindi, and Swahili, making it accessible across regions. The initiative is part of a broader plan to enhance voice technology for agricultural advisory. 
  4. Tech for Her: 
- Tech for Her empowers women farmers in Bihar and Kenya, focusing on tomatoes and cattle. Accessible via IVR, WhatsApp, and a mobile app, the platform uses LLM-powered intent and entity recognition for personalized chatbot interactions and speech-enabled IVR for voice support. AI-based video generation further enhances engagement. Available in English, Hindi, and Swahili, it caters to the specific needs of women in agriculture.</t>
+ Tech for Her empowers women farmers in Bihar and Kenya, focusing on tomatoes and cattle. Accessible via IVR, WhatsApp, and a mobile app, the platform uses LLM-powered intent and entity recognition for personalized chatbot interactions and speech-enabled IVR for voice support. AI-based video generation further enhances engagement. Available in English, Hindi, and Swahili, it caters to the specific needs of women in agriculture.
+5. Opportunity International/Digifarm:
+WhatsApp based bot in Kenya that emerged out of a custom-built solution tested in Malawi.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6935,7 +6937,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners (https://viamo.io/contact/), Tech for Her (contact@agrevolution.in), DynAg, Digifarm, Opportunity International (info@oid.org)</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">

</xml_diff>

<commit_message>
Sheet update 2026-06-29 08:45:33 UTC (#111)
Co-authored-by: GitHub Actions (Sheet Update) <actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -4762,7 +4762,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in), Dr. Philipp Olbrich (philipp.olbrich@giz.de)</t>
+          <t>Dr. Prasanta Ghosh (prasantag@iisc.ac.in)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -6909,7 +6909,9 @@
  3. Viamo and Partners: 
  This platform targets farmers in Kenya and Bihar, focusing on beans and wheat, respectively. Using IVR, SMS, and WhatsApp, the platform is built on a RAG pipeline powered by LLMs, with potential for intent and entity recognition. Machine translation and speech-enabled IVR support English, Hindi, and Swahili, making it accessible across regions. The initiative is part of a broader plan to enhance voice technology for agricultural advisory. 
  4. Tech for Her: 
- Tech for Her empowers women farmers in Bihar and Kenya, focusing on tomatoes and cattle. Accessible via IVR, WhatsApp, and a mobile app, the platform uses LLM-powered intent and entity recognition for personalized chatbot interactions and speech-enabled IVR for voice support. AI-based video generation further enhances engagement. Available in English, Hindi, and Swahili, it caters to the specific needs of women in agriculture.</t>
+ Tech for Her empowers women farmers in Bihar and Kenya, focusing on tomatoes and cattle. Accessible via IVR, WhatsApp, and a mobile app, the platform uses LLM-powered intent and entity recognition for personalized chatbot interactions and speech-enabled IVR for voice support. AI-based video generation further enhances engagement. Available in English, Hindi, and Swahili, it caters to the specific needs of women in agriculture.
+5. Opportunity International/Digifarm:
+WhatsApp based bot in Kenya that emerged out of a custom-built solution tested in Malawi.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6935,7 +6937,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners, Tech for Her, DynAg, Digifarm, Opportunity International</t>
+          <t>Digital Green (info@digitalgreentrust.org), Viamo and Partners (https://viamo.io/contact/), Tech for Her (contact@agrevolution.in), DynAg, Digifarm, Opportunity International (info@oid.org)</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">

</xml_diff>